<commit_message>
🤖 Daily run: 2026-08-05 14:11
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -16,7 +16,7 @@
     <sheet name="Perfis" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$N$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$N$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Perfil'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Perfil'!$1:$1</definedName>
@@ -566,7 +566,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 04/08/2026 às 16:56</t>
+          <t>Gerado em 05/08/2026 às 14:06</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6">
@@ -693,7 +693,7 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19">
@@ -709,7 +709,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Engenheiro Dados</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="B20" s="6" t="n">
@@ -731,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -865,9 +865,7 @@
       <c r="J2" s="13" t="n">
         <v>46250</v>
       </c>
-      <c r="K2" s="14" t="n">
-        <v>150000</v>
-      </c>
+      <c r="K2" s="14" t="inlineStr"/>
       <c r="L2" s="15" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1210,7 +1208,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Engenheiro Dados</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="E8" s="12" t="n">
@@ -1543,9 +1541,7 @@
       <c r="J13" s="21" t="n">
         <v>46252</v>
       </c>
-      <c r="K13" s="22" t="n">
-        <v>58600</v>
-      </c>
+      <c r="K13" s="22" t="inlineStr"/>
       <c r="L13" s="23" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1738,27 +1734,29 @@
     </row>
     <row r="17">
       <c r="A17" s="17" t="n">
-        <v>146290</v>
+        <v>146288</v>
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>TR DPA/PNUD 001/2026 - Suporte técnico especializado para fortalecimento de Mecanismos Integrados de Atendimento à RIDEs e à Faixa de Fronteira.</t>
+          <t xml:space="preserve"> BRA23/004 - TR 004/2026 - Consultoria Nacional pessoa física para elaborar estudo sobre favelas e comunidades urbanas do município de Niterói</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="E17" s="20" t="inlineStr"/>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="n">
+        <v>0.3</v>
+      </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G17" s="18" t="inlineStr">
@@ -1768,17 +1766,17 @@
       </c>
       <c r="H17" s="18" t="inlineStr">
         <is>
-          <t>Brasília</t>
+          <t>Remoto com possibilidade de atividades presenciais</t>
         </is>
       </c>
       <c r="I17" s="21" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="J17" s="21" t="n">
-        <v>46248</v>
+        <v>46252</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>101000</v>
+        <v>86112</v>
       </c>
       <c r="L17" s="23" t="inlineStr">
         <is>
@@ -1787,7 +1785,7 @@
       </c>
       <c r="M17" s="19" t="inlineStr">
         <is>
-          <t>prodocbra23018@sudeco.gov.br</t>
+          <t>prodoc.ssagi@seplag.niteroi.rj.gov.br</t>
         </is>
       </c>
       <c r="N17" s="24" t="inlineStr">
@@ -1798,64 +1796,184 @@
     </row>
     <row r="18">
       <c r="A18" s="9" t="n">
+        <v>146289</v>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>BRA23/004 - TR 003/2026 - Contratação de Consultoria Nacional pessoa física para elaborar estudo sobre mulheres e desigualdade de gênero no município de Niterói</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Física (PF)</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>Remoto com possibilidade de atividades presenciais</t>
+        </is>
+      </c>
+      <c r="I18" s="13" t="n">
+        <v>46239</v>
+      </c>
+      <c r="J18" s="13" t="n">
+        <v>46252</v>
+      </c>
+      <c r="K18" s="14" t="n">
+        <v>74880</v>
+      </c>
+      <c r="L18" s="15" t="inlineStr">
+        <is>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="M18" s="11" t="inlineStr">
+        <is>
+          <t>prodoc.ssagi@seplag.niteroi.rj.gov.br</t>
+        </is>
+      </c>
+      <c r="N18" s="16" t="inlineStr">
+        <is>
+          <t>https://parceiros.undp.org.br/opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="n">
+        <v>146290</v>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>TR DPA/PNUD 001/2026 - Suporte técnico especializado para fortalecimento de Mecanismos Integrados de Atendimento à RIDEs e à Faixa de Fronteira.</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="inlineStr">
+        <is>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="E19" s="20" t="inlineStr"/>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>Não classificada</t>
+        </is>
+      </c>
+      <c r="G19" s="18" t="inlineStr">
+        <is>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="H19" s="18" t="inlineStr">
+        <is>
+          <t>Brasília</t>
+        </is>
+      </c>
+      <c r="I19" s="21" t="n">
+        <v>46238</v>
+      </c>
+      <c r="J19" s="21" t="n">
+        <v>46248</v>
+      </c>
+      <c r="K19" s="22" t="inlineStr"/>
+      <c r="L19" s="23" t="inlineStr">
+        <is>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="M19" s="19" t="inlineStr">
+        <is>
+          <t>prodocbra23018@sudeco.gov.br</t>
+        </is>
+      </c>
+      <c r="N19" s="24" t="inlineStr">
+        <is>
+          <t>https://parceiros.undp.org.br/opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="n">
         <v>146292</v>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>UNDP-BRA-01222 - IC - Consultoria Técnica Especializada em Planos Nacionais de Adaptação (COP 30)</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr">
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>Edital Genérico / IC</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>Não Classificado</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr"/>
-      <c r="F18" s="10" t="inlineStr">
+      <c r="E20" s="12" t="inlineStr"/>
+      <c r="F20" s="10" t="inlineStr">
         <is>
           <t>Não classificada</t>
         </is>
       </c>
-      <c r="G18" s="10" t="inlineStr">
+      <c r="G20" s="10" t="inlineStr">
         <is>
           <t>PNUD (Direto)</t>
         </is>
       </c>
-      <c r="H18" s="10" t="inlineStr">
+      <c r="H20" s="10" t="inlineStr">
         <is>
           <t>Trabalho remoto, com possibilidade de viagens</t>
         </is>
       </c>
-      <c r="I18" s="13" t="n">
+      <c r="I20" s="13" t="n">
         <v>46238</v>
       </c>
-      <c r="J18" s="13" t="n">
+      <c r="J20" s="13" t="n">
         <v>46247</v>
       </c>
-      <c r="K18" s="14" t="inlineStr"/>
-      <c r="L18" s="15" t="inlineStr">
+      <c r="K20" s="14" t="inlineStr"/>
+      <c r="L20" s="15" t="inlineStr">
         <is>
           <t>Aprovada</t>
         </is>
       </c>
-      <c r="M18" s="11" t="inlineStr">
+      <c r="M20" s="11" t="inlineStr">
         <is>
           <t>ic.procurement.br@undp.org</t>
         </is>
       </c>
-      <c r="N18" s="16" t="inlineStr">
+      <c r="N20" s="16" t="inlineStr">
         <is>
           <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N18"/>
+  <autoFilter ref="A1:N20"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
@@ -1874,6 +1992,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -1912,7 +2032,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -1928,7 +2048,7 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>Engenheiro Dados</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="B4" s="9" t="n">
@@ -1974,7 +2094,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
@@ -2046,7 +2166,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -2056,7 +2176,7 @@
         </is>
       </c>
       <c r="B3" s="17" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -2066,7 +2186,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -2082,17 +2202,17 @@
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>Economia / Finanças Públicas</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Economia / Finanças Públicas</t>
         </is>
       </c>
       <c r="B7" s="17" t="n">
@@ -2102,7 +2222,7 @@
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="B8" s="9" t="n">
@@ -2164,17 +2284,17 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>TCU</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="18" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>TCU</t>
         </is>
       </c>
       <c r="B5" s="17" t="n">
@@ -2226,7 +2346,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
@@ -2237,45 +2357,45 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Engenheiro Dados</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="B3" s="17" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C3" s="18" t="inlineStr">
         <is>
-          <t>Engenheiro de Dados (Eng. Química + Ciência da Computação), 5 anos em pipelines ETL, Spark/Databricks/Azure e web scraping</t>
+          <t>Analista de BI (Engenharia da Computação + Técnico em Computação), 5+ anos em Power BI/SQL, 3 anos com dados públicos, econômicos e sociais</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Pesquisador Computacao</t>
+          <t>Engenheiro Dados</t>
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>Pesquisador acadêmico com foco em computação, dados e metodologia científica</t>
+          <t>Engenheiro de Dados (Eng. Química + Ciência da Computação), 5 anos em pipelines ETL, Spark/Databricks/Azure e web scraping</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Pesquisador Computacao</t>
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>Analista de BI (Engenharia da Computação + Técnico em Computação), 5+ anos em Power BI/SQL, 3 anos com dados públicos, econômicos e sociais</t>
+          <t>Pesquisador acadêmico com foco em computação, dados e metodologia científica</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-08-06 14:11
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -16,7 +16,7 @@
     <sheet name="Perfis" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$N$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$N$22</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Perfil'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Perfil'!$1:$1</definedName>
@@ -566,7 +566,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 05/08/2026 às 14:06</t>
+          <t>Gerado em 06/08/2026 às 14:05</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6">
@@ -693,7 +693,7 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19">
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -731,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1775,9 +1775,7 @@
       <c r="J17" s="21" t="n">
         <v>46252</v>
       </c>
-      <c r="K17" s="22" t="n">
-        <v>86112</v>
-      </c>
+      <c r="K17" s="22" t="inlineStr"/>
       <c r="L17" s="23" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1837,9 +1835,7 @@
       <c r="J18" s="13" t="n">
         <v>46252</v>
       </c>
-      <c r="K18" s="14" t="n">
-        <v>74880</v>
-      </c>
+      <c r="K18" s="14" t="inlineStr"/>
       <c r="L18" s="15" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1972,8 +1968,128 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="17" t="n">
+        <v>146295</v>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>IC - UNDP-BRA-01224 - Consultoria (pessoa física) para planejamento estratégico de roteiro internacional de missões para  diálogos sobre segurança cibernética no judiciário</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Física (PF)</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="E21" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados</t>
+        </is>
+      </c>
+      <c r="G21" s="18" t="inlineStr">
+        <is>
+          <t>PNUD (Direto)</t>
+        </is>
+      </c>
+      <c r="H21" s="18" t="inlineStr">
+        <is>
+          <t>Remoto. (Notar: na data de término, o edital se encerra às 17h de Brasília)</t>
+        </is>
+      </c>
+      <c r="I21" s="21" t="n">
+        <v>46239</v>
+      </c>
+      <c r="J21" s="21" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K21" s="22" t="inlineStr"/>
+      <c r="L21" s="23" t="inlineStr">
+        <is>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="M21" s="19" t="inlineStr">
+        <is>
+          <t>ic.procurement.br@undp.org</t>
+        </is>
+      </c>
+      <c r="N21" s="24" t="inlineStr">
+        <is>
+          <t>https://parceiros.undp.org.br/opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="n">
+        <v>146296</v>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>IC - UNDP-BRA-01226 - Consultoria para avaliação final do Projeto BRA/20/019</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>Edital Genérico / IC</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>PNUD (Direto)</t>
+        </is>
+      </c>
+      <c r="H22" s="10" t="inlineStr">
+        <is>
+          <t>Remoto (notar: na data de término, a negociação se encerra às 17h)</t>
+        </is>
+      </c>
+      <c r="I22" s="13" t="n">
+        <v>46239</v>
+      </c>
+      <c r="J22" s="13" t="n">
+        <v>46253</v>
+      </c>
+      <c r="K22" s="14" t="inlineStr"/>
+      <c r="L22" s="15" t="inlineStr">
+        <is>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="M22" s="11" t="inlineStr">
+        <is>
+          <t>ic.procurement.br@undp.org</t>
+        </is>
+      </c>
+      <c r="N22" s="16" t="inlineStr">
+        <is>
+          <t>https://parceiros.undp.org.br/opportunities</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N20"/>
+  <autoFilter ref="A1:N22"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
@@ -1994,6 +2110,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -2032,7 +2150,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
@@ -2052,7 +2170,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2094,7 +2212,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -2104,7 +2222,7 @@
         </is>
       </c>
       <c r="B3" s="17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -2166,7 +2284,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -2186,7 +2304,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -2278,7 +2396,7 @@
         </is>
       </c>
       <c r="B3" s="17" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -2346,7 +2464,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
@@ -2361,7 +2479,7 @@
         </is>
       </c>
       <c r="B3" s="17" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C3" s="18" t="inlineStr">
         <is>
@@ -2376,7 +2494,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
@@ -2391,7 +2509,7 @@
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-08-07 13:05
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -566,7 +566,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 06/08/2026 às 14:05</t>
+          <t>Gerado em 07/08/2026 às 13:00</t>
         </is>
       </c>
     </row>
@@ -693,13 +693,13 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Engenheiro Dados</t>
         </is>
       </c>
       <c r="B19" s="6" t="n">
@@ -709,11 +709,11 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Engenheiro Dados</t>
         </is>
       </c>
       <c r="E8" s="12" t="n">
@@ -1318,11 +1318,11 @@
     </row>
     <row r="10">
       <c r="A10" s="9" t="n">
-        <v>146277</v>
+        <v>146279</v>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>IC - UNDP-BRA-01210 - Consultoria para análise de financiamento climático (COP30)</t>
+          <t>UNDP-BRA-01215 - IC - Consultoria para sistematização da atuação de grupos especiais da COP30</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
@@ -1350,14 +1350,14 @@
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>Trabalho remoto, com possibilidade de viagens</t>
+          <t>Brasília. (Notar: na data de término, o edital se encerra às 17h de Brasília)</t>
         </is>
       </c>
       <c r="I10" s="13" t="n">
-        <v>46230</v>
+        <v>46231</v>
       </c>
       <c r="J10" s="13" t="n">
-        <v>46240</v>
+        <v>46245</v>
       </c>
       <c r="K10" s="14" t="inlineStr"/>
       <c r="L10" s="15" t="inlineStr">
@@ -1378,16 +1378,16 @@
     </row>
     <row r="11">
       <c r="A11" s="17" t="n">
-        <v>146279</v>
+        <v>146268</v>
       </c>
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>UNDP-BRA-01215 - IC - Consultoria para sistematização da atuação de grupos especiais da COP30</t>
+          <t>PROJETO BRA 23/023 - TR 125/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA ELABORAÇÃO DE ESTUDO SOBRE OS IMPACTOS DA DIGITALIZAÇÃO DOCUMENTAL E DO ARMAZENAMENTO EM NUVEM.</t>
         </is>
       </c>
       <c r="C11" s="18" t="inlineStr">
         <is>
-          <t>Edital Genérico / IC</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1396,7 +1396,7 @@
         </is>
       </c>
       <c r="E11" s="20" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
@@ -1405,21 +1405,23 @@
       </c>
       <c r="G11" s="18" t="inlineStr">
         <is>
-          <t>PNUD (Direto)</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="H11" s="18" t="inlineStr">
         <is>
-          <t>Brasília. (Notar: na data de término, o edital se encerra às 17h de Brasília)</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="I11" s="21" t="n">
-        <v>46231</v>
+        <v>46237</v>
       </c>
       <c r="J11" s="21" t="n">
-        <v>46245</v>
-      </c>
-      <c r="K11" s="22" t="inlineStr"/>
+        <v>46252</v>
+      </c>
+      <c r="K11" s="22" t="n">
+        <v>53000</v>
+      </c>
       <c r="L11" s="23" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1427,7 +1429,7 @@
       </c>
       <c r="M11" s="19" t="inlineStr">
         <is>
-          <t>ic.procurement.br@undp.org</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="N11" s="24" t="inlineStr">
@@ -1438,16 +1440,16 @@
     </row>
     <row r="12">
       <c r="A12" s="9" t="n">
-        <v>146268</v>
+        <v>146280</v>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 125/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA ELABORAÇÃO DE ESTUDO SOBRE OS IMPACTOS DA DIGITALIZAÇÃO DOCUMENTAL E DO ARMAZENAMENTO EM NUVEM.</t>
+          <t>PROJETO BRA 23/023 - TR 86/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ELABORAÇÃO DA PROPOSTA DE CAPACITAÇÃO DO CENSO AGROPECUÁRIO NAS CADEIAS DE INFORMÁTICA E ADMINISTRATIVA.</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1456,11 +1458,11 @@
         </is>
       </c>
       <c r="E12" s="12" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
@@ -1479,9 +1481,7 @@
       <c r="J12" s="13" t="n">
         <v>46252</v>
       </c>
-      <c r="K12" s="14" t="n">
-        <v>53000</v>
-      </c>
+      <c r="K12" s="14" t="inlineStr"/>
       <c r="L12" s="15" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1500,16 +1500,16 @@
     </row>
     <row r="13">
       <c r="A13" s="17" t="n">
-        <v>146280</v>
+        <v>146281</v>
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 86/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ELABORAÇÃO DA PROPOSTA DE CAPACITAÇÃO DO CENSO AGROPECUÁRIO NAS CADEIAS DE INFORMÁTICA E ADMINISTRATIVA.</t>
+          <t>IC - UNDP-BRA-01217 - Consultoria pessoa física para implementação do Formulário Nacional de Avaliação de Risco (FONAR) e do Formulário Rogéria</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1522,24 +1522,20 @@
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G13" s="18" t="inlineStr">
         <is>
-          <t>IBGE</t>
-        </is>
-      </c>
-      <c r="H13" s="18" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>PNUD (Direto)</t>
+        </is>
+      </c>
+      <c r="H13" s="18" t="inlineStr"/>
       <c r="I13" s="21" t="n">
-        <v>46237</v>
+        <v>46232</v>
       </c>
       <c r="J13" s="21" t="n">
-        <v>46252</v>
+        <v>46245</v>
       </c>
       <c r="K13" s="22" t="inlineStr"/>
       <c r="L13" s="23" t="inlineStr">
@@ -1549,7 +1545,7 @@
       </c>
       <c r="M13" s="19" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>ic.procurement.br@undp.org</t>
         </is>
       </c>
       <c r="N13" s="24" t="inlineStr">
@@ -1560,11 +1556,11 @@
     </row>
     <row r="14">
       <c r="A14" s="9" t="n">
-        <v>146281</v>
+        <v>146282</v>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>IC - UNDP-BRA-01217 - Consultoria pessoa física para implementação do Formulário Nacional de Avaliação de Risco (FONAR) e do Formulário Rogéria</t>
+          <t>IC - UNDP-BRA-01218 - Consultoria pessoa física para implementação do Formulário Nacional de Avaliação de Risco (FONAR) e do Formulário Rogéria em João Pessoa</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
@@ -1590,7 +1586,11 @@
           <t>PNUD (Direto)</t>
         </is>
       </c>
-      <c r="H14" s="10" t="inlineStr"/>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>João Pessoa. (Notar: na data de término, o edital se encerra às 17h de Brasília)</t>
+        </is>
+      </c>
       <c r="I14" s="13" t="n">
         <v>46232</v>
       </c>
@@ -1616,29 +1616,27 @@
     </row>
     <row r="15">
       <c r="A15" s="17" t="n">
-        <v>146282</v>
+        <v>146287</v>
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>IC - UNDP-BRA-01218 - Consultoria pessoa física para implementação do Formulário Nacional de Avaliação de Risco (FONAR) e do Formulário Rogéria em João Pessoa</t>
+          <t>IC - UNDP-BRA-01223 - Consultoria especializada em recrutamento e seleção</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Economista</t>
-        </is>
-      </c>
-      <c r="E15" s="20" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="E15" s="20" t="inlineStr"/>
       <c r="F15" s="18" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="G15" s="18" t="inlineStr">
@@ -1648,14 +1646,14 @@
       </c>
       <c r="H15" s="18" t="inlineStr">
         <is>
-          <t>João Pessoa. (Notar: na data de término, o edital se encerra às 17h de Brasília)</t>
+          <t>Remoto. (Notar: na data de término, o edital se encerra às 17h de Brasília)</t>
         </is>
       </c>
       <c r="I15" s="21" t="n">
-        <v>46232</v>
+        <v>46234</v>
       </c>
       <c r="J15" s="21" t="n">
-        <v>46245</v>
+        <v>46248</v>
       </c>
       <c r="K15" s="22" t="inlineStr"/>
       <c r="L15" s="23" t="inlineStr">
@@ -1676,44 +1674,46 @@
     </row>
     <row r="16">
       <c r="A16" s="9" t="n">
-        <v>146287</v>
+        <v>146288</v>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>IC - UNDP-BRA-01223 - Consultoria especializada em recrutamento e seleção</t>
+          <t xml:space="preserve"> BRA23/004 - TR 004/2026 - Consultoria Nacional pessoa física para elaborar estudo sobre favelas e comunidades urbanas do município de Niterói</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="E16" s="12" t="inlineStr"/>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="n">
+        <v>0.3</v>
+      </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>PNUD (Direto)</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>Remoto. (Notar: na data de término, o edital se encerra às 17h de Brasília)</t>
+          <t>Remoto com possibilidade de atividades presenciais</t>
         </is>
       </c>
       <c r="I16" s="13" t="n">
-        <v>46234</v>
+        <v>46239</v>
       </c>
       <c r="J16" s="13" t="n">
-        <v>46248</v>
+        <v>46252</v>
       </c>
       <c r="K16" s="14" t="inlineStr"/>
       <c r="L16" s="15" t="inlineStr">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="M16" s="11" t="inlineStr">
         <is>
-          <t>ic.procurement.br@undp.org</t>
+          <t>prodoc.ssagi@seplag.niteroi.rj.gov.br</t>
         </is>
       </c>
       <c r="N16" s="16" t="inlineStr">
@@ -1734,11 +1734,11 @@
     </row>
     <row r="17">
       <c r="A17" s="17" t="n">
-        <v>146288</v>
+        <v>146289</v>
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> BRA23/004 - TR 004/2026 - Consultoria Nacional pessoa física para elaborar estudo sobre favelas e comunidades urbanas do município de Niterói</t>
+          <t>BRA23/004 - TR 003/2026 - Contratação de Consultoria Nacional pessoa física para elaborar estudo sobre mulheres e desigualdade de gênero no município de Niterói</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
@@ -1756,7 +1756,7 @@
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G17" s="18" t="inlineStr">
@@ -1794,29 +1794,27 @@
     </row>
     <row r="18">
       <c r="A18" s="9" t="n">
-        <v>146289</v>
+        <v>146290</v>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>BRA23/004 - TR 003/2026 - Contratação de Consultoria Nacional pessoa física para elaborar estudo sobre mulheres e desigualdade de gênero no município de Niterói</t>
+          <t>TR DPA/PNUD 001/2026 - Suporte técnico especializado para fortalecimento de Mecanismos Integrados de Atendimento à RIDEs e à Faixa de Fronteira.</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Economista</t>
-        </is>
-      </c>
-      <c r="E18" s="12" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr"/>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
@@ -1826,14 +1824,14 @@
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>Remoto com possibilidade de atividades presenciais</t>
+          <t>Brasília</t>
         </is>
       </c>
       <c r="I18" s="13" t="n">
-        <v>46239</v>
+        <v>46238</v>
       </c>
       <c r="J18" s="13" t="n">
-        <v>46252</v>
+        <v>46248</v>
       </c>
       <c r="K18" s="14" t="inlineStr"/>
       <c r="L18" s="15" t="inlineStr">
@@ -1843,7 +1841,7 @@
       </c>
       <c r="M18" s="11" t="inlineStr">
         <is>
-          <t>prodoc.ssagi@seplag.niteroi.rj.gov.br</t>
+          <t>prodocbra23018@sudeco.gov.br</t>
         </is>
       </c>
       <c r="N18" s="16" t="inlineStr">
@@ -1854,16 +1852,16 @@
     </row>
     <row r="19">
       <c r="A19" s="17" t="n">
-        <v>146290</v>
+        <v>146292</v>
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>TR DPA/PNUD 001/2026 - Suporte técnico especializado para fortalecimento de Mecanismos Integrados de Atendimento à RIDEs e à Faixa de Fronteira.</t>
+          <t>UNDP-BRA-01222 - IC - Consultoria Técnica Especializada em Planos Nacionais de Adaptação (COP 30)</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Edital Genérico / IC</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -1879,19 +1877,19 @@
       </c>
       <c r="G19" s="18" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>PNUD (Direto)</t>
         </is>
       </c>
       <c r="H19" s="18" t="inlineStr">
         <is>
-          <t>Brasília</t>
+          <t>Trabalho remoto, com possibilidade de viagens</t>
         </is>
       </c>
       <c r="I19" s="21" t="n">
         <v>46238</v>
       </c>
       <c r="J19" s="21" t="n">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="K19" s="22" t="inlineStr"/>
       <c r="L19" s="23" t="inlineStr">
@@ -1901,7 +1899,7 @@
       </c>
       <c r="M19" s="19" t="inlineStr">
         <is>
-          <t>prodocbra23018@sudeco.gov.br</t>
+          <t>ic.procurement.br@undp.org</t>
         </is>
       </c>
       <c r="N19" s="24" t="inlineStr">
@@ -1912,27 +1910,29 @@
     </row>
     <row r="20">
       <c r="A20" s="9" t="n">
-        <v>146292</v>
+        <v>146295</v>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>UNDP-BRA-01222 - IC - Consultoria Técnica Especializada em Planos Nacionais de Adaptação (COP 30)</t>
+          <t>IC - UNDP-BRA-01224 - Consultoria (pessoa física) para planejamento estratégico de roteiro internacional de missões para  diálogos sobre segurança cibernética no judiciário</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Edital Genérico / IC</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="E20" s="12" t="inlineStr"/>
+          <t>Engenheiro Dados</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="n">
+        <v>0.3</v>
+      </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
@@ -1942,14 +1942,14 @@
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>Trabalho remoto, com possibilidade de viagens</t>
+          <t>Remoto. (Notar: na data de término, o edital se encerra às 17h de Brasília)</t>
         </is>
       </c>
       <c r="I20" s="13" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="J20" s="13" t="n">
-        <v>46247</v>
+        <v>46253</v>
       </c>
       <c r="K20" s="14" t="inlineStr"/>
       <c r="L20" s="15" t="inlineStr">
@@ -1970,21 +1970,21 @@
     </row>
     <row r="21">
       <c r="A21" s="17" t="n">
-        <v>146295</v>
+        <v>146296</v>
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>IC - UNDP-BRA-01224 - Consultoria (pessoa física) para planejamento estratégico de roteiro internacional de missões para  diálogos sobre segurança cibernética no judiciário</t>
+          <t>IC - UNDP-BRA-01226 - Consultoria para avaliação final do Projeto BRA/20/019</t>
         </is>
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Edital Genérico / IC</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="E21" s="20" t="n">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="F21" s="18" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G21" s="18" t="inlineStr">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="H21" s="18" t="inlineStr">
         <is>
-          <t>Remoto. (Notar: na data de término, o edital se encerra às 17h de Brasília)</t>
+          <t>Remoto (notar: na data de término, a negociação se encerra às 17h)</t>
         </is>
       </c>
       <c r="I21" s="21" t="n">
@@ -2030,21 +2030,21 @@
     </row>
     <row r="22">
       <c r="A22" s="9" t="n">
-        <v>146296</v>
+        <v>146301</v>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>IC - UNDP-BRA-01226 - Consultoria para avaliação final do Projeto BRA/20/019</t>
+          <t>Edital 01/2026 - Relatório ao Protocolo Adicional à Convenção Americana sobre Direitos Humanos em matéria de Direitos Econômicos, Sociais e Culturais – San Salvador</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>Edital Genérico / IC</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Engenheiro Dados</t>
         </is>
       </c>
       <c r="E22" s="12" t="n">
@@ -2052,26 +2052,28 @@
       </c>
       <c r="F22" s="10" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
-          <t>PNUD (Direto)</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t>Remoto (notar: na data de término, a negociação se encerra às 17h)</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="I22" s="13" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="J22" s="13" t="n">
-        <v>46253</v>
-      </c>
-      <c r="K22" s="14" t="inlineStr"/>
+        <v>46244</v>
+      </c>
+      <c r="K22" s="14" t="n">
+        <v>53000</v>
+      </c>
       <c r="L22" s="15" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -2079,7 +2081,7 @@
       </c>
       <c r="M22" s="11" t="inlineStr">
         <is>
-          <t>ic.procurement.br@undp.org</t>
+          <t>cgsimore@mdh.gov.br</t>
         </is>
       </c>
       <c r="N22" s="16" t="inlineStr">
@@ -2150,13 +2152,13 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="18" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Engenheiro Dados</t>
         </is>
       </c>
       <c r="B3" s="17" t="n">
@@ -2166,11 +2168,11 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -2212,7 +2214,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -2222,7 +2224,7 @@
         </is>
       </c>
       <c r="B3" s="17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -2284,7 +2286,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
@@ -2294,7 +2296,7 @@
         </is>
       </c>
       <c r="B3" s="17" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -2320,17 +2322,17 @@
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Economia / Finanças Públicas</t>
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>Economia / Finanças Públicas</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="B7" s="17" t="n">
@@ -2340,7 +2342,7 @@
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="B8" s="9" t="n">
@@ -2396,7 +2398,7 @@
         </is>
       </c>
       <c r="B3" s="17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -2406,7 +2408,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -2464,7 +2466,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
@@ -2475,7 +2477,7 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Engenheiro Dados</t>
         </is>
       </c>
       <c r="B3" s="17" t="n">
@@ -2483,37 +2485,37 @@
       </c>
       <c r="C3" s="18" t="inlineStr">
         <is>
-          <t>Analista de BI (Engenharia da Computação + Técnico em Computação), 5+ anos em Power BI/SQL, 3 anos com dados públicos, econômicos e sociais</t>
+          <t>Engenheiro de Dados (Eng. Química + Ciência da Computação), 5 anos em pipelines ETL, Spark/Databricks/Azure e web scraping</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Engenheiro Dados</t>
+          <t>Pesquisador Computacao</t>
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>Engenheiro de Dados (Eng. Química + Ciência da Computação), 5 anos em pipelines ETL, Spark/Databricks/Azure e web scraping</t>
+          <t>Pesquisador acadêmico com foco em computação, dados e metodologia científica</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Pesquisador Computacao</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>Pesquisador acadêmico com foco em computação, dados e metodologia científica</t>
+          <t>Analista de BI (Engenharia da Computação + Técnico em Computação), 5+ anos em Power BI/SQL, 3 anos com dados públicos, econômicos e sociais</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-08-12 13:12
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -16,7 +16,7 @@
     <sheet name="Perfis" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$N$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$N$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Perfil'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Perfil'!$1:$1</definedName>
@@ -566,7 +566,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 07/08/2026 às 13:00</t>
+          <t>Gerado em 12/08/2026 às 13:06</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6">
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>53000</v>
+        <v>80.64</v>
       </c>
     </row>
     <row r="13">
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>62287.5</v>
+        <v>55375.62666666667</v>
       </c>
     </row>
     <row r="15">
@@ -693,27 +693,27 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Engenheiro Dados</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -731,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Engenheiro Dados</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="E8" s="12" t="n">
@@ -1318,16 +1318,16 @@
     </row>
     <row r="10">
       <c r="A10" s="9" t="n">
-        <v>146279</v>
+        <v>146268</v>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>UNDP-BRA-01215 - IC - Consultoria para sistematização da atuação de grupos especiais da COP30</t>
+          <t>PROJETO BRA 23/023 - TR 125/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA ELABORAÇÃO DE ESTUDO SOBRE OS IMPACTOS DA DIGITALIZAÇÃO DOCUMENTAL E DO ARMAZENAMENTO EM NUVEM.</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>Edital Genérico / IC</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1336,7 +1336,7 @@
         </is>
       </c>
       <c r="E10" s="12" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="F10" s="10" t="inlineStr">
         <is>
@@ -1345,21 +1345,23 @@
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>PNUD (Direto)</t>
+          <t>IBGE</t>
         </is>
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>Brasília. (Notar: na data de término, o edital se encerra às 17h de Brasília)</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="I10" s="13" t="n">
-        <v>46231</v>
+        <v>46237</v>
       </c>
       <c r="J10" s="13" t="n">
-        <v>46245</v>
-      </c>
-      <c r="K10" s="14" t="inlineStr"/>
+        <v>46252</v>
+      </c>
+      <c r="K10" s="14" t="n">
+        <v>53000</v>
+      </c>
       <c r="L10" s="15" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1367,7 +1369,7 @@
       </c>
       <c r="M10" s="11" t="inlineStr">
         <is>
-          <t>ic.procurement.br@undp.org</t>
+          <t>projetos.especiais@ibge.gov.br</t>
         </is>
       </c>
       <c r="N10" s="16" t="inlineStr">
@@ -1378,16 +1380,16 @@
     </row>
     <row r="11">
       <c r="A11" s="17" t="n">
-        <v>146268</v>
+        <v>146280</v>
       </c>
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 125/2026 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA (PESSOA FÍSICA) PARA ELABORAÇÃO DE ESTUDO SOBRE OS IMPACTOS DA DIGITALIZAÇÃO DOCUMENTAL E DO ARMAZENAMENTO EM NUVEM.</t>
+          <t>PROJETO BRA 23/023 - TR 86/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ELABORAÇÃO DA PROPOSTA DE CAPACITAÇÃO DO CENSO AGROPECUÁRIO NAS CADEIAS DE INFORMÁTICA E ADMINISTRATIVA.</t>
         </is>
       </c>
       <c r="C11" s="18" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1396,11 +1398,11 @@
         </is>
       </c>
       <c r="E11" s="20" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G11" s="18" t="inlineStr">
@@ -1419,9 +1421,7 @@
       <c r="J11" s="21" t="n">
         <v>46252</v>
       </c>
-      <c r="K11" s="22" t="n">
-        <v>53000</v>
-      </c>
+      <c r="K11" s="22" t="inlineStr"/>
       <c r="L11" s="23" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1440,11 +1440,11 @@
     </row>
     <row r="12">
       <c r="A12" s="9" t="n">
-        <v>146280</v>
+        <v>146287</v>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>PROJETO BRA 23/023 - TR 86/26 - CONTRATAÇÃO DE CONSULTORIA ESPECIALIZADA PARA ELABORAÇÃO DA PROPOSTA DE CAPACITAÇÃO DO CENSO AGROPECUÁRIO NAS CADEIAS DE INFORMÁTICA E ADMINISTRATIVA.</t>
+          <t>IC - UNDP-BRA-01223 - Consultoria especializada em recrutamento e seleção</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
@@ -1454,32 +1454,30 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Economista</t>
-        </is>
-      </c>
-      <c r="E12" s="12" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr"/>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>IBGE</t>
+          <t>PNUD (Direto)</t>
         </is>
       </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Remoto. (Notar: na data de término, o edital se encerra às 17h de Brasília)</t>
         </is>
       </c>
       <c r="I12" s="13" t="n">
-        <v>46237</v>
+        <v>46234</v>
       </c>
       <c r="J12" s="13" t="n">
-        <v>46252</v>
+        <v>46248</v>
       </c>
       <c r="K12" s="14" t="inlineStr"/>
       <c r="L12" s="15" t="inlineStr">
@@ -1489,7 +1487,7 @@
       </c>
       <c r="M12" s="11" t="inlineStr">
         <is>
-          <t>projetos.especiais@ibge.gov.br</t>
+          <t>ic.procurement.br@undp.org</t>
         </is>
       </c>
       <c r="N12" s="16" t="inlineStr">
@@ -1500,11 +1498,11 @@
     </row>
     <row r="13">
       <c r="A13" s="17" t="n">
-        <v>146281</v>
+        <v>146288</v>
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>IC - UNDP-BRA-01217 - Consultoria pessoa física para implementação do Formulário Nacional de Avaliação de Risco (FONAR) e do Formulário Rogéria</t>
+          <t xml:space="preserve"> BRA23/004 - TR 004/2026 - Consultoria Nacional pessoa física para elaborar estudo sobre favelas e comunidades urbanas do município de Niterói</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
@@ -1522,20 +1520,24 @@
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G13" s="18" t="inlineStr">
         <is>
-          <t>PNUD (Direto)</t>
-        </is>
-      </c>
-      <c r="H13" s="18" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="H13" s="18" t="inlineStr">
+        <is>
+          <t>Remoto com possibilidade de atividades presenciais</t>
+        </is>
+      </c>
       <c r="I13" s="21" t="n">
-        <v>46232</v>
+        <v>46239</v>
       </c>
       <c r="J13" s="21" t="n">
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="K13" s="22" t="inlineStr"/>
       <c r="L13" s="23" t="inlineStr">
@@ -1545,7 +1547,7 @@
       </c>
       <c r="M13" s="19" t="inlineStr">
         <is>
-          <t>ic.procurement.br@undp.org</t>
+          <t>prodoc.ssagi@seplag.niteroi.rj.gov.br</t>
         </is>
       </c>
       <c r="N13" s="24" t="inlineStr">
@@ -1556,11 +1558,11 @@
     </row>
     <row r="14">
       <c r="A14" s="9" t="n">
-        <v>146282</v>
+        <v>146289</v>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>IC - UNDP-BRA-01218 - Consultoria pessoa física para implementação do Formulário Nacional de Avaliação de Risco (FONAR) e do Formulário Rogéria em João Pessoa</t>
+          <t>BRA23/004 - TR 003/2026 - Contratação de Consultoria Nacional pessoa física para elaborar estudo sobre mulheres e desigualdade de gênero no município de Niterói</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
@@ -1578,24 +1580,24 @@
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>PNUD (Direto)</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t>João Pessoa. (Notar: na data de término, o edital se encerra às 17h de Brasília)</t>
+          <t>Remoto com possibilidade de atividades presenciais</t>
         </is>
       </c>
       <c r="I14" s="13" t="n">
-        <v>46232</v>
+        <v>46239</v>
       </c>
       <c r="J14" s="13" t="n">
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="K14" s="14" t="inlineStr"/>
       <c r="L14" s="15" t="inlineStr">
@@ -1605,7 +1607,7 @@
       </c>
       <c r="M14" s="11" t="inlineStr">
         <is>
-          <t>ic.procurement.br@undp.org</t>
+          <t>prodoc.ssagi@seplag.niteroi.rj.gov.br</t>
         </is>
       </c>
       <c r="N14" s="16" t="inlineStr">
@@ -1616,16 +1618,16 @@
     </row>
     <row r="15">
       <c r="A15" s="17" t="n">
-        <v>146287</v>
+        <v>146290</v>
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>IC - UNDP-BRA-01223 - Consultoria especializada em recrutamento e seleção</t>
+          <t>TR DPA/PNUD 001/2026 - Suporte técnico especializado para fortalecimento de Mecanismos Integrados de Atendimento à RIDEs e à Faixa de Fronteira.</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1641,16 +1643,16 @@
       </c>
       <c r="G15" s="18" t="inlineStr">
         <is>
-          <t>PNUD (Direto)</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="H15" s="18" t="inlineStr">
         <is>
-          <t>Remoto. (Notar: na data de término, o edital se encerra às 17h de Brasília)</t>
+          <t>Brasília</t>
         </is>
       </c>
       <c r="I15" s="21" t="n">
-        <v>46234</v>
+        <v>46238</v>
       </c>
       <c r="J15" s="21" t="n">
         <v>46248</v>
@@ -1663,7 +1665,7 @@
       </c>
       <c r="M15" s="19" t="inlineStr">
         <is>
-          <t>ic.procurement.br@undp.org</t>
+          <t>prodocbra23018@sudeco.gov.br</t>
         </is>
       </c>
       <c r="N15" s="24" t="inlineStr">
@@ -1674,46 +1676,44 @@
     </row>
     <row r="16">
       <c r="A16" s="9" t="n">
-        <v>146288</v>
+        <v>146292</v>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> BRA23/004 - TR 004/2026 - Consultoria Nacional pessoa física para elaborar estudo sobre favelas e comunidades urbanas do município de Niterói</t>
+          <t>UNDP-BRA-01222 - IC - Consultoria Técnica Especializada em Planos Nacionais de Adaptação (COP 30)</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Edital Genérico / IC</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Economista</t>
-        </is>
-      </c>
-      <c r="E16" s="12" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr"/>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>PNUD (Direto)</t>
         </is>
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>Remoto com possibilidade de atividades presenciais</t>
+          <t>Trabalho remoto, com possibilidade de viagens</t>
         </is>
       </c>
       <c r="I16" s="13" t="n">
-        <v>46239</v>
+        <v>46238</v>
       </c>
       <c r="J16" s="13" t="n">
-        <v>46252</v>
+        <v>46247</v>
       </c>
       <c r="K16" s="14" t="inlineStr"/>
       <c r="L16" s="15" t="inlineStr">
@@ -1723,7 +1723,7 @@
       </c>
       <c r="M16" s="11" t="inlineStr">
         <is>
-          <t>prodoc.ssagi@seplag.niteroi.rj.gov.br</t>
+          <t>ic.procurement.br@undp.org</t>
         </is>
       </c>
       <c r="N16" s="16" t="inlineStr">
@@ -1734,16 +1734,16 @@
     </row>
     <row r="17">
       <c r="A17" s="17" t="n">
-        <v>146289</v>
+        <v>146294</v>
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>BRA23/004 - TR 003/2026 - Contratação de Consultoria Nacional pessoa física para elaborar estudo sobre mulheres e desigualdade de gênero no município de Niterói</t>
+          <t>Contratação de consultoria técnica especializada para elaboração e desenvolvimento de solução educacional voltada à formação de lideranças em todos os níveis organizacionais do Conselho Administrativo de Defesa Econômica (Cade), mediante a produção de cursos customizados e objetos de aprendizagem digitais alinhados aos objetivos estratégicos, à missão, à visão e aos valores da Autarquia.</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1756,7 +1756,7 @@
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G17" s="18" t="inlineStr">
@@ -1766,16 +1766,18 @@
       </c>
       <c r="H17" s="18" t="inlineStr">
         <is>
-          <t>Remoto com possibilidade de atividades presenciais</t>
+          <t xml:space="preserve"> Remoto</t>
         </is>
       </c>
       <c r="I17" s="21" t="n">
-        <v>46239</v>
+        <v>46245</v>
       </c>
       <c r="J17" s="21" t="n">
-        <v>46252</v>
-      </c>
-      <c r="K17" s="22" t="inlineStr"/>
+        <v>46251</v>
+      </c>
+      <c r="K17" s="22" t="n">
+        <v>80640</v>
+      </c>
       <c r="L17" s="23" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1783,7 +1785,7 @@
       </c>
       <c r="M17" s="19" t="inlineStr">
         <is>
-          <t>prodoc.ssagi@seplag.niteroi.rj.gov.br</t>
+          <t>prodoc@cade.gov.br</t>
         </is>
       </c>
       <c r="N17" s="24" t="inlineStr">
@@ -1794,44 +1796,46 @@
     </row>
     <row r="18">
       <c r="A18" s="9" t="n">
-        <v>146290</v>
+        <v>146295</v>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>TR DPA/PNUD 001/2026 - Suporte técnico especializado para fortalecimento de Mecanismos Integrados de Atendimento à RIDEs e à Faixa de Fronteira.</t>
+          <t>IC - UNDP-BRA-01224 - Consultoria (pessoa física) para planejamento estratégico de roteiro internacional de missões para  diálogos sobre segurança cibernética no judiciário</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="E18" s="12" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="n">
+        <v>0.3</v>
+      </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>PNUD (Direto)</t>
         </is>
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>Brasília</t>
+          <t>Remoto. (Notar: na data de término, o edital se encerra às 17h de Brasília)</t>
         </is>
       </c>
       <c r="I18" s="13" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="J18" s="13" t="n">
-        <v>46248</v>
+        <v>46253</v>
       </c>
       <c r="K18" s="14" t="inlineStr"/>
       <c r="L18" s="15" t="inlineStr">
@@ -1841,7 +1845,7 @@
       </c>
       <c r="M18" s="11" t="inlineStr">
         <is>
-          <t>prodocbra23018@sudeco.gov.br</t>
+          <t>ic.procurement.br@undp.org</t>
         </is>
       </c>
       <c r="N18" s="16" t="inlineStr">
@@ -1852,11 +1856,11 @@
     </row>
     <row r="19">
       <c r="A19" s="17" t="n">
-        <v>146292</v>
+        <v>146296</v>
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>UNDP-BRA-01222 - IC - Consultoria Técnica Especializada em Planos Nacionais de Adaptação (COP 30)</t>
+          <t>IC - UNDP-BRA-01226 - Consultoria para avaliação final do Projeto BRA/20/019</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
@@ -1866,13 +1870,15 @@
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="E19" s="20" t="inlineStr"/>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="E19" s="20" t="n">
+        <v>0.3</v>
+      </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G19" s="18" t="inlineStr">
@@ -1882,14 +1888,14 @@
       </c>
       <c r="H19" s="18" t="inlineStr">
         <is>
-          <t>Trabalho remoto, com possibilidade de viagens</t>
+          <t>Remoto (notar: na data de término, a negociação se encerra às 17h)</t>
         </is>
       </c>
       <c r="I19" s="21" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="J19" s="21" t="n">
-        <v>46247</v>
+        <v>46253</v>
       </c>
       <c r="K19" s="22" t="inlineStr"/>
       <c r="L19" s="23" t="inlineStr">
@@ -1910,48 +1916,48 @@
     </row>
     <row r="20">
       <c r="A20" s="9" t="n">
-        <v>146295</v>
+        <v>146303</v>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>IC - UNDP-BRA-01224 - Consultoria (pessoa física) para planejamento estratégico de roteiro internacional de missões para  diálogos sobre segurança cibernética no judiciário</t>
+          <t>Consultoria técnica especializada para estruturação, validação e implantação assistida do Processo Institucional de Due Diligence de Integridade da Secretaria do Tesouro Nacional</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Engenheiro Dados</t>
-        </is>
-      </c>
-      <c r="E20" s="12" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr"/>
       <c r="F20" s="10" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>PNUD (Direto)</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>Remoto. (Notar: na data de término, o edital se encerra às 17h de Brasília)</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="I20" s="13" t="n">
-        <v>46239</v>
+        <v>46246</v>
       </c>
       <c r="J20" s="13" t="n">
-        <v>46253</v>
-      </c>
-      <c r="K20" s="14" t="inlineStr"/>
+        <v>46257</v>
+      </c>
+      <c r="K20" s="14" t="n">
+        <v>110707.2</v>
+      </c>
       <c r="L20" s="15" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1959,7 +1965,7 @@
       </c>
       <c r="M20" s="11" t="inlineStr">
         <is>
-          <t>ic.procurement.br@undp.org</t>
+          <t>ucp.codin.df.stn@tesouro.gov.br</t>
         </is>
       </c>
       <c r="N20" s="16" t="inlineStr">
@@ -1968,130 +1974,8 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="17" t="n">
-        <v>146296</v>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>IC - UNDP-BRA-01226 - Consultoria para avaliação final do Projeto BRA/20/019</t>
-        </is>
-      </c>
-      <c r="C21" s="18" t="inlineStr">
-        <is>
-          <t>Edital Genérico / IC</t>
-        </is>
-      </c>
-      <c r="D21" s="19" t="inlineStr">
-        <is>
-          <t>Economista</t>
-        </is>
-      </c>
-      <c r="E21" s="20" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F21" s="18" t="inlineStr">
-        <is>
-          <t>Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="G21" s="18" t="inlineStr">
-        <is>
-          <t>PNUD (Direto)</t>
-        </is>
-      </c>
-      <c r="H21" s="18" t="inlineStr">
-        <is>
-          <t>Remoto (notar: na data de término, a negociação se encerra às 17h)</t>
-        </is>
-      </c>
-      <c r="I21" s="21" t="n">
-        <v>46239</v>
-      </c>
-      <c r="J21" s="21" t="n">
-        <v>46253</v>
-      </c>
-      <c r="K21" s="22" t="inlineStr"/>
-      <c r="L21" s="23" t="inlineStr">
-        <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="M21" s="19" t="inlineStr">
-        <is>
-          <t>ic.procurement.br@undp.org</t>
-        </is>
-      </c>
-      <c r="N21" s="24" t="inlineStr">
-        <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="n">
-        <v>146301</v>
-      </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>Edital 01/2026 - Relatório ao Protocolo Adicional à Convenção Americana sobre Direitos Humanos em matéria de Direitos Econômicos, Sociais e Culturais – San Salvador</t>
-        </is>
-      </c>
-      <c r="C22" s="10" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Física (PF)</t>
-        </is>
-      </c>
-      <c r="D22" s="11" t="inlineStr">
-        <is>
-          <t>Engenheiro Dados</t>
-        </is>
-      </c>
-      <c r="E22" s="12" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F22" s="10" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados</t>
-        </is>
-      </c>
-      <c r="G22" s="10" t="inlineStr">
-        <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="H22" s="10" t="inlineStr">
-        <is>
-          <t>Território Nacional</t>
-        </is>
-      </c>
-      <c r="I22" s="13" t="n">
-        <v>46240</v>
-      </c>
-      <c r="J22" s="13" t="n">
-        <v>46244</v>
-      </c>
-      <c r="K22" s="14" t="n">
-        <v>53000</v>
-      </c>
-      <c r="L22" s="15" t="inlineStr">
-        <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="M22" s="11" t="inlineStr">
-        <is>
-          <t>cgsimore@mdh.gov.br</t>
-        </is>
-      </c>
-      <c r="N22" s="16" t="inlineStr">
-        <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N22"/>
+  <autoFilter ref="A1:N20"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
@@ -2112,8 +1996,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -2152,27 +2034,27 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="18" t="inlineStr">
         <is>
-          <t>Engenheiro Dados</t>
+          <t>Não Classificado</t>
         </is>
       </c>
       <c r="B3" s="17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2214,13 +2096,13 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="18" t="inlineStr">
         <is>
-          <t>Edital Genérico / IC</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="B3" s="17" t="n">
@@ -2240,11 +2122,11 @@
     <row r="5">
       <c r="A5" s="18" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Edital Genérico / IC</t>
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2286,7 +2168,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
@@ -2296,7 +2178,7 @@
         </is>
       </c>
       <c r="B3" s="17" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -2306,7 +2188,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -2316,7 +2198,7 @@
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -2394,17 +2276,17 @@
     <row r="3">
       <c r="A3" s="18" t="inlineStr">
         <is>
-          <t>PNUD (Direto)</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="B3" s="17" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>PNUD (Direto)</t>
         </is>
       </c>
       <c r="B4" s="9" t="n">
@@ -2466,7 +2348,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
@@ -2477,45 +2359,45 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Engenheiro Dados</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="B3" s="17" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C3" s="18" t="inlineStr">
         <is>
-          <t>Engenheiro de Dados (Eng. Química + Ciência da Computação), 5 anos em pipelines ETL, Spark/Databricks/Azure e web scraping</t>
+          <t>Analista de BI (Engenharia da Computação + Técnico em Computação), 5+ anos em Power BI/SQL, 3 anos com dados públicos, econômicos e sociais</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Pesquisador Computacao</t>
+          <t>Engenheiro Dados</t>
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>Pesquisador acadêmico com foco em computação, dados e metodologia científica</t>
+          <t>Engenheiro de Dados (Eng. Química + Ciência da Computação), 5 anos em pipelines ETL, Spark/Databricks/Azure e web scraping</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Pesquisador Computacao</t>
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>Analista de BI (Engenharia da Computação + Técnico em Computação), 5+ anos em Power BI/SQL, 3 anos com dados públicos, econômicos e sociais</t>
+          <t>Pesquisador acadêmico com foco em computação, dados e metodologia científica</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-08-15 04:11
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -16,15 +16,15 @@
     <sheet name="Perfis" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$N$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$N$23</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Perfil'!$A$1:$B$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Perfil'!$A$1:$B$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Perfil'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Por_Tipo'!$A$1:$B$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Por_Tipo'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Por_Area'!$A$1:$B$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Por_Area'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Orgao'!$A$1:$B$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Orgao'!$A$1:$B$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Por_Orgao'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Perfis'!$A$1:$C$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Perfis'!$1:$1</definedName>
@@ -549,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -566,7 +566,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 12/08/2026 às 13:06</t>
+          <t>Gerado em 15/08/2026 às 04:06</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6">
@@ -617,7 +617,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -689,11 +689,11 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19">
@@ -703,17 +703,7 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -731,7 +721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -838,7 +828,7 @@
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="E2" s="12" t="n">
@@ -898,7 +888,7 @@
       </c>
       <c r="D3" s="19" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="E3" s="20" t="n">
@@ -960,7 +950,7 @@
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="E4" s="12" t="n">
@@ -1022,7 +1012,7 @@
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="E5" s="20" t="n">
@@ -1084,7 +1074,7 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="E6" s="12" t="n">
@@ -1146,7 +1136,7 @@
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="E7" s="20" t="n">
@@ -1270,7 +1260,7 @@
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="E9" s="20" t="n">
@@ -1332,7 +1322,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="E10" s="12" t="n">
@@ -1394,7 +1384,7 @@
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="E11" s="20" t="n">
@@ -1440,44 +1430,46 @@
     </row>
     <row r="12">
       <c r="A12" s="9" t="n">
-        <v>146287</v>
+        <v>146288</v>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>IC - UNDP-BRA-01223 - Consultoria especializada em recrutamento e seleção</t>
+          <t xml:space="preserve"> BRA23/004 - TR 004/2026 - Consultoria Nacional pessoa física para elaborar estudo sobre favelas e comunidades urbanas do município de Niterói</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="E12" s="12" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="n">
+        <v>0.3</v>
+      </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>PNUD (Direto)</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
-          <t>Remoto. (Notar: na data de término, o edital se encerra às 17h de Brasília)</t>
+          <t>Remoto com possibilidade de atividades presenciais</t>
         </is>
       </c>
       <c r="I12" s="13" t="n">
-        <v>46234</v>
+        <v>46239</v>
       </c>
       <c r="J12" s="13" t="n">
-        <v>46248</v>
+        <v>46252</v>
       </c>
       <c r="K12" s="14" t="inlineStr"/>
       <c r="L12" s="15" t="inlineStr">
@@ -1487,7 +1479,7 @@
       </c>
       <c r="M12" s="11" t="inlineStr">
         <is>
-          <t>ic.procurement.br@undp.org</t>
+          <t>prodoc.ssagi@seplag.niteroi.rj.gov.br</t>
         </is>
       </c>
       <c r="N12" s="16" t="inlineStr">
@@ -1498,11 +1490,11 @@
     </row>
     <row r="13">
       <c r="A13" s="17" t="n">
-        <v>146288</v>
+        <v>146289</v>
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> BRA23/004 - TR 004/2026 - Consultoria Nacional pessoa física para elaborar estudo sobre favelas e comunidades urbanas do município de Niterói</t>
+          <t>BRA23/004 - TR 003/2026 - Contratação de Consultoria Nacional pessoa física para elaborar estudo sobre mulheres e desigualdade de gênero no município de Niterói</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
@@ -1512,7 +1504,7 @@
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="E13" s="20" t="n">
@@ -1520,7 +1512,7 @@
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G13" s="18" t="inlineStr">
@@ -1558,21 +1550,21 @@
     </row>
     <row r="14">
       <c r="A14" s="9" t="n">
-        <v>146289</v>
+        <v>146294</v>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>BRA23/004 - TR 003/2026 - Contratação de Consultoria Nacional pessoa física para elaborar estudo sobre mulheres e desigualdade de gênero no município de Niterói</t>
+          <t>Contratação de consultoria técnica especializada para elaboração e desenvolvimento de solução educacional voltada à formação de lideranças em todos os níveis organizacionais do Conselho Administrativo de Defesa Econômica (Cade), mediante a produção de cursos customizados e objetos de aprendizagem digitais alinhados aos objetivos estratégicos, à missão, à visão e aos valores da Autarquia.</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="E14" s="12" t="n">
@@ -1580,7 +1572,7 @@
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
@@ -1590,16 +1582,18 @@
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t>Remoto com possibilidade de atividades presenciais</t>
+          <t xml:space="preserve"> Remoto</t>
         </is>
       </c>
       <c r="I14" s="13" t="n">
-        <v>46239</v>
+        <v>46245</v>
       </c>
       <c r="J14" s="13" t="n">
-        <v>46252</v>
-      </c>
-      <c r="K14" s="14" t="inlineStr"/>
+        <v>46251</v>
+      </c>
+      <c r="K14" s="14" t="n">
+        <v>80.64</v>
+      </c>
       <c r="L14" s="15" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1607,7 +1601,7 @@
       </c>
       <c r="M14" s="11" t="inlineStr">
         <is>
-          <t>prodoc.ssagi@seplag.niteroi.rj.gov.br</t>
+          <t>prodoc@cade.gov.br</t>
         </is>
       </c>
       <c r="N14" s="16" t="inlineStr">
@@ -1618,44 +1612,46 @@
     </row>
     <row r="15">
       <c r="A15" s="17" t="n">
-        <v>146290</v>
+        <v>146295</v>
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>TR DPA/PNUD 001/2026 - Suporte técnico especializado para fortalecimento de Mecanismos Integrados de Atendimento à RIDEs e à Faixa de Fronteira.</t>
+          <t>IC - UNDP-BRA-01224 - Consultoria (pessoa física) para planejamento estratégico de roteiro internacional de missões para  diálogos sobre segurança cibernética no judiciário</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="E15" s="20" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="E15" s="20" t="n">
+        <v>0.3</v>
+      </c>
       <c r="F15" s="18" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="G15" s="18" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>PNUD (Direto)</t>
         </is>
       </c>
       <c r="H15" s="18" t="inlineStr">
         <is>
-          <t>Brasília</t>
+          <t>Remoto. (Notar: na data de término, o edital se encerra às 17h de Brasília)</t>
         </is>
       </c>
       <c r="I15" s="21" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="J15" s="21" t="n">
-        <v>46248</v>
+        <v>46253</v>
       </c>
       <c r="K15" s="22" t="inlineStr"/>
       <c r="L15" s="23" t="inlineStr">
@@ -1665,7 +1661,7 @@
       </c>
       <c r="M15" s="19" t="inlineStr">
         <is>
-          <t>prodocbra23018@sudeco.gov.br</t>
+          <t>ic.procurement.br@undp.org</t>
         </is>
       </c>
       <c r="N15" s="24" t="inlineStr">
@@ -1676,11 +1672,11 @@
     </row>
     <row r="16">
       <c r="A16" s="9" t="n">
-        <v>146292</v>
+        <v>146296</v>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>UNDP-BRA-01222 - IC - Consultoria Técnica Especializada em Planos Nacionais de Adaptação (COP 30)</t>
+          <t>IC - UNDP-BRA-01226 - Consultoria para avaliação final do Projeto BRA/20/019</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
@@ -1690,13 +1686,15 @@
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="E16" s="12" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="n">
+        <v>0.3</v>
+      </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
@@ -1706,14 +1704,14 @@
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>Trabalho remoto, com possibilidade de viagens</t>
+          <t>Remoto (notar: na data de término, a negociação se encerra às 17h)</t>
         </is>
       </c>
       <c r="I16" s="13" t="n">
-        <v>46238</v>
+        <v>46239</v>
       </c>
       <c r="J16" s="13" t="n">
-        <v>46247</v>
+        <v>46253</v>
       </c>
       <c r="K16" s="14" t="inlineStr"/>
       <c r="L16" s="15" t="inlineStr">
@@ -1734,11 +1732,11 @@
     </row>
     <row r="17">
       <c r="A17" s="17" t="n">
-        <v>146294</v>
+        <v>146303</v>
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>Contratação de consultoria técnica especializada para elaboração e desenvolvimento de solução educacional voltada à formação de lideranças em todos os níveis organizacionais do Conselho Administrativo de Defesa Econômica (Cade), mediante a produção de cursos customizados e objetos de aprendizagem digitais alinhados aos objetivos estratégicos, à missão, à visão e aos valores da Autarquia.</t>
+          <t>Consultoria técnica especializada para estruturação, validação e implantação assistida do Processo Institucional de Due Diligence de Integridade da Secretaria do Tesouro Nacional</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
@@ -1748,15 +1746,13 @@
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Economista</t>
-        </is>
-      </c>
-      <c r="E17" s="20" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="inlineStr"/>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="G17" s="18" t="inlineStr">
@@ -1766,18 +1762,16 @@
       </c>
       <c r="H17" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Remoto</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="I17" s="21" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="J17" s="21" t="n">
-        <v>46251</v>
-      </c>
-      <c r="K17" s="22" t="n">
-        <v>80640</v>
-      </c>
+        <v>46257</v>
+      </c>
+      <c r="K17" s="22" t="inlineStr"/>
       <c r="L17" s="23" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1785,7 +1779,7 @@
       </c>
       <c r="M17" s="19" t="inlineStr">
         <is>
-          <t>prodoc@cade.gov.br</t>
+          <t>ucp.codin.df.stn@tesouro.gov.br</t>
         </is>
       </c>
       <c r="N17" s="24" t="inlineStr">
@@ -1796,11 +1790,11 @@
     </row>
     <row r="18">
       <c r="A18" s="9" t="n">
-        <v>146295</v>
+        <v>146311</v>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>IC - UNDP-BRA-01224 - Consultoria (pessoa física) para planejamento estratégico de roteiro internacional de missões para  diálogos sobre segurança cibernética no judiciário</t>
+          <t>Edital nº 19/2026 - Contratação de Consultoria Individual para o desenvolvimento, documentação e compilação de bases de dados dos módulos econômico e de distribuição de renda do modelo MIRA</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
@@ -1823,21 +1817,23 @@
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>PNUD (Direto)</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>Remoto. (Notar: na data de término, o edital se encerra às 17h de Brasília)</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="I18" s="13" t="n">
-        <v>46239</v>
+        <v>46248</v>
       </c>
       <c r="J18" s="13" t="n">
-        <v>46253</v>
-      </c>
-      <c r="K18" s="14" t="inlineStr"/>
+        <v>46266</v>
+      </c>
+      <c r="K18" s="14" t="n">
+        <v>120000</v>
+      </c>
       <c r="L18" s="15" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1845,7 +1841,7 @@
       </c>
       <c r="M18" s="11" t="inlineStr">
         <is>
-          <t>ic.procurement.br@undp.org</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="N18" s="16" t="inlineStr">
@@ -1856,48 +1852,48 @@
     </row>
     <row r="19">
       <c r="A19" s="17" t="n">
-        <v>146296</v>
+        <v>146312</v>
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>IC - UNDP-BRA-01226 - Consultoria para avaliação final do Projeto BRA/20/019</t>
+          <t>Edital nº 20/2026 - Contratação de Consultor Individual para o desenvolvimento, documentação e aplicação do módulo econômico do modelo MIRA, com foco na calibração de parâmetros, regionalização e estimação da Matriz de Absorção de Investimentos</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>Edital Genérico / IC</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Economista</t>
-        </is>
-      </c>
-      <c r="E19" s="20" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="E19" s="20" t="inlineStr"/>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="G19" s="18" t="inlineStr">
         <is>
-          <t>PNUD (Direto)</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="H19" s="18" t="inlineStr">
         <is>
-          <t>Remoto (notar: na data de término, a negociação se encerra às 17h)</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="I19" s="21" t="n">
-        <v>46239</v>
+        <v>46248</v>
       </c>
       <c r="J19" s="21" t="n">
-        <v>46253</v>
-      </c>
-      <c r="K19" s="22" t="inlineStr"/>
+        <v>46266</v>
+      </c>
+      <c r="K19" s="22" t="n">
+        <v>130000</v>
+      </c>
       <c r="L19" s="23" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1905,7 +1901,7 @@
       </c>
       <c r="M19" s="19" t="inlineStr">
         <is>
-          <t>ic.procurement.br@undp.org</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="N19" s="24" t="inlineStr">
@@ -1916,16 +1912,16 @@
     </row>
     <row r="20">
       <c r="A20" s="9" t="n">
-        <v>146303</v>
+        <v>146317</v>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Consultoria técnica especializada para estruturação, validação e implantação assistida do Processo Institucional de Due Diligence de Integridade da Secretaria do Tesouro Nacional</t>
+          <t>Edital nº 21/2026 - Contratação de Consultoria Individual para o desenvolvimento metodológico e a integração dos módulos de emissões de GEE e consumo de energia no modelo MIRA</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -1941,22 +1937,22 @@
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>REMOTO</t>
         </is>
       </c>
       <c r="I20" s="13" t="n">
-        <v>46246</v>
+        <v>46248</v>
       </c>
       <c r="J20" s="13" t="n">
-        <v>46257</v>
+        <v>46266</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>110707.2</v>
+        <v>120000</v>
       </c>
       <c r="L20" s="15" t="inlineStr">
         <is>
@@ -1965,7 +1961,7 @@
       </c>
       <c r="M20" s="11" t="inlineStr">
         <is>
-          <t>ucp.codin.df.stn@tesouro.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="N20" s="16" t="inlineStr">
@@ -1974,8 +1970,188 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="17" t="n">
+        <v>146318</v>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Edital nº 23/2026 - Contratação de consultor individual para a Elaboração do Guia Prático de Oficinas Colaborativas</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Física (PF)</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="E21" s="20" t="inlineStr"/>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>Não classificada</t>
+        </is>
+      </c>
+      <c r="G21" s="18" t="inlineStr">
+        <is>
+          <t>MGI</t>
+        </is>
+      </c>
+      <c r="H21" s="18" t="inlineStr">
+        <is>
+          <t>REMOTO</t>
+        </is>
+      </c>
+      <c r="I21" s="21" t="n">
+        <v>46248</v>
+      </c>
+      <c r="J21" s="21" t="n">
+        <v>46266</v>
+      </c>
+      <c r="K21" s="22" t="n">
+        <v>100000</v>
+      </c>
+      <c r="L21" s="23" t="inlineStr">
+        <is>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="M21" s="19" t="inlineStr">
+        <is>
+          <t>prodoc.mgi@gestao.gov.br</t>
+        </is>
+      </c>
+      <c r="N21" s="24" t="inlineStr">
+        <is>
+          <t>https://parceiros.undp.org.br/opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="n">
+        <v>146319</v>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Edital nº 22/2026 – Contratação de Consultoria Individual para o desenvolvimento metodológico e a integração dos módulos de emissões de GEE e consumo de água no modelo MIRA</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Física (PF)</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr"/>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>Não classificada</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>MGI</t>
+        </is>
+      </c>
+      <c r="H22" s="10" t="inlineStr">
+        <is>
+          <t>remoto</t>
+        </is>
+      </c>
+      <c r="I22" s="13" t="n">
+        <v>46248</v>
+      </c>
+      <c r="J22" s="13" t="n">
+        <v>46266</v>
+      </c>
+      <c r="K22" s="14" t="n">
+        <v>120000</v>
+      </c>
+      <c r="L22" s="15" t="inlineStr">
+        <is>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="M22" s="11" t="inlineStr">
+        <is>
+          <t>prodoc.mgi@gestao.gov.br</t>
+        </is>
+      </c>
+      <c r="N22" s="16" t="inlineStr">
+        <is>
+          <t>https://parceiros.undp.org.br/opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="n">
+        <v>146320</v>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Edital nº 24/2026 – Contratação de Consultoria individual para desenvolvimento de projeto gráfico  e diagramação do Relatório de Gestão Integrado </t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Física (PF)</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="E23" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="G23" s="18" t="inlineStr">
+        <is>
+          <t>MGI</t>
+        </is>
+      </c>
+      <c r="H23" s="18" t="inlineStr">
+        <is>
+          <t>remoto</t>
+        </is>
+      </c>
+      <c r="I23" s="21" t="n">
+        <v>46248</v>
+      </c>
+      <c r="J23" s="21" t="n">
+        <v>46266</v>
+      </c>
+      <c r="K23" s="22" t="inlineStr"/>
+      <c r="L23" s="23" t="inlineStr">
+        <is>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="M23" s="19" t="inlineStr">
+        <is>
+          <t>prodoc.mgi@gestao.gov.br</t>
+        </is>
+      </c>
+      <c r="N23" s="24" t="inlineStr">
+        <is>
+          <t>https://parceiros.undp.org.br/opportunities</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N20"/>
+  <autoFilter ref="A1:N23"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
@@ -1996,6 +2172,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -2008,7 +2187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2030,11 +2209,11 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -2044,21 +2223,11 @@
         </is>
       </c>
       <c r="B3" s="17" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B4"/>
+  <autoFilter ref="A1:B3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -2096,7 +2265,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3">
@@ -2106,7 +2275,7 @@
         </is>
       </c>
       <c r="B3" s="17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -2116,7 +2285,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -2126,7 +2295,7 @@
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2168,7 +2337,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -2188,7 +2357,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -2198,7 +2367,7 @@
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -2244,7 +2413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2276,17 +2445,17 @@
     <row r="3">
       <c r="A3" s="18" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="B3" s="17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>PNUD (Direto)</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="B4" s="9" t="n">
@@ -2296,15 +2465,25 @@
     <row r="5">
       <c r="A5" s="18" t="inlineStr">
         <is>
+          <t>PNUD (Direto)</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
           <t>TCU</t>
         </is>
       </c>
-      <c r="B5" s="17" t="n">
+      <c r="B6" s="9" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B5"/>
+  <autoFilter ref="A1:B6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -2344,22 +2523,22 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>Economista com stack técnica em análise de dados e políticas públicas, sem pós-graduação</t>
+          <t>Analista de BI (Engenharia da Computação + Técnico em Computação), 5+ anos em Power BI/SQL, 3 anos com dados públicos, econômicos e sociais</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Pesquisador Computacao</t>
         </is>
       </c>
       <c r="B3" s="17" t="n">
@@ -2367,37 +2546,37 @@
       </c>
       <c r="C3" s="18" t="inlineStr">
         <is>
-          <t>Analista de BI (Engenharia da Computação + Técnico em Computação), 5+ anos em Power BI/SQL, 3 anos com dados públicos, econômicos e sociais</t>
+          <t>Pesquisador acadêmico com foco em computação, dados e metodologia científica</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Engenheiro Dados</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>Engenheiro de Dados (Eng. Química + Ciência da Computação), 5 anos em pipelines ETL, Spark/Databricks/Azure e web scraping</t>
+          <t>Economista com stack técnica em análise de dados e políticas públicas, sem pós-graduação</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Pesquisador Computacao</t>
+          <t>Engenheiro Dados</t>
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>Pesquisador acadêmico com foco em computação, dados e metodologia científica</t>
+          <t>Engenheiro de Dados (Eng. Química + Ciência da Computação), 5 anos em pipelines ETL, Spark/Databricks/Azure e web scraping</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-08-22 12:43
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -16,7 +16,7 @@
     <sheet name="Perfis" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$N$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$N$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Perfil'!$A$1:$B$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Perfil'!$1:$1</definedName>
@@ -24,7 +24,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Por_Tipo'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Por_Area'!$A$1:$B$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Por_Area'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Orgao'!$A$1:$B$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Orgao'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Por_Orgao'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Perfis'!$A$1:$C$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Perfis'!$1:$1</definedName>
@@ -563,7 +563,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 20/08/2026 às 12:45</t>
+          <t>Gerado em 22/08/2026 às 12:36</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -660,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1090,9 +1090,7 @@
       <c r="J7" s="20" t="n">
         <v>46267</v>
       </c>
-      <c r="K7" s="21" t="n">
-        <v>83030.39999999999</v>
-      </c>
+      <c r="K7" s="21" t="inlineStr"/>
       <c r="L7" s="22" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1343,8 +1341,128 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="8" t="n">
+        <v>146336</v>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>UNDP-BRA-01232 - Benchmark Internacional e Análise de Adaptabilidade de Modelos Federativos de Gestão de Pessoas ao Contexto Brasileiro</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Física (PF)</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>PNUD (Direto)</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Home based</t>
+        </is>
+      </c>
+      <c r="I12" s="12" t="n">
+        <v>46255</v>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>46268</v>
+      </c>
+      <c r="K12" s="13" t="inlineStr"/>
+      <c r="L12" s="14" t="inlineStr">
+        <is>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="M12" s="10" t="inlineStr">
+        <is>
+          <t>ic.procurement.br@undp.org</t>
+        </is>
+      </c>
+      <c r="N12" s="15" t="inlineStr">
+        <is>
+          <t>https://parceiros.undp.org.br/opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="n">
+        <v>146337</v>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>IC UNDP-BRA-01228 - Benchmarking, modelagem federativa e análise de viabilidade institucional</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Física (PF)</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F13" s="17" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="G13" s="17" t="inlineStr">
+        <is>
+          <t>PNUD (Direto)</t>
+        </is>
+      </c>
+      <c r="H13" s="17" t="inlineStr">
+        <is>
+          <t>Home based</t>
+        </is>
+      </c>
+      <c r="I13" s="20" t="n">
+        <v>46255</v>
+      </c>
+      <c r="J13" s="20" t="n">
+        <v>46268</v>
+      </c>
+      <c r="K13" s="21" t="inlineStr"/>
+      <c r="L13" s="22" t="inlineStr">
+        <is>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="M13" s="18" t="inlineStr">
+        <is>
+          <t>aquisicoes.cbo.br@undp.org</t>
+        </is>
+      </c>
+      <c r="N13" s="23" t="inlineStr">
+        <is>
+          <t>https://parceiros.undp.org.br/opportunities</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N11"/>
+  <autoFilter ref="A1:N13"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
@@ -1356,6 +1474,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -1394,7 +1514,7 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3">
@@ -1446,7 +1566,7 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
@@ -1494,31 +1614,31 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="17" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -1528,7 +1648,7 @@
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -1554,7 +1674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1593,8 +1713,18 @@
         <v>4</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>PNUD (Direto)</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B3"/>
+  <autoFilter ref="A1:B4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -1638,7 +1768,7 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C2" s="9" t="inlineStr">
         <is>
@@ -1653,7 +1783,7 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C3" s="17" t="inlineStr">
         <is>
@@ -1668,7 +1798,7 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
@@ -1683,7 +1813,7 @@
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C5" s="17" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-08-24 12:53
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -16,13 +16,13 @@
     <sheet name="Perfis" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$N$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$N$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Perfil'!$A$1:$B$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Perfil'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Por_Tipo'!$A$1:$B$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Por_Tipo'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Por_Area'!$A$1:$B$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Por_Area'!$A$1:$B$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Por_Area'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Orgao'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Por_Orgao'!$1:$1</definedName>
@@ -563,7 +563,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 22/08/2026 às 12:36</t>
+          <t>Gerado em 24/08/2026 às 12:47</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -632,7 +632,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -660,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -753,11 +753,11 @@
     </row>
     <row r="2">
       <c r="A2" s="8" t="n">
-        <v>146288</v>
+        <v>146311</v>
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> BRA23/004 - TR 004/2026 - Consultoria Nacional pessoa física para elaborar estudo sobre favelas e comunidades urbanas do município de Niterói</t>
+          <t>Edital nº 19/2026 - Contratação de Consultoria Individual para o desenvolvimento, documentação e compilação de bases de dados dos módulos econômico e de distribuição de renda do modelo MIRA</t>
         </is>
       </c>
       <c r="C2" s="9" t="inlineStr">
@@ -775,24 +775,24 @@
       </c>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="G2" s="9" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>Remoto com possibilidade de atividades presenciais</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="I2" s="12" t="n">
-        <v>46239</v>
+        <v>46248</v>
       </c>
       <c r="J2" s="12" t="n">
-        <v>46257</v>
+        <v>46266</v>
       </c>
       <c r="K2" s="13" t="inlineStr"/>
       <c r="L2" s="14" t="inlineStr">
@@ -802,7 +802,7 @@
       </c>
       <c r="M2" s="10" t="inlineStr">
         <is>
-          <t>prodoc.ssagi@seplag.niteroi.rj.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="N2" s="15" t="inlineStr">
@@ -813,11 +813,11 @@
     </row>
     <row r="3">
       <c r="A3" s="16" t="n">
-        <v>146289</v>
+        <v>146312</v>
       </c>
       <c r="B3" s="17" t="inlineStr">
         <is>
-          <t>BRA23/004 - TR 003/2026 - Contratação de Consultoria Nacional pessoa física para elaborar estudo sobre mulheres e desigualdade de gênero no município de Niterói</t>
+          <t>Edital nº 20/2026 - Contratação de Consultor Individual para o desenvolvimento, documentação e aplicação do módulo econômico do modelo MIRA, com foco na calibração de parâmetros, regionalização e estimação da Matriz de Absorção de Investimentos</t>
         </is>
       </c>
       <c r="C3" s="17" t="inlineStr">
@@ -827,32 +827,30 @@
       </c>
       <c r="D3" s="18" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="E3" s="19" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="E3" s="19" t="inlineStr"/>
       <c r="F3" s="17" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="G3" s="17" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="H3" s="17" t="inlineStr">
         <is>
-          <t>Remoto com possibilidade de atividades presenciais</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="I3" s="20" t="n">
-        <v>46239</v>
+        <v>46248</v>
       </c>
       <c r="J3" s="20" t="n">
-        <v>46257</v>
+        <v>46266</v>
       </c>
       <c r="K3" s="21" t="inlineStr"/>
       <c r="L3" s="22" t="inlineStr">
@@ -862,7 +860,7 @@
       </c>
       <c r="M3" s="18" t="inlineStr">
         <is>
-          <t>prodoc.ssagi@seplag.niteroi.rj.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="N3" s="23" t="inlineStr">
@@ -873,11 +871,11 @@
     </row>
     <row r="4">
       <c r="A4" s="8" t="n">
-        <v>146303</v>
+        <v>146313</v>
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Consultoria técnica especializada para estruturação, validação e implantação assistida do Processo Institucional de Due Diligence de Integridade da Secretaria do Tesouro Nacional</t>
+          <t>Consultoria técnica especializada para desenvolvimento de proposta de governança e curadoria da Base de Conhecimento destinada ao suporte de soluções de Inteligência Artificial da área de Integridade da Secretaria do Tesouro Nacional</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
@@ -887,13 +885,15 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="E4" s="11" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>0.3</v>
+      </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
@@ -907,10 +907,10 @@
         </is>
       </c>
       <c r="I4" s="12" t="n">
-        <v>46246</v>
+        <v>46254</v>
       </c>
       <c r="J4" s="12" t="n">
-        <v>46257</v>
+        <v>46267</v>
       </c>
       <c r="K4" s="13" t="inlineStr"/>
       <c r="L4" s="14" t="inlineStr">
@@ -931,11 +931,11 @@
     </row>
     <row r="5">
       <c r="A5" s="16" t="n">
-        <v>146311</v>
+        <v>146317</v>
       </c>
       <c r="B5" s="17" t="inlineStr">
         <is>
-          <t>Edital nº 19/2026 - Contratação de Consultoria Individual para o desenvolvimento, documentação e compilação de bases de dados dos módulos econômico e de distribuição de renda do modelo MIRA</t>
+          <t>Edital nº 21/2026 - Contratação de Consultoria Individual para o desenvolvimento metodológico e a integração dos módulos de emissões de GEE e consumo de energia no modelo MIRA</t>
         </is>
       </c>
       <c r="C5" s="17" t="inlineStr">
@@ -945,15 +945,13 @@
       </c>
       <c r="D5" s="18" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="E5" s="19" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="E5" s="19" t="inlineStr"/>
       <c r="F5" s="17" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="G5" s="17" t="inlineStr">
@@ -963,7 +961,7 @@
       </c>
       <c r="H5" s="17" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>REMOTO</t>
         </is>
       </c>
       <c r="I5" s="20" t="n">
@@ -991,11 +989,11 @@
     </row>
     <row r="6">
       <c r="A6" s="8" t="n">
-        <v>146312</v>
+        <v>146318</v>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Edital nº 20/2026 - Contratação de Consultor Individual para o desenvolvimento, documentação e aplicação do módulo econômico do modelo MIRA, com foco na calibração de parâmetros, regionalização e estimação da Matriz de Absorção de Investimentos</t>
+          <t>Edital nº 23/2026 - Contratação de consultor individual para a Elaboração do Guia Prático de Oficinas Colaborativas</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -1021,7 +1019,7 @@
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>REMOTO</t>
         </is>
       </c>
       <c r="I6" s="12" t="n">
@@ -1049,46 +1047,44 @@
     </row>
     <row r="7">
       <c r="A7" s="16" t="n">
-        <v>146313</v>
+        <v>146319</v>
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>Consultoria técnica especializada para desenvolvimento de proposta de governança e curadoria da Base de Conhecimento destinada ao suporte de soluções de Inteligência Artificial da área de Integridade da Secretaria do Tesouro Nacional</t>
+          <t>Edital nº 22/2026 – Contratação de Consultoria Individual para o desenvolvimento metodológico e a integração dos módulos de emissões de GEE e consumo de água no modelo MIRA</t>
         </is>
       </c>
       <c r="C7" s="17" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="D7" s="18" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="E7" s="19" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="inlineStr"/>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="H7" s="17" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>remoto</t>
         </is>
       </c>
       <c r="I7" s="20" t="n">
-        <v>46254</v>
+        <v>46248</v>
       </c>
       <c r="J7" s="20" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="K7" s="21" t="inlineStr"/>
       <c r="L7" s="22" t="inlineStr">
@@ -1098,7 +1094,7 @@
       </c>
       <c r="M7" s="18" t="inlineStr">
         <is>
-          <t>ucp.codin.df.stn@tesouro.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="N7" s="23" t="inlineStr">
@@ -1109,11 +1105,11 @@
     </row>
     <row r="8">
       <c r="A8" s="8" t="n">
-        <v>146317</v>
+        <v>146320</v>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Edital nº 21/2026 - Contratação de Consultoria Individual para o desenvolvimento metodológico e a integração dos módulos de emissões de GEE e consumo de energia no modelo MIRA</t>
+          <t xml:space="preserve">Edital nº 24/2026 – Contratação de Consultoria individual para desenvolvimento de projeto gráfico  e diagramação do Relatório de Gestão Integrado </t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -1123,13 +1119,15 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="E8" s="11" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>0.3</v>
+      </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -1139,7 +1137,7 @@
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>remoto</t>
         </is>
       </c>
       <c r="I8" s="12" t="n">
@@ -1167,11 +1165,11 @@
     </row>
     <row r="9">
       <c r="A9" s="16" t="n">
-        <v>146318</v>
+        <v>146326</v>
       </c>
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>Edital nº 23/2026 - Contratação de consultor individual para a Elaboração do Guia Prático de Oficinas Colaborativas</t>
+          <t>Edital nº 02/2026 – Metodologia para monitoramento das decisões da Corte Interamericana de Direitos Humanos</t>
         </is>
       </c>
       <c r="C9" s="17" t="inlineStr">
@@ -1181,32 +1179,36 @@
       </c>
       <c r="D9" s="18" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="E9" s="19" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>0.3</v>
+      </c>
       <c r="F9" s="17" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="H9" s="17" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="I9" s="20" t="n">
-        <v>46248</v>
+        <v>46258</v>
       </c>
       <c r="J9" s="20" t="n">
-        <v>46266</v>
-      </c>
-      <c r="K9" s="21" t="inlineStr"/>
+        <v>46274</v>
+      </c>
+      <c r="K9" s="21" t="n">
+        <v>81000</v>
+      </c>
       <c r="L9" s="22" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1214,7 +1216,7 @@
       </c>
       <c r="M9" s="18" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>ccidh@mdh.gov.br</t>
         </is>
       </c>
       <c r="N9" s="23" t="inlineStr">
@@ -1225,11 +1227,11 @@
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
-        <v>146319</v>
+        <v>146327</v>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Edital nº 22/2026 – Contratação de Consultoria Individual para o desenvolvimento metodológico e a integração dos módulos de emissões de GEE e consumo de água no modelo MIRA</t>
+          <t>Edital nº 3/2026 – Metodologia para monitoramento de recomendações e decisões da Comissão Interamericana de Direitos Humanos</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -1239,32 +1241,36 @@
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="E10" s="11" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>0.3</v>
+      </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="H10" s="9" t="inlineStr">
         <is>
-          <t>remoto</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="I10" s="12" t="n">
-        <v>46248</v>
+        <v>46258</v>
       </c>
       <c r="J10" s="12" t="n">
-        <v>46266</v>
-      </c>
-      <c r="K10" s="13" t="inlineStr"/>
+        <v>46274</v>
+      </c>
+      <c r="K10" s="13" t="n">
+        <v>81000</v>
+      </c>
       <c r="L10" s="14" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1272,7 +1278,7 @@
       </c>
       <c r="M10" s="10" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>ccidh@mdh.gov.br</t>
         </is>
       </c>
       <c r="N10" s="15" t="inlineStr">
@@ -1283,11 +1289,11 @@
     </row>
     <row r="11">
       <c r="A11" s="16" t="n">
-        <v>146320</v>
+        <v>146332</v>
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edital nº 24/2026 – Contratação de Consultoria individual para desenvolvimento de projeto gráfico  e diagramação do Relatório de Gestão Integrado </t>
+          <t>Edital nº 04/2026 - Segundo Plano da Política Nacional de RCN</t>
         </is>
       </c>
       <c r="C11" s="17" t="inlineStr">
@@ -1305,26 +1311,28 @@
       </c>
       <c r="F11" s="17" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G11" s="17" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="H11" s="17" t="inlineStr">
         <is>
-          <t>remoto</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="I11" s="20" t="n">
-        <v>46248</v>
+        <v>46258</v>
       </c>
       <c r="J11" s="20" t="n">
-        <v>46266</v>
-      </c>
-      <c r="K11" s="21" t="inlineStr"/>
+        <v>46274</v>
+      </c>
+      <c r="K11" s="21" t="n">
+        <v>60000</v>
+      </c>
       <c r="L11" s="22" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1332,7 +1340,7 @@
       </c>
       <c r="M11" s="18" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>rcn_cidadania@mdh.gov.br</t>
         </is>
       </c>
       <c r="N11" s="23" t="inlineStr">
@@ -1343,16 +1351,16 @@
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
-        <v>146336</v>
+        <v>146335</v>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>UNDP-BRA-01232 - Benchmark Internacional e Análise de Adaptabilidade de Modelos Federativos de Gestão de Pessoas ao Contexto Brasileiro</t>
+          <t>Consultoria técnica especializada para avaliação das capacidades institucionais da Secretaria do Tesouro Nacional (STN)</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
@@ -1365,26 +1373,28 @@
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>PNUD (Direto)</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>Home based</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="I12" s="12" t="n">
-        <v>46255</v>
+        <v>46258</v>
       </c>
       <c r="J12" s="12" t="n">
-        <v>46268</v>
-      </c>
-      <c r="K12" s="13" t="inlineStr"/>
+        <v>46271</v>
+      </c>
+      <c r="K12" s="13" t="n">
+        <v>77495.03999999999</v>
+      </c>
       <c r="L12" s="14" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1392,7 +1402,7 @@
       </c>
       <c r="M12" s="10" t="inlineStr">
         <is>
-          <t>ic.procurement.br@undp.org</t>
+          <t>ucp.codin.df.stn@tesouro.gov.br</t>
         </is>
       </c>
       <c r="N12" s="15" t="inlineStr">
@@ -1403,11 +1413,11 @@
     </row>
     <row r="13">
       <c r="A13" s="16" t="n">
-        <v>146337</v>
+        <v>146336</v>
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>IC UNDP-BRA-01228 - Benchmarking, modelagem federativa e análise de viabilidade institucional</t>
+          <t>UNDP-BRA-01232 - Benchmark Internacional e Análise de Adaptabilidade de Modelos Federativos de Gestão de Pessoas ao Contexto Brasileiro</t>
         </is>
       </c>
       <c r="C13" s="17" t="inlineStr">
@@ -1452,17 +1462,77 @@
       </c>
       <c r="M13" s="18" t="inlineStr">
         <is>
+          <t>ic.procurement.br@undp.org</t>
+        </is>
+      </c>
+      <c r="N13" s="23" t="inlineStr">
+        <is>
+          <t>https://parceiros.undp.org.br/opportunities</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n">
+        <v>146337</v>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>IC UNDP-BRA-01228 - Benchmarking, modelagem federativa e análise de viabilidade institucional</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Física (PF)</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>PNUD (Direto)</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>Home based</t>
+        </is>
+      </c>
+      <c r="I14" s="12" t="n">
+        <v>46255</v>
+      </c>
+      <c r="J14" s="12" t="n">
+        <v>46268</v>
+      </c>
+      <c r="K14" s="13" t="inlineStr"/>
+      <c r="L14" s="14" t="inlineStr">
+        <is>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="M14" s="10" t="inlineStr">
+        <is>
           <t>aquisicoes.cbo.br@undp.org</t>
         </is>
       </c>
-      <c r="N13" s="23" t="inlineStr">
+      <c r="N14" s="15" t="inlineStr">
         <is>
           <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N13"/>
+  <autoFilter ref="A1:N14"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
@@ -1476,6 +1546,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -1514,7 +1585,7 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -1524,7 +1595,7 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1566,7 +1637,7 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3">
@@ -1592,7 +1663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1618,7 +1689,7 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -1628,13 +1699,13 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="B4" s="8" t="n">
@@ -1644,25 +1715,15 @@
     <row r="5">
       <c r="A5" s="17" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="B5" s="16" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="n">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:B6"/>
+  <autoFilter ref="A1:B5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -1710,7 +1771,7 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -1768,7 +1829,7 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C2" s="9" t="inlineStr">
         <is>
@@ -1783,7 +1844,7 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3" s="17" t="inlineStr">
         <is>
@@ -1798,7 +1859,7 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
@@ -1813,7 +1874,7 @@
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C5" s="17" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-08-26 12:53
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$60</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 25/08/2026 às 12:55</t>
+          <t>Gerado em 26/08/2026 às 12:51</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
@@ -644,21 +644,21 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>PNUD</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>PNUD</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24">
@@ -762,7 +762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O57"/>
+  <dimension ref="A1:O60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2054,12 +2054,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:7155091d-98d5-4ce4-df16-08df01dbdf45</t>
+          <t>unesco:8a4f297f-a7f6-4db9-ebd4-08defdee4813</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ4024 - EDITAL Nº03/2026 - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 34/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2069,13 +2069,15 @@
       </c>
       <c r="E21" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F21" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2085,10 +2087,10 @@
       </c>
       <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="22" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
@@ -2111,17 +2113,17 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:3ace2443-618f-4dcd-3f59-08def87d335c</t>
+          <t>unesco:1ade5265-d185-4752-ebd5-08defdee4813</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ1085 - Edital nº 03/2026 - 02 vagas - Consultores Individuais</t>
+          <t>914BRZ1159 - Publicação Edital 35/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -2134,7 +2136,7 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Saúde, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2144,10 +2146,10 @@
       </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46251</v>
+        <v>46260</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46260</v>
+        <v>46264</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2170,17 +2172,17 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:be7dda96-d11c-4774-ed52-08defa0191b8</t>
+          <t>unesco:e6ba376a-8848-485f-3f37-08defeb303ea</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
+          <t>914BRZ1163 - Publicação -  Edital 67/2026 - 01 Vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E23" s="20" t="inlineStr">
@@ -2193,7 +2195,7 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2203,10 +2205,10 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46257</v>
+        <v>46260</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46264</v>
+        <v>46266</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2229,17 +2231,17 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:5a9d0c82-e38a-483b-ed53-08defa0191b8</t>
+          <t>unesco:7155091d-98d5-4ce4-df16-08df01dbdf45</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 18/2026 (REPUBLICAÇÃO)</t>
+          <t>914BRZ4024 - EDITAL Nº03/2026 - Consultor Individual</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
@@ -2260,10 +2262,10 @@
       </c>
       <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46257</v>
+        <v>46259</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
@@ -2286,28 +2288,30 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:902f516e-135f-4244-ed50-08defa0191b8</t>
+          <t>unesco:3ace2443-618f-4dcd-3f59-08def87d335c</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3061 - EDITAL Nº 12/2026 - 01 VAGA - CONSULTOR INDIVIDUAL - REPUBLICAÇAO</t>
+          <t>Projeto 914BRZ1085 - Edital nº 03/2026 - 02 vagas - Consultores Individuais</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Saúde, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2317,7 +2321,7 @@
       </c>
       <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46255</v>
+        <v>46251</v>
       </c>
       <c r="K25" s="22" t="n">
         <v>46260</v>
@@ -2338,17 +2342,17 @@
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
+          <t>unesco:be7dda96-d11c-4774-ed52-08defa0191b8</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
+          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2362,7 +2366,7 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
@@ -2371,53 +2375,43 @@
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I26" s="11" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr"/>
       <c r="J26" s="14" t="n">
-        <v>46213</v>
+        <v>46257</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46217</v>
-      </c>
-      <c r="L26" s="15" t="n">
-        <v>144000</v>
-      </c>
+        <v>46264</v>
+      </c>
+      <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N26" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N26" s="12" t="inlineStr"/>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
+          <t>unesco:5a9d0c82-e38a-483b-ed53-08defa0191b8</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
+          <t>Projeto 914BRZ3051 - EDITAL 18/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2427,116 +2421,94 @@
       </c>
       <c r="E27" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F27" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F27" s="21" t="inlineStr"/>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I27" s="19" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I27" s="19" t="inlineStr"/>
       <c r="J27" s="22" t="n">
-        <v>46216</v>
+        <v>46257</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46223</v>
-      </c>
-      <c r="L27" s="23" t="n">
-        <v>133000</v>
-      </c>
+        <v>46264</v>
+      </c>
+      <c r="L27" s="23" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N27" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N27" s="20" t="inlineStr"/>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-03-territorios-criativos-e-educacao-tr-13051</t>
+          <t>unesco:902f516e-135f-4244-ed50-08defa0191b8</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-03 – Territórios Criativos e Educação – TR 13051</t>
+          <t>914BRZ3061 - EDITAL Nº 12/2026 - 01 VAGA - CONSULTOR INDIVIDUAL - REPUBLICAÇAO</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F28" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="inlineStr"/>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I28" s="11" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr"/>
       <c r="J28" s="14" t="n">
-        <v>46204</v>
+        <v>46255</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46209</v>
+        <v>46260</v>
       </c>
       <c r="L28" s="15" t="inlineStr"/>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N28" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N28" s="12" t="inlineStr"/>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-03-territorios-criativos-e-educacao-tr-13051/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -2617,12 +2589,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-03-territorios-criativos-e-educacao-tr-13051</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEC/BRA/24 – TR 13056</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-03 – Territórios Criativos e Educação – TR 13051</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2640,7 +2612,7 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2654,10 +2626,10 @@
         </is>
       </c>
       <c r="J30" s="14" t="n">
+        <v>46204</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>46209</v>
-      </c>
-      <c r="K30" s="14" t="n">
-        <v>46214</v>
       </c>
       <c r="L30" s="15" t="inlineStr"/>
       <c r="M30" s="9" t="inlineStr">
@@ -2672,7 +2644,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-03-territorios-criativos-e-educacao-tr-13051/</t>
         </is>
       </c>
     </row>
@@ -2684,17 +2656,17 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
@@ -2707,12 +2679,12 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I31" s="19" t="inlineStr">
@@ -2721,17 +2693,17 @@
         </is>
       </c>
       <c r="J31" s="22" t="n">
+        <v>46213</v>
+      </c>
+      <c r="K31" s="22" t="n">
         <v>46217</v>
       </c>
-      <c r="K31" s="22" t="n">
-        <v>46222</v>
-      </c>
       <c r="L31" s="23" t="n">
-        <v>77100</v>
+        <v>144000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N31" s="20" t="inlineStr">
@@ -2741,7 +2713,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
         </is>
       </c>
     </row>
@@ -2753,12 +2725,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEC/BRA/24 – TR 13056</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2772,16 +2744,16 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
@@ -2790,17 +2762,15 @@
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46220</v>
+        <v>46209</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46225</v>
-      </c>
-      <c r="L32" s="15" t="n">
-        <v>58800</v>
-      </c>
+        <v>46214</v>
+      </c>
+      <c r="L32" s="15" t="inlineStr"/>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N32" s="12" t="inlineStr">
@@ -2810,7 +2780,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056/</t>
         </is>
       </c>
     </row>
@@ -2822,12 +2792,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2841,11 +2811,11 @@
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
@@ -2855,19 +2825,21 @@
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46220</v>
-      </c>
-      <c r="L33" s="23" t="inlineStr"/>
+        <v>46223</v>
+      </c>
+      <c r="L33" s="23" t="n">
+        <v>133000</v>
+      </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N33" s="20" t="inlineStr">
@@ -2877,7 +2849,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
         </is>
       </c>
     </row>
@@ -2889,17 +2861,17 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -2908,11 +2880,11 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -2926,15 +2898,17 @@
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46221</v>
+        <v>46220</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46224</v>
-      </c>
-      <c r="L34" s="15" t="inlineStr"/>
+        <v>46225</v>
+      </c>
+      <c r="L34" s="15" t="n">
+        <v>58800</v>
+      </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -2944,7 +2918,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
         </is>
       </c>
     </row>
@@ -2956,17 +2930,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -2975,11 +2949,11 @@
         </is>
       </c>
       <c r="F35" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -2993,17 +2967,15 @@
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46223</v>
+        <v>46221</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46238</v>
-      </c>
-      <c r="L35" s="23" t="n">
-        <v>100000</v>
-      </c>
+        <v>46224</v>
+      </c>
+      <c r="L35" s="23" t="inlineStr"/>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N35" s="20" t="inlineStr">
@@ -3013,7 +2985,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
         </is>
       </c>
     </row>
@@ -3025,12 +2997,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR 12970</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3048,7 +3020,7 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3058,14 +3030,14 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46183</v>
+        <v>46213</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46188</v>
+        <v>46220</v>
       </c>
       <c r="L36" s="15" t="inlineStr"/>
       <c r="M36" s="9" t="inlineStr">
@@ -3080,7 +3052,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
         </is>
       </c>
     </row>
@@ -3092,12 +3064,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3115,27 +3087,27 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46225</v>
+        <v>46217</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46229</v>
+        <v>46222</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>114600</v>
+        <v>77100</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3149,7 +3121,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
         </is>
       </c>
     </row>
@@ -3161,17 +3133,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3194,21 +3166,21 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Brasília DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46227</v>
+        <v>46223</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46231</v>
+        <v>46238</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
@@ -3218,7 +3190,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
         </is>
       </c>
     </row>
@@ -3230,12 +3202,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3253,31 +3225,31 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46233</v>
+        <v>46231</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>288000</v>
+        <v>150000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
@@ -3287,7 +3259,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -3299,17 +3271,17 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
@@ -3318,11 +3290,11 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.343</v>
+        <v>0.4</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3332,17 +3304,17 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46232</v>
+        <v>46224</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46238</v>
+        <v>46233</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>30000</v>
+        <v>288000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3356,7 +3328,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -3368,12 +3340,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR 12970</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3387,11 +3359,11 @@
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3401,21 +3373,19 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46232</v>
+        <v>46183</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46237</v>
-      </c>
-      <c r="L41" s="23" t="n">
-        <v>288000</v>
-      </c>
+        <v>46188</v>
+      </c>
+      <c r="L41" s="23" t="inlineStr"/>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
@@ -3425,7 +3395,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970/</t>
         </is>
       </c>
     </row>
@@ -3437,12 +3407,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3452,33 +3422,35 @@
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F42" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F42" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46232</v>
+        <v>46225</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46238</v>
+        <v>46229</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>30000</v>
+        <v>114600</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3492,7 +3464,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
         </is>
       </c>
     </row>
@@ -3504,17 +3476,17 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
@@ -3523,45 +3495,45 @@
         </is>
       </c>
       <c r="F43" s="21" t="n">
-        <v>0.4</v>
+        <v>0.343</v>
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46208</v>
+        <v>46232</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46259</v>
+        <v>46238</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>500000</v>
+        <v>30000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -3573,12 +3545,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3588,15 +3560,13 @@
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F44" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F44" s="13" t="inlineStr"/>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
@@ -3606,17 +3576,17 @@
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>204000</v>
+        <v>30000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
@@ -3630,7 +3600,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -3642,12 +3612,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3665,7 +3635,7 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
@@ -3675,7 +3645,7 @@
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
@@ -3685,7 +3655,7 @@
         <v>46245</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>204000</v>
+        <v>80000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
@@ -3699,7 +3669,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -3711,12 +3681,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3734,7 +3704,7 @@
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3744,7 +3714,7 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
@@ -3754,7 +3724,7 @@
         <v>46245</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>80000</v>
+        <v>100000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3768,7 +3738,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3849,12 +3819,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3872,7 +3842,7 @@
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
@@ -3892,7 +3862,7 @@
         <v>46245</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>100000</v>
+        <v>204000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3906,7 +3876,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -3918,17 +3888,17 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
@@ -3941,41 +3911,41 @@
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46244</v>
+        <v>46232</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46300</v>
+        <v>46237</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>350000</v>
+        <v>288000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -3987,17 +3957,17 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
@@ -4010,41 +3980,41 @@
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46244</v>
+        <v>46240</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46296</v>
+        <v>46245</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>935000</v>
+        <v>204000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -4056,17 +4026,17 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
@@ -4079,41 +4049,41 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46246</v>
+        <v>46244</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46257</v>
+        <v>46300</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>54000</v>
+        <v>350000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4125,17 +4095,17 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
@@ -4148,41 +4118,41 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46246</v>
+        <v>46244</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46257</v>
+        <v>46296</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>54000</v>
+        <v>935000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4194,12 +4164,12 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -4209,37 +4179,37 @@
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F53" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F53" s="21" t="inlineStr"/>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46246</v>
+        <v>46227</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L53" s="23" t="inlineStr"/>
+        <v>46252</v>
+      </c>
+      <c r="L53" s="23" t="n">
+        <v>286000</v>
+      </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N53" s="20" t="inlineStr">
@@ -4249,7 +4219,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -4261,12 +4231,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4276,13 +4246,15 @@
       </c>
       <c r="E54" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F54" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F54" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
@@ -4292,17 +4264,17 @@
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46227</v>
+        <v>46246</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46252</v>
+        <v>46257</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>286000</v>
+        <v>54000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
@@ -4316,7 +4288,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -4328,12 +4300,12 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
@@ -4351,7 +4323,7 @@
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
@@ -4385,7 +4357,7 @@
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -4397,12 +4369,12 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
@@ -4416,35 +4388,33 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46252</v>
+        <v>46246</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L56" s="15" t="n">
-        <v>60000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L56" s="15" t="inlineStr"/>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
@@ -4454,7 +4424,7 @@
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -4466,17 +4436,17 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
@@ -4489,46 +4459,253 @@
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+        </is>
+      </c>
+      <c r="H57" s="19" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I57" s="19" t="inlineStr">
+        <is>
+          <t>Porto Alegre/RS</t>
+        </is>
+      </c>
+      <c r="J57" s="22" t="n">
+        <v>46246</v>
+      </c>
+      <c r="K57" s="22" t="n">
+        <v>46257</v>
+      </c>
+      <c r="L57" s="23" t="n">
+        <v>54000</v>
+      </c>
+      <c r="M57" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N57" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O57" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+        </is>
+      </c>
+      <c r="E58" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F58" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G58" s="11" t="inlineStr">
+        <is>
           <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
-      <c r="H57" s="19" t="inlineStr">
+      <c r="H58" s="11" t="inlineStr">
         <is>
           <t>OEI/BRA</t>
         </is>
       </c>
-      <c r="I57" s="19" t="inlineStr">
+      <c r="I58" s="11" t="inlineStr">
         <is>
           <t>Recife - PE</t>
         </is>
       </c>
-      <c r="J57" s="22" t="n">
+      <c r="J58" s="14" t="n">
         <v>46251</v>
       </c>
-      <c r="K57" s="22" t="n">
+      <c r="K58" s="14" t="n">
         <v>46256</v>
       </c>
-      <c r="L57" s="23" t="n">
+      <c r="L58" s="15" t="n">
         <v>50000</v>
       </c>
-      <c r="M57" s="17" t="inlineStr">
+      <c r="M58" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
         </is>
       </c>
-      <c r="N57" s="20" t="inlineStr">
+      <c r="N58" s="12" t="inlineStr">
         <is>
           <t>selecao.bra@oei.int</t>
         </is>
       </c>
-      <c r="O57" s="24" t="inlineStr">
+      <c r="O58" s="16" t="inlineStr">
         <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B59" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+        </is>
+      </c>
+      <c r="C59" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+        </is>
+      </c>
+      <c r="D59" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E59" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F59" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G59" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados</t>
+        </is>
+      </c>
+      <c r="H59" s="19" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I59" s="19" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
+      <c r="J59" s="22" t="n">
+        <v>46252</v>
+      </c>
+      <c r="K59" s="22" t="n">
+        <v>46259</v>
+      </c>
+      <c r="L59" s="23" t="n">
+        <v>60000</v>
+      </c>
+      <c r="M59" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N59" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O59" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B60" s="10" t="inlineStr">
+        <is>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E60" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F60" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G60" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados</t>
+        </is>
+      </c>
+      <c r="H60" s="11" t="inlineStr">
+        <is>
+          <t>OEI/MDHC</t>
+        </is>
+      </c>
+      <c r="I60" s="11" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="J60" s="14" t="n">
+        <v>46208</v>
+      </c>
+      <c r="K60" s="14" t="n">
+        <v>46259</v>
+      </c>
+      <c r="L60" s="15" t="n">
+        <v>500000</v>
+      </c>
+      <c r="M60" s="9" t="inlineStr">
+        <is>
+          <t>En presentación</t>
+        </is>
+      </c>
+      <c r="N60" s="12" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O60" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O57"/>
+  <autoFilter ref="A1:O60"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4586,6 +4763,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4630,21 +4810,21 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Pnud</t>
+          <t>Unesco</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Unesco</t>
+          <t>Pnud</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -4686,7 +4866,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3">
@@ -4748,7 +4928,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -4810,7 +4990,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3">
@@ -4820,7 +5000,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
@@ -4830,7 +5010,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5">
@@ -4928,21 +5108,21 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -5030,7 +5210,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5045,7 +5225,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5060,7 +5240,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5075,7 +5255,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-08-27 21:51
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 26/08/2026 às 12:51</t>
+          <t>Gerado em 27/08/2026 às 21:49</t>
         </is>
       </c>
     </row>
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -1822,12 +1822,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:ede6b983-4c99-440a-4777-08def936f411</t>
+          <t>unesco:eb67e949-3d0c-4334-df1b-08df01dbdf45</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ1154 - Edital 03/2026 - 01 perfil - Consultoria Individual </t>
+          <t>586RLA2002 - Edital 002/2026 - 1 vaga</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Saúde</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1855,10 +1855,10 @@
       </c>
       <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46251</v>
+        <v>46261</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46264</v>
+        <v>46272</v>
       </c>
       <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
@@ -1881,12 +1881,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:4ad4b204-cf32-4060-4778-08def936f411</t>
+          <t>unesco:ede6b983-4c99-440a-4777-08def936f411</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1154 - Edital 04/2026 - 01 perfil - Consultoria Individual</t>
+          <t xml:space="preserve">914BRZ1154 - Edital 03/2026 - 01 perfil - Consultoria Individual </t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1896,13 +1896,15 @@
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Saúde</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1938,12 +1940,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
+          <t>unesco:4ad4b204-cf32-4060-4778-08def936f411</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1154 - Edital 04/2026 - 01 perfil - Consultoria Individual</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -1953,15 +1955,13 @@
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F19" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="inlineStr"/>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -1971,10 +1971,10 @@
       </c>
       <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46253</v>
+        <v>46251</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46269</v>
+        <v>46264</v>
       </c>
       <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
@@ -1997,12 +1997,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:e7ac82d3-849f-4a69-8cae-08defc5a5785</t>
+          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 33/2026 - 2 vagas - Consultor Individual</t>
+          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2012,13 +2012,15 @@
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2028,10 +2030,10 @@
       </c>
       <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46258</v>
+        <v>46253</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46264</v>
+        <v>46269</v>
       </c>
       <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
@@ -2054,12 +2056,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:8a4f297f-a7f6-4db9-ebd4-08defdee4813</t>
+          <t>unesco:e7ac82d3-849f-4a69-8cae-08defc5a5785</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 34/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 33/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2069,15 +2071,13 @@
       </c>
       <c r="E21" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F21" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="inlineStr"/>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2087,7 +2087,7 @@
       </c>
       <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="22" t="n">
-        <v>46260</v>
+        <v>46258</v>
       </c>
       <c r="K21" s="22" t="n">
         <v>46264</v>
@@ -2113,12 +2113,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:1ade5265-d185-4752-ebd5-08defdee4813</t>
+          <t>unesco:8a4f297f-a7f6-4db9-ebd4-08defdee4813</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 35/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 34/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2136,7 +2136,7 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2172,12 +2172,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:e6ba376a-8848-485f-3f37-08defeb303ea</t>
+          <t>unesco:1ade5265-d185-4752-ebd5-08defdee4813</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1163 - Publicação -  Edital 67/2026 - 01 Vaga - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 35/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2208,7 +2208,7 @@
         <v>46260</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46266</v>
+        <v>46264</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2231,12 +2231,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:7155091d-98d5-4ce4-df16-08df01dbdf45</t>
+          <t>unesco:e6ba376a-8848-485f-3f37-08defeb303ea</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ4024 - EDITAL Nº03/2026 - Consultor Individual</t>
+          <t>914BRZ1163 - Publicação -  Edital 67/2026 - 01 Vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2246,13 +2246,15 @@
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F24" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2262,10 +2264,10 @@
       </c>
       <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
@@ -2288,30 +2290,28 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:3ace2443-618f-4dcd-3f59-08def87d335c</t>
+          <t>unesco:7155091d-98d5-4ce4-df16-08df01dbdf45</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ1085 - Edital nº 03/2026 - 02 vagas - Consultores Individuais</t>
+          <t>914BRZ4024 - EDITAL Nº03/2026 - Consultor Individual</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="inlineStr"/>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Saúde, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2321,10 +2321,10 @@
       </c>
       <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46251</v>
+        <v>46259</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46260</v>
+        <v>46265</v>
       </c>
       <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
@@ -2347,17 +2347,17 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:be7dda96-d11c-4774-ed52-08defa0191b8</t>
+          <t>unesco:9ecb033c-d905-4f6f-df1e-08df01dbdf45</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
+          <t>914BRZ4027 - Edital 54/2026 - Arquitetura e Urbanismo</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
@@ -2370,7 +2370,7 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2380,10 +2380,10 @@
       </c>
       <c r="I26" s="11" t="inlineStr"/>
       <c r="J26" s="14" t="n">
-        <v>46257</v>
+        <v>46261</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
@@ -2406,28 +2406,30 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:5a9d0c82-e38a-483b-ed53-08defa0191b8</t>
+          <t>unesco:be7dda96-d11c-4774-ed52-08defa0191b8</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 18/2026 (REPUBLICAÇÃO)</t>
+          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F27" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F27" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2463,17 +2465,17 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>unesco:902f516e-135f-4244-ed50-08defa0191b8</t>
+          <t>unesco:5a9d0c82-e38a-483b-ed53-08defa0191b8</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3061 - EDITAL Nº 12/2026 - 01 VAGA - CONSULTOR INDIVIDUAL - REPUBLICAÇAO</t>
+          <t>Projeto 914BRZ3051 - EDITAL 18/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -2494,10 +2496,10 @@
       </c>
       <c r="I28" s="11" t="inlineStr"/>
       <c r="J28" s="14" t="n">
-        <v>46255</v>
+        <v>46257</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46260</v>
+        <v>46264</v>
       </c>
       <c r="L28" s="15" t="inlineStr"/>
       <c r="M28" s="9" t="inlineStr">
@@ -2520,17 +2522,17 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13067</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
@@ -2543,7 +2545,7 @@
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2553,17 +2555,17 @@
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Secretaria de Estado da Educação  SEED-PR</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46212</v>
+        <v>46216</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46224</v>
+        <v>46223</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>150000</v>
+        <v>133000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
@@ -2577,7 +2579,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
         </is>
       </c>
     </row>
@@ -2656,12 +2658,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13067</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2679,7 +2681,7 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2689,21 +2691,21 @@
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Secretaria de Estado da Educação  SEED-PR</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46213</v>
+        <v>46212</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46217</v>
+        <v>46224</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>144000</v>
+        <v>150000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N31" s="20" t="inlineStr">
@@ -2713,7 +2715,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067/</t>
         </is>
       </c>
     </row>
@@ -2792,17 +2794,17 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
@@ -2815,7 +2817,7 @@
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
@@ -2825,21 +2827,21 @@
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46216</v>
+        <v>46213</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46223</v>
+        <v>46217</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>133000</v>
+        <v>144000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N33" s="20" t="inlineStr">
@@ -2849,7 +2851,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
         </is>
       </c>
     </row>
@@ -2861,12 +2863,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2880,11 +2882,11 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -2898,17 +2900,15 @@
         </is>
       </c>
       <c r="J34" s="14" t="n">
+        <v>46213</v>
+      </c>
+      <c r="K34" s="14" t="n">
         <v>46220</v>
       </c>
-      <c r="K34" s="14" t="n">
-        <v>46225</v>
-      </c>
-      <c r="L34" s="15" t="n">
-        <v>58800</v>
-      </c>
+      <c r="L34" s="15" t="inlineStr"/>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -2918,7 +2918,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
         </is>
       </c>
     </row>
@@ -2930,17 +2930,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -2949,11 +2949,11 @@
         </is>
       </c>
       <c r="F35" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -2967,15 +2967,17 @@
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46221</v>
+        <v>46220</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46224</v>
-      </c>
-      <c r="L35" s="23" t="inlineStr"/>
+        <v>46225</v>
+      </c>
+      <c r="L35" s="23" t="n">
+        <v>58800</v>
+      </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N35" s="20" t="inlineStr">
@@ -2985,7 +2987,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
         </is>
       </c>
     </row>
@@ -2997,17 +2999,17 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
@@ -3020,7 +3022,7 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3034,15 +3036,15 @@
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46213</v>
+        <v>46221</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46220</v>
+        <v>46224</v>
       </c>
       <c r="L36" s="15" t="inlineStr"/>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N36" s="12" t="inlineStr">
@@ -3052,7 +3054,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
         </is>
       </c>
     </row>
@@ -3202,12 +3204,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR 12970</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3221,7 +3223,7 @@
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
@@ -3235,18 +3237,16 @@
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Brasília DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46227</v>
+        <v>46183</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46231</v>
-      </c>
-      <c r="L39" s="23" t="n">
-        <v>150000</v>
-      </c>
+        <v>46188</v>
+      </c>
+      <c r="L39" s="23" t="inlineStr"/>
       <c r="M39" s="17" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
@@ -3259,7 +3259,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970/</t>
         </is>
       </c>
     </row>
@@ -3271,12 +3271,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3294,27 +3294,27 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46233</v>
+        <v>46229</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>288000</v>
+        <v>114600</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3328,7 +3328,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
         </is>
       </c>
     </row>
@@ -3340,12 +3340,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR 12970</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3359,7 +3359,7 @@
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
@@ -3373,16 +3373,18 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46183</v>
+        <v>46227</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46188</v>
-      </c>
-      <c r="L41" s="23" t="inlineStr"/>
+        <v>46231</v>
+      </c>
+      <c r="L41" s="23" t="n">
+        <v>150000</v>
+      </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
@@ -3395,7 +3397,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -3407,12 +3409,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3430,27 +3432,27 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46225</v>
+        <v>46224</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46229</v>
+        <v>46233</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>114600</v>
+        <v>288000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3464,7 +3466,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -3476,30 +3478,28 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F43" s="21" t="n">
-        <v>0.343</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F43" s="21" t="inlineStr"/>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -3545,28 +3545,30 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F44" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F44" s="13" t="n">
+        <v>0.343</v>
+      </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
@@ -3600,7 +3602,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -3612,12 +3614,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3635,27 +3637,27 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46245</v>
+        <v>46237</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>80000</v>
+        <v>288000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
@@ -3669,7 +3671,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -3681,12 +3683,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3704,7 +3706,7 @@
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3724,7 +3726,7 @@
         <v>46245</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>100000</v>
+        <v>204000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3738,7 +3740,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -3750,12 +3752,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3773,7 +3775,7 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
@@ -3793,7 +3795,7 @@
         <v>46245</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>80000</v>
+        <v>204000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
@@ -3807,7 +3809,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -3819,12 +3821,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3842,7 +3844,7 @@
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
@@ -3862,7 +3864,7 @@
         <v>46245</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>204000</v>
+        <v>80000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3876,7 +3878,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -3888,17 +3890,17 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
@@ -3911,41 +3913,41 @@
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46232</v>
+        <v>46244</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46237</v>
+        <v>46296</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>288000</v>
+        <v>935000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -3957,12 +3959,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -3990,7 +3992,7 @@
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
@@ -4000,7 +4002,7 @@
         <v>46245</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>204000</v>
+        <v>80000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
@@ -4014,7 +4016,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -4026,64 +4028,62 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F51" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F51" s="21" t="inlineStr"/>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46244</v>
+        <v>46227</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46300</v>
+        <v>46252</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>350000</v>
+        <v>286000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -4095,17 +4095,17 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
@@ -4123,36 +4123,36 @@
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46244</v>
+        <v>46240</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46296</v>
+        <v>46245</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>935000</v>
+        <v>100000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -4164,62 +4164,64 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F53" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F53" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46227</v>
+        <v>46244</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46252</v>
+        <v>46300</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>286000</v>
+        <v>350000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N53" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4231,12 +4233,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4250,35 +4252,33 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
         <v>46246</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46257</v>
-      </c>
-      <c r="L54" s="15" t="n">
-        <v>54000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L54" s="15" t="inlineStr"/>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
@@ -4288,7 +4288,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -4369,12 +4369,12 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
@@ -4388,33 +4388,35 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
         <v>46246</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L56" s="15" t="inlineStr"/>
+        <v>46257</v>
+      </c>
+      <c r="L56" s="15" t="n">
+        <v>54000</v>
+      </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
@@ -4424,7 +4426,7 @@
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -4436,17 +4438,17 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
@@ -4459,7 +4461,7 @@
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
@@ -4469,17 +4471,17 @@
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46257</v>
+        <v>46256</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
@@ -4493,7 +4495,7 @@
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -4505,17 +4507,17 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
@@ -4528,7 +4530,7 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
@@ -4538,17 +4540,17 @@
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46256</v>
+        <v>46259</v>
       </c>
       <c r="L58" s="15" t="n">
-        <v>50000</v>
+        <v>60000</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
@@ -4562,7 +4564,7 @@
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -4574,12 +4576,12 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
@@ -4597,7 +4599,7 @@
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
@@ -4607,21 +4609,21 @@
       </c>
       <c r="I59" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J59" s="22" t="n">
-        <v>46252</v>
+        <v>46246</v>
       </c>
       <c r="K59" s="22" t="n">
-        <v>46259</v>
+        <v>46272</v>
       </c>
       <c r="L59" s="23" t="n">
-        <v>60000</v>
+        <v>54000</v>
       </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N59" s="20" t="inlineStr">
@@ -4631,7 +4633,7 @@
       </c>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -4866,7 +4868,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3">
@@ -4876,7 +4878,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -4918,7 +4920,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
@@ -4928,7 +4930,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -5000,7 +5002,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4">
@@ -5010,7 +5012,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
@@ -5020,7 +5022,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -5046,7 +5048,7 @@
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Direito / Jurídico</t>
         </is>
       </c>
       <c r="B8" s="10" t="n">
@@ -5056,11 +5058,11 @@
     <row r="9">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Direito / Jurídico</t>
+          <t>Saúde</t>
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -5210,7 +5212,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5225,7 +5227,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5240,7 +5242,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5255,7 +5257,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-08-28 21:48
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$65</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 27/08/2026 às 21:49</t>
+          <t>Gerado em 28/08/2026 às 21:46</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="24">
@@ -762,7 +762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O60"/>
+  <dimension ref="A1:O65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1699,17 +1699,15 @@
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>unesco:cce39a92-3e1c-4533-6f2c-08def7ab12e1</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="n">
+        <v>146346</v>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3057 - Edital nº 03/2026 - 1 vaga - Consultor individual</t>
+          <t>Contratação de consultor (a) individual para assessoramento técnico especializado à consolidação, redação técnica e estruturação dos mecanismos de governança do Plano Estadual de Educação do Piauí 2026-2036</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1727,48 +1725,56 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I15" s="19" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I15" s="19" t="inlineStr">
+        <is>
+          <t>Home based</t>
+        </is>
+      </c>
       <c r="J15" s="22" t="n">
-        <v>46258</v>
+        <v>46262</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46262</v>
-      </c>
-      <c r="L15" s="23" t="inlineStr"/>
+        <v>46276</v>
+      </c>
+      <c r="L15" s="23" t="n">
+        <v>79200</v>
+      </c>
       <c r="M15" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N15" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N15" s="20" t="inlineStr">
+        <is>
+          <t>ugest@seduc.pi.gov.br</t>
+        </is>
+      </c>
       <c r="O15" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>unesco:07727145-a919-4540-98cd-08dee32d8e84</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>146347</v>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ5019 - Edital 3/2026 - 01 vaga - Consultor Individual</t>
+          <t>Contratação de consultor (a) individual para apoiar tecnicamente a Superintendência de Ensino na realização das Olimpíadas do Conhecimento</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1791,26 +1797,36 @@
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I16" s="11" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>Home based</t>
+        </is>
+      </c>
       <c r="J16" s="14" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46265</v>
-      </c>
-      <c r="L16" s="15" t="inlineStr"/>
+        <v>46276</v>
+      </c>
+      <c r="L16" s="15" t="n">
+        <v>51000</v>
+      </c>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N16" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N16" s="12" t="inlineStr">
+        <is>
+          <t>ugest@seduc.pi.gov.br</t>
+        </is>
+      </c>
       <c r="O16" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -1822,12 +1838,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:eb67e949-3d0c-4334-df1b-08df01dbdf45</t>
+          <t>unesco:cce39a92-3e1c-4533-6f2c-08def7ab12e1</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>586RLA2002 - Edital 002/2026 - 1 vaga</t>
+          <t>914BRZ3057 - Edital nº 03/2026 - 1 vaga - Consultor individual</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1845,7 +1861,7 @@
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1855,10 +1871,10 @@
       </c>
       <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46261</v>
+        <v>46258</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46272</v>
+        <v>46262</v>
       </c>
       <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
@@ -1881,12 +1897,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:ede6b983-4c99-440a-4777-08def936f411</t>
+          <t>unesco:07727145-a919-4540-98cd-08dee32d8e84</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ1154 - Edital 03/2026 - 01 perfil - Consultoria Individual </t>
+          <t>914BRZ5019 - Edital 3/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1904,7 +1920,7 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Saúde</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1914,10 +1930,10 @@
       </c>
       <c r="I18" s="11" t="inlineStr"/>
       <c r="J18" s="14" t="n">
-        <v>46251</v>
+        <v>46255</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
@@ -1940,12 +1956,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:4ad4b204-cf32-4060-4778-08def936f411</t>
+          <t>unesco:eb67e949-3d0c-4334-df1b-08df01dbdf45</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1154 - Edital 04/2026 - 01 perfil - Consultoria Individual</t>
+          <t>586RLA2002 - Edital 002/2026 - 1 vaga</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -1955,13 +1971,15 @@
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F19" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -1971,10 +1989,10 @@
       </c>
       <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46251</v>
+        <v>46261</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46264</v>
+        <v>46272</v>
       </c>
       <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
@@ -1997,12 +2015,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
+          <t>unesco:ede6b983-4c99-440a-4777-08def936f411</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
+          <t xml:space="preserve">914BRZ1154 - Edital 03/2026 - 01 perfil - Consultoria Individual </t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2020,7 +2038,7 @@
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Saúde</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2030,10 +2048,10 @@
       </c>
       <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46253</v>
+        <v>46251</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46269</v>
+        <v>46264</v>
       </c>
       <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
@@ -2056,12 +2074,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:e7ac82d3-849f-4a69-8cae-08defc5a5785</t>
+          <t>unesco:4ad4b204-cf32-4060-4778-08def936f411</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 33/2026 - 2 vagas - Consultor Individual</t>
+          <t>914BRZ1154 - Edital 04/2026 - 01 perfil - Consultoria Individual</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2087,7 +2105,7 @@
       </c>
       <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="22" t="n">
-        <v>46258</v>
+        <v>46251</v>
       </c>
       <c r="K21" s="22" t="n">
         <v>46264</v>
@@ -2113,12 +2131,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:8a4f297f-a7f6-4db9-ebd4-08defdee4813</t>
+          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 34/2026 - 1 vaga - Consultor Individual</t>
+          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2146,10 +2164,10 @@
       </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46260</v>
+        <v>46253</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46264</v>
+        <v>46269</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2172,12 +2190,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:1ade5265-d185-4752-ebd5-08defdee4813</t>
+          <t>unesco:e7ac82d3-849f-4a69-8cae-08defc5a5785</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 35/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 33/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2187,15 +2205,13 @@
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F23" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="inlineStr"/>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2205,7 +2221,7 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46260</v>
+        <v>46258</v>
       </c>
       <c r="K23" s="22" t="n">
         <v>46264</v>
@@ -2231,12 +2247,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:e6ba376a-8848-485f-3f37-08defeb303ea</t>
+          <t>unesco:8a4f297f-a7f6-4db9-ebd4-08defdee4813</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1163 - Publicação -  Edital 67/2026 - 01 Vaga - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 34/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2267,7 +2283,7 @@
         <v>46260</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46266</v>
+        <v>46264</v>
       </c>
       <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
@@ -2290,12 +2306,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:7155091d-98d5-4ce4-df16-08df01dbdf45</t>
+          <t>unesco:1ade5265-d185-4752-ebd5-08defdee4813</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ4024 - EDITAL Nº03/2026 - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 35/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2305,13 +2321,15 @@
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F25" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2321,10 +2339,10 @@
       </c>
       <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
@@ -2347,12 +2365,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:9ecb033c-d905-4f6f-df1e-08df01dbdf45</t>
+          <t>unesco:e6ba376a-8848-485f-3f37-08defeb303ea</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 54/2026 - Arquitetura e Urbanismo</t>
+          <t>914BRZ1163 - Publicação -  Edital 67/2026 - 01 Vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2370,7 +2388,7 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2380,10 +2398,10 @@
       </c>
       <c r="I26" s="11" t="inlineStr"/>
       <c r="J26" s="14" t="n">
-        <v>46261</v>
+        <v>46260</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
@@ -2406,30 +2424,28 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:be7dda96-d11c-4774-ed52-08defa0191b8</t>
+          <t>unesco:7155091d-98d5-4ce4-df16-08df01dbdf45</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
+          <t>914BRZ4024 - EDITAL Nº03/2026 - Consultor Individual</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F27" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F27" s="21" t="inlineStr"/>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2439,10 +2455,10 @@
       </c>
       <c r="I27" s="19" t="inlineStr"/>
       <c r="J27" s="22" t="n">
-        <v>46257</v>
+        <v>46259</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="L27" s="23" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr">
@@ -2465,28 +2481,30 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>unesco:5a9d0c82-e38a-483b-ed53-08defa0191b8</t>
+          <t>unesco:4fda0c36-f1a0-41f6-3f3a-08defeb303ea</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 18/2026 (REPUBLICAÇÃO)</t>
+          <t>914BRZ1155 - EDITAL Nº 47/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F28" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2496,10 +2514,10 @@
       </c>
       <c r="I28" s="11" t="inlineStr"/>
       <c r="J28" s="14" t="n">
-        <v>46257</v>
+        <v>46262</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46264</v>
+        <v>46268</v>
       </c>
       <c r="L28" s="15" t="inlineStr"/>
       <c r="M28" s="9" t="inlineStr">
@@ -2517,22 +2535,22 @@
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
+          <t>unesco:4db2e20b-a2e2-4074-00dc-08deff7b5e96</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
+          <t>914BRZ1155 - EDITAL Nº 49/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
@@ -2541,67 +2559,57 @@
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I29" s="19" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I29" s="19" t="inlineStr"/>
       <c r="J29" s="22" t="n">
-        <v>46216</v>
+        <v>46262</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46223</v>
-      </c>
-      <c r="L29" s="23" t="n">
-        <v>133000</v>
-      </c>
+        <v>46268</v>
+      </c>
+      <c r="L29" s="23" t="inlineStr"/>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N29" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N29" s="20" t="inlineStr"/>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-03-territorios-criativos-e-educacao-tr-13051</t>
+          <t>unesco:ecd2379c-2ba5-488f-00dd-08deff7b5e96</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-03 – Territórios Criativos e Educação – TR 13051</t>
+          <t>914BRZ1155 - EDITAL Nº 50/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2614,61 +2622,53 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I30" s="11" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="inlineStr"/>
       <c r="J30" s="14" t="n">
-        <v>46204</v>
+        <v>46262</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46209</v>
+        <v>46268</v>
       </c>
       <c r="L30" s="15" t="inlineStr"/>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N30" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N30" s="12" t="inlineStr"/>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-03-territorios-criativos-e-educacao-tr-13051/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067</t>
+          <t>unesco:9ecb033c-d905-4f6f-df1e-08df01dbdf45</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13067</t>
+          <t>914BRZ4027 - Edital 54/2026 - Arquitetura e Urbanismo</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
@@ -2677,7 +2677,7 @@
         </is>
       </c>
       <c r="F31" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
@@ -2686,58 +2686,48 @@
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I31" s="19" t="inlineStr">
-        <is>
-          <t>Secretaria de Estado da Educação  SEED-PR</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I31" s="19" t="inlineStr"/>
       <c r="J31" s="22" t="n">
-        <v>46212</v>
+        <v>46261</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46224</v>
-      </c>
-      <c r="L31" s="23" t="n">
-        <v>150000</v>
-      </c>
+        <v>46265</v>
+      </c>
+      <c r="L31" s="23" t="inlineStr"/>
       <c r="M31" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N31" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N31" s="20" t="inlineStr"/>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056</t>
+          <t>unesco:be7dda96-d11c-4774-ed52-08defa0191b8</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEC/BRA/24 – TR 13056</t>
+          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
@@ -2750,108 +2740,88 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I32" s="11" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I32" s="11" t="inlineStr"/>
       <c r="J32" s="14" t="n">
-        <v>46209</v>
+        <v>46257</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46214</v>
+        <v>46264</v>
       </c>
       <c r="L32" s="15" t="inlineStr"/>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N32" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N32" s="12" t="inlineStr"/>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
+          <t>unesco:5a9d0c82-e38a-483b-ed53-08defa0191b8</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
+          <t>Projeto 914BRZ3051 - EDITAL 18/2026 (REPUBLICAÇÃO)</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E33" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F33" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F33" s="21" t="inlineStr"/>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I33" s="19" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I33" s="19" t="inlineStr"/>
       <c r="J33" s="22" t="n">
-        <v>46213</v>
+        <v>46257</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46217</v>
-      </c>
-      <c r="L33" s="23" t="n">
-        <v>144000</v>
-      </c>
+        <v>46264</v>
+      </c>
+      <c r="L33" s="23" t="inlineStr"/>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N33" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N33" s="20" t="inlineStr"/>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -2863,17 +2833,17 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13067</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -2882,11 +2852,11 @@
         </is>
       </c>
       <c r="F34" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -2896,19 +2866,21 @@
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Secretaria de Estado da Educação  SEED-PR</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46213</v>
+        <v>46212</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46220</v>
-      </c>
-      <c r="L34" s="15" t="inlineStr"/>
+        <v>46224</v>
+      </c>
+      <c r="L34" s="15" t="n">
+        <v>150000</v>
+      </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -2918,7 +2890,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067/</t>
         </is>
       </c>
     </row>
@@ -2930,12 +2902,12 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEC/BRA/24 – TR 13056</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -2949,16 +2921,16 @@
         </is>
       </c>
       <c r="F35" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
@@ -2967,17 +2939,15 @@
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46220</v>
+        <v>46209</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46225</v>
-      </c>
-      <c r="L35" s="23" t="n">
-        <v>58800</v>
-      </c>
+        <v>46214</v>
+      </c>
+      <c r="L35" s="23" t="inlineStr"/>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N35" s="20" t="inlineStr">
@@ -2987,7 +2957,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056/</t>
         </is>
       </c>
     </row>
@@ -2999,17 +2969,17 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
@@ -3018,11 +2988,11 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3032,19 +3002,21 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46221</v>
+        <v>46216</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46224</v>
-      </c>
-      <c r="L36" s="15" t="inlineStr"/>
+        <v>46223</v>
+      </c>
+      <c r="L36" s="15" t="n">
+        <v>133000</v>
+      </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N36" s="12" t="inlineStr">
@@ -3054,7 +3026,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
         </is>
       </c>
     </row>
@@ -3066,12 +3038,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-03-territorios-criativos-e-educacao-tr-13051</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-03 – Territórios Criativos e Educação – TR 13051</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3085,11 +3057,11 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3103,17 +3075,15 @@
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46217</v>
+        <v>46204</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46222</v>
-      </c>
-      <c r="L37" s="23" t="n">
-        <v>77100</v>
-      </c>
+        <v>46209</v>
+      </c>
+      <c r="L37" s="23" t="inlineStr"/>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N37" s="20" t="inlineStr">
@@ -3123,7 +3093,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-03-territorios-criativos-e-educacao-tr-13051/</t>
         </is>
       </c>
     </row>
@@ -3135,17 +3105,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3158,7 +3128,7 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3172,17 +3142,17 @@
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46223</v>
+        <v>46213</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46238</v>
+        <v>46217</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>100000</v>
+        <v>144000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
@@ -3192,7 +3162,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
         </is>
       </c>
     </row>
@@ -3204,12 +3174,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR 12970</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3223,11 +3193,11 @@
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3237,19 +3207,21 @@
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46183</v>
+        <v>46220</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46188</v>
-      </c>
-      <c r="L39" s="23" t="inlineStr"/>
+        <v>46225</v>
+      </c>
+      <c r="L39" s="23" t="n">
+        <v>58800</v>
+      </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
@@ -3259,7 +3231,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
         </is>
       </c>
     </row>
@@ -3271,17 +3243,17 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
@@ -3290,11 +3262,11 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3304,21 +3276,19 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46225</v>
+        <v>46221</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46229</v>
-      </c>
-      <c r="L40" s="15" t="n">
-        <v>114600</v>
-      </c>
+        <v>46224</v>
+      </c>
+      <c r="L40" s="15" t="inlineStr"/>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
@@ -3328,7 +3298,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
         </is>
       </c>
     </row>
@@ -3340,12 +3310,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3359,11 +3329,11 @@
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3373,18 +3343,16 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Brasília DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46227</v>
+        <v>46213</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46231</v>
-      </c>
-      <c r="L41" s="23" t="n">
-        <v>150000</v>
-      </c>
+        <v>46220</v>
+      </c>
+      <c r="L41" s="23" t="inlineStr"/>
       <c r="M41" s="17" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
@@ -3397,7 +3365,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
         </is>
       </c>
     </row>
@@ -3409,12 +3377,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3432,7 +3400,7 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3442,17 +3410,17 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46224</v>
+        <v>46217</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46233</v>
+        <v>46222</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>288000</v>
+        <v>77100</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3466,7 +3434,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
         </is>
       </c>
     </row>
@@ -3478,48 +3446,50 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F43" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F43" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46232</v>
+        <v>46223</v>
       </c>
       <c r="K43" s="22" t="n">
         <v>46238</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>30000</v>
+        <v>100000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
@@ -3533,7 +3503,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
         </is>
       </c>
     </row>
@@ -3545,17 +3515,17 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
@@ -3564,31 +3534,31 @@
         </is>
       </c>
       <c r="F44" s="13" t="n">
-        <v>0.343</v>
+        <v>0.4</v>
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46232</v>
+        <v>46225</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46238</v>
+        <v>46229</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>30000</v>
+        <v>114600</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
@@ -3602,7 +3572,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
         </is>
       </c>
     </row>
@@ -3614,12 +3584,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR 12970</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3633,11 +3603,11 @@
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
@@ -3647,21 +3617,19 @@
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46232</v>
+        <v>46183</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46237</v>
-      </c>
-      <c r="L45" s="23" t="n">
-        <v>288000</v>
-      </c>
+        <v>46188</v>
+      </c>
+      <c r="L45" s="23" t="inlineStr"/>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
@@ -3671,7 +3639,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970/</t>
         </is>
       </c>
     </row>
@@ -3683,12 +3651,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3711,26 +3679,26 @@
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46240</v>
+        <v>46227</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46245</v>
+        <v>46231</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>204000</v>
+        <v>150000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
@@ -3740,7 +3708,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -3752,12 +3720,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3775,7 +3743,7 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
@@ -3785,17 +3753,17 @@
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46240</v>
+        <v>46224</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46245</v>
+        <v>46233</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>204000</v>
+        <v>288000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
@@ -3809,7 +3777,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -3821,12 +3789,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3836,15 +3804,13 @@
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F48" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F48" s="13" t="inlineStr"/>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
@@ -3854,17 +3820,17 @@
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>80000</v>
+        <v>30000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3878,7 +3844,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -3890,17 +3856,17 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
@@ -3909,45 +3875,45 @@
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.4</v>
+        <v>0.343</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46244</v>
+        <v>46232</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46296</v>
+        <v>46238</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>935000</v>
+        <v>30000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -3959,12 +3925,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -3982,27 +3948,27 @@
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46245</v>
+        <v>46237</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>80000</v>
+        <v>288000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
@@ -4016,7 +3982,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -4028,12 +3994,12 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -4043,33 +4009,35 @@
       </c>
       <c r="E51" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F51" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F51" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46227</v>
+        <v>46240</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46252</v>
+        <v>46245</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>286000</v>
+        <v>80000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
@@ -4083,7 +4051,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -4164,17 +4132,17 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
@@ -4187,41 +4155,41 @@
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46244</v>
+        <v>46240</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46300</v>
+        <v>46245</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>350000</v>
+        <v>80000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N53" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -4233,12 +4201,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4252,11 +4220,11 @@
         </is>
       </c>
       <c r="F54" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
@@ -4266,19 +4234,21 @@
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L54" s="15" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L54" s="15" t="n">
+        <v>204000</v>
+      </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
@@ -4288,7 +4258,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -4300,12 +4270,12 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
@@ -4323,27 +4293,27 @@
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46257</v>
+        <v>46245</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>54000</v>
+        <v>204000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
@@ -4357,7 +4327,7 @@
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -4369,17 +4339,17 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
@@ -4392,41 +4362,41 @@
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46246</v>
+        <v>46244</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46257</v>
+        <v>46300</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>54000</v>
+        <v>350000</v>
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4438,17 +4408,17 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
@@ -4461,7 +4431,7 @@
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
@@ -4471,17 +4441,17 @@
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
@@ -4495,7 +4465,7 @@
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -4507,17 +4477,17 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
@@ -4530,41 +4500,41 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46252</v>
+        <v>46244</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46259</v>
+        <v>46296</v>
       </c>
       <c r="L58" s="15" t="n">
-        <v>60000</v>
+        <v>935000</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N58" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4576,12 +4546,12 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
@@ -4599,7 +4569,7 @@
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
@@ -4616,14 +4586,14 @@
         <v>46246</v>
       </c>
       <c r="K59" s="22" t="n">
-        <v>46272</v>
+        <v>46257</v>
       </c>
       <c r="L59" s="23" t="n">
         <v>54000</v>
       </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N59" s="20" t="inlineStr">
@@ -4633,7 +4603,7 @@
       </c>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -4645,69 +4615,410 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E60" s="12" t="inlineStr">
+        <is>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F60" s="13" t="inlineStr"/>
+      <c r="G60" s="11" t="inlineStr">
+        <is>
+          <t>Não classificada</t>
+        </is>
+      </c>
+      <c r="H60" s="11" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I60" s="11" t="inlineStr">
+        <is>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+        </is>
+      </c>
+      <c r="J60" s="14" t="n">
+        <v>46227</v>
+      </c>
+      <c r="K60" s="14" t="n">
+        <v>46252</v>
+      </c>
+      <c r="L60" s="15" t="n">
+        <v>286000</v>
+      </c>
+      <c r="M60" s="9" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N60" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O60" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B61" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+        </is>
+      </c>
+      <c r="C61" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+        </is>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E61" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F61" s="21" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G61" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H61" s="19" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I61" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - DF | Híbrido</t>
+        </is>
+      </c>
+      <c r="J61" s="22" t="n">
+        <v>46246</v>
+      </c>
+      <c r="K61" s="22" t="n">
+        <v>46250</v>
+      </c>
+      <c r="L61" s="23" t="inlineStr"/>
+      <c r="M61" s="17" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N61" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O61" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+        </is>
+      </c>
+      <c r="C62" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+        </is>
+      </c>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+        </is>
+      </c>
+      <c r="E62" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F62" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G62" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H62" s="11" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I62" s="11" t="inlineStr">
+        <is>
+          <t>Recife - PE</t>
+        </is>
+      </c>
+      <c r="J62" s="14" t="n">
+        <v>46251</v>
+      </c>
+      <c r="K62" s="14" t="n">
+        <v>46256</v>
+      </c>
+      <c r="L62" s="15" t="n">
+        <v>50000</v>
+      </c>
+      <c r="M62" s="9" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N62" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O62" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B63" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+        </is>
+      </c>
+      <c r="C63" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+        </is>
+      </c>
+      <c r="D63" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E63" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F63" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G63" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados</t>
+        </is>
+      </c>
+      <c r="H63" s="19" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I63" s="19" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
+      <c r="J63" s="22" t="n">
+        <v>46252</v>
+      </c>
+      <c r="K63" s="22" t="n">
+        <v>46259</v>
+      </c>
+      <c r="L63" s="23" t="n">
+        <v>60000</v>
+      </c>
+      <c r="M63" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N63" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O63" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B64" s="10" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+        </is>
+      </c>
+      <c r="C64" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+        </is>
+      </c>
+      <c r="D64" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E64" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F64" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G64" s="11" t="inlineStr">
+        <is>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+        </is>
+      </c>
+      <c r="H64" s="11" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I64" s="11" t="inlineStr">
+        <is>
+          <t>Porto Alegre/RS</t>
+        </is>
+      </c>
+      <c r="J64" s="14" t="n">
+        <v>46246</v>
+      </c>
+      <c r="K64" s="14" t="n">
+        <v>46272</v>
+      </c>
+      <c r="L64" s="15" t="n">
+        <v>54000</v>
+      </c>
+      <c r="M64" s="9" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N64" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O64" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B65" s="18" t="inlineStr">
+        <is>
           <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
-      <c r="C60" s="11" t="inlineStr">
+      <c r="C65" s="19" t="inlineStr">
         <is>
           <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
-      <c r="D60" s="11" t="inlineStr">
+      <c r="D65" s="19" t="inlineStr">
         <is>
           <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
-      <c r="E60" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F60" s="13" t="n">
+      <c r="E65" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F65" s="21" t="n">
         <v>0.4</v>
       </c>
-      <c r="G60" s="11" t="inlineStr">
+      <c r="G65" s="19" t="inlineStr">
         <is>
           <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
-      <c r="H60" s="11" t="inlineStr">
+      <c r="H65" s="19" t="inlineStr">
         <is>
           <t>OEI/MDHC</t>
         </is>
       </c>
-      <c r="I60" s="11" t="inlineStr">
+      <c r="I65" s="19" t="inlineStr">
         <is>
           <t>Nacional</t>
         </is>
       </c>
-      <c r="J60" s="14" t="n">
+      <c r="J65" s="22" t="n">
         <v>46208</v>
       </c>
-      <c r="K60" s="14" t="n">
+      <c r="K65" s="22" t="n">
         <v>46259</v>
       </c>
-      <c r="L60" s="15" t="n">
+      <c r="L65" s="23" t="n">
         <v>500000</v>
       </c>
-      <c r="M60" s="9" t="inlineStr">
+      <c r="M65" s="17" t="inlineStr">
         <is>
           <t>En presentación</t>
         </is>
       </c>
-      <c r="N60" s="12" t="inlineStr">
+      <c r="N65" s="20" t="inlineStr">
         <is>
           <t>compras.bra@oei.int</t>
         </is>
       </c>
-      <c r="O60" s="16" t="inlineStr">
+      <c r="O65" s="24" t="inlineStr">
         <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O60"/>
+  <autoFilter ref="A1:O65"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4768,6 +5079,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId64"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4816,7 +5132,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4">
@@ -4826,7 +5142,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -4868,7 +5184,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3">
@@ -4916,21 +5232,21 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4">
@@ -4992,7 +5308,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3">
@@ -5002,7 +5318,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
@@ -5012,7 +5328,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5">
@@ -5028,17 +5344,17 @@
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Economia / Finanças Públicas</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Economia / Finanças Públicas</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
@@ -5100,7 +5416,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
@@ -5110,11 +5426,11 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4">
@@ -5130,21 +5446,21 @@
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -5212,7 +5528,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5227,7 +5543,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5242,7 +5558,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5257,7 +5573,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-08-31 18:52
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,11 +17,11 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$58</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Por_Perfil'!$A$1:$B$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Por_Perfil'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Por_Perfil'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Por_Tipo'!$A$1:$B$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Por_Tipo'!$1:$1</definedName>
@@ -552,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 28/08/2026 às 21:46</t>
+          <t>Gerado em 31/08/2026 às 18:50</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6">
@@ -644,21 +644,21 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>PNUD</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>PNUD</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>175942.3076923077</v>
+        <v>170537.0370370371</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>114600</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,17 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -762,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O65"/>
+  <dimension ref="A1:O58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1744,9 +1754,7 @@
       <c r="K15" s="22" t="n">
         <v>46276</v>
       </c>
-      <c r="L15" s="23" t="n">
-        <v>79200</v>
-      </c>
+      <c r="L15" s="23" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1811,9 +1819,7 @@
       <c r="K16" s="14" t="n">
         <v>46276</v>
       </c>
-      <c r="L16" s="15" t="n">
-        <v>51000</v>
-      </c>
+      <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1838,12 +1844,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:cce39a92-3e1c-4533-6f2c-08def7ab12e1</t>
+          <t>unesco:07727145-a919-4540-98cd-08dee32d8e84</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3057 - Edital nº 03/2026 - 1 vaga - Consultor individual</t>
+          <t>914BRZ5019 - Edital 3/2026 - 01 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1861,7 +1867,7 @@
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1871,10 +1877,10 @@
       </c>
       <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46258</v>
+        <v>46255</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
@@ -1897,12 +1903,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:07727145-a919-4540-98cd-08dee32d8e84</t>
+          <t>unesco:eb67e949-3d0c-4334-df1b-08df01dbdf45</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ5019 - Edital 3/2026 - 01 vaga - Consultor Individual</t>
+          <t>586RLA2002 - Edital 002/2026 - 1 vaga</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1920,7 +1926,7 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1930,10 +1936,10 @@
       </c>
       <c r="I18" s="11" t="inlineStr"/>
       <c r="J18" s="14" t="n">
-        <v>46255</v>
+        <v>46261</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46265</v>
+        <v>46272</v>
       </c>
       <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
@@ -1956,12 +1962,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:eb67e949-3d0c-4334-df1b-08df01dbdf45</t>
+          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>586RLA2002 - Edital 002/2026 - 1 vaga</t>
+          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -1979,7 +1985,7 @@
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -1989,10 +1995,10 @@
       </c>
       <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46261</v>
+        <v>46253</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46272</v>
+        <v>46269</v>
       </c>
       <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
@@ -2015,12 +2021,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:ede6b983-4c99-440a-4777-08def936f411</t>
+          <t>unesco:17177a8d-bde0-4a60-df1c-08df01dbdf45</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">914BRZ1154 - Edital 03/2026 - 01 perfil - Consultoria Individual </t>
+          <t>914BRZ1159 - Publicação Edital 36/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2038,7 +2044,7 @@
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Saúde</t>
+          <t>Saúde, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2048,10 +2054,10 @@
       </c>
       <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46251</v>
+        <v>46265</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46264</v>
+        <v>46271</v>
       </c>
       <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
@@ -2074,12 +2080,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:4ad4b204-cf32-4060-4778-08def936f411</t>
+          <t>unesco:e6ba376a-8848-485f-3f37-08defeb303ea</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1154 - Edital 04/2026 - 01 perfil - Consultoria Individual</t>
+          <t>914BRZ1163 - Publicação -  Edital 67/2026 - 01 Vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2089,13 +2095,15 @@
       </c>
       <c r="E21" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F21" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2105,10 +2113,10 @@
       </c>
       <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="22" t="n">
-        <v>46251</v>
+        <v>46260</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46264</v>
+        <v>46266</v>
       </c>
       <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
@@ -2131,12 +2139,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
+          <t>unesco:7155091d-98d5-4ce4-df16-08df01dbdf45</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ4024 - EDITAL Nº03/2026 - Consultor Individual</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2146,15 +2154,13 @@
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr"/>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2164,10 +2170,10 @@
       </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46253</v>
+        <v>46259</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46269</v>
+        <v>46265</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2190,12 +2196,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:e7ac82d3-849f-4a69-8cae-08defc5a5785</t>
+          <t>unesco:4fda0c36-f1a0-41f6-3f3a-08defeb303ea</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 33/2026 - 2 vagas - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 47/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2205,13 +2211,15 @@
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F23" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2221,10 +2229,10 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46258</v>
+        <v>46262</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46264</v>
+        <v>46268</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2247,12 +2255,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:8a4f297f-a7f6-4db9-ebd4-08defdee4813</t>
+          <t>unesco:4db2e20b-a2e2-4074-00dc-08deff7b5e96</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 34/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 49/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2270,7 +2278,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2280,10 +2288,10 @@
       </c>
       <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46264</v>
+        <v>46268</v>
       </c>
       <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
@@ -2306,12 +2314,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:1ade5265-d185-4752-ebd5-08defdee4813</t>
+          <t>unesco:ecd2379c-2ba5-488f-00dd-08deff7b5e96</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 35/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 50/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2329,7 +2337,7 @@
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2339,10 +2347,10 @@
       </c>
       <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46260</v>
+        <v>46262</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46264</v>
+        <v>46268</v>
       </c>
       <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
@@ -2365,12 +2373,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:e6ba376a-8848-485f-3f37-08defeb303ea</t>
+          <t>unesco:9ecb033c-d905-4f6f-df1e-08df01dbdf45</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1163 - Publicação -  Edital 67/2026 - 01 Vaga - Consultor Individual</t>
+          <t>914BRZ4027 - Edital 54/2026 - Arquitetura e Urbanismo</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2388,7 +2396,7 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2398,10 +2406,10 @@
       </c>
       <c r="I26" s="11" t="inlineStr"/>
       <c r="J26" s="14" t="n">
-        <v>46260</v>
+        <v>46261</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
@@ -2419,79 +2427,89 @@
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:7155091d-98d5-4ce4-df16-08df01dbdf45</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>914BRZ4024 - EDITAL Nº03/2026 - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEC/BRA/24 – TR 13056</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F27" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F27" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I27" s="19" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I27" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J27" s="22" t="n">
-        <v>46259</v>
+        <v>46209</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46265</v>
+        <v>46214</v>
       </c>
       <c r="L27" s="23" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N27" s="20" t="inlineStr"/>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N27" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>unesco:4fda0c36-f1a0-41f6-3f3a-08defeb303ea</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 47/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13067</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -2500,57 +2518,67 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I28" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr">
+        <is>
+          <t>Secretaria de Estado da Educação  SEED-PR</t>
+        </is>
+      </c>
       <c r="J28" s="14" t="n">
-        <v>46262</v>
+        <v>46212</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46268</v>
-      </c>
-      <c r="L28" s="15" t="inlineStr"/>
+        <v>46224</v>
+      </c>
+      <c r="L28" s="15" t="n">
+        <v>150000</v>
+      </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N28" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N28" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>unesco:4db2e20b-a2e2-4074-00dc-08deff7b5e96</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 49/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
@@ -2559,57 +2587,67 @@
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I29" s="19" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I29" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J29" s="22" t="n">
-        <v>46262</v>
+        <v>46217</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46268</v>
-      </c>
-      <c r="L29" s="23" t="inlineStr"/>
+        <v>46222</v>
+      </c>
+      <c r="L29" s="23" t="n">
+        <v>77100</v>
+      </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N29" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N29" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>unesco:ecd2379c-2ba5-488f-00dd-08deff7b5e96</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 50/2026 - 2 vagas - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2618,57 +2656,67 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I30" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J30" s="14" t="n">
-        <v>46262</v>
+        <v>46213</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46268</v>
-      </c>
-      <c r="L30" s="15" t="inlineStr"/>
+        <v>46217</v>
+      </c>
+      <c r="L30" s="15" t="n">
+        <v>144000</v>
+      </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N30" s="12" t="inlineStr"/>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N30" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>unesco:9ecb033c-d905-4f6f-df1e-08df01dbdf45</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 54/2026 - Arquitetura e Urbanismo</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
@@ -2681,53 +2729,61 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I31" s="19" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I31" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J31" s="22" t="n">
-        <v>46261</v>
+        <v>46213</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46265</v>
+        <v>46220</v>
       </c>
       <c r="L31" s="23" t="inlineStr"/>
       <c r="M31" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N31" s="20" t="inlineStr"/>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N31" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>unesco:be7dda96-d11c-4774-ed52-08defa0191b8</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 17/2026 (REPUBLICAÇÃO)</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
@@ -2736,52 +2792,62 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I32" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I32" s="11" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
       <c r="J32" s="14" t="n">
-        <v>46257</v>
+        <v>46216</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46264</v>
-      </c>
-      <c r="L32" s="15" t="inlineStr"/>
+        <v>46223</v>
+      </c>
+      <c r="L32" s="15" t="n">
+        <v>133000</v>
+      </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N32" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N32" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>unesco:5a9d0c82-e38a-483b-ed53-08defa0191b8</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3051 - EDITAL 18/2026 (REPUBLICAÇÃO)</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR 12970</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2791,37 +2857,47 @@
       </c>
       <c r="E33" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F33" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F33" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I33" s="19" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I33" s="19" t="inlineStr">
+        <is>
+          <t>Recife - PE</t>
+        </is>
+      </c>
       <c r="J33" s="22" t="n">
-        <v>46257</v>
+        <v>46183</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46264</v>
+        <v>46188</v>
       </c>
       <c r="L33" s="23" t="inlineStr"/>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N33" s="20" t="inlineStr"/>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N33" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970/</t>
         </is>
       </c>
     </row>
@@ -2833,17 +2909,17 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13067</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -2856,7 +2932,7 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -2866,17 +2942,17 @@
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Secretaria de Estado da Educação  SEED-PR</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46212</v>
+        <v>46220</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46224</v>
+        <v>46225</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>150000</v>
+        <v>58800</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
@@ -2890,7 +2966,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
         </is>
       </c>
     </row>
@@ -2902,17 +2978,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEC/BRA/24 – TR 13056</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -2925,12 +3001,12 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
@@ -2939,15 +3015,15 @@
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46209</v>
+        <v>46221</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46214</v>
+        <v>46224</v>
       </c>
       <c r="L35" s="23" t="inlineStr"/>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N35" s="20" t="inlineStr">
@@ -2957,7 +3033,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
         </is>
       </c>
     </row>
@@ -2969,17 +3045,17 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
@@ -2992,7 +3068,7 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3002,17 +3078,17 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46216</v>
+        <v>46223</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46223</v>
+        <v>46238</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>133000</v>
+        <v>100000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3026,7 +3102,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
         </is>
       </c>
     </row>
@@ -3038,12 +3114,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-03-territorios-criativos-e-educacao-tr-13051</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO FP-26-03 – Territórios Criativos e Educação – TR 13051</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3057,33 +3133,35 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46204</v>
+        <v>46225</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46209</v>
-      </c>
-      <c r="L37" s="23" t="inlineStr"/>
+        <v>46229</v>
+      </c>
+      <c r="L37" s="23" t="n">
+        <v>114600</v>
+      </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N37" s="20" t="inlineStr">
@@ -3093,7 +3171,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-fp-26-03-territorios-criativos-e-educacao-tr-13051/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
         </is>
       </c>
     </row>
@@ -3105,17 +3183,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3128,7 +3206,7 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3138,17 +3216,17 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46213</v>
+        <v>46227</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46217</v>
+        <v>46231</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>144000</v>
+        <v>150000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3162,7 +3240,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -3174,12 +3252,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3197,27 +3275,27 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46220</v>
+        <v>46224</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>58800</v>
+        <v>288000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3231,7 +3309,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -3243,52 +3321,52 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F40" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="inlineStr"/>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46221</v>
+        <v>46232</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46224</v>
-      </c>
-      <c r="L40" s="15" t="inlineStr"/>
+        <v>46238</v>
+      </c>
+      <c r="L40" s="15" t="n">
+        <v>30000</v>
+      </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
@@ -3298,7 +3376,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -3310,17 +3388,17 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
@@ -3329,33 +3407,35 @@
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.3</v>
+        <v>0.343</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46213</v>
+        <v>46232</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46220</v>
-      </c>
-      <c r="L41" s="23" t="inlineStr"/>
+        <v>46238</v>
+      </c>
+      <c r="L41" s="23" t="n">
+        <v>30000</v>
+      </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
@@ -3365,7 +3445,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -3377,12 +3457,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3414,13 +3494,13 @@
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46217</v>
+        <v>46240</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46222</v>
+        <v>46245</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>77100</v>
+        <v>204000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3434,7 +3514,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -3446,17 +3526,17 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
@@ -3469,7 +3549,7 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
@@ -3479,17 +3559,17 @@
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46223</v>
+        <v>46232</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46238</v>
+        <v>46237</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>100000</v>
+        <v>288000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
@@ -3503,7 +3583,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -3515,12 +3595,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3538,27 +3618,27 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46225</v>
+        <v>46240</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46229</v>
+        <v>46245</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>114600</v>
+        <v>100000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
@@ -3572,7 +3652,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3584,17 +3664,17 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR 12970</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
@@ -3603,30 +3683,32 @@
         </is>
       </c>
       <c r="F45" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46183</v>
+        <v>46244</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46188</v>
-      </c>
-      <c r="L45" s="23" t="inlineStr"/>
+        <v>46300</v>
+      </c>
+      <c r="L45" s="23" t="n">
+        <v>350000</v>
+      </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
@@ -3634,12 +3716,12 @@
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3651,12 +3733,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3674,31 +3756,31 @@
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Brasília DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46227</v>
+        <v>46240</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46231</v>
+        <v>46245</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>150000</v>
+        <v>204000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
@@ -3708,7 +3790,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -3720,12 +3802,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3743,7 +3825,7 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
@@ -3753,17 +3835,17 @@
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46224</v>
+        <v>46240</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46233</v>
+        <v>46245</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>288000</v>
+        <v>80000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
@@ -3777,7 +3859,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -3789,62 +3871,64 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F48" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F48" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46232</v>
+        <v>46244</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46238</v>
+        <v>46296</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>30000</v>
+        <v>935000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N48" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -3856,17 +3940,17 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
@@ -3875,11 +3959,11 @@
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.343</v>
+        <v>0.4</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
@@ -3889,17 +3973,17 @@
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>30000</v>
+        <v>80000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
@@ -3913,7 +3997,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -3925,12 +4009,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -3940,15 +4024,13 @@
       </c>
       <c r="E50" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F50" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F50" s="13" t="inlineStr"/>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
@@ -3958,17 +4040,17 @@
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46232</v>
+        <v>46227</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46237</v>
+        <v>46252</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>288000</v>
+        <v>286000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
@@ -3982,7 +4064,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3994,12 +4076,12 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -4013,7 +4095,7 @@
         </is>
       </c>
       <c r="F51" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
@@ -4027,21 +4109,19 @@
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46245</v>
-      </c>
-      <c r="L51" s="23" t="n">
-        <v>80000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L51" s="23" t="inlineStr"/>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
@@ -4051,7 +4131,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -4063,12 +4143,12 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -4086,27 +4166,27 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>100000</v>
+        <v>54000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
@@ -4120,7 +4200,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -4132,12 +4212,12 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -4155,27 +4235,27 @@
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>80000</v>
+        <v>54000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
@@ -4189,7 +4269,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -4201,17 +4281,17 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
@@ -4224,27 +4304,27 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46240</v>
+        <v>46251</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46245</v>
+        <v>46256</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>204000</v>
+        <v>50000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
@@ -4258,7 +4338,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -4270,12 +4350,12 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
@@ -4293,27 +4373,27 @@
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46240</v>
+        <v>46252</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46245</v>
+        <v>46259</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>204000</v>
+        <v>60000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
@@ -4327,7 +4407,7 @@
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -4339,12 +4419,12 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
@@ -4362,7 +4442,7 @@
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
@@ -4376,17 +4456,17 @@
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46244</v>
+        <v>46208</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46300</v>
+        <v>46259</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>350000</v>
+        <v>500000</v>
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
@@ -4396,7 +4476,7 @@
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4408,22 +4488,22 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F57" s="21" t="n">
@@ -4431,27 +4511,27 @@
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46246</v>
+        <v>46265</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46257</v>
+        <v>46270</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
@@ -4465,7 +4545,7 @@
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -4477,17 +4557,17 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
@@ -4500,27 +4580,27 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46244</v>
+        <v>46246</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46296</v>
+        <v>46272</v>
       </c>
       <c r="L58" s="15" t="n">
-        <v>935000</v>
+        <v>54000</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
@@ -4529,496 +4609,17 @@
       </c>
       <c r="N58" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B59" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
-        </is>
-      </c>
-      <c r="C59" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
-        </is>
-      </c>
-      <c r="D59" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E59" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F59" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G59" s="19" t="inlineStr">
-        <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H59" s="19" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I59" s="19" t="inlineStr">
-        <is>
-          <t>Porto Alegre/RS</t>
-        </is>
-      </c>
-      <c r="J59" s="22" t="n">
-        <v>46246</v>
-      </c>
-      <c r="K59" s="22" t="n">
-        <v>46257</v>
-      </c>
-      <c r="L59" s="23" t="n">
-        <v>54000</v>
-      </c>
-      <c r="M59" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N59" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O59" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B60" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
-        </is>
-      </c>
-      <c r="C60" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
-        </is>
-      </c>
-      <c r="D60" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E60" s="12" t="inlineStr">
-        <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F60" s="13" t="inlineStr"/>
-      <c r="G60" s="11" t="inlineStr">
-        <is>
-          <t>Não classificada</t>
-        </is>
-      </c>
-      <c r="H60" s="11" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I60" s="11" t="inlineStr">
-        <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
-        </is>
-      </c>
-      <c r="J60" s="14" t="n">
-        <v>46227</v>
-      </c>
-      <c r="K60" s="14" t="n">
-        <v>46252</v>
-      </c>
-      <c r="L60" s="15" t="n">
-        <v>286000</v>
-      </c>
-      <c r="M60" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N60" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O60" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B61" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
-        </is>
-      </c>
-      <c r="C61" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
-        </is>
-      </c>
-      <c r="D61" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E61" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F61" s="21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G61" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
-        </is>
-      </c>
-      <c r="H61" s="19" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I61" s="19" t="inlineStr">
-        <is>
-          <t>Brasília - DF | Híbrido</t>
-        </is>
-      </c>
-      <c r="J61" s="22" t="n">
-        <v>46246</v>
-      </c>
-      <c r="K61" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L61" s="23" t="inlineStr"/>
-      <c r="M61" s="17" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N61" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O61" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B62" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
-        </is>
-      </c>
-      <c r="C62" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
-        </is>
-      </c>
-      <c r="D62" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
-        </is>
-      </c>
-      <c r="E62" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F62" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G62" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H62" s="11" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I62" s="11" t="inlineStr">
-        <is>
-          <t>Recife - PE</t>
-        </is>
-      </c>
-      <c r="J62" s="14" t="n">
-        <v>46251</v>
-      </c>
-      <c r="K62" s="14" t="n">
-        <v>46256</v>
-      </c>
-      <c r="L62" s="15" t="n">
-        <v>50000</v>
-      </c>
-      <c r="M62" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N62" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O62" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B63" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
-        </is>
-      </c>
-      <c r="C63" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
-        </is>
-      </c>
-      <c r="D63" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E63" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F63" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G63" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados</t>
-        </is>
-      </c>
-      <c r="H63" s="19" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I63" s="19" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="J63" s="22" t="n">
-        <v>46252</v>
-      </c>
-      <c r="K63" s="22" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L63" s="23" t="n">
-        <v>60000</v>
-      </c>
-      <c r="M63" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N63" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O63" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B64" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
-        </is>
-      </c>
-      <c r="C64" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
-        </is>
-      </c>
-      <c r="D64" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E64" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F64" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G64" s="11" t="inlineStr">
-        <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
-        </is>
-      </c>
-      <c r="H64" s="11" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I64" s="11" t="inlineStr">
-        <is>
-          <t>Porto Alegre/RS</t>
-        </is>
-      </c>
-      <c r="J64" s="14" t="n">
-        <v>46246</v>
-      </c>
-      <c r="K64" s="14" t="n">
-        <v>46272</v>
-      </c>
-      <c r="L64" s="15" t="n">
-        <v>54000</v>
-      </c>
-      <c r="M64" s="9" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N64" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O64" s="16" t="inlineStr">
-        <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B65" s="18" t="inlineStr">
-        <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
-        </is>
-      </c>
-      <c r="C65" s="19" t="inlineStr">
-        <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
-        </is>
-      </c>
-      <c r="D65" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
-        </is>
-      </c>
-      <c r="E65" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F65" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G65" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados</t>
-        </is>
-      </c>
-      <c r="H65" s="19" t="inlineStr">
-        <is>
-          <t>OEI/MDHC</t>
-        </is>
-      </c>
-      <c r="I65" s="19" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="J65" s="22" t="n">
-        <v>46208</v>
-      </c>
-      <c r="K65" s="22" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L65" s="23" t="n">
-        <v>500000</v>
-      </c>
-      <c r="M65" s="17" t="inlineStr">
-        <is>
-          <t>En presentación</t>
-        </is>
-      </c>
-      <c r="N65" s="20" t="inlineStr">
-        <is>
-          <t>compras.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O65" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:O65"/>
+  <autoFilter ref="A1:O58"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -5077,13 +4678,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId64"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -5128,21 +4722,21 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Unesco</t>
+          <t>Pnud</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Pnud</t>
+          <t>Unesco</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -5158,7 +4752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5184,7 +4778,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3">
@@ -5194,11 +4788,21 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>10</v>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B3"/>
+  <autoFilter ref="A1:B4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -5236,7 +4840,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
@@ -5246,7 +4850,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -5256,7 +4860,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -5308,7 +4912,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3">
@@ -5318,7 +4922,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4">
@@ -5338,7 +4942,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -5348,7 +4952,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -5358,7 +4962,7 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -5416,7 +5020,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
@@ -5426,21 +5030,21 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -5528,7 +5132,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5543,7 +5147,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5558,7 +5162,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5573,7 +5177,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-01 16:10
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$64</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 31/08/2026 às 18:50</t>
+          <t>Gerado em 01/09/2026 às 16:07</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6">
@@ -644,21 +644,21 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>PNUD</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>PNUD</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O58"/>
+  <dimension ref="A1:O64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1844,12 +1844,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:07727145-a919-4540-98cd-08dee32d8e84</t>
+          <t>unesco:5d64862a-264d-475d-5f8e-08df036d3e00</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ5019 - Edital 3/2026 - 01 vaga - Consultor Individual</t>
+          <t>4BRZ4025 - Edital 18/2026 - Consultor Individual (1 Vaga)  REPUBLICAÇÃO</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1859,15 +1859,13 @@
       </c>
       <c r="E17" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F17" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="inlineStr"/>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1877,10 +1875,10 @@
       </c>
       <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46255</v>
+        <v>46266</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46265</v>
+        <v>46270</v>
       </c>
       <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
@@ -2139,12 +2137,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:7155091d-98d5-4ce4-df16-08df01dbdf45</t>
+          <t>unesco:b324319d-9f96-425f-8caf-08defc5a5785</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ4024 - EDITAL Nº03/2026 - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 48/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2154,13 +2152,15 @@
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F22" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2170,10 +2170,10 @@
       </c>
       <c r="I22" s="11" t="inlineStr"/>
       <c r="J22" s="14" t="n">
-        <v>46259</v>
+        <v>46266</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46265</v>
+        <v>46274</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2196,12 +2196,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:4fda0c36-f1a0-41f6-3f3a-08defeb303ea</t>
+          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 47/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2229,10 +2229,10 @@
       </c>
       <c r="I23" s="19" t="inlineStr"/>
       <c r="J23" s="22" t="n">
-        <v>46262</v>
+        <v>46266</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46268</v>
+        <v>46274</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2255,12 +2255,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:4db2e20b-a2e2-4074-00dc-08deff7b5e96</t>
+          <t>unesco:5c1d62c6-1efa-431c-b9e2-08df0436270c</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 49/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 54/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2288,10 +2288,10 @@
       </c>
       <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46262</v>
+        <v>46266</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46268</v>
+        <v>46273</v>
       </c>
       <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
@@ -2314,12 +2314,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:ecd2379c-2ba5-488f-00dd-08deff7b5e96</t>
+          <t>unesco:c9020343-9d28-49e3-b9e3-08df0436270c</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 50/2026 - 2 vagas - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 52/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2347,10 +2347,10 @@
       </c>
       <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46262</v>
+        <v>46266</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46268</v>
+        <v>46273</v>
       </c>
       <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
@@ -2373,12 +2373,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:9ecb033c-d905-4f6f-df1e-08df01dbdf45</t>
+          <t>unesco:b74745df-a51d-41c1-b9e5-08df0436270c</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 54/2026 - Arquitetura e Urbanismo</t>
+          <t>914BRZ1155 - EDITAL Nº 55/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2396,7 +2396,7 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2406,10 +2406,10 @@
       </c>
       <c r="I26" s="11" t="inlineStr"/>
       <c r="J26" s="14" t="n">
-        <v>46261</v>
+        <v>46266</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46265</v>
+        <v>46273</v>
       </c>
       <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
@@ -2427,22 +2427,22 @@
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056</t>
+          <t>unesco:f4efa11a-ea51-47cf-b9e7-08df0436270c</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEC/BRA/24 – TR 13056</t>
+          <t>914BRZ1155 - EDITAL Nº 56/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
@@ -2455,61 +2455,53 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I27" s="19" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I27" s="19" t="inlineStr"/>
       <c r="J27" s="22" t="n">
-        <v>46209</v>
+        <v>46266</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46214</v>
+        <v>46273</v>
       </c>
       <c r="L27" s="23" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N27" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N27" s="20" t="inlineStr"/>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067</t>
+          <t>unesco:6f0bebf7-7be2-4b29-17c5-08df04786cdd</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13067</t>
+          <t>914BRZ1155 - EDITAL Nº 53/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -2518,67 +2510,57 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I28" s="11" t="inlineStr">
-        <is>
-          <t>Secretaria de Estado da Educação  SEED-PR</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr"/>
       <c r="J28" s="14" t="n">
-        <v>46212</v>
+        <v>46266</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46224</v>
-      </c>
-      <c r="L28" s="15" t="n">
-        <v>150000</v>
-      </c>
+        <v>46273</v>
+      </c>
+      <c r="L28" s="15" t="inlineStr"/>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N28" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N28" s="12" t="inlineStr"/>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
+          <t>unesco:4fda0c36-f1a0-41f6-3f3a-08defeb303ea</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
+          <t>914BRZ1155 - EDITAL Nº 47/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
@@ -2587,67 +2569,57 @@
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I29" s="19" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I29" s="19" t="inlineStr"/>
       <c r="J29" s="22" t="n">
-        <v>46217</v>
+        <v>46262</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46222</v>
-      </c>
-      <c r="L29" s="23" t="n">
-        <v>77100</v>
-      </c>
+        <v>46268</v>
+      </c>
+      <c r="L29" s="23" t="inlineStr"/>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N29" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N29" s="20" t="inlineStr"/>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
+          <t>unesco:4db2e20b-a2e2-4074-00dc-08deff7b5e96</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
+          <t>914BRZ1155 - EDITAL Nº 49/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2656,7 +2628,7 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
@@ -2665,58 +2637,48 @@
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I30" s="11" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="inlineStr"/>
       <c r="J30" s="14" t="n">
-        <v>46213</v>
+        <v>46262</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46217</v>
-      </c>
-      <c r="L30" s="15" t="n">
-        <v>144000</v>
-      </c>
+        <v>46268</v>
+      </c>
+      <c r="L30" s="15" t="inlineStr"/>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N30" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N30" s="12" t="inlineStr"/>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
+          <t>unesco:ecd2379c-2ba5-488f-00dd-08deff7b5e96</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
+          <t>914BRZ1155 - EDITAL Nº 50/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
@@ -2729,61 +2691,53 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I31" s="19" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I31" s="19" t="inlineStr"/>
       <c r="J31" s="22" t="n">
-        <v>46213</v>
+        <v>46262</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46220</v>
+        <v>46268</v>
       </c>
       <c r="L31" s="23" t="inlineStr"/>
       <c r="M31" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N31" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N31" s="20" t="inlineStr"/>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
+          <t>unesco:11c715d6-1d36-4c54-5f8f-08df036d3e00</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
+          <t>914BRZ4027 - Edital 55/2026 - Ciências Sociais</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
@@ -2792,45 +2746,35 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I32" s="11" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I32" s="11" t="inlineStr"/>
       <c r="J32" s="14" t="n">
-        <v>46216</v>
+        <v>46266</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46223</v>
-      </c>
-      <c r="L32" s="15" t="n">
-        <v>133000</v>
-      </c>
+        <v>46271</v>
+      </c>
+      <c r="L32" s="15" t="inlineStr"/>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N32" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N32" s="12" t="inlineStr"/>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -2842,12 +2786,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR 12970</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2861,11 +2805,11 @@
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
@@ -2875,19 +2819,21 @@
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46183</v>
+        <v>46216</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46188</v>
-      </c>
-      <c r="L33" s="23" t="inlineStr"/>
+        <v>46223</v>
+      </c>
+      <c r="L33" s="23" t="n">
+        <v>133000</v>
+      </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N33" s="20" t="inlineStr">
@@ -2897,7 +2843,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
         </is>
       </c>
     </row>
@@ -2909,17 +2855,17 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -2932,7 +2878,7 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -2946,17 +2892,17 @@
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46220</v>
+        <v>46213</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46225</v>
+        <v>46217</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>58800</v>
+        <v>144000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -2966,7 +2912,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
         </is>
       </c>
     </row>
@@ -2978,17 +2924,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -3001,7 +2947,7 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3015,15 +2961,15 @@
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46221</v>
+        <v>46213</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="L35" s="23" t="inlineStr"/>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N35" s="20" t="inlineStr">
@@ -3033,7 +2979,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
         </is>
       </c>
     </row>
@@ -3045,17 +2991,17 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
@@ -3073,7 +3019,7 @@
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
@@ -3082,13 +3028,13 @@
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46223</v>
+        <v>46217</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46238</v>
+        <v>46222</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>100000</v>
+        <v>77100</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3102,7 +3048,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
         </is>
       </c>
     </row>
@@ -3114,12 +3060,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEC/BRA/24 – TR 13056</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3133,35 +3079,33 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46225</v>
+        <v>46209</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46229</v>
-      </c>
-      <c r="L37" s="23" t="n">
-        <v>114600</v>
-      </c>
+        <v>46214</v>
+      </c>
+      <c r="L37" s="23" t="inlineStr"/>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N37" s="20" t="inlineStr">
@@ -3171,7 +3115,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056/</t>
         </is>
       </c>
     </row>
@@ -3183,17 +3127,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13067</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3206,7 +3150,7 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3216,21 +3160,21 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Brasília DF</t>
+          <t>Secretaria de Estado da Educação  SEED-PR</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46227</v>
+        <v>46212</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46231</v>
+        <v>46224</v>
       </c>
       <c r="L38" s="15" t="n">
         <v>150000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
@@ -3240,7 +3184,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067/</t>
         </is>
       </c>
     </row>
@@ -3252,12 +3196,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3275,27 +3219,27 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46233</v>
+        <v>46225</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>288000</v>
+        <v>58800</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3309,7 +3253,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
         </is>
       </c>
     </row>
@@ -3321,52 +3265,52 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F40" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46232</v>
+        <v>46221</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46238</v>
-      </c>
-      <c r="L40" s="15" t="n">
-        <v>30000</v>
-      </c>
+        <v>46224</v>
+      </c>
+      <c r="L40" s="15" t="inlineStr"/>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
@@ -3376,7 +3320,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
         </is>
       </c>
     </row>
@@ -3388,17 +3332,17 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR 12970</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
@@ -3407,35 +3351,33 @@
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.343</v>
+        <v>0.3</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46232</v>
+        <v>46183</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46238</v>
-      </c>
-      <c r="L41" s="23" t="n">
-        <v>30000</v>
-      </c>
+        <v>46188</v>
+      </c>
+      <c r="L41" s="23" t="inlineStr"/>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
@@ -3445,7 +3387,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970/</t>
         </is>
       </c>
     </row>
@@ -3457,17 +3399,17 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
@@ -3485,7 +3427,7 @@
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
@@ -3494,13 +3436,13 @@
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46240</v>
+        <v>46223</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>204000</v>
+        <v>100000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3514,7 +3456,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
         </is>
       </c>
     </row>
@@ -3526,12 +3468,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3549,7 +3491,7 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
@@ -3559,17 +3501,17 @@
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46232</v>
+        <v>46225</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46237</v>
+        <v>46229</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>288000</v>
+        <v>114600</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
@@ -3583,7 +3525,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
         </is>
       </c>
     </row>
@@ -3595,12 +3537,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3618,31 +3560,31 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46240</v>
+        <v>46227</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46245</v>
+        <v>46231</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>100000</v>
+        <v>150000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
@@ -3652,7 +3594,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -3664,17 +3606,17 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
@@ -3687,41 +3629,41 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46244</v>
+        <v>46224</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46300</v>
+        <v>46233</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>350000</v>
+        <v>288000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -3733,12 +3675,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3748,15 +3690,13 @@
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F46" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F46" s="13" t="inlineStr"/>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3766,17 +3706,17 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>204000</v>
+        <v>30000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3790,7 +3730,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -3802,12 +3742,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3825,27 +3765,27 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46245</v>
+        <v>46237</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>80000</v>
+        <v>288000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
@@ -3859,7 +3799,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -3871,17 +3811,17 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
@@ -3890,45 +3830,45 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.4</v>
+        <v>0.343</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46244</v>
+        <v>46232</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46296</v>
+        <v>46238</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>935000</v>
+        <v>30000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N48" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -3940,12 +3880,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -3963,7 +3903,7 @@
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
@@ -3983,7 +3923,7 @@
         <v>46245</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>80000</v>
+        <v>204000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
@@ -3997,7 +3937,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -4009,12 +3949,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4024,33 +3964,35 @@
       </c>
       <c r="E50" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F50" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F50" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46227</v>
+        <v>46240</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46252</v>
+        <v>46245</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>286000</v>
+        <v>204000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
@@ -4064,7 +4006,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -4076,12 +4018,12 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -4095,7 +4037,7 @@
         </is>
       </c>
       <c r="F51" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
@@ -4109,19 +4051,21 @@
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L51" s="23" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L51" s="23" t="n">
+        <v>80000</v>
+      </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
@@ -4131,7 +4075,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -4143,17 +4087,17 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
@@ -4166,41 +4110,41 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46246</v>
+        <v>46244</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46257</v>
+        <v>46300</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>54000</v>
+        <v>350000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4212,12 +4156,12 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -4235,27 +4179,27 @@
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46257</v>
+        <v>46245</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>54000</v>
+        <v>80000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
@@ -4269,7 +4213,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -4281,17 +4225,17 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
@@ -4304,27 +4248,27 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46251</v>
+        <v>46240</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46256</v>
+        <v>46245</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>50000</v>
+        <v>100000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
@@ -4338,7 +4282,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -4350,17 +4294,17 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
@@ -4373,41 +4317,41 @@
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46252</v>
+        <v>46244</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46259</v>
+        <v>46296</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>60000</v>
+        <v>935000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N55" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4419,17 +4363,17 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
@@ -4438,45 +4382,43 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46208</v>
+        <v>46246</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L56" s="15" t="n">
-        <v>500000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L56" s="15" t="inlineStr"/>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -4488,50 +4430,48 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
-        </is>
-      </c>
-      <c r="F57" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F57" s="21" t="inlineStr"/>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46265</v>
+        <v>46227</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46270</v>
+        <v>46252</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>30000</v>
+        <v>286000</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
@@ -4545,7 +4485,7 @@
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -4557,12 +4497,12 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
@@ -4580,7 +4520,7 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
@@ -4597,29 +4537,443 @@
         <v>46246</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46272</v>
+        <v>46257</v>
       </c>
       <c r="L58" s="15" t="n">
         <v>54000</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N58" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O58" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B59" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+        </is>
+      </c>
+      <c r="C59" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+        </is>
+      </c>
+      <c r="D59" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+        </is>
+      </c>
+      <c r="E59" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F59" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G59" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H59" s="19" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I59" s="19" t="inlineStr">
+        <is>
+          <t>Recife - PE</t>
+        </is>
+      </c>
+      <c r="J59" s="22" t="n">
+        <v>46251</v>
+      </c>
+      <c r="K59" s="22" t="n">
+        <v>46256</v>
+      </c>
+      <c r="L59" s="23" t="n">
+        <v>50000</v>
+      </c>
+      <c r="M59" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N59" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O59" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B60" s="10" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E60" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F60" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G60" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H60" s="11" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I60" s="11" t="inlineStr">
+        <is>
+          <t>Porto Alegre/RS</t>
+        </is>
+      </c>
+      <c r="J60" s="14" t="n">
+        <v>46246</v>
+      </c>
+      <c r="K60" s="14" t="n">
+        <v>46257</v>
+      </c>
+      <c r="L60" s="15" t="n">
+        <v>54000</v>
+      </c>
+      <c r="M60" s="9" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N60" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O60" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B61" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+        </is>
+      </c>
+      <c r="C61" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+        </is>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E61" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F61" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G61" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados</t>
+        </is>
+      </c>
+      <c r="H61" s="19" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I61" s="19" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
+      <c r="J61" s="22" t="n">
+        <v>46252</v>
+      </c>
+      <c r="K61" s="22" t="n">
+        <v>46259</v>
+      </c>
+      <c r="L61" s="23" t="n">
+        <v>60000</v>
+      </c>
+      <c r="M61" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N61" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O61" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+        </is>
+      </c>
+      <c r="C62" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+        </is>
+      </c>
+      <c r="D62" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Física (PF)</t>
+        </is>
+      </c>
+      <c r="E62" s="12" t="inlineStr">
+        <is>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="F62" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G62" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+        </is>
+      </c>
+      <c r="H62" s="11" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I62" s="11" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J62" s="14" t="n">
+        <v>46265</v>
+      </c>
+      <c r="K62" s="14" t="n">
+        <v>46270</v>
+      </c>
+      <c r="L62" s="15" t="n">
+        <v>30000</v>
+      </c>
+      <c r="M62" s="9" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N62" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O62" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B63" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+        </is>
+      </c>
+      <c r="C63" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+        </is>
+      </c>
+      <c r="D63" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E63" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F63" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G63" s="19" t="inlineStr">
+        <is>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+        </is>
+      </c>
+      <c r="H63" s="19" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I63" s="19" t="inlineStr">
+        <is>
+          <t>Porto Alegre/RS</t>
+        </is>
+      </c>
+      <c r="J63" s="22" t="n">
+        <v>46246</v>
+      </c>
+      <c r="K63" s="22" t="n">
+        <v>46272</v>
+      </c>
+      <c r="L63" s="23" t="n">
+        <v>54000</v>
+      </c>
+      <c r="M63" s="17" t="inlineStr">
+        <is>
           <t>En fase de apresentação</t>
         </is>
       </c>
-      <c r="N58" s="12" t="inlineStr">
+      <c r="N63" s="20" t="inlineStr">
         <is>
           <t>selecao.bra@oei.int</t>
         </is>
       </c>
-      <c r="O58" s="16" t="inlineStr">
+      <c r="O63" s="24" t="inlineStr">
         <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B64" s="10" t="inlineStr">
+        <is>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+        </is>
+      </c>
+      <c r="C64" s="11" t="inlineStr">
+        <is>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+        </is>
+      </c>
+      <c r="D64" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E64" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F64" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G64" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados</t>
+        </is>
+      </c>
+      <c r="H64" s="11" t="inlineStr">
+        <is>
+          <t>OEI/MDHC</t>
+        </is>
+      </c>
+      <c r="I64" s="11" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="J64" s="14" t="n">
+        <v>46208</v>
+      </c>
+      <c r="K64" s="14" t="n">
+        <v>46259</v>
+      </c>
+      <c r="L64" s="15" t="n">
+        <v>500000</v>
+      </c>
+      <c r="M64" s="9" t="inlineStr">
+        <is>
+          <t>En presentación</t>
+        </is>
+      </c>
+      <c r="N64" s="12" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O64" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O58"/>
+  <autoFilter ref="A1:O64"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4678,6 +5032,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId63"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4722,21 +5082,21 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Pnud</t>
+          <t>Unesco</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Unesco</t>
+          <t>Pnud</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -4778,7 +5138,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3">
@@ -4840,7 +5200,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
@@ -4912,7 +5272,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
@@ -4922,7 +5282,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4">
@@ -4932,7 +5292,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5">
@@ -4972,7 +5332,7 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -5030,21 +5390,21 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -5132,7 +5492,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5147,7 +5507,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5162,7 +5522,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5177,7 +5537,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-02 16:05
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$60</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -27,7 +27,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Por_Tipo'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Area'!$A$1:$B$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Por_Area'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Por_Orgao'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Perfis'!$A$1:$C$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Perfis'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 01/09/2026 às 16:07</t>
+          <t>Gerado em 02/09/2026 às 16:03</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="17">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>30000</v>
+        <v>55</v>
       </c>
     </row>
     <row r="18">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>170537.0370370371</v>
+        <v>161191.5517241379</v>
       </c>
     </row>
     <row r="20">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O64"/>
+  <dimension ref="A1:O60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -876,16 +876,16 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>146311</v>
+        <v>146313</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 19/2026 - Contratação de Consultoria Individual para o desenvolvimento, documentação e compilação de bases de dados dos módulos econômico e de distribuição de renda do modelo MIRA</t>
+          <t>Consultoria técnica especializada para desenvolvimento de proposta de governança e curadoria da Base de Conhecimento destinada ao suporte de soluções de Inteligência Artificial da área de Integridade da Secretaria do Tesouro Nacional</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E2" s="12" t="inlineStr">
@@ -898,12 +898,12 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H2" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I2" s="11" t="inlineStr">
@@ -912,10 +912,10 @@
         </is>
       </c>
       <c r="J2" s="14" t="n">
-        <v>46248</v>
+        <v>46254</v>
       </c>
       <c r="K2" s="14" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="L2" s="15" t="inlineStr"/>
       <c r="M2" s="9" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="N2" s="12" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>ucp.codin.df.stn@tesouro.gov.br</t>
         </is>
       </c>
       <c r="O2" s="16" t="inlineStr">
@@ -941,11 +941,11 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>146312</v>
+        <v>146326</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 20/2026 - Contratação de Consultor Individual para o desenvolvimento, documentação e aplicação do módulo econômico do modelo MIRA, com foco na calibração de parâmetros, regionalização e estimação da Matriz de Absorção de Investimentos</t>
+          <t>Edital nº 02/2026 – Metodologia para monitoramento das decisões da Corte Interamericana de Direitos Humanos</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
@@ -955,30 +955,32 @@
       </c>
       <c r="E3" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F3" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F3" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G3" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H3" s="19" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I3" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J3" s="22" t="n">
-        <v>46248</v>
+        <v>46258</v>
       </c>
       <c r="K3" s="22" t="n">
-        <v>46266</v>
+        <v>46274</v>
       </c>
       <c r="L3" s="23" t="inlineStr"/>
       <c r="M3" s="17" t="inlineStr">
@@ -988,7 +990,7 @@
       </c>
       <c r="N3" s="20" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>ccidh@mdh.gov.br</t>
         </is>
       </c>
       <c r="O3" s="24" t="inlineStr">
@@ -1004,16 +1006,16 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146313</v>
+        <v>146327</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Consultoria técnica especializada para desenvolvimento de proposta de governança e curadoria da Base de Conhecimento destinada ao suporte de soluções de Inteligência Artificial da área de Integridade da Secretaria do Tesouro Nacional</t>
+          <t>Edital nº 3/2026 – Metodologia para monitoramento de recomendações e decisões da Comissão Interamericana de Direitos Humanos</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E4" s="12" t="inlineStr">
@@ -1026,7 +1028,7 @@
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr">
@@ -1036,14 +1038,14 @@
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
-        <v>46254</v>
+        <v>46258</v>
       </c>
       <c r="K4" s="14" t="n">
-        <v>46267</v>
+        <v>46274</v>
       </c>
       <c r="L4" s="15" t="inlineStr"/>
       <c r="M4" s="9" t="inlineStr">
@@ -1053,7 +1055,7 @@
       </c>
       <c r="N4" s="12" t="inlineStr">
         <is>
-          <t>ucp.codin.df.stn@tesouro.gov.br</t>
+          <t>ccidh@mdh.gov.br</t>
         </is>
       </c>
       <c r="O4" s="16" t="inlineStr">
@@ -1069,11 +1071,11 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146317</v>
+        <v>146332</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 21/2026 - Contratação de Consultoria Individual para o desenvolvimento metodológico e a integração dos módulos de emissões de GEE e consumo de energia no modelo MIRA</t>
+          <t>Edital nº 04/2026 - Segundo Plano da Política Nacional de RCN</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -1083,30 +1085,32 @@
       </c>
       <c r="E5" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F5" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F5" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J5" s="22" t="n">
-        <v>46248</v>
+        <v>46258</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46266</v>
+        <v>46274</v>
       </c>
       <c r="L5" s="23" t="inlineStr"/>
       <c r="M5" s="17" t="inlineStr">
@@ -1116,7 +1120,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>rcn_cidadania@mdh.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1132,44 +1136,46 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146318</v>
+        <v>146335</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 23/2026 - Contratação de consultor individual para a Elaboração do Guia Prático de Oficinas Colaborativas</t>
+          <t>Consultoria técnica especializada para avaliação das capacidades institucionais da Secretaria do Tesouro Nacional (STN)</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F6" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>REMOTO</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
-        <v>46248</v>
+        <v>46258</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>46266</v>
+        <v>46271</v>
       </c>
       <c r="L6" s="15" t="inlineStr"/>
       <c r="M6" s="9" t="inlineStr">
@@ -1179,7 +1185,7 @@
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>ucp.codin.df.stn@tesouro.gov.br</t>
         </is>
       </c>
       <c r="O6" s="16" t="inlineStr">
@@ -1195,11 +1201,11 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146319</v>
+        <v>146336</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 22/2026 – Contratação de Consultoria Individual para o desenvolvimento metodológico e a integração dos módulos de emissões de GEE e consumo de água no modelo MIRA</t>
+          <t>UNDP-BRA-01232 - Benchmark Internacional e Análise de Adaptabilidade de Modelos Federativos de Gestão de Pessoas ao Contexto Brasileiro</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1209,30 +1215,32 @@
       </c>
       <c r="E7" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F7" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F7" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H7" s="19" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>PNUD (Direto)</t>
         </is>
       </c>
       <c r="I7" s="19" t="inlineStr">
         <is>
-          <t>remoto</t>
+          <t>Home based</t>
         </is>
       </c>
       <c r="J7" s="22" t="n">
-        <v>46248</v>
+        <v>46255</v>
       </c>
       <c r="K7" s="22" t="n">
-        <v>46266</v>
+        <v>46268</v>
       </c>
       <c r="L7" s="23" t="inlineStr"/>
       <c r="M7" s="17" t="inlineStr">
@@ -1242,7 +1250,7 @@
       </c>
       <c r="N7" s="20" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>ic.procurement.br@undp.org</t>
         </is>
       </c>
       <c r="O7" s="24" t="inlineStr">
@@ -1258,11 +1266,11 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146320</v>
+        <v>146337</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edital nº 24/2026 – Contratação de Consultoria individual para desenvolvimento de projeto gráfico  e diagramação do Relatório de Gestão Integrado </t>
+          <t>IC UNDP-BRA-01228 - Benchmarking, modelagem federativa e análise de viabilidade institucional</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1280,24 +1288,24 @@
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>PNUD (Direto)</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>remoto</t>
+          <t>Home based</t>
         </is>
       </c>
       <c r="J8" s="14" t="n">
-        <v>46248</v>
+        <v>46255</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>46266</v>
+        <v>46268</v>
       </c>
       <c r="L8" s="15" t="inlineStr"/>
       <c r="M8" s="9" t="inlineStr">
@@ -1307,7 +1315,7 @@
       </c>
       <c r="N8" s="12" t="inlineStr">
         <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
+          <t>aquisicoes.cbo.br@undp.org</t>
         </is>
       </c>
       <c r="O8" s="16" t="inlineStr">
@@ -1323,11 +1331,11 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146326</v>
+        <v>146346</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 02/2026 – Metodologia para monitoramento das decisões da Corte Interamericana de Direitos Humanos</t>
+          <t>Contratação de consultor (a) individual para assessoramento técnico especializado à consolidação, redação técnica e estruturação dos mecanismos de governança do Plano Estadual de Educação do Piauí 2026-2036</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -1355,14 +1363,14 @@
       </c>
       <c r="I9" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Home based</t>
         </is>
       </c>
       <c r="J9" s="22" t="n">
-        <v>46258</v>
+        <v>46262</v>
       </c>
       <c r="K9" s="22" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="L9" s="23" t="inlineStr"/>
       <c r="M9" s="17" t="inlineStr">
@@ -1372,7 +1380,7 @@
       </c>
       <c r="N9" s="20" t="inlineStr">
         <is>
-          <t>ccidh@mdh.gov.br</t>
+          <t>ugest@seduc.pi.gov.br</t>
         </is>
       </c>
       <c r="O9" s="24" t="inlineStr">
@@ -1388,11 +1396,11 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>146327</v>
+        <v>146347</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 3/2026 – Metodologia para monitoramento de recomendações e decisões da Comissão Interamericana de Direitos Humanos</t>
+          <t>Contratação de consultor (a) individual para apoiar tecnicamente a Superintendência de Ensino na realização das Olimpíadas do Conhecimento</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1410,7 +1418,7 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -1420,14 +1428,14 @@
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Home based</t>
         </is>
       </c>
       <c r="J10" s="14" t="n">
-        <v>46258</v>
+        <v>46262</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="L10" s="15" t="inlineStr"/>
       <c r="M10" s="9" t="inlineStr">
@@ -1437,7 +1445,7 @@
       </c>
       <c r="N10" s="12" t="inlineStr">
         <is>
-          <t>ccidh@mdh.gov.br</t>
+          <t>ugest@seduc.pi.gov.br</t>
         </is>
       </c>
       <c r="O10" s="16" t="inlineStr">
@@ -1453,16 +1461,16 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>146332</v>
+        <v>146349</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 04/2026 - Segundo Plano da Política Nacional de RCN</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA PARA O DESENVOLVIMENTO DE TECNOLOGIA APLICADA AO OBSERVATÓRIO DO NORDESTE</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E11" s="20" t="inlineStr">
@@ -1475,7 +1483,7 @@
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
@@ -1485,16 +1493,18 @@
       </c>
       <c r="I11" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>HOME OFFICE</t>
         </is>
       </c>
       <c r="J11" s="22" t="n">
-        <v>46258</v>
+        <v>46267</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46274</v>
-      </c>
-      <c r="L11" s="23" t="inlineStr"/>
+        <v>46278</v>
+      </c>
+      <c r="L11" s="23" t="n">
+        <v>200000</v>
+      </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1502,7 +1512,7 @@
       </c>
       <c r="N11" s="20" t="inlineStr">
         <is>
-          <t>rcn_cidadania@mdh.gov.br</t>
+          <t>curriculos@consorcionordeste.gov.br</t>
         </is>
       </c>
       <c r="O11" s="24" t="inlineStr">
@@ -1518,16 +1528,16 @@
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>146335</v>
+        <v>146350</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Consultoria técnica especializada para avaliação das capacidades institucionais da Secretaria do Tesouro Nacional (STN)</t>
+          <t xml:space="preserve">Contratação de consultoria individual (pessoa física) para elaboração de estudo analítico, voltado ao mapeamento de empreendimentos vinculados à transição energética em execução ou em fase de planejamento e de seu potencial impacto sobre territórios quilombolas na Região Sudeste </t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -1540,7 +1550,7 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
@@ -1554,12 +1564,14 @@
         </is>
       </c>
       <c r="J12" s="14" t="n">
-        <v>46258</v>
+        <v>46266</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>46271</v>
-      </c>
-      <c r="L12" s="15" t="inlineStr"/>
+        <v>46272</v>
+      </c>
+      <c r="L12" s="15" t="n">
+        <v>55000</v>
+      </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1567,7 +1579,7 @@
       </c>
       <c r="N12" s="12" t="inlineStr">
         <is>
-          <t>ucp.codin.df.stn@tesouro.gov.br</t>
+          <t>dqc@igualdaderacial.gov.br</t>
         </is>
       </c>
       <c r="O12" s="16" t="inlineStr">
@@ -1579,15 +1591,17 @@
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="n">
-        <v>146336</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>unesco:5d64862a-264d-475d-5f8e-08df036d3e00</t>
+        </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>UNDP-BRA-01232 - Benchmark Internacional e Análise de Adaptabilidade de Modelos Federativos de Gestão de Pessoas ao Contexto Brasileiro</t>
+          <t>4BRZ4025 - Edital 18/2026 - Consultor Individual (1 Vaga)  REPUBLICAÇÃO</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1597,62 +1611,54 @@
       </c>
       <c r="E13" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F13" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F13" s="21" t="inlineStr"/>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
         <is>
-          <t>PNUD (Direto)</t>
-        </is>
-      </c>
-      <c r="I13" s="19" t="inlineStr">
-        <is>
-          <t>Home based</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I13" s="19" t="inlineStr"/>
       <c r="J13" s="22" t="n">
-        <v>46255</v>
+        <v>46266</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46268</v>
+        <v>46270</v>
       </c>
       <c r="L13" s="23" t="inlineStr"/>
       <c r="M13" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N13" s="20" t="inlineStr">
-        <is>
-          <t>ic.procurement.br@undp.org</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N13" s="20" t="inlineStr"/>
       <c r="O13" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="n">
-        <v>146337</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>unesco:eb67e949-3d0c-4334-df1b-08df01dbdf45</t>
+        </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>IC UNDP-BRA-01228 - Benchmarking, modelagem federativa e análise de viabilidade institucional</t>
+          <t>586RLA2002 - Edital 002/2026 - 1 vaga</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1670,54 +1676,48 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>PNUD (Direto)</t>
-        </is>
-      </c>
-      <c r="I14" s="11" t="inlineStr">
-        <is>
-          <t>Home based</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="14" t="n">
-        <v>46255</v>
+        <v>46261</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46268</v>
+        <v>46272</v>
       </c>
       <c r="L14" s="15" t="inlineStr"/>
       <c r="M14" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N14" s="12" t="inlineStr">
-        <is>
-          <t>aquisicoes.cbo.br@undp.org</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N14" s="12" t="inlineStr"/>
       <c r="O14" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B15" s="18" t="n">
-        <v>146346</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
+        </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor (a) individual para assessoramento técnico especializado à consolidação, redação técnica e estruturação dos mecanismos de governança do Plano Estadual de Educação do Piauí 2026-2036</t>
+          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1735,54 +1735,48 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="I15" s="19" t="inlineStr">
-        <is>
-          <t>Home based</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46262</v>
+        <v>46253</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46276</v>
+        <v>46269</v>
       </c>
       <c r="L15" s="23" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N15" s="20" t="inlineStr">
-        <is>
-          <t>ugest@seduc.pi.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N15" s="20" t="inlineStr"/>
       <c r="O15" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="n">
-        <v>146347</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>unesco:17177a8d-bde0-4a60-df1c-08df01dbdf45</t>
+        </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor (a) individual para apoiar tecnicamente a Superintendência de Ensino na realização das Olimpíadas do Conhecimento</t>
+          <t>914BRZ1159 - Publicação Edital 36/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1800,39 +1794,31 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Saúde, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="I16" s="11" t="inlineStr">
-        <is>
-          <t>Home based</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46262</v>
+        <v>46265</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46276</v>
+        <v>46271</v>
       </c>
       <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N16" s="12" t="inlineStr">
-        <is>
-          <t>ugest@seduc.pi.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N16" s="12" t="inlineStr"/>
       <c r="O16" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -1844,12 +1830,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:5d64862a-264d-475d-5f8e-08df036d3e00</t>
+          <t>unesco:b324319d-9f96-425f-8caf-08defc5a5785</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>4BRZ4025 - Edital 18/2026 - Consultor Individual (1 Vaga)  REPUBLICAÇÃO</t>
+          <t>914BRZ1155 - EDITAL Nº 48/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1859,13 +1845,15 @@
       </c>
       <c r="E17" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F17" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1878,7 +1866,7 @@
         <v>46266</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46270</v>
+        <v>46274</v>
       </c>
       <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
@@ -1901,12 +1889,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:eb67e949-3d0c-4334-df1b-08df01dbdf45</t>
+          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>586RLA2002 - Edital 002/2026 - 1 vaga</t>
+          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1924,7 +1912,7 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1934,10 +1922,10 @@
       </c>
       <c r="I18" s="11" t="inlineStr"/>
       <c r="J18" s="14" t="n">
-        <v>46261</v>
+        <v>46266</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46272</v>
+        <v>46274</v>
       </c>
       <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
@@ -1960,12 +1948,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
+          <t>unesco:5c1d62c6-1efa-431c-b9e2-08df0436270c</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 54/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -1983,7 +1971,7 @@
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -1993,10 +1981,10 @@
       </c>
       <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46253</v>
+        <v>46266</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46269</v>
+        <v>46273</v>
       </c>
       <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
@@ -2019,12 +2007,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:17177a8d-bde0-4a60-df1c-08df01dbdf45</t>
+          <t>unesco:c9020343-9d28-49e3-b9e3-08df0436270c</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 36/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 52/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2042,7 +2030,7 @@
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Saúde, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2052,10 +2040,10 @@
       </c>
       <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46271</v>
+        <v>46273</v>
       </c>
       <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
@@ -2078,12 +2066,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:e6ba376a-8848-485f-3f37-08defeb303ea</t>
+          <t>unesco:b74745df-a51d-41c1-b9e5-08df0436270c</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1163 - Publicação -  Edital 67/2026 - 01 Vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 55/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2111,10 +2099,10 @@
       </c>
       <c r="I21" s="19" t="inlineStr"/>
       <c r="J21" s="22" t="n">
-        <v>46260</v>
+        <v>46266</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46266</v>
+        <v>46273</v>
       </c>
       <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
@@ -2137,12 +2125,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:b324319d-9f96-425f-8caf-08defc5a5785</t>
+          <t>unesco:f4efa11a-ea51-47cf-b9e7-08df0436270c</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 48/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 56/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2160,7 +2148,7 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2173,7 +2161,7 @@
         <v>46266</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
@@ -2196,12 +2184,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
+          <t>unesco:6f0bebf7-7be2-4b29-17c5-08df04786cdd</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 53/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2219,7 +2207,7 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2232,7 +2220,7 @@
         <v>46266</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="L23" s="23" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr">
@@ -2255,12 +2243,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:5c1d62c6-1efa-431c-b9e2-08df0436270c</t>
+          <t>unesco:4fda0c36-f1a0-41f6-3f3a-08defeb303ea</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 54/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 47/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2278,7 +2266,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2288,10 +2276,10 @@
       </c>
       <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46266</v>
+        <v>46262</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46273</v>
+        <v>46268</v>
       </c>
       <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
@@ -2314,12 +2302,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:c9020343-9d28-49e3-b9e3-08df0436270c</t>
+          <t>unesco:4db2e20b-a2e2-4074-00dc-08deff7b5e96</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 52/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 49/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2337,7 +2325,7 @@
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2347,10 +2335,10 @@
       </c>
       <c r="I25" s="19" t="inlineStr"/>
       <c r="J25" s="22" t="n">
-        <v>46266</v>
+        <v>46262</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46273</v>
+        <v>46268</v>
       </c>
       <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
@@ -2373,12 +2361,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:b74745df-a51d-41c1-b9e5-08df0436270c</t>
+          <t>unesco:ecd2379c-2ba5-488f-00dd-08deff7b5e96</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 55/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 50/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2396,7 +2384,7 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2406,10 +2394,10 @@
       </c>
       <c r="I26" s="11" t="inlineStr"/>
       <c r="J26" s="14" t="n">
-        <v>46266</v>
+        <v>46262</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46273</v>
+        <v>46268</v>
       </c>
       <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
@@ -2432,12 +2420,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:f4efa11a-ea51-47cf-b9e7-08df0436270c</t>
+          <t>unesco:11c715d6-1d36-4c54-5f8f-08df036d3e00</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 56/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ4027 - Edital 55/2026 - Ciências Sociais</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2455,7 +2443,7 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2468,7 +2456,7 @@
         <v>46266</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46273</v>
+        <v>46271</v>
       </c>
       <c r="L27" s="23" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr">
@@ -2486,22 +2474,22 @@
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>unesco:6f0bebf7-7be2-4b29-17c5-08df04786cdd</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 53/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -2510,57 +2498,67 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I28" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J28" s="14" t="n">
-        <v>46266</v>
+        <v>46213</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46273</v>
-      </c>
-      <c r="L28" s="15" t="inlineStr"/>
+        <v>46217</v>
+      </c>
+      <c r="L28" s="15" t="n">
+        <v>144000</v>
+      </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N28" s="12" t="inlineStr"/>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N28" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>unesco:4fda0c36-f1a0-41f6-3f3a-08defeb303ea</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 47/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
@@ -2569,57 +2567,67 @@
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I29" s="19" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I29" s="19" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
       <c r="J29" s="22" t="n">
-        <v>46262</v>
+        <v>46216</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46268</v>
-      </c>
-      <c r="L29" s="23" t="inlineStr"/>
+        <v>46223</v>
+      </c>
+      <c r="L29" s="23" t="n">
+        <v>133000</v>
+      </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N29" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N29" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>unesco:4db2e20b-a2e2-4074-00dc-08deff7b5e96</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 49/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2637,48 +2645,56 @@
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I30" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J30" s="14" t="n">
-        <v>46262</v>
+        <v>46213</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46268</v>
+        <v>46220</v>
       </c>
       <c r="L30" s="15" t="inlineStr"/>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N30" s="12" t="inlineStr"/>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N30" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>unesco:ecd2379c-2ba5-488f-00dd-08deff7b5e96</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 50/2026 - 2 vagas - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13067</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
@@ -2687,57 +2703,67 @@
         </is>
       </c>
       <c r="F31" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I31" s="19" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I31" s="19" t="inlineStr">
+        <is>
+          <t>Secretaria de Estado da Educação  SEED-PR</t>
+        </is>
+      </c>
       <c r="J31" s="22" t="n">
-        <v>46262</v>
+        <v>46212</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46268</v>
-      </c>
-      <c r="L31" s="23" t="inlineStr"/>
+        <v>46224</v>
+      </c>
+      <c r="L31" s="23" t="n">
+        <v>150000</v>
+      </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N31" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N31" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067/</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>unesco:11c715d6-1d36-4c54-5f8f-08df036d3e00</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 55/2026 - Ciências Sociais</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
@@ -2746,35 +2772,45 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I32" s="11" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I32" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J32" s="14" t="n">
-        <v>46266</v>
+        <v>46217</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46271</v>
-      </c>
-      <c r="L32" s="15" t="inlineStr"/>
+        <v>46222</v>
+      </c>
+      <c r="L32" s="15" t="n">
+        <v>77100</v>
+      </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N32" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N32" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
         </is>
       </c>
     </row>
@@ -2786,12 +2822,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEC/BRA/24 – TR 13056</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2805,35 +2841,33 @@
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46216</v>
+        <v>46209</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46223</v>
-      </c>
-      <c r="L33" s="23" t="n">
-        <v>133000</v>
-      </c>
+        <v>46214</v>
+      </c>
+      <c r="L33" s="23" t="inlineStr"/>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N33" s="20" t="inlineStr">
@@ -2843,7 +2877,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056/</t>
         </is>
       </c>
     </row>
@@ -2855,17 +2889,17 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -2878,7 +2912,7 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -2888,21 +2922,21 @@
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46213</v>
+        <v>46225</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46217</v>
+        <v>46229</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>144000</v>
+        <v>114600</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N34" s="12" t="inlineStr">
@@ -2912,7 +2946,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
         </is>
       </c>
     </row>
@@ -2924,17 +2958,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -2943,11 +2977,11 @@
         </is>
       </c>
       <c r="F35" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -2961,15 +2995,17 @@
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46213</v>
+        <v>46223</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46220</v>
-      </c>
-      <c r="L35" s="23" t="inlineStr"/>
+        <v>46238</v>
+      </c>
+      <c r="L35" s="23" t="n">
+        <v>100000</v>
+      </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N35" s="20" t="inlineStr">
@@ -2979,7 +3015,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
         </is>
       </c>
     </row>
@@ -2991,12 +3027,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3014,12 +3050,12 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
@@ -3028,13 +3064,13 @@
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46217</v>
+        <v>46220</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46222</v>
+        <v>46225</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>77100</v>
+        <v>58800</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3048,7 +3084,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
         </is>
       </c>
     </row>
@@ -3060,12 +3096,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEC/BRA/24 – TR 13056</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR 12970</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3088,19 +3124,19 @@
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46209</v>
+        <v>46183</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46214</v>
+        <v>46188</v>
       </c>
       <c r="L37" s="23" t="inlineStr"/>
       <c r="M37" s="17" t="inlineStr">
@@ -3115,7 +3151,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970/</t>
         </is>
       </c>
     </row>
@@ -3127,12 +3163,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13067</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3146,11 +3182,11 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3160,21 +3196,19 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Secretaria de Estado da Educação  SEED-PR</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46212</v>
+        <v>46221</v>
       </c>
       <c r="K38" s="14" t="n">
         <v>46224</v>
       </c>
-      <c r="L38" s="15" t="n">
-        <v>150000</v>
-      </c>
+      <c r="L38" s="15" t="inlineStr"/>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
@@ -3184,7 +3218,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
         </is>
       </c>
     </row>
@@ -3196,12 +3230,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3219,7 +3253,7 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3229,21 +3263,21 @@
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46220</v>
+        <v>46227</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46225</v>
+        <v>46231</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>58800</v>
+        <v>150000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
@@ -3253,7 +3287,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -3265,17 +3299,17 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
@@ -3284,33 +3318,35 @@
         </is>
       </c>
       <c r="F40" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46221</v>
+        <v>46224</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46224</v>
-      </c>
-      <c r="L40" s="15" t="inlineStr"/>
+        <v>46233</v>
+      </c>
+      <c r="L40" s="15" t="n">
+        <v>288000</v>
+      </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
@@ -3320,7 +3356,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -3332,17 +3368,17 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR 12970</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
@@ -3351,33 +3387,35 @@
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.3</v>
+        <v>0.343</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46183</v>
+        <v>46232</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46188</v>
-      </c>
-      <c r="L41" s="23" t="inlineStr"/>
+        <v>46238</v>
+      </c>
+      <c r="L41" s="23" t="n">
+        <v>30000</v>
+      </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
@@ -3387,7 +3425,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -3399,50 +3437,48 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F42" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F42" s="13" t="inlineStr"/>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46223</v>
+        <v>46232</v>
       </c>
       <c r="K42" s="14" t="n">
         <v>46238</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>100000</v>
+        <v>30000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3456,7 +3492,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -3468,12 +3504,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3491,7 +3527,7 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
@@ -3501,17 +3537,17 @@
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46229</v>
+        <v>46237</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>114600</v>
+        <v>288000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
@@ -3525,7 +3561,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -3537,12 +3573,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3565,26 +3601,26 @@
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Brasília DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46227</v>
+        <v>46240</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46231</v>
+        <v>46245</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>150000</v>
+        <v>204000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N44" s="12" t="inlineStr">
@@ -3594,7 +3630,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -3606,12 +3642,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3629,7 +3665,7 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
@@ -3639,17 +3675,17 @@
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46224</v>
+        <v>46240</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46233</v>
+        <v>46245</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>288000</v>
+        <v>80000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
@@ -3663,7 +3699,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -3675,12 +3711,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3690,13 +3726,15 @@
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F46" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F46" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3706,17 +3744,17 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>30000</v>
+        <v>204000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3730,7 +3768,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -3742,17 +3780,17 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E47" s="20" t="inlineStr">
@@ -3765,41 +3803,41 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46232</v>
+        <v>46244</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46237</v>
+        <v>46296</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>288000</v>
+        <v>935000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -3811,50 +3849,48 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F48" s="13" t="n">
-        <v>0.343</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F48" s="13" t="inlineStr"/>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46232</v>
+        <v>46227</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46238</v>
+        <v>46252</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>30000</v>
+        <v>286000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3868,7 +3904,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3880,17 +3916,17 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
@@ -3903,41 +3939,41 @@
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46240</v>
+        <v>46244</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46245</v>
+        <v>46300</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>204000</v>
+        <v>350000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3949,12 +3985,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -3968,11 +4004,11 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
@@ -3982,21 +4018,19 @@
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46245</v>
-      </c>
-      <c r="L50" s="15" t="n">
-        <v>204000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L50" s="15" t="inlineStr"/>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
@@ -4006,7 +4040,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -4018,12 +4052,12 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -4041,7 +4075,7 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
@@ -4051,7 +4085,7 @@
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
@@ -4075,7 +4109,7 @@
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -4087,17 +4121,17 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
@@ -4115,36 +4149,36 @@
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46244</v>
+        <v>46240</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46300</v>
+        <v>46245</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>350000</v>
+        <v>100000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -4156,12 +4190,12 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -4179,27 +4213,27 @@
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>80000</v>
+        <v>54000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
@@ -4213,7 +4247,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -4225,12 +4259,12 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
@@ -4248,27 +4282,27 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>100000</v>
+        <v>54000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
@@ -4282,7 +4316,7 @@
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -4294,17 +4328,17 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
@@ -4317,41 +4351,41 @@
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46244</v>
+        <v>46251</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46296</v>
+        <v>46256</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>935000</v>
+        <v>50000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N55" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -4363,12 +4397,12 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
@@ -4382,33 +4416,35 @@
         </is>
       </c>
       <c r="F56" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46246</v>
+        <v>46252</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L56" s="15" t="inlineStr"/>
+        <v>46259</v>
+      </c>
+      <c r="L56" s="15" t="n">
+        <v>60000</v>
+      </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N56" s="12" t="inlineStr">
@@ -4418,7 +4454,7 @@
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -4430,62 +4466,64 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F57" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F57" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46227</v>
+        <v>46208</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46252</v>
+        <v>46259</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>286000</v>
+        <v>500000</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N57" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4497,12 +4535,12 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
@@ -4520,7 +4558,7 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
@@ -4537,14 +4575,14 @@
         <v>46246</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46257</v>
+        <v>46272</v>
       </c>
       <c r="L58" s="15" t="n">
         <v>54000</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N58" s="12" t="inlineStr">
@@ -4554,7 +4592,7 @@
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -4566,22 +4604,22 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E59" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F59" s="21" t="n">
@@ -4589,27 +4627,27 @@
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I59" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J59" s="22" t="n">
-        <v>46251</v>
+        <v>46265</v>
       </c>
       <c r="K59" s="22" t="n">
-        <v>46256</v>
+        <v>46270</v>
       </c>
       <c r="L59" s="23" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
@@ -4623,7 +4661,7 @@
       </c>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -4635,12 +4673,12 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
@@ -4658,7 +4696,7 @@
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H60" s="11" t="inlineStr">
@@ -4668,17 +4706,17 @@
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J60" s="14" t="n">
-        <v>46246</v>
+        <v>46266</v>
       </c>
       <c r="K60" s="14" t="n">
-        <v>46257</v>
+        <v>46275</v>
       </c>
       <c r="L60" s="15" t="n">
-        <v>54000</v>
+        <v>70000</v>
       </c>
       <c r="M60" s="9" t="inlineStr">
         <is>
@@ -4692,288 +4730,12 @@
       </c>
       <c r="O60" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B61" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
-        </is>
-      </c>
-      <c r="C61" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
-        </is>
-      </c>
-      <c r="D61" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E61" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F61" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G61" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados</t>
-        </is>
-      </c>
-      <c r="H61" s="19" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I61" s="19" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="J61" s="22" t="n">
-        <v>46252</v>
-      </c>
-      <c r="K61" s="22" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L61" s="23" t="n">
-        <v>60000</v>
-      </c>
-      <c r="M61" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N61" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O61" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B62" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
-        </is>
-      </c>
-      <c r="C62" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
-        </is>
-      </c>
-      <c r="D62" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Física (PF)</t>
-        </is>
-      </c>
-      <c r="E62" s="12" t="inlineStr">
-        <is>
-          <t>Economista</t>
-        </is>
-      </c>
-      <c r="F62" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G62" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
-        </is>
-      </c>
-      <c r="H62" s="11" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I62" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="J62" s="14" t="n">
-        <v>46265</v>
-      </c>
-      <c r="K62" s="14" t="n">
-        <v>46270</v>
-      </c>
-      <c r="L62" s="15" t="n">
-        <v>30000</v>
-      </c>
-      <c r="M62" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N62" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O62" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B63" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
-        </is>
-      </c>
-      <c r="C63" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
-        </is>
-      </c>
-      <c r="D63" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E63" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F63" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G63" s="19" t="inlineStr">
-        <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
-        </is>
-      </c>
-      <c r="H63" s="19" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I63" s="19" t="inlineStr">
-        <is>
-          <t>Porto Alegre/RS</t>
-        </is>
-      </c>
-      <c r="J63" s="22" t="n">
-        <v>46246</v>
-      </c>
-      <c r="K63" s="22" t="n">
-        <v>46272</v>
-      </c>
-      <c r="L63" s="23" t="n">
-        <v>54000</v>
-      </c>
-      <c r="M63" s="17" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N63" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O63" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B64" s="10" t="inlineStr">
-        <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
-        </is>
-      </c>
-      <c r="C64" s="11" t="inlineStr">
-        <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
-        </is>
-      </c>
-      <c r="D64" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
-        </is>
-      </c>
-      <c r="E64" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F64" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G64" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados</t>
-        </is>
-      </c>
-      <c r="H64" s="11" t="inlineStr">
-        <is>
-          <t>OEI/MDHC</t>
-        </is>
-      </c>
-      <c r="I64" s="11" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="J64" s="14" t="n">
-        <v>46208</v>
-      </c>
-      <c r="K64" s="14" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L64" s="15" t="n">
-        <v>500000</v>
-      </c>
-      <c r="M64" s="9" t="inlineStr">
-        <is>
-          <t>En presentación</t>
-        </is>
-      </c>
-      <c r="N64" s="12" t="inlineStr">
-        <is>
-          <t>compras.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O64" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O64"/>
+  <autoFilter ref="A1:O60"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -5034,10 +4796,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId63"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -5076,7 +4834,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3">
@@ -5086,7 +4844,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -5096,7 +4854,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -5148,7 +4906,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -5200,7 +4958,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
@@ -5210,7 +4968,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -5220,7 +4978,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -5282,7 +5040,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4">
@@ -5298,31 +5056,31 @@
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Meio Ambiente / Clima / Geografia</t>
+          <t>Economia / Finanças Públicas</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Economia / Finanças Públicas</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -5358,7 +5116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5384,7 +5142,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3">
@@ -5394,7 +5152,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -5414,41 +5172,31 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>PNUD (Direto)</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>PNUD (Direto)</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="n">
         <v>2</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B8"/>
+  <autoFilter ref="A1:B7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -5507,7 +5255,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-03 15:53
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$61</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 02/09/2026 às 16:03</t>
+          <t>Gerado em 03/09/2026 às 15:51</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O60"/>
+  <dimension ref="A1:O61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -876,16 +876,16 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>146313</v>
+        <v>146326</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>Consultoria técnica especializada para desenvolvimento de proposta de governança e curadoria da Base de Conhecimento destinada ao suporte de soluções de Inteligência Artificial da área de Integridade da Secretaria do Tesouro Nacional</t>
+          <t>Edital nº 02/2026 – Metodologia para monitoramento das decisões da Corte Interamericana de Direitos Humanos</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E2" s="12" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H2" s="11" t="inlineStr">
@@ -908,14 +908,14 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Território Nacional</t>
         </is>
       </c>
       <c r="J2" s="14" t="n">
-        <v>46254</v>
+        <v>46258</v>
       </c>
       <c r="K2" s="14" t="n">
-        <v>46267</v>
+        <v>46274</v>
       </c>
       <c r="L2" s="15" t="inlineStr"/>
       <c r="M2" s="9" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="N2" s="12" t="inlineStr">
         <is>
-          <t>ucp.codin.df.stn@tesouro.gov.br</t>
+          <t>ccidh@mdh.gov.br</t>
         </is>
       </c>
       <c r="O2" s="16" t="inlineStr">
@@ -941,11 +941,11 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>146326</v>
+        <v>146327</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 02/2026 – Metodologia para monitoramento das decisões da Corte Interamericana de Direitos Humanos</t>
+          <t>Edital nº 3/2026 – Metodologia para monitoramento de recomendações e decisões da Comissão Interamericana de Direitos Humanos</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
@@ -1006,11 +1006,11 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146327</v>
+        <v>146332</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 3/2026 – Metodologia para monitoramento de recomendações e decisões da Comissão Interamericana de Direitos Humanos</t>
+          <t>Edital nº 04/2026 - Segundo Plano da Política Nacional de RCN</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="N4" s="12" t="inlineStr">
         <is>
-          <t>ccidh@mdh.gov.br</t>
+          <t>rcn_cidadania@mdh.gov.br</t>
         </is>
       </c>
       <c r="O4" s="16" t="inlineStr">
@@ -1071,16 +1071,16 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146332</v>
+        <v>146335</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 04/2026 - Segundo Plano da Política Nacional de RCN</t>
+          <t>Consultoria técnica especializada para avaliação das capacidades institucionais da Secretaria do Tesouro Nacional (STN)</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E5" s="20" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
@@ -1103,14 +1103,14 @@
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J5" s="22" t="n">
         <v>46258</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46274</v>
+        <v>46271</v>
       </c>
       <c r="L5" s="23" t="inlineStr"/>
       <c r="M5" s="17" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>rcn_cidadania@mdh.gov.br</t>
+          <t>ucp.codin.df.stn@tesouro.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1136,16 +1136,16 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146335</v>
+        <v>146336</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Consultoria técnica especializada para avaliação das capacidades institucionais da Secretaria do Tesouro Nacional (STN)</t>
+          <t>UNDP-BRA-01232 - Benchmark Internacional e Análise de Adaptabilidade de Modelos Federativos de Gestão de Pessoas ao Contexto Brasileiro</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -1158,24 +1158,24 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>PNUD (Direto)</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Home based</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
-        <v>46258</v>
+        <v>46255</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>46271</v>
+        <v>46268</v>
       </c>
       <c r="L6" s="15" t="inlineStr"/>
       <c r="M6" s="9" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
-          <t>ucp.codin.df.stn@tesouro.gov.br</t>
+          <t>ic.procurement.br@undp.org</t>
         </is>
       </c>
       <c r="O6" s="16" t="inlineStr">
@@ -1201,11 +1201,11 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146336</v>
+        <v>146337</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>UNDP-BRA-01232 - Benchmark Internacional e Análise de Adaptabilidade de Modelos Federativos de Gestão de Pessoas ao Contexto Brasileiro</t>
+          <t>IC UNDP-BRA-01228 - Benchmarking, modelagem federativa e análise de viabilidade institucional</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="N7" s="20" t="inlineStr">
         <is>
-          <t>ic.procurement.br@undp.org</t>
+          <t>aquisicoes.cbo.br@undp.org</t>
         </is>
       </c>
       <c r="O7" s="24" t="inlineStr">
@@ -1266,16 +1266,16 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146337</v>
+        <v>146343</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>IC UNDP-BRA-01228 - Benchmarking, modelagem federativa e análise de viabilidade institucional</t>
+          <t>TR 005/2026 - ASPAD - MDA - Contratação de consultoria especializada para participação social no Plano Safra da Agricultura Familiar</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -1288,26 +1288,28 @@
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>PNUD (Direto)</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Home based</t>
+          <t>Brasília/DF</t>
         </is>
       </c>
       <c r="J8" s="14" t="n">
-        <v>46255</v>
+        <v>46268</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>46268</v>
-      </c>
-      <c r="L8" s="15" t="inlineStr"/>
+        <v>46277</v>
+      </c>
+      <c r="L8" s="15" t="n">
+        <v>130000</v>
+      </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1315,7 +1317,7 @@
       </c>
       <c r="N8" s="12" t="inlineStr">
         <is>
-          <t>aquisicoes.cbo.br@undp.org</t>
+          <t>cgctf.editais@mda.gov.br</t>
         </is>
       </c>
       <c r="O8" s="16" t="inlineStr">
@@ -1502,9 +1504,7 @@
       <c r="K11" s="22" t="n">
         <v>46278</v>
       </c>
-      <c r="L11" s="23" t="n">
-        <v>200000</v>
-      </c>
+      <c r="L11" s="23" t="inlineStr"/>
       <c r="M11" s="17" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1570,7 +1570,7 @@
         <v>46272</v>
       </c>
       <c r="L12" s="15" t="n">
-        <v>55000</v>
+        <v>55</v>
       </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
@@ -1653,12 +1653,12 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>unesco:eb67e949-3d0c-4334-df1b-08df01dbdf45</t>
+          <t>unesco:1d72ac67-6c7d-4a8b-dd78-08df0757caed</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>586RLA2002 - Edital 002/2026 - 1 vaga</t>
+          <t>914BRZ1154 - Edital 05/2026 - 01 perfil - Consultoria Individual</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1676,7 +1676,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1686,10 +1686,10 @@
       </c>
       <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="14" t="n">
-        <v>46261</v>
+        <v>46268</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46272</v>
+        <v>46278</v>
       </c>
       <c r="L14" s="15" t="inlineStr"/>
       <c r="M14" s="9" t="inlineStr">
@@ -1712,12 +1712,12 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
+          <t>unesco:eb67e949-3d0c-4334-df1b-08df01dbdf45</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
+          <t>586RLA2002 - Edital 002/2026 - 1 vaga</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
@@ -1745,10 +1745,10 @@
       </c>
       <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46253</v>
+        <v>46261</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="L15" s="23" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr">
@@ -1771,12 +1771,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:17177a8d-bde0-4a60-df1c-08df01dbdf45</t>
+          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 36/2026 - 1 vaga - Consultor Individual</t>
+          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Saúde, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1804,10 +1804,10 @@
       </c>
       <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46265</v>
+        <v>46253</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46271</v>
+        <v>46269</v>
       </c>
       <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
@@ -1830,12 +1830,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:b324319d-9f96-425f-8caf-08defc5a5785</t>
+          <t>unesco:17177a8d-bde0-4a60-df1c-08df01dbdf45</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 48/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 36/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Saúde, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1863,10 +1863,10 @@
       </c>
       <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46266</v>
+        <v>46265</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46274</v>
+        <v>46271</v>
       </c>
       <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
@@ -1889,12 +1889,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
+          <t>unesco:b324319d-9f96-425f-8caf-08defc5a5785</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 48/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1912,7 +1912,7 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1948,12 +1948,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:5c1d62c6-1efa-431c-b9e2-08df0436270c</t>
+          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 54/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -1971,7 +1971,7 @@
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -1984,7 +1984,7 @@
         <v>46266</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
@@ -2007,12 +2007,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:c9020343-9d28-49e3-b9e3-08df0436270c</t>
+          <t>unesco:5c1d62c6-1efa-431c-b9e2-08df0436270c</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 52/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 54/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2066,12 +2066,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:b74745df-a51d-41c1-b9e5-08df0436270c</t>
+          <t>unesco:c9020343-9d28-49e3-b9e3-08df0436270c</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 55/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 52/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2125,12 +2125,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:f4efa11a-ea51-47cf-b9e7-08df0436270c</t>
+          <t>unesco:b74745df-a51d-41c1-b9e5-08df0436270c</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 56/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 55/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2148,7 +2148,7 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2184,12 +2184,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:6f0bebf7-7be2-4b29-17c5-08df04786cdd</t>
+          <t>unesco:f4efa11a-ea51-47cf-b9e7-08df0436270c</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 53/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 56/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2243,12 +2243,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:4fda0c36-f1a0-41f6-3f3a-08defeb303ea</t>
+          <t>unesco:6f0bebf7-7be2-4b29-17c5-08df04786cdd</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 47/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 53/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2276,10 +2276,10 @@
       </c>
       <c r="I24" s="11" t="inlineStr"/>
       <c r="J24" s="14" t="n">
-        <v>46262</v>
+        <v>46266</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46268</v>
+        <v>46273</v>
       </c>
       <c r="L24" s="15" t="inlineStr"/>
       <c r="M24" s="9" t="inlineStr">
@@ -2302,12 +2302,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:4db2e20b-a2e2-4074-00dc-08deff7b5e96</t>
+          <t>unesco:4fda0c36-f1a0-41f6-3f3a-08defeb303ea</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 49/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 47/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2361,12 +2361,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:ecd2379c-2ba5-488f-00dd-08deff7b5e96</t>
+          <t>unesco:4db2e20b-a2e2-4074-00dc-08deff7b5e96</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 50/2026 - 2 vagas - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 49/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2420,12 +2420,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:11c715d6-1d36-4c54-5f8f-08df036d3e00</t>
+          <t>unesco:ecd2379c-2ba5-488f-00dd-08deff7b5e96</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 55/2026 - Ciências Sociais</t>
+          <t>914BRZ1155 - EDITAL Nº 50/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2453,10 +2453,10 @@
       </c>
       <c r="I27" s="19" t="inlineStr"/>
       <c r="J27" s="22" t="n">
-        <v>46266</v>
+        <v>46262</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46271</v>
+        <v>46268</v>
       </c>
       <c r="L27" s="23" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr">
@@ -2474,22 +2474,22 @@
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
+          <t>unesco:11c715d6-1d36-4c54-5f8f-08df036d3e00</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
+          <t>914BRZ4027 - Edital 55/2026 - Ciências Sociais</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -2498,45 +2498,35 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I28" s="11" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr"/>
       <c r="J28" s="14" t="n">
-        <v>46213</v>
+        <v>46266</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46217</v>
-      </c>
-      <c r="L28" s="15" t="n">
-        <v>144000</v>
-      </c>
+        <v>46271</v>
+      </c>
+      <c r="L28" s="15" t="inlineStr"/>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N28" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N28" s="12" t="inlineStr"/>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -2548,12 +2538,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEC/BRA/24 – TR 13056</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2567,35 +2557,33 @@
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46216</v>
+        <v>46209</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46223</v>
-      </c>
-      <c r="L29" s="23" t="n">
-        <v>133000</v>
-      </c>
+        <v>46214</v>
+      </c>
+      <c r="L29" s="23" t="inlineStr"/>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N29" s="20" t="inlineStr">
@@ -2605,7 +2593,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056/</t>
         </is>
       </c>
     </row>
@@ -2617,17 +2605,17 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13067</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2636,11 +2624,11 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2650,19 +2638,21 @@
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Secretaria de Estado da Educação  SEED-PR</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46213</v>
+        <v>46212</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46220</v>
-      </c>
-      <c r="L30" s="15" t="inlineStr"/>
+        <v>46224</v>
+      </c>
+      <c r="L30" s="15" t="n">
+        <v>150000</v>
+      </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N30" s="12" t="inlineStr">
@@ -2672,7 +2662,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067/</t>
         </is>
       </c>
     </row>
@@ -2684,17 +2674,17 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13067</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E31" s="20" t="inlineStr">
@@ -2703,11 +2693,11 @@
         </is>
       </c>
       <c r="F31" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2717,21 +2707,19 @@
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Secretaria de Estado da Educação  SEED-PR</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46224</v>
-      </c>
-      <c r="L31" s="23" t="n">
-        <v>150000</v>
-      </c>
+        <v>46220</v>
+      </c>
+      <c r="L31" s="23" t="inlineStr"/>
       <c r="M31" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N31" s="20" t="inlineStr">
@@ -2741,7 +2729,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
         </is>
       </c>
     </row>
@@ -2753,17 +2741,17 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
@@ -2776,12 +2764,12 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
@@ -2790,17 +2778,17 @@
         </is>
       </c>
       <c r="J32" s="14" t="n">
+        <v>46213</v>
+      </c>
+      <c r="K32" s="14" t="n">
         <v>46217</v>
       </c>
-      <c r="K32" s="14" t="n">
-        <v>46222</v>
-      </c>
       <c r="L32" s="15" t="n">
-        <v>77100</v>
+        <v>144000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N32" s="12" t="inlineStr">
@@ -2810,7 +2798,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
         </is>
       </c>
     </row>
@@ -2822,12 +2810,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEC/BRA/24 – TR 13056</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2841,33 +2829,35 @@
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46209</v>
+        <v>46216</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46214</v>
-      </c>
-      <c r="L33" s="23" t="inlineStr"/>
+        <v>46223</v>
+      </c>
+      <c r="L33" s="23" t="n">
+        <v>133000</v>
+      </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N33" s="20" t="inlineStr">
@@ -2877,7 +2867,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
         </is>
       </c>
     </row>
@@ -2889,12 +2879,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2912,27 +2902,27 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46225</v>
+        <v>46217</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46229</v>
+        <v>46222</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>114600</v>
+        <v>77100</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
@@ -2946,7 +2936,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
         </is>
       </c>
     </row>
@@ -2958,17 +2948,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR 12970</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -2977,7 +2967,7 @@
         </is>
       </c>
       <c r="F35" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
@@ -2991,21 +2981,19 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46223</v>
+        <v>46183</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46238</v>
-      </c>
-      <c r="L35" s="23" t="n">
-        <v>100000</v>
-      </c>
+        <v>46188</v>
+      </c>
+      <c r="L35" s="23" t="inlineStr"/>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N35" s="20" t="inlineStr">
@@ -3015,7 +3003,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970/</t>
         </is>
       </c>
     </row>
@@ -3027,17 +3015,17 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
@@ -3046,11 +3034,11 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3064,17 +3052,15 @@
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46220</v>
+        <v>46221</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46225</v>
-      </c>
-      <c r="L36" s="15" t="n">
-        <v>58800</v>
-      </c>
+        <v>46224</v>
+      </c>
+      <c r="L36" s="15" t="inlineStr"/>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N36" s="12" t="inlineStr">
@@ -3084,7 +3070,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
         </is>
       </c>
     </row>
@@ -3096,12 +3082,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR 12970</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3115,11 +3101,11 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3129,19 +3115,21 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46183</v>
+        <v>46220</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46188</v>
-      </c>
-      <c r="L37" s="23" t="inlineStr"/>
+        <v>46225</v>
+      </c>
+      <c r="L37" s="23" t="n">
+        <v>58800</v>
+      </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N37" s="20" t="inlineStr">
@@ -3151,7 +3139,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
         </is>
       </c>
     </row>
@@ -3163,17 +3151,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3182,11 +3170,11 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3196,19 +3184,21 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46221</v>
+        <v>46225</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46224</v>
-      </c>
-      <c r="L38" s="15" t="inlineStr"/>
+        <v>46229</v>
+      </c>
+      <c r="L38" s="15" t="n">
+        <v>114600</v>
+      </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
@@ -3218,7 +3208,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
         </is>
       </c>
     </row>
@@ -3230,17 +3220,17 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
@@ -3263,21 +3253,21 @@
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Brasília DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46227</v>
+        <v>46223</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46231</v>
+        <v>46238</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
@@ -3287,7 +3277,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
         </is>
       </c>
     </row>
@@ -3299,12 +3289,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3322,31 +3312,31 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46224</v>
+        <v>46227</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46233</v>
+        <v>46231</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>288000</v>
+        <v>150000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
@@ -3356,7 +3346,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -3368,17 +3358,17 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
@@ -3387,11 +3377,11 @@
         </is>
       </c>
       <c r="F41" s="21" t="n">
-        <v>0.343</v>
+        <v>0.4</v>
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3401,17 +3391,17 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46232</v>
+        <v>46224</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46238</v>
+        <v>46233</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>30000</v>
+        <v>288000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3425,7 +3415,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -3437,28 +3427,30 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F42" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F42" s="13" t="n">
+        <v>0.343</v>
+      </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3492,7 +3484,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -3504,12 +3496,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3519,35 +3511,33 @@
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F43" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F43" s="21" t="inlineStr"/>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
         <v>46232</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>288000</v>
+        <v>30000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
@@ -3561,7 +3551,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -3573,12 +3563,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3596,27 +3586,27 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46245</v>
+        <v>46237</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>204000</v>
+        <v>288000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
@@ -3630,7 +3620,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -3642,12 +3632,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3665,7 +3655,7 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
@@ -3685,7 +3675,7 @@
         <v>46245</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>80000</v>
+        <v>204000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
@@ -3699,7 +3689,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -3780,17 +3770,17 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E47" s="20" t="inlineStr">
@@ -3808,36 +3798,36 @@
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46244</v>
+        <v>46240</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46296</v>
+        <v>46245</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>935000</v>
+        <v>80000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -3849,12 +3839,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3864,33 +3854,35 @@
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F48" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F48" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46227</v>
+        <v>46240</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46252</v>
+        <v>46245</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>286000</v>
+        <v>100000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
@@ -3904,7 +3896,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3916,17 +3908,17 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E49" s="20" t="inlineStr">
@@ -3939,41 +3931,41 @@
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46244</v>
+        <v>46240</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46300</v>
+        <v>46245</v>
       </c>
       <c r="L49" s="23" t="n">
-        <v>350000</v>
+        <v>80000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -3985,17 +3977,17 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
@@ -4004,7 +3996,7 @@
         </is>
       </c>
       <c r="F50" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
@@ -4013,21 +4005,23 @@
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46246</v>
+        <v>46244</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L50" s="15" t="inlineStr"/>
+        <v>46300</v>
+      </c>
+      <c r="L50" s="15" t="n">
+        <v>350000</v>
+      </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
@@ -4035,12 +4029,12 @@
       </c>
       <c r="N50" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4052,17 +4046,17 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
@@ -4075,41 +4069,41 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46240</v>
+        <v>46244</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46245</v>
+        <v>46296</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>80000</v>
+        <v>935000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -4121,12 +4115,12 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -4140,7 +4134,7 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
@@ -4154,21 +4148,19 @@
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46245</v>
-      </c>
-      <c r="L52" s="15" t="n">
-        <v>100000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L52" s="15" t="inlineStr"/>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
@@ -4178,7 +4170,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -4190,12 +4182,12 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -4205,15 +4197,13 @@
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F53" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F53" s="21" t="inlineStr"/>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
@@ -4223,17 +4213,17 @@
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46246</v>
+        <v>46227</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46257</v>
+        <v>46252</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>54000</v>
+        <v>286000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
@@ -4247,7 +4237,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -4328,17 +4318,17 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E55" s="20" t="inlineStr">
@@ -4351,7 +4341,7 @@
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
@@ -4361,17 +4351,17 @@
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J55" s="22" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="L55" s="23" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
@@ -4385,7 +4375,7 @@
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -4397,17 +4387,17 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
@@ -4420,7 +4410,7 @@
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
@@ -4430,17 +4420,17 @@
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46252</v>
+        <v>46251</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
@@ -4454,7 +4444,7 @@
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -4466,17 +4456,17 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E57" s="20" t="inlineStr">
@@ -4494,36 +4484,36 @@
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46208</v>
+        <v>46252</v>
       </c>
       <c r="K57" s="22" t="n">
         <v>46259</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>500000</v>
+        <v>60000</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N57" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -4535,22 +4525,22 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C58" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F58" s="13" t="n">
@@ -4558,31 +4548,31 @@
       </c>
       <c r="G58" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H58" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I58" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J58" s="14" t="n">
-        <v>46246</v>
+        <v>46265</v>
       </c>
       <c r="K58" s="14" t="n">
-        <v>46272</v>
+        <v>46270</v>
       </c>
       <c r="L58" s="15" t="n">
-        <v>54000</v>
+        <v>30000</v>
       </c>
       <c r="M58" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N58" s="12" t="inlineStr">
@@ -4592,7 +4582,7 @@
       </c>
       <c r="O58" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -4604,22 +4594,22 @@
       </c>
       <c r="B59" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E59" s="20" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F59" s="21" t="n">
@@ -4627,41 +4617,41 @@
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I59" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J59" s="22" t="n">
-        <v>46265</v>
+        <v>46208</v>
       </c>
       <c r="K59" s="22" t="n">
-        <v>46270</v>
+        <v>46259</v>
       </c>
       <c r="L59" s="23" t="n">
-        <v>30000</v>
+        <v>500000</v>
       </c>
       <c r="M59" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N59" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4673,12 +4663,12 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
@@ -4696,46 +4686,115 @@
       </c>
       <c r="G60" s="11" t="inlineStr">
         <is>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+        </is>
+      </c>
+      <c r="H60" s="11" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I60" s="11" t="inlineStr">
+        <is>
+          <t>Porto Alegre/RS</t>
+        </is>
+      </c>
+      <c r="J60" s="14" t="n">
+        <v>46246</v>
+      </c>
+      <c r="K60" s="14" t="n">
+        <v>46272</v>
+      </c>
+      <c r="L60" s="15" t="n">
+        <v>54000</v>
+      </c>
+      <c r="M60" s="9" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N60" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O60" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B61" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+        </is>
+      </c>
+      <c r="C61" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+        </is>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E61" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F61" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G61" s="19" t="inlineStr">
+        <is>
           <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
-      <c r="H60" s="11" t="inlineStr">
+      <c r="H61" s="19" t="inlineStr">
         <is>
           <t>OEI/BRA</t>
         </is>
       </c>
-      <c r="I60" s="11" t="inlineStr">
+      <c r="I61" s="19" t="inlineStr">
         <is>
           <t>São Paulo - SP</t>
         </is>
       </c>
-      <c r="J60" s="14" t="n">
+      <c r="J61" s="22" t="n">
         <v>46266</v>
       </c>
-      <c r="K60" s="14" t="n">
+      <c r="K61" s="22" t="n">
         <v>46275</v>
       </c>
-      <c r="L60" s="15" t="n">
+      <c r="L61" s="23" t="n">
         <v>70000</v>
       </c>
-      <c r="M60" s="9" t="inlineStr">
+      <c r="M61" s="17" t="inlineStr">
         <is>
           <t>En evaluación</t>
         </is>
       </c>
-      <c r="N60" s="12" t="inlineStr">
+      <c r="N61" s="20" t="inlineStr">
         <is>
           <t>selecao.bra@oei.int</t>
         </is>
       </c>
-      <c r="O60" s="16" t="inlineStr">
+      <c r="O61" s="24" t="inlineStr">
         <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O60"/>
+  <autoFilter ref="A1:O61"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4796,6 +4855,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4844,7 +4904,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
@@ -4896,7 +4956,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3">
@@ -4958,7 +5018,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3">
@@ -4968,7 +5028,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4">
@@ -4978,7 +5038,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -5026,21 +5086,21 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4">
@@ -5050,7 +5110,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5">
@@ -5152,7 +5212,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
@@ -5240,7 +5300,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5255,7 +5315,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5270,7 +5330,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5285,7 +5345,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-04 15:53
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$57</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -27,7 +27,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Por_Tipo'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Area'!$A$1:$B$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Por_Area'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Por_Orgao'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Perfis'!$A$1:$C$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Perfis'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 03/09/2026 às 15:51</t>
+          <t>Gerado em 04/09/2026 às 15:49</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O61"/>
+  <dimension ref="A1:O57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1136,16 +1136,16 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146336</v>
+        <v>146343</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>UNDP-BRA-01232 - Benchmark Internacional e Análise de Adaptabilidade de Modelos Federativos de Gestão de Pessoas ao Contexto Brasileiro</t>
+          <t>TR 005/2026 - ASPAD - MDA - Contratação de consultoria especializada para participação social no Plano Safra da Agricultura Familiar</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -1158,24 +1158,24 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>PNUD (Direto)</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Home based</t>
+          <t>Brasília/DF</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
-        <v>46255</v>
+        <v>46268</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>46268</v>
+        <v>46277</v>
       </c>
       <c r="L6" s="15" t="inlineStr"/>
       <c r="M6" s="9" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
-          <t>ic.procurement.br@undp.org</t>
+          <t>cgctf.editais@mda.gov.br</t>
         </is>
       </c>
       <c r="O6" s="16" t="inlineStr">
@@ -1201,11 +1201,11 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146337</v>
+        <v>146346</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>IC UNDP-BRA-01228 - Benchmarking, modelagem federativa e análise de viabilidade institucional</t>
+          <t>Contratação de consultor (a) individual para assessoramento técnico especializado à consolidação, redação técnica e estruturação dos mecanismos de governança do Plano Estadual de Educação do Piauí 2026-2036</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="H7" s="19" t="inlineStr">
         <is>
-          <t>PNUD (Direto)</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="I7" s="19" t="inlineStr">
@@ -1237,10 +1237,10 @@
         </is>
       </c>
       <c r="J7" s="22" t="n">
-        <v>46255</v>
+        <v>46262</v>
       </c>
       <c r="K7" s="22" t="n">
-        <v>46268</v>
+        <v>46276</v>
       </c>
       <c r="L7" s="23" t="inlineStr"/>
       <c r="M7" s="17" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="N7" s="20" t="inlineStr">
         <is>
-          <t>aquisicoes.cbo.br@undp.org</t>
+          <t>ugest@seduc.pi.gov.br</t>
         </is>
       </c>
       <c r="O7" s="24" t="inlineStr">
@@ -1266,16 +1266,16 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146343</v>
+        <v>146347</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>TR 005/2026 - ASPAD - MDA - Contratação de consultoria especializada para participação social no Plano Safra da Agricultura Familiar</t>
+          <t>Contratação de consultor (a) individual para apoiar tecnicamente a Superintendência de Ensino na realização das Olimpíadas do Conhecimento</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
@@ -1298,18 +1298,16 @@
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Brasília/DF</t>
+          <t>Home based</t>
         </is>
       </c>
       <c r="J8" s="14" t="n">
-        <v>46268</v>
+        <v>46262</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>46277</v>
-      </c>
-      <c r="L8" s="15" t="n">
-        <v>130000</v>
-      </c>
+        <v>46276</v>
+      </c>
+      <c r="L8" s="15" t="inlineStr"/>
       <c r="M8" s="9" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1317,7 +1315,7 @@
       </c>
       <c r="N8" s="12" t="inlineStr">
         <is>
-          <t>cgctf.editais@mda.gov.br</t>
+          <t>ugest@seduc.pi.gov.br</t>
         </is>
       </c>
       <c r="O8" s="16" t="inlineStr">
@@ -1333,16 +1331,16 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146346</v>
+        <v>146349</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor (a) individual para assessoramento técnico especializado à consolidação, redação técnica e estruturação dos mecanismos de governança do Plano Estadual de Educação do Piauí 2026-2036</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA PARA O DESENVOLVIMENTO DE TECNOLOGIA APLICADA AO OBSERVATÓRIO DO NORDESTE</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E9" s="20" t="inlineStr">
@@ -1355,7 +1353,7 @@
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
@@ -1365,14 +1363,14 @@
       </c>
       <c r="I9" s="19" t="inlineStr">
         <is>
-          <t>Home based</t>
+          <t>HOME OFFICE</t>
         </is>
       </c>
       <c r="J9" s="22" t="n">
-        <v>46262</v>
+        <v>46267</v>
       </c>
       <c r="K9" s="22" t="n">
-        <v>46276</v>
+        <v>46278</v>
       </c>
       <c r="L9" s="23" t="inlineStr"/>
       <c r="M9" s="17" t="inlineStr">
@@ -1382,7 +1380,7 @@
       </c>
       <c r="N9" s="20" t="inlineStr">
         <is>
-          <t>ugest@seduc.pi.gov.br</t>
+          <t>curriculos@consorcionordeste.gov.br</t>
         </is>
       </c>
       <c r="O9" s="24" t="inlineStr">
@@ -1398,11 +1396,11 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>146347</v>
+        <v>146350</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor (a) individual para apoiar tecnicamente a Superintendência de Ensino na realização das Olimpíadas do Conhecimento</t>
+          <t xml:space="preserve">Contratação de consultoria individual (pessoa física) para elaboração de estudo analítico, voltado ao mapeamento de empreendimentos vinculados à transição energética em execução ou em fase de planejamento e de seu potencial impacto sobre territórios quilombolas na Região Sudeste </t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1420,7 +1418,7 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -1430,16 +1428,18 @@
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>Home based</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J10" s="14" t="n">
-        <v>46262</v>
+        <v>46266</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>46276</v>
-      </c>
-      <c r="L10" s="15" t="inlineStr"/>
+        <v>46272</v>
+      </c>
+      <c r="L10" s="15" t="n">
+        <v>55</v>
+      </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1447,7 +1447,7 @@
       </c>
       <c r="N10" s="12" t="inlineStr">
         <is>
-          <t>ugest@seduc.pi.gov.br</t>
+          <t>dqc@igualdaderacial.gov.br</t>
         </is>
       </c>
       <c r="O10" s="16" t="inlineStr">
@@ -1459,20 +1459,22 @@
     <row r="11">
       <c r="A11" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="n">
-        <v>146349</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>unesco:11c715d6-1d36-4c54-5f8f-08df036d3e00</t>
+        </is>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>BRA/23/006 - CONSULTORIA TÉCNICA PARA O DESENVOLVIMENTO DE TECNOLOGIA APLICADA AO OBSERVATÓRIO DO NORDESTE</t>
+          <t>914BRZ4027 - Edital 55/2026 - Ciências Sociais</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E11" s="20" t="inlineStr">
@@ -1485,54 +1487,48 @@
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="I11" s="19" t="inlineStr">
-        <is>
-          <t>HOME OFFICE</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I11" s="19" t="inlineStr"/>
       <c r="J11" s="22" t="n">
-        <v>46267</v>
+        <v>46266</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46278</v>
+        <v>46271</v>
       </c>
       <c r="L11" s="23" t="inlineStr"/>
       <c r="M11" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N11" s="20" t="inlineStr">
-        <is>
-          <t>curriculos@consorcionordeste.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N11" s="20" t="inlineStr"/>
       <c r="O11" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="n">
-        <v>146350</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>unesco:5d64862a-264d-475d-5f8e-08df036d3e00</t>
+        </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contratação de consultoria individual (pessoa física) para elaboração de estudo analítico, voltado ao mapeamento de empreendimentos vinculados à transição energética em execução ou em fase de planejamento e de seu potencial impacto sobre territórios quilombolas na Região Sudeste </t>
+          <t>4BRZ4025 - Edital 18/2026 - Consultor Individual (1 Vaga)  REPUBLICAÇÃO</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1542,49 +1538,37 @@
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F12" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr"/>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="I12" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr"/>
       <c r="J12" s="14" t="n">
         <v>46266</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>46272</v>
-      </c>
-      <c r="L12" s="15" t="n">
-        <v>55</v>
-      </c>
+        <v>46270</v>
+      </c>
+      <c r="L12" s="15" t="inlineStr"/>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N12" s="12" t="inlineStr">
-        <is>
-          <t>dqc@igualdaderacial.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N12" s="12" t="inlineStr"/>
       <c r="O12" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -1596,12 +1580,12 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>unesco:5d64862a-264d-475d-5f8e-08df036d3e00</t>
+          <t>unesco:1d72ac67-6c7d-4a8b-dd78-08df0757caed</t>
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>4BRZ4025 - Edital 18/2026 - Consultor Individual (1 Vaga)  REPUBLICAÇÃO</t>
+          <t>914BRZ1154 - Edital 05/2026 - 01 perfil - Consultoria Individual</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1611,13 +1595,15 @@
       </c>
       <c r="E13" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F13" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F13" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
@@ -1627,10 +1613,10 @@
       </c>
       <c r="I13" s="19" t="inlineStr"/>
       <c r="J13" s="22" t="n">
-        <v>46266</v>
+        <v>46268</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46270</v>
+        <v>46278</v>
       </c>
       <c r="L13" s="23" t="inlineStr"/>
       <c r="M13" s="17" t="inlineStr">
@@ -1653,12 +1639,12 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>unesco:1d72ac67-6c7d-4a8b-dd78-08df0757caed</t>
+          <t>unesco:eb67e949-3d0c-4334-df1b-08df01dbdf45</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1154 - Edital 05/2026 - 01 perfil - Consultoria Individual</t>
+          <t>586RLA2002 - Edital 002/2026 - 1 vaga</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1676,7 +1662,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1686,10 +1672,10 @@
       </c>
       <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="14" t="n">
-        <v>46268</v>
+        <v>46261</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46278</v>
+        <v>46272</v>
       </c>
       <c r="L14" s="15" t="inlineStr"/>
       <c r="M14" s="9" t="inlineStr">
@@ -1712,12 +1698,12 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>unesco:eb67e949-3d0c-4334-df1b-08df01dbdf45</t>
+          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>586RLA2002 - Edital 002/2026 - 1 vaga</t>
+          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1735,7 +1721,7 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
@@ -1745,10 +1731,10 @@
       </c>
       <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46261</v>
+        <v>46253</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46272</v>
+        <v>46269</v>
       </c>
       <c r="L15" s="23" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr">
@@ -1771,12 +1757,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
+          <t>unesco:17177a8d-bde0-4a60-df1c-08df01dbdf45</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 36/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1794,7 +1780,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Saúde, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1804,10 +1790,10 @@
       </c>
       <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46253</v>
+        <v>46265</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46269</v>
+        <v>46271</v>
       </c>
       <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
@@ -1830,12 +1816,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:17177a8d-bde0-4a60-df1c-08df01dbdf45</t>
+          <t>unesco:b324319d-9f96-425f-8caf-08defc5a5785</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 36/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 48/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1853,7 +1839,7 @@
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Saúde, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1863,10 +1849,10 @@
       </c>
       <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46271</v>
+        <v>46274</v>
       </c>
       <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
@@ -1889,12 +1875,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:b324319d-9f96-425f-8caf-08defc5a5785</t>
+          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 48/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1912,7 +1898,7 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1948,12 +1934,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
+          <t>unesco:b0920c88-ab66-4545-2ead-08df08e94b75</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual</t>
+          <t xml:space="preserve">Projeto 914BRZ3050 - Edital N° 04/2026 - Consultor Individual </t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -1971,7 +1957,7 @@
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -1981,10 +1967,10 @@
       </c>
       <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46266</v>
+        <v>46269</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
@@ -2297,22 +2283,22 @@
     <row r="25">
       <c r="A25" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>unesco:4fda0c36-f1a0-41f6-3f3a-08defeb303ea</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 47/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E25" s="20" t="inlineStr">
@@ -2325,53 +2311,61 @@
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I25" s="19" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I25" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J25" s="22" t="n">
-        <v>46262</v>
+        <v>46213</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46268</v>
+        <v>46220</v>
       </c>
       <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N25" s="20" t="inlineStr"/>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N25" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>unesco:4db2e20b-a2e2-4074-00dc-08deff7b5e96</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 49/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13067</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
@@ -2380,57 +2374,67 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I26" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr">
+        <is>
+          <t>Secretaria de Estado da Educação  SEED-PR</t>
+        </is>
+      </c>
       <c r="J26" s="14" t="n">
-        <v>46262</v>
+        <v>46212</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46268</v>
-      </c>
-      <c r="L26" s="15" t="inlineStr"/>
+        <v>46224</v>
+      </c>
+      <c r="L26" s="15" t="n">
+        <v>150000</v>
+      </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N26" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N26" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>unesco:ecd2379c-2ba5-488f-00dd-08deff7b5e96</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 50/2026 - 2 vagas - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEC/BRA/24 – TR 13056</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
@@ -2443,53 +2447,61 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I27" s="19" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I27" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J27" s="22" t="n">
-        <v>46262</v>
+        <v>46209</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46268</v>
+        <v>46214</v>
       </c>
       <c r="L27" s="23" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N27" s="20" t="inlineStr"/>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N27" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056/</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>unesco:11c715d6-1d36-4c54-5f8f-08df036d3e00</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 55/2026 - Ciências Sociais</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -2498,35 +2510,45 @@
         </is>
       </c>
       <c r="F28" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I28" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J28" s="14" t="n">
-        <v>46266</v>
+        <v>46213</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46271</v>
-      </c>
-      <c r="L28" s="15" t="inlineStr"/>
+        <v>46217</v>
+      </c>
+      <c r="L28" s="15" t="n">
+        <v>144000</v>
+      </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N28" s="12" t="inlineStr"/>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N28" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
         </is>
       </c>
     </row>
@@ -2538,12 +2560,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEC/BRA/24 – TR 13056</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2557,33 +2579,35 @@
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46209</v>
+        <v>46216</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46214</v>
-      </c>
-      <c r="L29" s="23" t="inlineStr"/>
+        <v>46223</v>
+      </c>
+      <c r="L29" s="23" t="n">
+        <v>133000</v>
+      </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N29" s="20" t="inlineStr">
@@ -2593,7 +2617,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
         </is>
       </c>
     </row>
@@ -2605,17 +2629,17 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13067</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2628,27 +2652,27 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Secretaria de Estado da Educação  SEED-PR</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46212</v>
+        <v>46217</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46224</v>
+        <v>46222</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>150000</v>
+        <v>77100</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
@@ -2662,7 +2686,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
         </is>
       </c>
     </row>
@@ -2674,12 +2698,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR 12970</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2697,7 +2721,7 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2707,14 +2731,14 @@
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46213</v>
+        <v>46183</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46220</v>
+        <v>46188</v>
       </c>
       <c r="L31" s="23" t="inlineStr"/>
       <c r="M31" s="17" t="inlineStr">
@@ -2729,7 +2753,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970/</t>
         </is>
       </c>
     </row>
@@ -2741,17 +2765,17 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
@@ -2764,7 +2788,7 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
@@ -2778,17 +2802,17 @@
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46213</v>
+        <v>46223</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46217</v>
+        <v>46238</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>144000</v>
+        <v>100000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N32" s="12" t="inlineStr">
@@ -2798,7 +2822,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
         </is>
       </c>
     </row>
@@ -2810,12 +2834,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2833,7 +2857,7 @@
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
@@ -2843,17 +2867,17 @@
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46216</v>
+        <v>46225</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46223</v>
+        <v>46229</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>133000</v>
+        <v>114600</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
@@ -2867,7 +2891,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
         </is>
       </c>
     </row>
@@ -2879,12 +2903,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2902,12 +2926,12 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
@@ -2916,13 +2940,13 @@
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46217</v>
+        <v>46220</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46222</v>
+        <v>46225</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>77100</v>
+        <v>58800</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
@@ -2936,7 +2960,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
         </is>
       </c>
     </row>
@@ -2948,17 +2972,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR 12970</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -2971,7 +2995,7 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -2981,19 +3005,19 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46183</v>
+        <v>46221</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46188</v>
+        <v>46224</v>
       </c>
       <c r="L35" s="23" t="inlineStr"/>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N35" s="20" t="inlineStr">
@@ -3003,7 +3027,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
         </is>
       </c>
     </row>
@@ -3015,17 +3039,17 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
@@ -3034,11 +3058,11 @@
         </is>
       </c>
       <c r="F36" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3048,19 +3072,21 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46221</v>
+        <v>46227</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46224</v>
-      </c>
-      <c r="L36" s="15" t="inlineStr"/>
+        <v>46231</v>
+      </c>
+      <c r="L36" s="15" t="n">
+        <v>150000</v>
+      </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N36" s="12" t="inlineStr">
@@ -3070,7 +3096,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -3082,12 +3108,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3105,27 +3131,27 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46220</v>
+        <v>46224</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>58800</v>
+        <v>288000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3139,7 +3165,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -3151,17 +3177,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3170,31 +3196,31 @@
         </is>
       </c>
       <c r="F38" s="13" t="n">
-        <v>0.4</v>
+        <v>0.343</v>
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46229</v>
+        <v>46238</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>114600</v>
+        <v>30000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3208,7 +3234,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -3220,17 +3246,17 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
@@ -3243,7 +3269,7 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3253,17 +3279,17 @@
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46223</v>
+        <v>46232</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46238</v>
+        <v>46237</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>100000</v>
+        <v>288000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3277,7 +3303,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -3289,12 +3315,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3304,39 +3330,37 @@
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F40" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="inlineStr"/>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Brasília DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46227</v>
+        <v>46232</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46231</v>
+        <v>46238</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>150000</v>
+        <v>30000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N40" s="12" t="inlineStr">
@@ -3346,7 +3370,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -3358,12 +3382,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3381,7 +3405,7 @@
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3391,17 +3415,17 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46224</v>
+        <v>46240</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46233</v>
+        <v>46245</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>288000</v>
+        <v>204000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3415,7 +3439,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -3427,17 +3451,17 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
@@ -3446,11 +3470,11 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.343</v>
+        <v>0.4</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3460,17 +3484,17 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>30000</v>
+        <v>204000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3484,7 +3508,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -3496,12 +3520,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3511,13 +3535,15 @@
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F43" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F43" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
@@ -3527,17 +3553,17 @@
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>30000</v>
+        <v>80000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
@@ -3551,7 +3577,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -3563,12 +3589,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3586,27 +3612,27 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46237</v>
+        <v>46245</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>288000</v>
+        <v>80000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
@@ -3620,7 +3646,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -3632,12 +3658,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3655,7 +3681,7 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
@@ -3675,7 +3701,7 @@
         <v>46245</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>204000</v>
+        <v>100000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
@@ -3689,7 +3715,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3701,17 +3727,17 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E46" s="12" t="inlineStr">
@@ -3724,41 +3750,41 @@
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46240</v>
+        <v>46244</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46245</v>
+        <v>46300</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>204000</v>
+        <v>350000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3770,12 +3796,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3785,35 +3811,33 @@
       </c>
       <c r="E47" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F47" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F47" s="21" t="inlineStr"/>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46240</v>
+        <v>46227</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>80000</v>
+        <v>286000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
@@ -3827,7 +3851,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3839,17 +3863,17 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
@@ -3867,36 +3891,36 @@
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46240</v>
+        <v>46244</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46245</v>
+        <v>46296</v>
       </c>
       <c r="L48" s="15" t="n">
-        <v>100000</v>
+        <v>935000</v>
       </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N48" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -3908,12 +3932,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -3927,11 +3951,11 @@
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
@@ -3941,21 +3965,19 @@
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46245</v>
-      </c>
-      <c r="L49" s="23" t="n">
-        <v>80000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L49" s="23" t="inlineStr"/>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
@@ -3965,7 +3987,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3977,17 +3999,17 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
@@ -4000,41 +4022,41 @@
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46244</v>
+        <v>46246</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46300</v>
+        <v>46257</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>350000</v>
+        <v>54000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N50" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -4046,17 +4068,17 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
@@ -4069,41 +4091,41 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46244</v>
+        <v>46251</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46296</v>
+        <v>46256</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>935000</v>
+        <v>50000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -4115,12 +4137,12 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -4134,33 +4156,35 @@
         </is>
       </c>
       <c r="F52" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
         <v>46246</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L52" s="15" t="inlineStr"/>
+        <v>46257</v>
+      </c>
+      <c r="L52" s="15" t="n">
+        <v>54000</v>
+      </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N52" s="12" t="inlineStr">
@@ -4170,7 +4194,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -4182,12 +4206,12 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -4197,13 +4221,15 @@
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F53" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F53" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
@@ -4213,17 +4239,17 @@
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46227</v>
+        <v>46252</v>
       </c>
       <c r="K53" s="22" t="n">
-        <v>46252</v>
+        <v>46259</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>286000</v>
+        <v>60000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
@@ -4237,7 +4263,7 @@
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -4249,17 +4275,17 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
@@ -4272,41 +4298,41 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46246</v>
+        <v>46208</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46257</v>
+        <v>46259</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>54000</v>
+        <v>500000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4318,12 +4344,12 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
@@ -4341,7 +4367,7 @@
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
@@ -4358,14 +4384,14 @@
         <v>46246</v>
       </c>
       <c r="K55" s="22" t="n">
-        <v>46257</v>
+        <v>46272</v>
       </c>
       <c r="L55" s="23" t="n">
         <v>54000</v>
       </c>
       <c r="M55" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N55" s="20" t="inlineStr">
@@ -4375,7 +4401,7 @@
       </c>
       <c r="O55" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -4387,22 +4413,22 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F56" s="13" t="n">
@@ -4410,27 +4436,27 @@
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46251</v>
+        <v>46265</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46256</v>
+        <v>46270</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
@@ -4444,7 +4470,7 @@
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -4456,12 +4482,12 @@
       </c>
       <c r="B57" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
@@ -4479,7 +4505,7 @@
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
@@ -4493,13 +4519,13 @@
         </is>
       </c>
       <c r="J57" s="22" t="n">
-        <v>46252</v>
+        <v>46266</v>
       </c>
       <c r="K57" s="22" t="n">
-        <v>46259</v>
+        <v>46275</v>
       </c>
       <c r="L57" s="23" t="n">
-        <v>60000</v>
+        <v>70000</v>
       </c>
       <c r="M57" s="17" t="inlineStr">
         <is>
@@ -4513,288 +4539,12 @@
       </c>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B58" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
-        </is>
-      </c>
-      <c r="C58" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
-        </is>
-      </c>
-      <c r="D58" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Física (PF)</t>
-        </is>
-      </c>
-      <c r="E58" s="12" t="inlineStr">
-        <is>
-          <t>Economista</t>
-        </is>
-      </c>
-      <c r="F58" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G58" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
-        </is>
-      </c>
-      <c r="H58" s="11" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I58" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="J58" s="14" t="n">
-        <v>46265</v>
-      </c>
-      <c r="K58" s="14" t="n">
-        <v>46270</v>
-      </c>
-      <c r="L58" s="15" t="n">
-        <v>30000</v>
-      </c>
-      <c r="M58" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N58" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O58" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B59" s="18" t="inlineStr">
-        <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
-        </is>
-      </c>
-      <c r="C59" s="19" t="inlineStr">
-        <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
-        </is>
-      </c>
-      <c r="D59" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
-        </is>
-      </c>
-      <c r="E59" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F59" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G59" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados</t>
-        </is>
-      </c>
-      <c r="H59" s="19" t="inlineStr">
-        <is>
-          <t>OEI/MDHC</t>
-        </is>
-      </c>
-      <c r="I59" s="19" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="J59" s="22" t="n">
-        <v>46208</v>
-      </c>
-      <c r="K59" s="22" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L59" s="23" t="n">
-        <v>500000</v>
-      </c>
-      <c r="M59" s="17" t="inlineStr">
-        <is>
-          <t>En presentación</t>
-        </is>
-      </c>
-      <c r="N59" s="20" t="inlineStr">
-        <is>
-          <t>compras.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O59" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B60" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
-        </is>
-      </c>
-      <c r="C60" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
-        </is>
-      </c>
-      <c r="D60" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E60" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F60" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G60" s="11" t="inlineStr">
-        <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
-        </is>
-      </c>
-      <c r="H60" s="11" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I60" s="11" t="inlineStr">
-        <is>
-          <t>Porto Alegre/RS</t>
-        </is>
-      </c>
-      <c r="J60" s="14" t="n">
-        <v>46246</v>
-      </c>
-      <c r="K60" s="14" t="n">
-        <v>46272</v>
-      </c>
-      <c r="L60" s="15" t="n">
-        <v>54000</v>
-      </c>
-      <c r="M60" s="9" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N60" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O60" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B61" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
-        </is>
-      </c>
-      <c r="C61" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
-        </is>
-      </c>
-      <c r="D61" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E61" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F61" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G61" s="19" t="inlineStr">
-        <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H61" s="19" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I61" s="19" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="J61" s="22" t="n">
-        <v>46266</v>
-      </c>
-      <c r="K61" s="22" t="n">
-        <v>46275</v>
-      </c>
-      <c r="L61" s="23" t="n">
-        <v>70000</v>
-      </c>
-      <c r="M61" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N61" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O61" s="24" t="inlineStr">
-        <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O61"/>
+  <autoFilter ref="A1:O57"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4852,10 +4602,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId60"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4904,7 +4650,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -4914,7 +4660,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -4956,7 +4702,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3">
@@ -5014,21 +4760,21 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
@@ -5086,21 +4832,21 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4">
@@ -5110,7 +4856,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
@@ -5120,7 +4866,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -5176,7 +4922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5212,7 +4958,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -5245,18 +4991,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>PNUD (Direto)</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="n">
-        <v>2</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:B7"/>
+  <autoFilter ref="A1:B6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -5300,7 +5036,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5315,7 +5051,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5330,7 +5066,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5345,7 +5081,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-05 14:44
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$56</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 04/09/2026 às 15:49</t>
+          <t>Gerado em 05/09/2026 às 14:39</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="24">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O57"/>
+  <dimension ref="A1:O56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1580,12 +1580,12 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>unesco:1d72ac67-6c7d-4a8b-dd78-08df0757caed</t>
+          <t>unesco:83caba6b-babf-4307-dd76-08df0757caed</t>
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1154 - Edital 05/2026 - 01 perfil - Consultoria Individual</t>
+          <t>914BRZ1164 - EDITAL 03/2026 - 2 VAGAS - Consultor Individual</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
@@ -1613,10 +1613,10 @@
       </c>
       <c r="I13" s="19" t="inlineStr"/>
       <c r="J13" s="22" t="n">
-        <v>46268</v>
+        <v>46270</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46278</v>
+        <v>46276</v>
       </c>
       <c r="L13" s="23" t="inlineStr"/>
       <c r="M13" s="17" t="inlineStr">
@@ -1639,12 +1639,12 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>unesco:eb67e949-3d0c-4334-df1b-08df01dbdf45</t>
+          <t>unesco:1d72ac67-6c7d-4a8b-dd78-08df0757caed</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>586RLA2002 - Edital 002/2026 - 1 vaga</t>
+          <t>914BRZ1154 - Edital 05/2026 - 01 perfil - Consultoria Individual</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1672,10 +1672,10 @@
       </c>
       <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="14" t="n">
-        <v>46261</v>
+        <v>46268</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46272</v>
+        <v>46278</v>
       </c>
       <c r="L14" s="15" t="inlineStr"/>
       <c r="M14" s="9" t="inlineStr">
@@ -1698,12 +1698,12 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
+          <t>unesco:eb67e949-3d0c-4334-df1b-08df01dbdf45</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
+          <t>586RLA2002 - Edital 002/2026 - 1 vaga</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1721,7 +1721,7 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
@@ -1731,10 +1731,10 @@
       </c>
       <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46253</v>
+        <v>46261</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="L15" s="23" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr">
@@ -2288,12 +2288,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2307,11 +2307,11 @@
         </is>
       </c>
       <c r="F25" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2321,19 +2321,21 @@
       </c>
       <c r="I25" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J25" s="22" t="n">
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46220</v>
-      </c>
-      <c r="L25" s="23" t="inlineStr"/>
+        <v>46223</v>
+      </c>
+      <c r="L25" s="23" t="n">
+        <v>133000</v>
+      </c>
       <c r="M25" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N25" s="20" t="inlineStr">
@@ -2343,7 +2345,7 @@
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
         </is>
       </c>
     </row>
@@ -2424,17 +2426,17 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEC/BRA/24 – TR 13056</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
@@ -2443,16 +2445,16 @@
         </is>
       </c>
       <c r="F27" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I27" s="19" t="inlineStr">
@@ -2461,12 +2463,14 @@
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46209</v>
+        <v>46213</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46214</v>
-      </c>
-      <c r="L27" s="23" t="inlineStr"/>
+        <v>46217</v>
+      </c>
+      <c r="L27" s="23" t="n">
+        <v>144000</v>
+      </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
@@ -2479,7 +2483,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-mec-bra-24-tr-13056/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
         </is>
       </c>
     </row>
@@ -2491,17 +2495,17 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -2514,12 +2518,12 @@
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I28" s="11" t="inlineStr">
@@ -2528,17 +2532,17 @@
         </is>
       </c>
       <c r="J28" s="14" t="n">
-        <v>46213</v>
+        <v>46217</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46217</v>
+        <v>46222</v>
       </c>
       <c r="L28" s="15" t="n">
-        <v>144000</v>
+        <v>77100</v>
       </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N28" s="12" t="inlineStr">
@@ -2548,7 +2552,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
         </is>
       </c>
     </row>
@@ -2560,12 +2564,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2579,11 +2583,11 @@
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2593,21 +2597,19 @@
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46216</v>
+        <v>46213</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46223</v>
-      </c>
-      <c r="L29" s="23" t="n">
-        <v>133000</v>
-      </c>
+        <v>46220</v>
+      </c>
+      <c r="L29" s="23" t="inlineStr"/>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N29" s="20" t="inlineStr">
@@ -2617,7 +2619,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
         </is>
       </c>
     </row>
@@ -2629,17 +2631,17 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2648,16 +2650,16 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
@@ -2666,17 +2668,15 @@
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46217</v>
+        <v>46221</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46222</v>
-      </c>
-      <c r="L30" s="15" t="n">
-        <v>77100</v>
-      </c>
+        <v>46224</v>
+      </c>
+      <c r="L30" s="15" t="inlineStr"/>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N30" s="12" t="inlineStr">
@@ -2686,7 +2686,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
         </is>
       </c>
     </row>
@@ -2972,17 +2972,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -2991,11 +2991,11 @@
         </is>
       </c>
       <c r="F35" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
@@ -3005,19 +3005,21 @@
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46221</v>
+        <v>46227</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46224</v>
-      </c>
-      <c r="L35" s="23" t="inlineStr"/>
+        <v>46231</v>
+      </c>
+      <c r="L35" s="23" t="n">
+        <v>150000</v>
+      </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N35" s="20" t="inlineStr">
@@ -3027,7 +3029,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -3039,12 +3041,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3062,31 +3064,31 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Brasília DF</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46227</v>
+        <v>46224</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46231</v>
+        <v>46233</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>150000</v>
+        <v>288000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N36" s="12" t="inlineStr">
@@ -3096,7 +3098,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -3108,17 +3110,17 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
@@ -3127,11 +3129,11 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.4</v>
+        <v>0.343</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3141,17 +3143,17 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46224</v>
+        <v>46232</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46233</v>
+        <v>46238</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>288000</v>
+        <v>30000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3165,7 +3167,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -3177,30 +3179,28 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F38" s="13" t="n">
-        <v>0.343</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F38" s="13" t="inlineStr"/>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -3315,12 +3315,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3330,13 +3330,15 @@
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F40" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3346,17 +3348,17 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>30000</v>
+        <v>204000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3370,7 +3372,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -3382,12 +3384,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3405,7 +3407,7 @@
       </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3439,7 +3441,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -3451,12 +3453,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3474,7 +3476,7 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3494,7 +3496,7 @@
         <v>46245</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>204000</v>
+        <v>100000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
@@ -3508,7 +3510,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3520,12 +3522,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3543,7 +3545,7 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
@@ -3553,7 +3555,7 @@
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
@@ -3577,7 +3579,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -3589,12 +3591,12 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
@@ -3612,7 +3614,7 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
@@ -3622,7 +3624,7 @@
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
@@ -3646,7 +3648,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -3658,17 +3660,17 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
@@ -3686,36 +3688,36 @@
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46240</v>
+        <v>46244</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46245</v>
+        <v>46300</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>100000</v>
+        <v>350000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3727,64 +3729,62 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F46" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F46" s="13" t="inlineStr"/>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46244</v>
+        <v>46227</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46300</v>
+        <v>46252</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>350000</v>
+        <v>286000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3796,62 +3796,64 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E47" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F47" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F47" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46227</v>
+        <v>46244</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46252</v>
+        <v>46296</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>286000</v>
+        <v>935000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -3863,17 +3865,17 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
@@ -3882,7 +3884,7 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
@@ -3891,23 +3893,21 @@
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46244</v>
+        <v>46246</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46296</v>
-      </c>
-      <c r="L48" s="15" t="n">
-        <v>935000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L48" s="15" t="inlineStr"/>
       <c r="M48" s="9" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
@@ -3915,12 +3915,12 @@
       </c>
       <c r="N48" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3932,12 +3932,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -3951,33 +3951,35 @@
         </is>
       </c>
       <c r="F49" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J49" s="22" t="n">
         <v>46246</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L49" s="23" t="inlineStr"/>
+        <v>46257</v>
+      </c>
+      <c r="L49" s="23" t="n">
+        <v>54000</v>
+      </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
@@ -3987,7 +3989,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3999,12 +4001,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4022,7 +4024,7 @@
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
@@ -4056,7 +4058,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -4137,12 +4139,12 @@
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D52" s="11" t="inlineStr">
@@ -4160,7 +4162,7 @@
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H52" s="11" t="inlineStr">
@@ -4170,17 +4172,17 @@
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J52" s="14" t="n">
-        <v>46246</v>
+        <v>46252</v>
       </c>
       <c r="K52" s="14" t="n">
-        <v>46257</v>
+        <v>46259</v>
       </c>
       <c r="L52" s="15" t="n">
-        <v>54000</v>
+        <v>60000</v>
       </c>
       <c r="M52" s="9" t="inlineStr">
         <is>
@@ -4194,7 +4196,7 @@
       </c>
       <c r="O52" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -4206,17 +4208,17 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E53" s="20" t="inlineStr">
@@ -4234,36 +4236,36 @@
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J53" s="22" t="n">
-        <v>46252</v>
+        <v>46208</v>
       </c>
       <c r="K53" s="22" t="n">
         <v>46259</v>
       </c>
       <c r="L53" s="23" t="n">
-        <v>60000</v>
+        <v>500000</v>
       </c>
       <c r="M53" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N53" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -4275,22 +4277,22 @@
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F54" s="13" t="n">
@@ -4298,41 +4300,41 @@
       </c>
       <c r="G54" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H54" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J54" s="14" t="n">
-        <v>46208</v>
+        <v>46265</v>
       </c>
       <c r="K54" s="14" t="n">
-        <v>46259</v>
+        <v>46270</v>
       </c>
       <c r="L54" s="15" t="n">
-        <v>500000</v>
+        <v>30000</v>
       </c>
       <c r="M54" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N54" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O54" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -4413,22 +4415,22 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F56" s="13" t="n">
@@ -4436,27 +4438,27 @@
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H56" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J56" s="14" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="K56" s="14" t="n">
-        <v>46270</v>
+        <v>46275</v>
       </c>
       <c r="L56" s="15" t="n">
-        <v>30000</v>
+        <v>70000</v>
       </c>
       <c r="M56" s="9" t="inlineStr">
         <is>
@@ -4470,81 +4472,12 @@
       </c>
       <c r="O56" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B57" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
-        </is>
-      </c>
-      <c r="C57" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
-        </is>
-      </c>
-      <c r="D57" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E57" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F57" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G57" s="19" t="inlineStr">
-        <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H57" s="19" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I57" s="19" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="J57" s="22" t="n">
-        <v>46266</v>
-      </c>
-      <c r="K57" s="22" t="n">
-        <v>46275</v>
-      </c>
-      <c r="L57" s="23" t="n">
-        <v>70000</v>
-      </c>
-      <c r="M57" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N57" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O57" s="24" t="inlineStr">
-        <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O57"/>
+  <autoFilter ref="A1:O56"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4601,7 +4534,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId56"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4640,7 +4572,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
@@ -4702,7 +4634,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3">
@@ -4760,17 +4692,17 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
@@ -4836,7 +4768,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3">
@@ -4846,7 +4778,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
@@ -4856,7 +4788,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5">
@@ -4968,7 +4900,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
@@ -5036,7 +4968,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -5051,7 +4983,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -5066,7 +4998,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5081,7 +5013,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-08 16:05
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$51</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -25,7 +25,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Por_Perfil'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Por_Tipo'!$A$1:$B$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Por_Tipo'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Area'!$A$1:$B$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Area'!$A$1:$B$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Por_Area'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Por_Orgao'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 05/09/2026 às 14:39</t>
+          <t>Gerado em 08/09/2026 às 16:03</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>55</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="18">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>161191.5517241379</v>
+        <v>167574.0740740741</v>
       </c>
     </row>
     <row r="20">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O56"/>
+  <dimension ref="A1:O51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1071,16 +1071,16 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146335</v>
+        <v>146343</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>Consultoria técnica especializada para avaliação das capacidades institucionais da Secretaria do Tesouro Nacional (STN)</t>
+          <t>TR 005/2026 - ASPAD - MDA - Contratação de consultoria especializada para participação social no Plano Safra da Agricultura Familiar</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E5" s="20" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
@@ -1103,14 +1103,14 @@
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>Brasília/DF</t>
         </is>
       </c>
       <c r="J5" s="22" t="n">
-        <v>46258</v>
+        <v>46268</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46271</v>
+        <v>46277</v>
       </c>
       <c r="L5" s="23" t="inlineStr"/>
       <c r="M5" s="17" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>ucp.codin.df.stn@tesouro.gov.br</t>
+          <t>cgctf.editais@mda.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1136,16 +1136,16 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146343</v>
+        <v>146346</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>TR 005/2026 - ASPAD - MDA - Contratação de consultoria especializada para participação social no Plano Safra da Agricultura Familiar</t>
+          <t>Contratação de consultor (a) individual para assessoramento técnico especializado à consolidação, redação técnica e estruturação dos mecanismos de governança do Plano Estadual de Educação do Piauí 2026-2036</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -1168,14 +1168,14 @@
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Brasília/DF</t>
+          <t>Home based</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
-        <v>46268</v>
+        <v>46262</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="L6" s="15" t="inlineStr"/>
       <c r="M6" s="9" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
-          <t>cgctf.editais@mda.gov.br</t>
+          <t>ugest@seduc.pi.gov.br</t>
         </is>
       </c>
       <c r="O6" s="16" t="inlineStr">
@@ -1201,11 +1201,11 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146346</v>
+        <v>146347</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor (a) individual para assessoramento técnico especializado à consolidação, redação técnica e estruturação dos mecanismos de governança do Plano Estadual de Educação do Piauí 2026-2036</t>
+          <t>Contratação de consultor (a) individual para apoiar tecnicamente a Superintendência de Ensino na realização das Olimpíadas do Conhecimento</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H7" s="19" t="inlineStr">
@@ -1266,16 +1266,16 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146347</v>
+        <v>146349</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor (a) individual para apoiar tecnicamente a Superintendência de Ensino na realização das Olimpíadas do Conhecimento</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA PARA O DESENVOLVIMENTO DE TECNOLOGIA APLICADA AO OBSERVATÓRIO DO NORDESTE</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
@@ -1298,14 +1298,14 @@
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Home based</t>
+          <t>HOME OFFICE</t>
         </is>
       </c>
       <c r="J8" s="14" t="n">
-        <v>46262</v>
+        <v>46267</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>46276</v>
+        <v>46278</v>
       </c>
       <c r="L8" s="15" t="inlineStr"/>
       <c r="M8" s="9" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="N8" s="12" t="inlineStr">
         <is>
-          <t>ugest@seduc.pi.gov.br</t>
+          <t>curriculos@consorcionordeste.gov.br</t>
         </is>
       </c>
       <c r="O8" s="16" t="inlineStr">
@@ -1331,16 +1331,16 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146349</v>
+        <v>146353</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>BRA/23/006 - CONSULTORIA TÉCNICA PARA O DESENVOLVIMENTO DE TECNOLOGIA APLICADA AO OBSERVATÓRIO DO NORDESTE</t>
+          <t>TR - Mobilização Territorial/2026 - Suporte técnico especializado para Avaliação de Efetividade e Metodologias para Mobilização Territorial e Acesso a Instrumentos de Desenvolvimento</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E9" s="20" t="inlineStr">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
@@ -1363,16 +1363,18 @@
       </c>
       <c r="I9" s="19" t="inlineStr">
         <is>
-          <t>HOME OFFICE</t>
+          <t>Região Centro Oeste</t>
         </is>
       </c>
       <c r="J9" s="22" t="n">
-        <v>46267</v>
+        <v>46273</v>
       </c>
       <c r="K9" s="22" t="n">
-        <v>46278</v>
-      </c>
-      <c r="L9" s="23" t="inlineStr"/>
+        <v>46283</v>
+      </c>
+      <c r="L9" s="23" t="n">
+        <v>180000</v>
+      </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1380,7 +1382,7 @@
       </c>
       <c r="N9" s="20" t="inlineStr">
         <is>
-          <t>curriculos@consorcionordeste.gov.br</t>
+          <t>prodocbra23018@sudeco.gov.br</t>
         </is>
       </c>
       <c r="O9" s="24" t="inlineStr">
@@ -1392,15 +1394,17 @@
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="n">
-        <v>146350</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>unesco:83caba6b-babf-4307-dd76-08df0757caed</t>
+        </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contratação de consultoria individual (pessoa física) para elaboração de estudo analítico, voltado ao mapeamento de empreendimentos vinculados à transição energética em execução ou em fase de planejamento e de seu potencial impacto sobre territórios quilombolas na Região Sudeste </t>
+          <t>914BRZ1164 - EDITAL 03/2026 - 2 VAGAS - Consultor Individual</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1418,41 +1422,31 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
-        </is>
-      </c>
-      <c r="I10" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr"/>
       <c r="J10" s="14" t="n">
-        <v>46266</v>
+        <v>46270</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>46272</v>
-      </c>
-      <c r="L10" s="15" t="n">
-        <v>55</v>
-      </c>
+        <v>46276</v>
+      </c>
+      <c r="L10" s="15" t="inlineStr"/>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N10" s="12" t="inlineStr">
-        <is>
-          <t>dqc@igualdaderacial.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N10" s="12" t="inlineStr"/>
       <c r="O10" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -1464,12 +1458,12 @@
       </c>
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>unesco:11c715d6-1d36-4c54-5f8f-08df036d3e00</t>
+          <t>unesco:1d72ac67-6c7d-4a8b-dd78-08df0757caed</t>
         </is>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>914BRZ4027 - Edital 55/2026 - Ciências Sociais</t>
+          <t>914BRZ1154 - Edital 05/2026 - 01 perfil - Consultoria Individual</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1487,7 +1481,7 @@
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
@@ -1497,10 +1491,10 @@
       </c>
       <c r="I11" s="19" t="inlineStr"/>
       <c r="J11" s="22" t="n">
-        <v>46266</v>
+        <v>46268</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46271</v>
+        <v>46278</v>
       </c>
       <c r="L11" s="23" t="inlineStr"/>
       <c r="M11" s="17" t="inlineStr">
@@ -1523,12 +1517,12 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>unesco:5d64862a-264d-475d-5f8e-08df036d3e00</t>
+          <t>unesco:b260be61-61f9-4226-2eb0-08df08e94b75</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>4BRZ4025 - Edital 18/2026 - Consultor Individual (1 Vaga)  REPUBLICAÇÃO</t>
+          <t>914BRZ3061 - EDITAL Nº 13/2026 - 01 VAGA - CONSULTOR INDIVIDUAL-REPUBLICACAO</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1554,10 +1548,10 @@
       </c>
       <c r="I12" s="11" t="inlineStr"/>
       <c r="J12" s="14" t="n">
-        <v>46266</v>
+        <v>46273</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>46270</v>
+        <v>46278</v>
       </c>
       <c r="L12" s="15" t="inlineStr"/>
       <c r="M12" s="9" t="inlineStr">
@@ -1580,12 +1574,12 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>unesco:83caba6b-babf-4307-dd76-08df0757caed</t>
+          <t>unesco:b324319d-9f96-425f-8caf-08defc5a5785</t>
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1164 - EDITAL 03/2026 - 2 VAGAS - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 48/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1603,7 +1597,7 @@
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
@@ -1613,10 +1607,10 @@
       </c>
       <c r="I13" s="19" t="inlineStr"/>
       <c r="J13" s="22" t="n">
-        <v>46270</v>
+        <v>46266</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46276</v>
+        <v>46274</v>
       </c>
       <c r="L13" s="23" t="inlineStr"/>
       <c r="M13" s="17" t="inlineStr">
@@ -1639,12 +1633,12 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>unesco:1d72ac67-6c7d-4a8b-dd78-08df0757caed</t>
+          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1154 - Edital 05/2026 - 01 perfil - Consultoria Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1662,7 +1656,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1672,10 +1666,10 @@
       </c>
       <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="14" t="n">
-        <v>46268</v>
+        <v>46266</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46278</v>
+        <v>46274</v>
       </c>
       <c r="L14" s="15" t="inlineStr"/>
       <c r="M14" s="9" t="inlineStr">
@@ -1698,12 +1692,12 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>unesco:eb67e949-3d0c-4334-df1b-08df01dbdf45</t>
+          <t>unesco:b0920c88-ab66-4545-2ead-08df08e94b75</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>586RLA2002 - Edital 002/2026 - 1 vaga</t>
+          <t xml:space="preserve">Projeto 914BRZ3050 - Edital N° 04/2026 - Consultor Individual </t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1721,7 +1715,7 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
@@ -1731,10 +1725,10 @@
       </c>
       <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46261</v>
+        <v>46269</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="L15" s="23" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr">
@@ -1757,12 +1751,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:17177a8d-bde0-4a60-df1c-08df01dbdf45</t>
+          <t>unesco:5c1d62c6-1efa-431c-b9e2-08df0436270c</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1159 - Publicação Edital 36/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 54/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1780,7 +1774,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Saúde, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1790,10 +1784,10 @@
       </c>
       <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46271</v>
+        <v>46273</v>
       </c>
       <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
@@ -1816,12 +1810,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:b324319d-9f96-425f-8caf-08defc5a5785</t>
+          <t>unesco:c9020343-9d28-49e3-b9e3-08df0436270c</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 48/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 52/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1839,7 +1833,7 @@
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1852,7 +1846,7 @@
         <v>46266</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
@@ -1875,12 +1869,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
+          <t>unesco:b74745df-a51d-41c1-b9e5-08df0436270c</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 55/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1898,7 +1892,7 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1911,7 +1905,7 @@
         <v>46266</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
@@ -1934,12 +1928,12 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:b0920c88-ab66-4545-2ead-08df08e94b75</t>
+          <t>unesco:f4efa11a-ea51-47cf-b9e7-08df0436270c</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Projeto 914BRZ3050 - Edital N° 04/2026 - Consultor Individual </t>
+          <t>914BRZ1155 - EDITAL Nº 56/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
@@ -1957,7 +1951,7 @@
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -1967,7 +1961,7 @@
       </c>
       <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46269</v>
+        <v>46266</v>
       </c>
       <c r="K19" s="22" t="n">
         <v>46273</v>
@@ -1993,12 +1987,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:5c1d62c6-1efa-431c-b9e2-08df0436270c</t>
+          <t>unesco:6f0bebf7-7be2-4b29-17c5-08df04786cdd</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 54/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 53/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2016,7 +2010,7 @@
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2047,22 +2041,22 @@
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>unesco:c9020343-9d28-49e3-b9e3-08df0436270c</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 52/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E21" s="20" t="inlineStr">
@@ -2071,57 +2065,67 @@
         </is>
       </c>
       <c r="F21" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I21" s="19" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I21" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J21" s="22" t="n">
-        <v>46266</v>
+        <v>46213</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46273</v>
-      </c>
-      <c r="L21" s="23" t="inlineStr"/>
+        <v>46217</v>
+      </c>
+      <c r="L21" s="23" t="n">
+        <v>144000</v>
+      </c>
       <c r="M21" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N21" s="20" t="inlineStr"/>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N21" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O21" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>unesco:b74745df-a51d-41c1-b9e5-08df0436270c</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 55/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -2134,53 +2138,61 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I22" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I22" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J22" s="14" t="n">
-        <v>46266</v>
+        <v>46213</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46273</v>
+        <v>46220</v>
       </c>
       <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N22" s="12" t="inlineStr"/>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N22" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>unesco:f4efa11a-ea51-47cf-b9e7-08df0436270c</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 56/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E23" s="20" t="inlineStr">
@@ -2189,57 +2201,67 @@
         </is>
       </c>
       <c r="F23" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I23" s="19" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I23" s="19" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
       <c r="J23" s="22" t="n">
-        <v>46266</v>
+        <v>46216</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46273</v>
-      </c>
-      <c r="L23" s="23" t="inlineStr"/>
+        <v>46223</v>
+      </c>
+      <c r="L23" s="23" t="n">
+        <v>133000</v>
+      </c>
       <c r="M23" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N23" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N23" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>unesco:6f0bebf7-7be2-4b29-17c5-08df04786cdd</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 53/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
@@ -2248,35 +2270,45 @@
         </is>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I24" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J24" s="14" t="n">
-        <v>46266</v>
+        <v>46220</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46273</v>
-      </c>
-      <c r="L24" s="15" t="inlineStr"/>
+        <v>46225</v>
+      </c>
+      <c r="L24" s="15" t="n">
+        <v>58800</v>
+      </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N24" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N24" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
         </is>
       </c>
     </row>
@@ -2288,12 +2320,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2311,27 +2343,27 @@
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I25" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J25" s="22" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46223</v>
+        <v>46222</v>
       </c>
       <c r="L25" s="23" t="n">
-        <v>133000</v>
+        <v>77100</v>
       </c>
       <c r="M25" s="17" t="inlineStr">
         <is>
@@ -2345,7 +2377,7 @@
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
         </is>
       </c>
     </row>
@@ -2357,12 +2389,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/001 – TR13067</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2376,11 +2408,11 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
@@ -2390,21 +2422,19 @@
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Secretaria de Estado da Educação  SEED-PR</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J26" s="14" t="n">
-        <v>46212</v>
+        <v>46221</v>
       </c>
       <c r="K26" s="14" t="n">
         <v>46224</v>
       </c>
-      <c r="L26" s="15" t="n">
-        <v>150000</v>
-      </c>
+      <c r="L26" s="15" t="inlineStr"/>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N26" s="12" t="inlineStr">
@@ -2414,7 +2444,7 @@
       </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-001-tr13067/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
         </is>
       </c>
     </row>
@@ -2426,17 +2456,17 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR 12970</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
@@ -2445,11 +2475,11 @@
         </is>
       </c>
       <c r="F27" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2459,18 +2489,16 @@
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46213</v>
+        <v>46183</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46217</v>
-      </c>
-      <c r="L27" s="23" t="n">
-        <v>144000</v>
-      </c>
+        <v>46188</v>
+      </c>
+      <c r="L27" s="23" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
@@ -2483,7 +2511,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970/</t>
         </is>
       </c>
     </row>
@@ -2495,12 +2523,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2523,26 +2551,26 @@
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
-        <v>46217</v>
+        <v>46227</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46222</v>
+        <v>46231</v>
       </c>
       <c r="L28" s="15" t="n">
-        <v>77100</v>
+        <v>150000</v>
       </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N28" s="12" t="inlineStr">
@@ -2552,7 +2580,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -2564,12 +2592,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2583,11 +2611,11 @@
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2597,19 +2625,21 @@
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46213</v>
+        <v>46225</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46220</v>
-      </c>
-      <c r="L29" s="23" t="inlineStr"/>
+        <v>46229</v>
+      </c>
+      <c r="L29" s="23" t="n">
+        <v>114600</v>
+      </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N29" s="20" t="inlineStr">
@@ -2619,7 +2649,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
         </is>
       </c>
     </row>
@@ -2631,17 +2661,17 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2650,11 +2680,11 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2668,15 +2698,17 @@
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46221</v>
+        <v>46223</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46224</v>
-      </c>
-      <c r="L30" s="15" t="inlineStr"/>
+        <v>46238</v>
+      </c>
+      <c r="L30" s="15" t="n">
+        <v>100000</v>
+      </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N30" s="12" t="inlineStr">
@@ -2686,7 +2718,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
         </is>
       </c>
     </row>
@@ -2698,12 +2730,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR 12970</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2717,33 +2749,35 @@
         </is>
       </c>
       <c r="F31" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46183</v>
+        <v>46224</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46188</v>
-      </c>
-      <c r="L31" s="23" t="inlineStr"/>
+        <v>46233</v>
+      </c>
+      <c r="L31" s="23" t="n">
+        <v>288000</v>
+      </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N31" s="20" t="inlineStr">
@@ -2753,7 +2787,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -2765,12 +2799,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2784,31 +2818,31 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.4</v>
+        <v>0.343</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46223</v>
+        <v>46232</v>
       </c>
       <c r="K32" s="14" t="n">
         <v>46238</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>100000</v>
+        <v>30000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2822,7 +2856,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -2834,12 +2868,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2849,35 +2883,33 @@
       </c>
       <c r="E33" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F33" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F33" s="21" t="inlineStr"/>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46229</v>
+        <v>46238</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>114600</v>
+        <v>30000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
@@ -2891,7 +2923,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -2903,12 +2935,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2926,7 +2958,7 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -2936,17 +2968,17 @@
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46220</v>
+        <v>46232</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46225</v>
+        <v>46237</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>58800</v>
+        <v>288000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
@@ -2960,7 +2992,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -2972,12 +3004,12 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -2995,31 +3027,31 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Brasília DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46227</v>
+        <v>46240</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46231</v>
+        <v>46245</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>150000</v>
+        <v>204000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N35" s="20" t="inlineStr">
@@ -3029,7 +3061,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -3041,12 +3073,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3064,7 +3096,7 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3074,17 +3106,17 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46224</v>
+        <v>46240</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46233</v>
+        <v>46245</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>288000</v>
+        <v>204000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3098,7 +3130,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -3110,17 +3142,17 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E37" s="20" t="inlineStr">
@@ -3129,11 +3161,11 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.343</v>
+        <v>0.4</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3143,17 +3175,17 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>30000</v>
+        <v>80000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3167,7 +3199,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -3179,12 +3211,12 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
@@ -3194,13 +3226,15 @@
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F38" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F38" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -3210,17 +3244,17 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>30000</v>
+        <v>80000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
@@ -3234,7 +3268,7 @@
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -3246,17 +3280,17 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
@@ -3269,41 +3303,41 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46232</v>
+        <v>46244</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46237</v>
+        <v>46296</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>288000</v>
+        <v>935000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -3315,12 +3349,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3338,7 +3372,7 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3358,7 +3392,7 @@
         <v>46245</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>204000</v>
+        <v>100000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3372,7 +3406,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3384,12 +3418,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3399,35 +3433,33 @@
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F41" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F41" s="21" t="inlineStr"/>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46240</v>
+        <v>46227</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>204000</v>
+        <v>286000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3441,7 +3473,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3453,12 +3485,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3472,7 +3504,7 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
@@ -3486,21 +3518,19 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46245</v>
-      </c>
-      <c r="L42" s="15" t="n">
-        <v>100000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L42" s="15" t="inlineStr"/>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
@@ -3510,7 +3540,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3522,12 +3552,12 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -3545,27 +3575,27 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>80000</v>
+        <v>54000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
@@ -3579,7 +3609,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3591,17 +3621,17 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
@@ -3614,27 +3644,27 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46240</v>
+        <v>46251</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46245</v>
+        <v>46256</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>80000</v>
+        <v>50000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
@@ -3648,7 +3678,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3660,17 +3690,17 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
@@ -3683,41 +3713,41 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46244</v>
+        <v>46246</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46300</v>
+        <v>46257</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>350000</v>
+        <v>54000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3729,12 +3759,12 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
@@ -3744,13 +3774,15 @@
       </c>
       <c r="E46" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F46" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F46" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
@@ -3760,17 +3792,17 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46227</v>
+        <v>46252</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46252</v>
+        <v>46259</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>286000</v>
+        <v>60000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
@@ -3784,7 +3816,7 @@
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3796,12 +3828,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3819,7 +3851,7 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
@@ -3833,17 +3865,17 @@
         </is>
       </c>
       <c r="J47" s="22" t="n">
-        <v>46244</v>
+        <v>46208</v>
       </c>
       <c r="K47" s="22" t="n">
-        <v>46296</v>
+        <v>46259</v>
       </c>
       <c r="L47" s="23" t="n">
-        <v>935000</v>
+        <v>500000</v>
       </c>
       <c r="M47" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N47" s="20" t="inlineStr">
@@ -3853,7 +3885,7 @@
       </c>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3865,30 +3897,30 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
@@ -3898,19 +3930,21 @@
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46246</v>
+        <v>46265</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L48" s="15" t="inlineStr"/>
+        <v>46270</v>
+      </c>
+      <c r="L48" s="15" t="n">
+        <v>30000</v>
+      </c>
       <c r="M48" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N48" s="12" t="inlineStr">
@@ -3920,7 +3954,7 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3932,12 +3966,12 @@
       </c>
       <c r="B49" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -3955,7 +3989,7 @@
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
@@ -3972,14 +4006,14 @@
         <v>46246</v>
       </c>
       <c r="K49" s="22" t="n">
-        <v>46257</v>
+        <v>46272</v>
       </c>
       <c r="L49" s="23" t="n">
         <v>54000</v>
       </c>
       <c r="M49" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N49" s="20" t="inlineStr">
@@ -3989,7 +4023,7 @@
       </c>
       <c r="O49" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -4001,12 +4035,12 @@
       </c>
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D50" s="11" t="inlineStr">
@@ -4024,7 +4058,7 @@
       </c>
       <c r="G50" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H50" s="11" t="inlineStr">
@@ -4034,17 +4068,17 @@
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J50" s="14" t="n">
-        <v>46246</v>
+        <v>46266</v>
       </c>
       <c r="K50" s="14" t="n">
-        <v>46257</v>
+        <v>46275</v>
       </c>
       <c r="L50" s="15" t="n">
-        <v>54000</v>
+        <v>70000</v>
       </c>
       <c r="M50" s="9" t="inlineStr">
         <is>
@@ -4058,7 +4092,7 @@
       </c>
       <c r="O50" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
@@ -4070,17 +4104,17 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E51" s="20" t="inlineStr">
@@ -4093,391 +4127,46 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J51" s="22" t="n">
-        <v>46251</v>
+        <v>46244</v>
       </c>
       <c r="K51" s="22" t="n">
-        <v>46256</v>
+        <v>46300</v>
       </c>
       <c r="L51" s="23" t="n">
-        <v>50000</v>
+        <v>350000</v>
       </c>
       <c r="M51" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N51" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O51" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B52" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
-        </is>
-      </c>
-      <c r="C52" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
-        </is>
-      </c>
-      <c r="D52" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E52" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F52" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G52" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados</t>
-        </is>
-      </c>
-      <c r="H52" s="11" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I52" s="11" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="J52" s="14" t="n">
-        <v>46252</v>
-      </c>
-      <c r="K52" s="14" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L52" s="15" t="n">
-        <v>60000</v>
-      </c>
-      <c r="M52" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N52" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O52" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B53" s="18" t="inlineStr">
-        <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
-        </is>
-      </c>
-      <c r="C53" s="19" t="inlineStr">
-        <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
-        </is>
-      </c>
-      <c r="D53" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
-        </is>
-      </c>
-      <c r="E53" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F53" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G53" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados</t>
-        </is>
-      </c>
-      <c r="H53" s="19" t="inlineStr">
-        <is>
-          <t>OEI/MDHC</t>
-        </is>
-      </c>
-      <c r="I53" s="19" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="J53" s="22" t="n">
-        <v>46208</v>
-      </c>
-      <c r="K53" s="22" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L53" s="23" t="n">
-        <v>500000</v>
-      </c>
-      <c r="M53" s="17" t="inlineStr">
-        <is>
-          <t>En presentación</t>
-        </is>
-      </c>
-      <c r="N53" s="20" t="inlineStr">
-        <is>
-          <t>compras.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O53" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B54" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
-        </is>
-      </c>
-      <c r="C54" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
-        </is>
-      </c>
-      <c r="D54" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Física (PF)</t>
-        </is>
-      </c>
-      <c r="E54" s="12" t="inlineStr">
-        <is>
-          <t>Economista</t>
-        </is>
-      </c>
-      <c r="F54" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G54" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
-        </is>
-      </c>
-      <c r="H54" s="11" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I54" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="J54" s="14" t="n">
-        <v>46265</v>
-      </c>
-      <c r="K54" s="14" t="n">
-        <v>46270</v>
-      </c>
-      <c r="L54" s="15" t="n">
-        <v>30000</v>
-      </c>
-      <c r="M54" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N54" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O54" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B55" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
-        </is>
-      </c>
-      <c r="C55" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
-        </is>
-      </c>
-      <c r="D55" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E55" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F55" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G55" s="19" t="inlineStr">
-        <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
-        </is>
-      </c>
-      <c r="H55" s="19" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I55" s="19" t="inlineStr">
-        <is>
-          <t>Porto Alegre/RS</t>
-        </is>
-      </c>
-      <c r="J55" s="22" t="n">
-        <v>46246</v>
-      </c>
-      <c r="K55" s="22" t="n">
-        <v>46272</v>
-      </c>
-      <c r="L55" s="23" t="n">
-        <v>54000</v>
-      </c>
-      <c r="M55" s="17" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N55" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O55" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B56" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
-        </is>
-      </c>
-      <c r="C56" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
-        </is>
-      </c>
-      <c r="D56" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E56" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F56" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G56" s="11" t="inlineStr">
-        <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H56" s="11" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I56" s="11" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="J56" s="14" t="n">
-        <v>46266</v>
-      </c>
-      <c r="K56" s="14" t="n">
-        <v>46275</v>
-      </c>
-      <c r="L56" s="15" t="n">
-        <v>70000</v>
-      </c>
-      <c r="M56" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N56" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O56" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O56"/>
+  <autoFilter ref="A1:O51"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4529,11 +4218,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId55"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4572,7 +4256,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3">
@@ -4582,7 +4266,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -4592,7 +4276,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -4634,7 +4318,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3">
@@ -4692,7 +4376,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
@@ -4702,11 +4386,11 @@
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
@@ -4716,7 +4400,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -4742,7 +4426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4778,7 +4462,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
@@ -4788,7 +4472,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5">
@@ -4831,18 +4515,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>Saúde</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="n">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:B9"/>
+  <autoFilter ref="A1:B8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -4880,7 +4554,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3">
@@ -4890,7 +4564,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -4910,7 +4584,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
@@ -4968,7 +4642,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -4983,7 +4657,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -4998,7 +4672,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -5013,7 +4687,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-09 16:02
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$45</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 08/09/2026 às 16:03</t>
+          <t>Gerado em 09/09/2026 às 15:59</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6">
@@ -638,27 +638,27 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>PNUD</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>PNUD</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>167574.0740740741</v>
+        <v>168480.7692307692</v>
       </c>
     </row>
     <row r="20">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O51"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1372,9 +1372,7 @@
       <c r="K9" s="22" t="n">
         <v>46283</v>
       </c>
-      <c r="L9" s="23" t="n">
-        <v>180000</v>
-      </c>
+      <c r="L9" s="23" t="inlineStr"/>
       <c r="M9" s="17" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1517,12 +1515,12 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>unesco:b260be61-61f9-4226-2eb0-08df08e94b75</t>
+          <t>unesco:b0920c88-ab66-4545-2ead-08df08e94b75</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3061 - EDITAL Nº 13/2026 - 01 VAGA - CONSULTOR INDIVIDUAL-REPUBLICACAO</t>
+          <t>Projeto 914BRZ3050 - Edital N° 04/2026 - Consultor Individual PRORROGAÇÃO</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1532,13 +1530,15 @@
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F12" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="I12" s="11" t="inlineStr"/>
       <c r="J12" s="14" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="K12" s="14" t="n">
         <v>46278</v>
@@ -1574,12 +1574,12 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>unesco:b324319d-9f96-425f-8caf-08defc5a5785</t>
+          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 48/2026 - 1 vaga - Consultor Individual</t>
+          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1597,7 +1597,7 @@
       </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
@@ -1607,10 +1607,10 @@
       </c>
       <c r="I13" s="19" t="inlineStr"/>
       <c r="J13" s="22" t="n">
-        <v>46266</v>
+        <v>46253</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="L13" s="23" t="inlineStr"/>
       <c r="M13" s="17" t="inlineStr">
@@ -1633,12 +1633,12 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
+          <t>unesco:b260be61-61f9-4226-2eb0-08df08e94b75</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual</t>
+          <t>914BRZ3061 - EDITAL Nº 13/2026 - 01 VAGA - CONSULTOR INDIVIDUAL-REPUBLICACAO</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1648,15 +1648,13 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F14" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr"/>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1666,10 +1664,10 @@
       </c>
       <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="14" t="n">
-        <v>46266</v>
+        <v>46273</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46274</v>
+        <v>46278</v>
       </c>
       <c r="L14" s="15" t="inlineStr"/>
       <c r="M14" s="9" t="inlineStr">
@@ -1692,12 +1690,12 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>unesco:b0920c88-ab66-4545-2ead-08df08e94b75</t>
+          <t>unesco:b324319d-9f96-425f-8caf-08defc5a5785</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Projeto 914BRZ3050 - Edital N° 04/2026 - Consultor Individual </t>
+          <t>914BRZ1155 - EDITAL Nº 48/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1715,7 +1713,7 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
@@ -1725,10 +1723,10 @@
       </c>
       <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46269</v>
+        <v>46266</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="L15" s="23" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr">
@@ -1751,12 +1749,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:5c1d62c6-1efa-431c-b9e2-08df0436270c</t>
+          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 54/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1774,7 +1772,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1787,7 +1785,7 @@
         <v>46266</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
@@ -1805,22 +1803,22 @@
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:c9020343-9d28-49e3-b9e3-08df0436270c</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 52/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E17" s="20" t="inlineStr">
@@ -1829,57 +1827,67 @@
         </is>
       </c>
       <c r="F17" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I17" s="19" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J17" s="22" t="n">
-        <v>46266</v>
+        <v>46217</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46273</v>
-      </c>
-      <c r="L17" s="23" t="inlineStr"/>
+        <v>46222</v>
+      </c>
+      <c r="L17" s="23" t="n">
+        <v>77100</v>
+      </c>
       <c r="M17" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N17" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N17" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O17" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:b74745df-a51d-41c1-b9e5-08df0436270c</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 55/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
@@ -1892,53 +1900,61 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I18" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J18" s="14" t="n">
-        <v>46266</v>
+        <v>46221</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46273</v>
+        <v>46224</v>
       </c>
       <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N18" s="12" t="inlineStr"/>
+          <t>En presentación</t>
+        </is>
+      </c>
+      <c r="N18" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O18" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:f4efa11a-ea51-47cf-b9e7-08df0436270c</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 56/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E19" s="20" t="inlineStr">
@@ -1947,57 +1963,67 @@
         </is>
       </c>
       <c r="F19" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I19" s="19" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
       <c r="J19" s="22" t="n">
-        <v>46266</v>
+        <v>46216</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46273</v>
-      </c>
-      <c r="L19" s="23" t="inlineStr"/>
+        <v>46223</v>
+      </c>
+      <c r="L19" s="23" t="n">
+        <v>133000</v>
+      </c>
       <c r="M19" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N19" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N19" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O19" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:6f0bebf7-7be2-4b29-17c5-08df04786cdd</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 53/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -2010,31 +2036,39 @@
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J20" s="14" t="n">
-        <v>46266</v>
+        <v>46213</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46273</v>
+        <v>46220</v>
       </c>
       <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N20" s="12" t="inlineStr"/>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N20" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O20" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
         </is>
       </c>
     </row>
@@ -2046,17 +2080,17 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13072</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E21" s="20" t="inlineStr">
@@ -2069,7 +2103,7 @@
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2083,17 +2117,17 @@
         </is>
       </c>
       <c r="J21" s="22" t="n">
-        <v>46213</v>
+        <v>46220</v>
       </c>
       <c r="K21" s="22" t="n">
-        <v>46217</v>
+        <v>46225</v>
       </c>
       <c r="L21" s="23" t="n">
-        <v>144000</v>
+        <v>58800</v>
       </c>
       <c r="M21" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N21" s="20" t="inlineStr">
@@ -2103,7 +2137,7 @@
       </c>
       <c r="O21" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13072/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
         </is>
       </c>
     </row>
@@ -2115,12 +2149,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2134,11 +2168,11 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2148,16 +2182,18 @@
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J22" s="14" t="n">
-        <v>46213</v>
+        <v>46227</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46220</v>
-      </c>
-      <c r="L22" s="15" t="inlineStr"/>
+        <v>46231</v>
+      </c>
+      <c r="L22" s="15" t="n">
+        <v>150000</v>
+      </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
@@ -2170,7 +2206,7 @@
       </c>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -2182,17 +2218,17 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E23" s="20" t="inlineStr">
@@ -2205,7 +2241,7 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2215,17 +2251,17 @@
       </c>
       <c r="I23" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J23" s="22" t="n">
-        <v>46216</v>
+        <v>46223</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46223</v>
+        <v>46238</v>
       </c>
       <c r="L23" s="23" t="n">
-        <v>133000</v>
+        <v>100000</v>
       </c>
       <c r="M23" s="17" t="inlineStr">
         <is>
@@ -2239,7 +2275,7 @@
       </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
         </is>
       </c>
     </row>
@@ -2251,12 +2287,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2274,27 +2310,27 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J24" s="14" t="n">
-        <v>46220</v>
+        <v>46224</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="L24" s="15" t="n">
-        <v>58800</v>
+        <v>288000</v>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
@@ -2308,7 +2344,7 @@
       </c>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -2320,12 +2356,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2343,27 +2379,27 @@
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I25" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J25" s="22" t="n">
-        <v>46217</v>
+        <v>46225</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46222</v>
+        <v>46229</v>
       </c>
       <c r="L25" s="23" t="n">
-        <v>77100</v>
+        <v>114600</v>
       </c>
       <c r="M25" s="17" t="inlineStr">
         <is>
@@ -2377,7 +2413,7 @@
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
         </is>
       </c>
     </row>
@@ -2389,17 +2425,17 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
@@ -2408,33 +2444,35 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.3</v>
+        <v>0.343</v>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J26" s="14" t="n">
-        <v>46221</v>
+        <v>46232</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46224</v>
-      </c>
-      <c r="L26" s="15" t="inlineStr"/>
+        <v>46238</v>
+      </c>
+      <c r="L26" s="15" t="n">
+        <v>30000</v>
+      </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N26" s="12" t="inlineStr">
@@ -2444,7 +2482,7 @@
       </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -2456,12 +2494,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR 12970</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2475,7 +2513,7 @@
         </is>
       </c>
       <c r="F27" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
@@ -2484,24 +2522,26 @@
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46183</v>
+        <v>46240</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46188</v>
-      </c>
-      <c r="L27" s="23" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L27" s="23" t="n">
+        <v>204000</v>
+      </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N27" s="20" t="inlineStr">
@@ -2511,7 +2551,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr-12970/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -2523,12 +2563,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2546,7 +2586,7 @@
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2556,21 +2596,21 @@
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Brasília DF</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
-        <v>46227</v>
+        <v>46232</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46231</v>
+        <v>46237</v>
       </c>
       <c r="L28" s="15" t="n">
-        <v>150000</v>
+        <v>288000</v>
       </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N28" s="12" t="inlineStr">
@@ -2580,7 +2620,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -2592,12 +2632,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2615,27 +2655,27 @@
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46225</v>
+        <v>46240</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46229</v>
+        <v>46245</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>114600</v>
+        <v>80000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
@@ -2649,7 +2689,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -2661,50 +2701,48 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F30" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="inlineStr"/>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46223</v>
+        <v>46232</v>
       </c>
       <c r="K30" s="14" t="n">
         <v>46238</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>100000</v>
+        <v>30000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
@@ -2718,7 +2756,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -2730,12 +2768,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2753,7 +2791,7 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2763,17 +2801,17 @@
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46224</v>
+        <v>46240</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46233</v>
+        <v>46245</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>288000</v>
+        <v>204000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2787,7 +2825,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -2799,17 +2837,17 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
@@ -2818,11 +2856,11 @@
         </is>
       </c>
       <c r="F32" s="13" t="n">
-        <v>0.343</v>
+        <v>0.4</v>
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
@@ -2832,17 +2870,17 @@
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K32" s="14" t="n">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>30000</v>
+        <v>80000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2856,7 +2894,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -2868,12 +2906,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2883,13 +2921,15 @@
       </c>
       <c r="E33" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F33" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F33" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
@@ -2899,21 +2939,19 @@
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46232</v>
+        <v>46246</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46238</v>
-      </c>
-      <c r="L33" s="23" t="n">
-        <v>30000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L33" s="23" t="inlineStr"/>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N33" s="20" t="inlineStr">
@@ -2923,7 +2961,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -2935,12 +2973,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2950,15 +2988,13 @@
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F34" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F34" s="13" t="inlineStr"/>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -2968,17 +3004,17 @@
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46232</v>
+        <v>46227</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46237</v>
+        <v>46252</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>288000</v>
+        <v>286000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
@@ -2992,7 +3028,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3004,12 +3040,12 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -3027,27 +3063,27 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>204000</v>
+        <v>54000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
@@ -3061,7 +3097,7 @@
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3073,12 +3109,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3096,7 +3132,7 @@
       </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -3116,7 +3152,7 @@
         <v>46245</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>204000</v>
+        <v>100000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3130,7 +3166,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3142,12 +3178,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3165,27 +3201,27 @@
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46245</v>
+        <v>46257</v>
       </c>
       <c r="L37" s="23" t="n">
-        <v>80000</v>
+        <v>54000</v>
       </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
@@ -3199,7 +3235,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3211,17 +3247,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3239,36 +3275,36 @@
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46240</v>
+        <v>46244</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46245</v>
+        <v>46296</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>80000</v>
+        <v>935000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -3280,17 +3316,17 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
@@ -3303,41 +3339,41 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46244</v>
+        <v>46251</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46296</v>
+        <v>46256</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>935000</v>
+        <v>50000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3349,12 +3385,12 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
@@ -3372,27 +3408,27 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46240</v>
+        <v>46252</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46245</v>
+        <v>46259</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>100000</v>
+        <v>60000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3406,7 +3442,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3418,62 +3454,64 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F41" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F41" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46227</v>
+        <v>46208</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46252</v>
+        <v>46259</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>286000</v>
+        <v>500000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3485,12 +3523,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3504,30 +3542,32 @@
         </is>
       </c>
       <c r="F42" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
         <v>46246</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L42" s="15" t="inlineStr"/>
+        <v>46272</v>
+      </c>
+      <c r="L42" s="15" t="n">
+        <v>54000</v>
+      </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
           <t>En fase de apresentação</t>
@@ -3540,7 +3580,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3552,17 +3592,17 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
@@ -3575,41 +3615,41 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46246</v>
+        <v>46244</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46257</v>
+        <v>46300</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>54000</v>
+        <v>350000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3621,22 +3661,22 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
@@ -3644,27 +3684,27 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46251</v>
+        <v>46265</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46256</v>
+        <v>46270</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
@@ -3678,7 +3718,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3690,12 +3730,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3713,7 +3753,7 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
@@ -3723,17 +3763,17 @@
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46246</v>
+        <v>46266</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46257</v>
+        <v>46275</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>54000</v>
+        <v>70000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
@@ -3747,426 +3787,12 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B46" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
-        </is>
-      </c>
-      <c r="C46" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
-        </is>
-      </c>
-      <c r="D46" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E46" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F46" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G46" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados</t>
-        </is>
-      </c>
-      <c r="H46" s="11" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I46" s="11" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="J46" s="14" t="n">
-        <v>46252</v>
-      </c>
-      <c r="K46" s="14" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L46" s="15" t="n">
-        <v>60000</v>
-      </c>
-      <c r="M46" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N46" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O46" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B47" s="18" t="inlineStr">
-        <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
-        </is>
-      </c>
-      <c r="C47" s="19" t="inlineStr">
-        <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
-        </is>
-      </c>
-      <c r="D47" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
-        </is>
-      </c>
-      <c r="E47" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F47" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G47" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados</t>
-        </is>
-      </c>
-      <c r="H47" s="19" t="inlineStr">
-        <is>
-          <t>OEI/MDHC</t>
-        </is>
-      </c>
-      <c r="I47" s="19" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="J47" s="22" t="n">
-        <v>46208</v>
-      </c>
-      <c r="K47" s="22" t="n">
-        <v>46259</v>
-      </c>
-      <c r="L47" s="23" t="n">
-        <v>500000</v>
-      </c>
-      <c r="M47" s="17" t="inlineStr">
-        <is>
-          <t>En presentación</t>
-        </is>
-      </c>
-      <c r="N47" s="20" t="inlineStr">
-        <is>
-          <t>compras.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O47" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B48" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
-        </is>
-      </c>
-      <c r="C48" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
-        </is>
-      </c>
-      <c r="D48" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Física (PF)</t>
-        </is>
-      </c>
-      <c r="E48" s="12" t="inlineStr">
-        <is>
-          <t>Economista</t>
-        </is>
-      </c>
-      <c r="F48" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G48" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
-        </is>
-      </c>
-      <c r="H48" s="11" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I48" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="J48" s="14" t="n">
-        <v>46265</v>
-      </c>
-      <c r="K48" s="14" t="n">
-        <v>46270</v>
-      </c>
-      <c r="L48" s="15" t="n">
-        <v>30000</v>
-      </c>
-      <c r="M48" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N48" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O48" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B49" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
-        </is>
-      </c>
-      <c r="C49" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
-        </is>
-      </c>
-      <c r="D49" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E49" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F49" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G49" s="19" t="inlineStr">
-        <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
-        </is>
-      </c>
-      <c r="H49" s="19" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I49" s="19" t="inlineStr">
-        <is>
-          <t>Porto Alegre/RS</t>
-        </is>
-      </c>
-      <c r="J49" s="22" t="n">
-        <v>46246</v>
-      </c>
-      <c r="K49" s="22" t="n">
-        <v>46272</v>
-      </c>
-      <c r="L49" s="23" t="n">
-        <v>54000</v>
-      </c>
-      <c r="M49" s="17" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N49" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O49" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B50" s="10" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
-        </is>
-      </c>
-      <c r="C50" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
-        </is>
-      </c>
-      <c r="D50" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E50" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F50" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G50" s="11" t="inlineStr">
-        <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H50" s="11" t="inlineStr">
-        <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I50" s="11" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
-      <c r="J50" s="14" t="n">
-        <v>46266</v>
-      </c>
-      <c r="K50" s="14" t="n">
-        <v>46275</v>
-      </c>
-      <c r="L50" s="15" t="n">
-        <v>70000</v>
-      </c>
-      <c r="M50" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N50" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O50" s="16" t="inlineStr">
-        <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B51" s="18" t="inlineStr">
-        <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
-        </is>
-      </c>
-      <c r="C51" s="19" t="inlineStr">
-        <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
-        </is>
-      </c>
-      <c r="D51" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
-        </is>
-      </c>
-      <c r="E51" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F51" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G51" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
-        </is>
-      </c>
-      <c r="H51" s="19" t="inlineStr">
-        <is>
-          <t>OEI/MDHC</t>
-        </is>
-      </c>
-      <c r="I51" s="19" t="inlineStr">
-        <is>
-          <t>Nacional</t>
-        </is>
-      </c>
-      <c r="J51" s="22" t="n">
-        <v>46244</v>
-      </c>
-      <c r="K51" s="22" t="n">
-        <v>46300</v>
-      </c>
-      <c r="L51" s="23" t="n">
-        <v>350000</v>
-      </c>
-      <c r="M51" s="17" t="inlineStr">
-        <is>
-          <t>En fase de apresentação</t>
-        </is>
-      </c>
-      <c r="N51" s="20" t="inlineStr">
-        <is>
-          <t>compras.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O51" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:O51"/>
+  <autoFilter ref="A1:O45"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4212,12 +3838,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4256,27 +3876,27 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>Unesco</t>
+          <t>Pnud</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>Pnud</t>
+          <t>Unesco</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -4318,7 +3938,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
@@ -4380,7 +4000,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3">
@@ -4390,7 +4010,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -4400,7 +4020,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -4452,7 +4072,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3">
@@ -4462,7 +4082,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -4472,7 +4092,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
@@ -4512,7 +4132,7 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -4554,13 +4174,13 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B3" s="18" t="n">
@@ -4570,21 +4190,21 @@
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>Não identificado</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -4642,7 +4262,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -4657,7 +4277,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -4672,7 +4292,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -4687,7 +4307,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-10 15:58
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 09/09/2026 às 15:59</t>
+          <t>Gerado em 10/09/2026 às 15:53</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>168480.7692307692</v>
+        <v>164092.5925925926</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>100000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O45"/>
+  <dimension ref="A1:O47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -876,16 +876,16 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>146326</v>
+        <v>146343</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 02/2026 – Metodologia para monitoramento das decisões da Corte Interamericana de Direitos Humanos</t>
+          <t>TR 005/2026 - ASPAD - MDA - Contratação de consultoria especializada para participação social no Plano Safra da Agricultura Familiar</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E2" s="12" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H2" s="11" t="inlineStr">
@@ -908,14 +908,14 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Brasília/DF</t>
         </is>
       </c>
       <c r="J2" s="14" t="n">
-        <v>46258</v>
+        <v>46268</v>
       </c>
       <c r="K2" s="14" t="n">
-        <v>46274</v>
+        <v>46277</v>
       </c>
       <c r="L2" s="15" t="inlineStr"/>
       <c r="M2" s="9" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="N2" s="12" t="inlineStr">
         <is>
-          <t>ccidh@mdh.gov.br</t>
+          <t>cgctf.editais@mda.gov.br</t>
         </is>
       </c>
       <c r="O2" s="16" t="inlineStr">
@@ -941,11 +941,11 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>146327</v>
+        <v>146346</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>Edital nº 3/2026 – Metodologia para monitoramento de recomendações e decisões da Comissão Interamericana de Direitos Humanos</t>
+          <t>Contratação de consultor (a) individual para assessoramento técnico especializado à consolidação, redação técnica e estruturação dos mecanismos de governança do Plano Estadual de Educação do Piauí 2026-2036</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
@@ -973,14 +973,14 @@
       </c>
       <c r="I3" s="19" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Home based</t>
         </is>
       </c>
       <c r="J3" s="22" t="n">
-        <v>46258</v>
+        <v>46262</v>
       </c>
       <c r="K3" s="22" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="L3" s="23" t="inlineStr"/>
       <c r="M3" s="17" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="N3" s="20" t="inlineStr">
         <is>
-          <t>ccidh@mdh.gov.br</t>
+          <t>ugest@seduc.pi.gov.br</t>
         </is>
       </c>
       <c r="O3" s="24" t="inlineStr">
@@ -1006,11 +1006,11 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146332</v>
+        <v>146347</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 04/2026 - Segundo Plano da Política Nacional de RCN</t>
+          <t>Contratação de consultor (a) individual para apoiar tecnicamente a Superintendência de Ensino na realização das Olimpíadas do Conhecimento</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr">
@@ -1038,14 +1038,14 @@
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Território Nacional</t>
+          <t>Home based</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
-        <v>46258</v>
+        <v>46262</v>
       </c>
       <c r="K4" s="14" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="L4" s="15" t="inlineStr"/>
       <c r="M4" s="9" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="N4" s="12" t="inlineStr">
         <is>
-          <t>rcn_cidadania@mdh.gov.br</t>
+          <t>ugest@seduc.pi.gov.br</t>
         </is>
       </c>
       <c r="O4" s="16" t="inlineStr">
@@ -1071,11 +1071,11 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146343</v>
+        <v>146349</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>TR 005/2026 - ASPAD - MDA - Contratação de consultoria especializada para participação social no Plano Safra da Agricultura Familiar</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA PARA O DESENVOLVIMENTO DE TECNOLOGIA APLICADA AO OBSERVATÓRIO DO NORDESTE</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
@@ -1103,14 +1103,14 @@
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
-          <t>Brasília/DF</t>
+          <t>HOME OFFICE</t>
         </is>
       </c>
       <c r="J5" s="22" t="n">
-        <v>46268</v>
+        <v>46267</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="L5" s="23" t="inlineStr"/>
       <c r="M5" s="17" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>cgctf.editais@mda.gov.br</t>
+          <t>curriculos@consorcionordeste.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1136,16 +1136,16 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146346</v>
+        <v>146353</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor (a) individual para assessoramento técnico especializado à consolidação, redação técnica e estruturação dos mecanismos de governança do Plano Estadual de Educação do Piauí 2026-2036</t>
+          <t>TR - Mobilização Territorial/2026 - Suporte técnico especializado para Avaliação de Efetividade e Metodologias para Mobilização Territorial e Acesso a Instrumentos de Desenvolvimento</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -1168,14 +1168,14 @@
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Home based</t>
+          <t>Região Centro Oeste</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
-        <v>46262</v>
+        <v>46273</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>46276</v>
+        <v>46283</v>
       </c>
       <c r="L6" s="15" t="inlineStr"/>
       <c r="M6" s="9" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
-          <t>ugest@seduc.pi.gov.br</t>
+          <t>prodocbra23018@sudeco.gov.br</t>
         </is>
       </c>
       <c r="O6" s="16" t="inlineStr">
@@ -1201,11 +1201,11 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146347</v>
+        <v>146368</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor (a) individual para apoiar tecnicamente a Superintendência de Ensino na realização das Olimpíadas do Conhecimento</t>
+          <t>Edital 6/2026- UGP-PNUD/SENAD</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1233,16 +1233,18 @@
       </c>
       <c r="I7" s="19" t="inlineStr">
         <is>
-          <t>Home based</t>
+          <t>null</t>
         </is>
       </c>
       <c r="J7" s="22" t="n">
-        <v>46262</v>
+        <v>46275</v>
       </c>
       <c r="K7" s="22" t="n">
-        <v>46276</v>
-      </c>
-      <c r="L7" s="23" t="inlineStr"/>
+        <v>46280</v>
+      </c>
+      <c r="L7" s="23" t="n">
+        <v>108000</v>
+      </c>
       <c r="M7" s="17" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1250,7 +1252,7 @@
       </c>
       <c r="N7" s="20" t="inlineStr">
         <is>
-          <t>ugest@seduc.pi.gov.br</t>
+          <t>cgep@mj.gov.br</t>
         </is>
       </c>
       <c r="O7" s="24" t="inlineStr">
@@ -1266,16 +1268,16 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146349</v>
+        <v>146367</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>BRA/23/006 - CONSULTORIA TÉCNICA PARA O DESENVOLVIMENTO DE TECNOLOGIA APLICADA AO OBSERVATÓRIO DO NORDESTE</t>
+          <t>EDITAL Nº 5/2026 - UGP-PNUD/SENAD</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -1288,7 +1290,7 @@
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
@@ -1298,16 +1300,18 @@
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>HOME OFFICE</t>
+          <t>Brasília/DF</t>
         </is>
       </c>
       <c r="J8" s="14" t="n">
-        <v>46267</v>
+        <v>46275</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>46278</v>
-      </c>
-      <c r="L8" s="15" t="inlineStr"/>
+        <v>46280</v>
+      </c>
+      <c r="L8" s="15" t="n">
+        <v>72000</v>
+      </c>
       <c r="M8" s="9" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1315,7 +1319,7 @@
       </c>
       <c r="N8" s="12" t="inlineStr">
         <is>
-          <t>curriculos@consorcionordeste.gov.br</t>
+          <t>cgep@mj.gov.br</t>
         </is>
       </c>
       <c r="O8" s="16" t="inlineStr">
@@ -1331,16 +1335,16 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146353</v>
+        <v>146365</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>TR - Mobilização Territorial/2026 - Suporte técnico especializado para Avaliação de Efetividade e Metodologias para Mobilização Territorial e Acesso a Instrumentos de Desenvolvimento</t>
+          <t>EDITAL Nº 4/2026 - UGP-PNUD/SENAD</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E9" s="20" t="inlineStr">
@@ -1353,7 +1357,7 @@
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
@@ -1363,16 +1367,18 @@
       </c>
       <c r="I9" s="19" t="inlineStr">
         <is>
-          <t>Região Centro Oeste</t>
+          <t>null</t>
         </is>
       </c>
       <c r="J9" s="22" t="n">
-        <v>46273</v>
+        <v>46275</v>
       </c>
       <c r="K9" s="22" t="n">
-        <v>46283</v>
-      </c>
-      <c r="L9" s="23" t="inlineStr"/>
+        <v>46280</v>
+      </c>
+      <c r="L9" s="23" t="n">
+        <v>102000</v>
+      </c>
       <c r="M9" s="17" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1380,7 +1386,7 @@
       </c>
       <c r="N9" s="20" t="inlineStr">
         <is>
-          <t>prodocbra23018@sudeco.gov.br</t>
+          <t>dpagi@mj.gov.br</t>
         </is>
       </c>
       <c r="O9" s="24" t="inlineStr">
@@ -1392,17 +1398,15 @@
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>unesco:83caba6b-babf-4307-dd76-08df0757caed</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>146364</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1164 - EDITAL 03/2026 - 2 VAGAS - Consultor Individual</t>
+          <t>EDITAL Nº 3/2026 - UGP-PNUD/SENAD</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1420,48 +1424,56 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I10" s="11" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
       <c r="J10" s="14" t="n">
-        <v>46270</v>
+        <v>46275</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>46276</v>
-      </c>
-      <c r="L10" s="15" t="inlineStr"/>
+        <v>46280</v>
+      </c>
+      <c r="L10" s="15" t="n">
+        <v>216000</v>
+      </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N10" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N10" s="12" t="inlineStr">
+        <is>
+          <t>dpagi@mj.gov.br</t>
+        </is>
+      </c>
       <c r="O10" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>unesco:1d72ac67-6c7d-4a8b-dd78-08df0757caed</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="n">
+        <v>146363</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1154 - Edital 05/2026 - 01 perfil - Consultoria Individual</t>
+          <t>EDITAL Nº 2/2026 - UGP-PNUD/SENAD</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1479,31 +1491,41 @@
       </c>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I11" s="19" t="inlineStr"/>
+          <t>Não identificado</t>
+        </is>
+      </c>
+      <c r="I11" s="19" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
       <c r="J11" s="22" t="n">
-        <v>46268</v>
+        <v>46275</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46278</v>
-      </c>
-      <c r="L11" s="23" t="inlineStr"/>
+        <v>46280</v>
+      </c>
+      <c r="L11" s="23" t="n">
+        <v>70000</v>
+      </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N11" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N11" s="20" t="inlineStr">
+        <is>
+          <t>senad@mj.gov.br</t>
+        </is>
+      </c>
       <c r="O11" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -1515,12 +1537,12 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>unesco:b0920c88-ab66-4545-2ead-08df08e94b75</t>
+          <t>unesco:5c1d62c6-1efa-431c-b9e2-08df0436270c</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3050 - Edital N° 04/2026 - Consultor Individual PRORROGAÇÃO</t>
+          <t>914BRZ1155 - EDITAL Nº 54/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1538,7 +1560,7 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
@@ -1574,12 +1596,12 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
+          <t>unesco:83caba6b-babf-4307-dd76-08df0757caed</t>
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1164 - EDITAL 03/2026 - 2 VAGAS - Consultor Individual</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1607,10 +1629,10 @@
       </c>
       <c r="I13" s="19" t="inlineStr"/>
       <c r="J13" s="22" t="n">
-        <v>46253</v>
+        <v>46270</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46283</v>
+        <v>46276</v>
       </c>
       <c r="L13" s="23" t="inlineStr"/>
       <c r="M13" s="17" t="inlineStr">
@@ -1633,12 +1655,12 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>unesco:b260be61-61f9-4226-2eb0-08df08e94b75</t>
+          <t>unesco:1d72ac67-6c7d-4a8b-dd78-08df0757caed</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3061 - EDITAL Nº 13/2026 - 01 VAGA - CONSULTOR INDIVIDUAL-REPUBLICACAO</t>
+          <t>914BRZ1154 - Edital 05/2026 - 01 perfil - Consultoria Individual</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1648,13 +1670,15 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F14" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1664,7 +1688,7 @@
       </c>
       <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="14" t="n">
-        <v>46273</v>
+        <v>46268</v>
       </c>
       <c r="K14" s="14" t="n">
         <v>46278</v>
@@ -1690,12 +1714,12 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>unesco:b324319d-9f96-425f-8caf-08defc5a5785</t>
+          <t>unesco:b0920c88-ab66-4545-2ead-08df08e94b75</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 48/2026 - 1 vaga - Consultor Individual</t>
+          <t>Projeto 914BRZ3050 - Edital N° 04/2026 - Consultor Individual PRORROGAÇÃO</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1713,7 +1737,7 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
@@ -1723,10 +1747,10 @@
       </c>
       <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46266</v>
+        <v>46274</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46274</v>
+        <v>46278</v>
       </c>
       <c r="L15" s="23" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr">
@@ -1749,12 +1773,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:7863ef0f-6e11-4770-df18-08df01dbdf45</t>
+          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 51/2026 - 3 vagas - Consultor Individual</t>
+          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1772,7 +1796,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1782,10 +1806,10 @@
       </c>
       <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46266</v>
+        <v>46253</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46274</v>
+        <v>46283</v>
       </c>
       <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
@@ -1803,69 +1827,57 @@
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
+          <t>unesco:b260be61-61f9-4226-2eb0-08df08e94b75</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
+          <t>914BRZ3061 - EDITAL Nº 13/2026 - 01 VAGA - CONSULTOR INDIVIDUAL-REPUBLICACAO</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E17" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F17" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="inlineStr"/>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I17" s="19" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46217</v>
+        <v>46273</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46222</v>
-      </c>
-      <c r="L17" s="23" t="n">
-        <v>77100</v>
-      </c>
+        <v>46278</v>
+      </c>
+      <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N17" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N17" s="20" t="inlineStr"/>
       <c r="O17" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -1877,17 +1889,17 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
@@ -1896,11 +1908,11 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1914,15 +1926,17 @@
         </is>
       </c>
       <c r="J18" s="14" t="n">
-        <v>46221</v>
+        <v>46220</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46224</v>
-      </c>
-      <c r="L18" s="15" t="inlineStr"/>
+        <v>46225</v>
+      </c>
+      <c r="L18" s="15" t="n">
+        <v>58800</v>
+      </c>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N18" s="12" t="inlineStr">
@@ -1932,7 +1946,7 @@
       </c>
       <c r="O18" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
         </is>
       </c>
     </row>
@@ -1944,17 +1958,17 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E19" s="20" t="inlineStr">
@@ -1963,11 +1977,11 @@
         </is>
       </c>
       <c r="F19" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
@@ -1977,21 +1991,19 @@
       </c>
       <c r="I19" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J19" s="22" t="n">
-        <v>46216</v>
+        <v>46221</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46223</v>
-      </c>
-      <c r="L19" s="23" t="n">
-        <v>133000</v>
-      </c>
+        <v>46224</v>
+      </c>
+      <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N19" s="20" t="inlineStr">
@@ -2001,7 +2013,7 @@
       </c>
       <c r="O19" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
         </is>
       </c>
     </row>
@@ -2013,12 +2025,12 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2032,11 +2044,11 @@
         </is>
       </c>
       <c r="F20" s="13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -2046,19 +2058,21 @@
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J20" s="14" t="n">
-        <v>46213</v>
+        <v>46216</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46220</v>
-      </c>
-      <c r="L20" s="15" t="inlineStr"/>
+        <v>46223</v>
+      </c>
+      <c r="L20" s="15" t="n">
+        <v>133000</v>
+      </c>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N20" s="12" t="inlineStr">
@@ -2068,7 +2082,7 @@
       </c>
       <c r="O20" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
         </is>
       </c>
     </row>
@@ -2080,12 +2094,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13074</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -2099,11 +2113,11 @@
         </is>
       </c>
       <c r="F21" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
@@ -2117,17 +2131,15 @@
         </is>
       </c>
       <c r="J21" s="22" t="n">
+        <v>46213</v>
+      </c>
+      <c r="K21" s="22" t="n">
         <v>46220</v>
       </c>
-      <c r="K21" s="22" t="n">
-        <v>46225</v>
-      </c>
-      <c r="L21" s="23" t="n">
-        <v>58800</v>
-      </c>
+      <c r="L21" s="23" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N21" s="20" t="inlineStr">
@@ -2137,7 +2149,7 @@
       </c>
       <c r="O21" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13074/</t>
         </is>
       </c>
     </row>
@@ -2149,12 +2161,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2177,26 +2189,26 @@
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>Brasília DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J22" s="14" t="n">
-        <v>46227</v>
+        <v>46217</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46231</v>
+        <v>46222</v>
       </c>
       <c r="L22" s="15" t="n">
-        <v>150000</v>
+        <v>77100</v>
       </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N22" s="12" t="inlineStr">
@@ -2206,7 +2218,7 @@
       </c>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
         </is>
       </c>
     </row>
@@ -2218,17 +2230,17 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E23" s="20" t="inlineStr">
@@ -2241,7 +2253,7 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
@@ -2251,17 +2263,17 @@
       </c>
       <c r="I23" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J23" s="22" t="n">
-        <v>46223</v>
+        <v>46225</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46238</v>
+        <v>46229</v>
       </c>
       <c r="L23" s="23" t="n">
-        <v>100000</v>
+        <v>114600</v>
       </c>
       <c r="M23" s="17" t="inlineStr">
         <is>
@@ -2275,7 +2287,7 @@
       </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
         </is>
       </c>
     </row>
@@ -2356,12 +2368,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -2379,7 +2391,7 @@
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2389,21 +2401,21 @@
       </c>
       <c r="I25" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J25" s="22" t="n">
-        <v>46225</v>
+        <v>46227</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="L25" s="23" t="n">
-        <v>114600</v>
+        <v>150000</v>
       </c>
       <c r="M25" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N25" s="20" t="inlineStr">
@@ -2413,7 +2425,7 @@
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -2425,12 +2437,12 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
@@ -2444,31 +2456,31 @@
         </is>
       </c>
       <c r="F26" s="13" t="n">
-        <v>0.343</v>
+        <v>0.4</v>
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J26" s="14" t="n">
-        <v>46232</v>
+        <v>46223</v>
       </c>
       <c r="K26" s="14" t="n">
         <v>46238</v>
       </c>
       <c r="L26" s="15" t="n">
-        <v>30000</v>
+        <v>100000</v>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
@@ -2482,7 +2494,7 @@
       </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
         </is>
       </c>
     </row>
@@ -2494,17 +2506,17 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
@@ -2513,11 +2525,11 @@
         </is>
       </c>
       <c r="F27" s="21" t="n">
-        <v>0.4</v>
+        <v>0.343</v>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2527,17 +2539,17 @@
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L27" s="23" t="n">
-        <v>204000</v>
+        <v>30000</v>
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
@@ -2551,7 +2563,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -2563,12 +2575,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2578,35 +2590,33 @@
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F28" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="inlineStr"/>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
         <v>46232</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="L28" s="15" t="n">
-        <v>288000</v>
+        <v>30000</v>
       </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
@@ -2620,7 +2630,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -2632,12 +2642,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2655,27 +2665,27 @@
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46245</v>
+        <v>46237</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>80000</v>
+        <v>288000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
@@ -2689,7 +2699,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -2701,12 +2711,12 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
@@ -2716,13 +2726,15 @@
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F30" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2732,17 +2744,17 @@
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>30000</v>
+        <v>204000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
@@ -2756,7 +2768,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -2768,12 +2780,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2791,7 +2803,7 @@
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2811,7 +2823,7 @@
         <v>46245</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>204000</v>
+        <v>80000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2825,7 +2837,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -2837,12 +2849,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2860,7 +2872,7 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
@@ -2870,7 +2882,7 @@
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J32" s="14" t="n">
@@ -2880,7 +2892,7 @@
         <v>46245</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>80000</v>
+        <v>204000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2894,7 +2906,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -2906,12 +2918,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2925,7 +2937,7 @@
         </is>
       </c>
       <c r="F33" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
@@ -2939,19 +2951,21 @@
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L33" s="23" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L33" s="23" t="n">
+        <v>100000</v>
+      </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N33" s="20" t="inlineStr">
@@ -2961,7 +2975,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -2973,12 +2987,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2988,33 +3002,35 @@
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F34" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F34" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
-        <v>46227</v>
+        <v>46240</v>
       </c>
       <c r="K34" s="14" t="n">
-        <v>46252</v>
+        <v>46245</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>286000</v>
+        <v>80000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
@@ -3028,7 +3044,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -3040,17 +3056,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -3063,41 +3079,41 @@
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46246</v>
+        <v>46244</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46257</v>
+        <v>46296</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>54000</v>
+        <v>935000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N35" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -3109,12 +3125,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3124,35 +3140,33 @@
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F36" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="inlineStr"/>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46240</v>
+        <v>46227</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>100000</v>
+        <v>286000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3166,7 +3180,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3178,12 +3192,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3197,35 +3211,33 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
         <v>46246</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46257</v>
-      </c>
-      <c r="L37" s="23" t="n">
-        <v>54000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L37" s="23" t="inlineStr"/>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N37" s="20" t="inlineStr">
@@ -3235,7 +3247,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3247,17 +3259,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3270,41 +3282,41 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46244</v>
+        <v>46246</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46296</v>
+        <v>46257</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>935000</v>
+        <v>54000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3316,17 +3328,17 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E39" s="20" t="inlineStr">
@@ -3339,7 +3351,7 @@
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
@@ -3349,17 +3361,17 @@
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="L39" s="23" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
@@ -3373,7 +3385,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3385,17 +3397,17 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
@@ -3408,7 +3420,7 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3418,17 +3430,17 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46252</v>
+        <v>46251</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46259</v>
+        <v>46256</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3442,7 +3454,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3454,17 +3466,17 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E41" s="20" t="inlineStr">
@@ -3482,36 +3494,36 @@
       </c>
       <c r="H41" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46208</v>
+        <v>46252</v>
       </c>
       <c r="K41" s="22" t="n">
         <v>46259</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>500000</v>
+        <v>60000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N41" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3523,17 +3535,17 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
@@ -3546,41 +3558,41 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46246</v>
+        <v>46208</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46272</v>
+        <v>46259</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>54000</v>
+        <v>500000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3592,17 +3604,17 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
@@ -3615,27 +3627,27 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46244</v>
+        <v>46246</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46300</v>
+        <v>46272</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>350000</v>
+        <v>54000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
@@ -3644,12 +3656,12 @@
       </c>
       <c r="N43" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3791,8 +3803,146 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="inlineStr">
+        <is>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+        </is>
+      </c>
+      <c r="E46" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F46" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G46" s="11" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+        </is>
+      </c>
+      <c r="H46" s="11" t="inlineStr">
+        <is>
+          <t>OEI/MDHC</t>
+        </is>
+      </c>
+      <c r="I46" s="11" t="inlineStr">
+        <is>
+          <t>Nacional</t>
+        </is>
+      </c>
+      <c r="J46" s="14" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K46" s="14" t="n">
+        <v>46300</v>
+      </c>
+      <c r="L46" s="15" t="n">
+        <v>350000</v>
+      </c>
+      <c r="M46" s="9" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N46" s="12" t="inlineStr">
+        <is>
+          <t>compras.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O46" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B47" s="18" t="inlineStr">
+        <is>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+        </is>
+      </c>
+      <c r="C47" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+        </is>
+      </c>
+      <c r="D47" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E47" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F47" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G47" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H47" s="19" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I47" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
+      <c r="J47" s="22" t="n">
+        <v>46275</v>
+      </c>
+      <c r="K47" s="22" t="n">
+        <v>46280</v>
+      </c>
+      <c r="L47" s="23" t="n">
+        <v>50000</v>
+      </c>
+      <c r="M47" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N47" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O47" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O45"/>
+  <autoFilter ref="A1:O47"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -3838,6 +3988,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId46"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -3876,7 +4028,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
@@ -3886,7 +4038,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -3896,7 +4048,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -3938,7 +4090,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3">
@@ -4000,7 +4152,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3">
@@ -4010,7 +4162,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
@@ -4072,7 +4224,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3">
@@ -4082,7 +4234,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4">
@@ -4184,7 +4336,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -4194,7 +4346,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -4204,7 +4356,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -4262,7 +4414,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -4277,7 +4429,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -4292,7 +4444,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -4307,7 +4459,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-11 16:03
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$51</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -27,7 +27,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Por_Tipo'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Por_Area'!$A$1:$B$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Por_Area'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Por_Orgao'!$A$1:$B$7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Por_Orgao'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Perfis'!$A$1:$C$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Perfis'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 10/09/2026 às 15:53</t>
+          <t>Gerado em 11/09/2026 às 15:56</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6">
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>164092.5925925926</v>
+        <v>164660.7142857143</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>80000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O47"/>
+  <dimension ref="A1:O51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1242,9 +1242,7 @@
       <c r="K7" s="22" t="n">
         <v>46280</v>
       </c>
-      <c r="L7" s="23" t="n">
-        <v>108000</v>
-      </c>
+      <c r="L7" s="23" t="inlineStr"/>
       <c r="M7" s="17" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1309,9 +1307,7 @@
       <c r="K8" s="14" t="n">
         <v>46280</v>
       </c>
-      <c r="L8" s="15" t="n">
-        <v>72000</v>
-      </c>
+      <c r="L8" s="15" t="inlineStr"/>
       <c r="M8" s="9" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1376,9 +1372,7 @@
       <c r="K9" s="22" t="n">
         <v>46280</v>
       </c>
-      <c r="L9" s="23" t="n">
-        <v>102000</v>
-      </c>
+      <c r="L9" s="23" t="inlineStr"/>
       <c r="M9" s="17" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1443,9 +1437,7 @@
       <c r="K10" s="14" t="n">
         <v>46280</v>
       </c>
-      <c r="L10" s="15" t="n">
-        <v>216000</v>
-      </c>
+      <c r="L10" s="15" t="inlineStr"/>
       <c r="M10" s="9" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1510,9 +1502,7 @@
       <c r="K11" s="22" t="n">
         <v>46280</v>
       </c>
-      <c r="L11" s="23" t="n">
-        <v>70000</v>
-      </c>
+      <c r="L11" s="23" t="inlineStr"/>
       <c r="M11" s="17" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1532,17 +1522,15 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>unesco:5c1d62c6-1efa-431c-b9e2-08df0436270c</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="n">
+        <v>146369</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 54/2026 - 1 vaga - Consultor Individual</t>
+          <t>Edital nº 29/2026 – Contratação de Consultoria Individual para o desenho institucional da Secretaria de Serviços Compartilhados (SSC/MGI)</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1552,56 +1540,62 @@
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F12" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr"/>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I12" s="11" t="inlineStr"/>
+          <t>MGI</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
       <c r="J12" s="14" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>46278</v>
-      </c>
-      <c r="L12" s="15" t="inlineStr"/>
+        <v>46290</v>
+      </c>
+      <c r="L12" s="15" t="n">
+        <v>120000</v>
+      </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N12" s="12" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N12" s="12" t="inlineStr">
+        <is>
+          <t>prodoc.mgi@gestao.gov.br</t>
+        </is>
+      </c>
       <c r="O12" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>unesco:83caba6b-babf-4307-dd76-08df0757caed</t>
-        </is>
+          <t>PNUD</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="n">
+        <v>146370</v>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1164 - EDITAL 03/2026 - 2 VAGAS - Consultor Individual</t>
+          <t xml:space="preserve">Edital nº 25/2026 – Contratação de Consultoria Individual para avaliar os efeitos de intervenções comportamentais (políticas fiscais e de arquitetura de escolha) em mercado experimental para promover escolhas alimentares mais saudáveis. </t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1611,39 +1605,47 @@
       </c>
       <c r="E13" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F13" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F13" s="21" t="inlineStr"/>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I13" s="19" t="inlineStr"/>
+          <t>MGI</t>
+        </is>
+      </c>
+      <c r="I13" s="19" t="inlineStr">
+        <is>
+          <t>REMOTO</t>
+        </is>
+      </c>
       <c r="J13" s="22" t="n">
-        <v>46270</v>
+        <v>46276</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46276</v>
-      </c>
-      <c r="L13" s="23" t="inlineStr"/>
+        <v>46290</v>
+      </c>
+      <c r="L13" s="23" t="n">
+        <v>126000</v>
+      </c>
       <c r="M13" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N13" s="20" t="inlineStr"/>
+          <t>Aprovada</t>
+        </is>
+      </c>
+      <c r="N13" s="20" t="inlineStr">
+        <is>
+          <t>prodoc.mgi@gestao.gov.br</t>
+        </is>
+      </c>
       <c r="O13" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://parceiros.undp.org.br/opportunities</t>
         </is>
       </c>
     </row>
@@ -1655,12 +1657,12 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>unesco:1d72ac67-6c7d-4a8b-dd78-08df0757caed</t>
+          <t>unesco:5c1d62c6-1efa-431c-b9e2-08df0436270c</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1154 - Edital 05/2026 - 01 perfil - Consultoria Individual</t>
+          <t>914BRZ1155 - EDITAL Nº 54/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1678,7 +1680,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1688,7 +1690,7 @@
       </c>
       <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="14" t="n">
-        <v>46268</v>
+        <v>46274</v>
       </c>
       <c r="K14" s="14" t="n">
         <v>46278</v>
@@ -1714,12 +1716,12 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>unesco:b0920c88-ab66-4545-2ead-08df08e94b75</t>
+          <t>unesco:83caba6b-babf-4307-dd76-08df0757caed</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3050 - Edital N° 04/2026 - Consultor Individual PRORROGAÇÃO</t>
+          <t>914BRZ1164 - EDITAL 03/2026 - 2 VAGAS - Consultor Individual</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1737,7 +1739,7 @@
       </c>
       <c r="G15" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H15" s="19" t="inlineStr">
@@ -1747,10 +1749,10 @@
       </c>
       <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46274</v>
+        <v>46270</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46278</v>
+        <v>46276</v>
       </c>
       <c r="L15" s="23" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr">
@@ -1773,12 +1775,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
+          <t>unesco:1d72ac67-6c7d-4a8b-dd78-08df0757caed</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1154 - Edital 05/2026 - 01 perfil - Consultoria Individual</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1796,7 +1798,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1806,10 +1808,10 @@
       </c>
       <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46253</v>
+        <v>46268</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>46283</v>
+        <v>46278</v>
       </c>
       <c r="L16" s="15" t="inlineStr"/>
       <c r="M16" s="9" t="inlineStr">
@@ -1832,12 +1834,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:b260be61-61f9-4226-2eb0-08df08e94b75</t>
+          <t>unesco:8c824e7b-7b9a-4a59-7ffc-08df082d82f3</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ3061 - EDITAL Nº 13/2026 - 01 VAGA - CONSULTOR INDIVIDUAL-REPUBLICACAO</t>
+          <t>914BRZ1163 - Publicação -  Edital 68/2026 - 01 Vaga consultor Individual</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1847,13 +1849,15 @@
       </c>
       <c r="E17" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F17" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F17" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1863,10 +1867,10 @@
       </c>
       <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46273</v>
+        <v>46276</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
@@ -1884,22 +1888,22 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
+          <t>unesco:b0920c88-ab66-4545-2ead-08df08e94b75</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
+          <t>Projeto 914BRZ3050 - Edital N° 04/2026 - Consultor Individual PRORROGAÇÃO</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
@@ -1908,67 +1912,57 @@
         </is>
       </c>
       <c r="F18" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I18" s="11" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr"/>
       <c r="J18" s="14" t="n">
-        <v>46220</v>
+        <v>46274</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>46225</v>
-      </c>
-      <c r="L18" s="15" t="n">
-        <v>58800</v>
-      </c>
+        <v>46278</v>
+      </c>
+      <c r="L18" s="15" t="inlineStr"/>
       <c r="M18" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N18" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N18" s="12" t="inlineStr"/>
       <c r="O18" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
+          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
+          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E19" s="20" t="inlineStr">
@@ -1981,108 +1975,88 @@
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I19" s="19" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="inlineStr"/>
       <c r="J19" s="22" t="n">
-        <v>46221</v>
+        <v>46253</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46224</v>
+        <v>46283</v>
       </c>
       <c r="L19" s="23" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
-        </is>
-      </c>
-      <c r="N19" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N19" s="20" t="inlineStr"/>
       <c r="O19" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>UNESCO</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
+          <t>unesco:b260be61-61f9-4226-2eb0-08df08e94b75</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
+          <t>914BRZ3061 - EDITAL Nº 13/2026 - 01 VAGA - CONSULTOR INDIVIDUAL-REPUBLICACAO</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr"/>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr">
-        <is>
-          <t>São Paulo - SP</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr"/>
       <c r="J20" s="14" t="n">
-        <v>46216</v>
+        <v>46273</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46223</v>
-      </c>
-      <c r="L20" s="15" t="n">
-        <v>133000</v>
-      </c>
+        <v>46278</v>
+      </c>
+      <c r="L20" s="15" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N20" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N20" s="12" t="inlineStr"/>
       <c r="O20" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -2161,12 +2135,12 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2184,27 +2158,27 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J22" s="14" t="n">
-        <v>46217</v>
+        <v>46216</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46222</v>
+        <v>46223</v>
       </c>
       <c r="L22" s="15" t="n">
-        <v>77100</v>
+        <v>133000</v>
       </c>
       <c r="M22" s="9" t="inlineStr">
         <is>
@@ -2218,7 +2192,7 @@
       </c>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
         </is>
       </c>
     </row>
@@ -2230,12 +2204,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2253,27 +2227,27 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I23" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J23" s="22" t="n">
-        <v>46225</v>
+        <v>46217</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46229</v>
+        <v>46222</v>
       </c>
       <c r="L23" s="23" t="n">
-        <v>114600</v>
+        <v>77100</v>
       </c>
       <c r="M23" s="17" t="inlineStr">
         <is>
@@ -2287,7 +2261,7 @@
       </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
         </is>
       </c>
     </row>
@@ -2299,12 +2273,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2322,27 +2296,27 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J24" s="14" t="n">
-        <v>46224</v>
+        <v>46220</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46233</v>
+        <v>46225</v>
       </c>
       <c r="L24" s="15" t="n">
-        <v>288000</v>
+        <v>58800</v>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
@@ -2356,7 +2330,7 @@
       </c>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
         </is>
       </c>
     </row>
@@ -2368,17 +2342,17 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E25" s="20" t="inlineStr">
@@ -2387,11 +2361,11 @@
         </is>
       </c>
       <c r="F25" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2401,21 +2375,19 @@
       </c>
       <c r="I25" s="19" t="inlineStr">
         <is>
-          <t>Brasília DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J25" s="22" t="n">
-        <v>46227</v>
+        <v>46221</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46231</v>
-      </c>
-      <c r="L25" s="23" t="n">
-        <v>150000</v>
-      </c>
+        <v>46224</v>
+      </c>
+      <c r="L25" s="23" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N25" s="20" t="inlineStr">
@@ -2425,7 +2397,7 @@
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
         </is>
       </c>
     </row>
@@ -2506,17 +2478,17 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E27" s="20" t="inlineStr">
@@ -2525,31 +2497,31 @@
         </is>
       </c>
       <c r="F27" s="21" t="n">
-        <v>0.343</v>
+        <v>0.4</v>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46232</v>
+        <v>46225</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46238</v>
+        <v>46229</v>
       </c>
       <c r="L27" s="23" t="n">
-        <v>30000</v>
+        <v>114600</v>
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
@@ -2563,7 +2535,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
         </is>
       </c>
     </row>
@@ -2575,12 +2547,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2590,13 +2562,15 @@
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F28" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2606,17 +2580,17 @@
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
-        <v>46232</v>
+        <v>46224</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46238</v>
+        <v>46233</v>
       </c>
       <c r="L28" s="15" t="n">
-        <v>30000</v>
+        <v>288000</v>
       </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
@@ -2630,7 +2604,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -2642,12 +2616,12 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
@@ -2665,7 +2639,7 @@
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
@@ -2675,21 +2649,21 @@
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46232</v>
+        <v>46227</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46237</v>
+        <v>46231</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>288000</v>
+        <v>150000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N29" s="20" t="inlineStr">
@@ -2699,7 +2673,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -2711,17 +2685,17 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2730,11 +2704,11 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.4</v>
+        <v>0.343</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2744,17 +2718,17 @@
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>204000</v>
+        <v>30000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
@@ -2768,7 +2742,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -2780,12 +2754,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2795,15 +2769,13 @@
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F31" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="inlineStr"/>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2813,17 +2785,17 @@
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>80000</v>
+        <v>30000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2837,7 +2809,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -2849,12 +2821,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2872,7 +2844,7 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
@@ -2906,7 +2878,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -2918,12 +2890,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2941,27 +2913,27 @@
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46240</v>
+        <v>46232</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46245</v>
+        <v>46237</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>100000</v>
+        <v>288000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
@@ -2975,7 +2947,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -2987,12 +2959,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -3010,7 +2982,7 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -3020,7 +2992,7 @@
       </c>
       <c r="I34" s="11" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J34" s="14" t="n">
@@ -3030,7 +3002,7 @@
         <v>46245</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>80000</v>
+        <v>204000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
@@ -3044,7 +3016,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -3056,17 +3028,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -3084,36 +3056,36 @@
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46244</v>
+        <v>46240</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46296</v>
+        <v>46245</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>935000</v>
+        <v>80000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N35" s="20" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -3125,12 +3097,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3140,33 +3112,35 @@
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F36" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46227</v>
+        <v>46240</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46252</v>
+        <v>46245</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>286000</v>
+        <v>100000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3180,7 +3154,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3192,12 +3166,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3211,11 +3185,11 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3225,19 +3199,21 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L37" s="23" t="inlineStr"/>
+        <v>46245</v>
+      </c>
+      <c r="L37" s="23" t="n">
+        <v>80000</v>
+      </c>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N37" s="20" t="inlineStr">
@@ -3247,7 +3223,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -3259,17 +3235,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3282,41 +3258,41 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46246</v>
+        <v>46244</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46257</v>
+        <v>46296</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>54000</v>
+        <v>935000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -3328,12 +3304,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3347,35 +3323,33 @@
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
         <v>46246</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46257</v>
-      </c>
-      <c r="L39" s="23" t="n">
-        <v>54000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L39" s="23" t="inlineStr"/>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
@@ -3385,7 +3359,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3397,17 +3371,17 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
@@ -3420,7 +3394,7 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3430,17 +3404,17 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46251</v>
+        <v>46246</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>50000</v>
+        <v>54000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3454,7 +3428,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3466,12 +3440,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3481,15 +3455,13 @@
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F41" s="21" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F41" s="21" t="inlineStr"/>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3499,17 +3471,17 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
+        <v>46227</v>
+      </c>
+      <c r="K41" s="22" t="n">
         <v>46252</v>
       </c>
-      <c r="K41" s="22" t="n">
-        <v>46259</v>
-      </c>
       <c r="L41" s="23" t="n">
-        <v>60000</v>
+        <v>286000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3523,7 +3495,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3535,17 +3507,17 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
@@ -3558,41 +3530,41 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J42" s="14" t="n">
-        <v>46208</v>
+        <v>46246</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46259</v>
+        <v>46257</v>
       </c>
       <c r="L42" s="15" t="n">
-        <v>500000</v>
+        <v>54000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3604,17 +3576,17 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
@@ -3627,7 +3599,7 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
@@ -3637,21 +3609,21 @@
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46272</v>
+        <v>46256</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
@@ -3661,7 +3633,7 @@
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3673,22 +3645,22 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Economista</t>
+          <t>Analista Powerbi</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
@@ -3696,27 +3668,27 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Remoto</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46265</v>
+        <v>46252</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46270</v>
+        <v>46259</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>30000</v>
+        <v>60000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
@@ -3730,7 +3702,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3742,17 +3714,17 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E45" s="20" t="inlineStr">
@@ -3765,41 +3737,41 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I45" s="19" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46266</v>
+        <v>46208</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46275</v>
+        <v>46259</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>70000</v>
+        <v>500000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3880,12 +3852,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13216</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -3903,46 +3875,322 @@
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H47" s="19" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I47" s="19" t="inlineStr">
+        <is>
+          <t>São Paulo - SP</t>
+        </is>
+      </c>
+      <c r="J47" s="22" t="n">
+        <v>46266</v>
+      </c>
+      <c r="K47" s="22" t="n">
+        <v>46283</v>
+      </c>
+      <c r="L47" s="23" t="n">
+        <v>70000</v>
+      </c>
+      <c r="M47" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N47" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O47" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13216/</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+        </is>
+      </c>
+      <c r="C48" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E48" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F48" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G48" s="11" t="inlineStr">
+        <is>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+        </is>
+      </c>
+      <c r="H48" s="11" t="inlineStr">
+        <is>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I48" s="11" t="inlineStr">
+        <is>
+          <t>Porto Alegre/RS</t>
+        </is>
+      </c>
+      <c r="J48" s="14" t="n">
+        <v>46246</v>
+      </c>
+      <c r="K48" s="14" t="n">
+        <v>46272</v>
+      </c>
+      <c r="L48" s="15" t="n">
+        <v>54000</v>
+      </c>
+      <c r="M48" s="9" t="inlineStr">
+        <is>
+          <t>En fase de apresentação</t>
+        </is>
+      </c>
+      <c r="N48" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O48" s="16" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B49" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
+        </is>
+      </c>
+      <c r="C49" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
+        </is>
+      </c>
+      <c r="D49" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria Pessoa Física (PF)</t>
+        </is>
+      </c>
+      <c r="E49" s="20" t="inlineStr">
+        <is>
+          <t>Economista</t>
+        </is>
+      </c>
+      <c r="F49" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G49" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
+        </is>
+      </c>
+      <c r="H49" s="19" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I49" s="19" t="inlineStr">
+        <is>
+          <t>Remoto</t>
+        </is>
+      </c>
+      <c r="J49" s="22" t="n">
+        <v>46265</v>
+      </c>
+      <c r="K49" s="22" t="n">
+        <v>46270</v>
+      </c>
+      <c r="L49" s="23" t="n">
+        <v>30000</v>
+      </c>
+      <c r="M49" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N49" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O49" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="inlineStr">
+        <is>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E50" s="12" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F50" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G50" s="11" t="inlineStr">
+        <is>
           <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
-      <c r="H47" s="19" t="inlineStr">
+      <c r="H50" s="11" t="inlineStr">
         <is>
           <t>OEI</t>
         </is>
       </c>
-      <c r="I47" s="19" t="inlineStr">
+      <c r="I50" s="11" t="inlineStr">
         <is>
           <t>Brasília - DF</t>
         </is>
       </c>
-      <c r="J47" s="22" t="n">
+      <c r="J50" s="14" t="n">
         <v>46275</v>
       </c>
-      <c r="K47" s="22" t="n">
+      <c r="K50" s="14" t="n">
         <v>46280</v>
       </c>
-      <c r="L47" s="23" t="n">
+      <c r="L50" s="15" t="n">
         <v>50000</v>
       </c>
-      <c r="M47" s="17" t="inlineStr">
+      <c r="M50" s="9" t="inlineStr">
         <is>
           <t>En evaluación</t>
         </is>
       </c>
-      <c r="N47" s="20" t="inlineStr">
+      <c r="N50" s="12" t="inlineStr">
         <is>
           <t>selecao.bra@oei.int</t>
         </is>
       </c>
-      <c r="O47" s="24" t="inlineStr">
+      <c r="O50" s="16" t="inlineStr">
         <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="B51" s="18" t="inlineStr">
+        <is>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
+        </is>
+      </c>
+      <c r="C51" s="19" t="inlineStr">
+        <is>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13238</t>
+        </is>
+      </c>
+      <c r="D51" s="19" t="inlineStr">
+        <is>
+          <t>Consultoria (tipo não especificado)</t>
+        </is>
+      </c>
+      <c r="E51" s="20" t="inlineStr">
+        <is>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F51" s="21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G51" s="19" t="inlineStr">
+        <is>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+        </is>
+      </c>
+      <c r="H51" s="19" t="inlineStr">
+        <is>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I51" s="19" t="inlineStr">
+        <is>
+          <t>Porto Alegre - RS</t>
+        </is>
+      </c>
+      <c r="J51" s="22" t="n">
+        <v>46275</v>
+      </c>
+      <c r="K51" s="22" t="n">
+        <v>46281</v>
+      </c>
+      <c r="L51" s="23" t="n">
+        <v>180000</v>
+      </c>
+      <c r="M51" s="17" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N51" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
+      <c r="O51" s="24" t="inlineStr">
+        <is>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O47"/>
+  <autoFilter ref="A1:O51"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -3990,6 +4238,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4028,7 +4280,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3">
@@ -4038,7 +4290,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
@@ -4048,7 +4300,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -4090,7 +4342,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3">
@@ -4100,7 +4352,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -4152,7 +4404,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -4162,7 +4414,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
@@ -4224,7 +4476,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3">
@@ -4244,7 +4496,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5">
@@ -4260,21 +4512,21 @@
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>Economia / Finanças Públicas</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Economia / Finanças Públicas</t>
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -4300,7 +4552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4336,7 +4588,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
@@ -4356,7 +4608,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -4369,8 +4621,18 @@
         <v>3</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>MGI</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B6"/>
+  <autoFilter ref="A1:B7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -4414,7 +4676,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -4429,7 +4691,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -4444,7 +4706,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -4459,7 +4721,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
🤖 Daily run: 2026-09-12 15:08
</commit_message>
<xml_diff>
--- a/analise_editais_pnud.xlsx
+++ b/analise_editais_pnud.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Perfis" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Editais'!$A$1:$O$48</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Editais'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Por_Fonte'!$A$1:$B$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Por_Fonte'!$1:$1</definedName>
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 11/09/2026 às 15:56</t>
+          <t>Gerado em 12/09/2026 às 15:02</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6">
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>164660.7142857143</v>
+        <v>165288.4615384615</v>
       </c>
     </row>
     <row r="20">
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>100000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="24">
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O51"/>
+  <dimension ref="A1:O48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -941,16 +941,16 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>146346</v>
+        <v>146349</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor (a) individual para assessoramento técnico especializado à consolidação, redação técnica e estruturação dos mecanismos de governança do Plano Estadual de Educação do Piauí 2026-2036</t>
+          <t>BRA/23/006 - CONSULTORIA TÉCNICA PARA O DESENVOLVIMENTO DE TECNOLOGIA APLICADA AO OBSERVATÓRIO DO NORDESTE</t>
         </is>
       </c>
       <c r="D3" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E3" s="20" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="G3" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H3" s="19" t="inlineStr">
@@ -973,14 +973,14 @@
       </c>
       <c r="I3" s="19" t="inlineStr">
         <is>
-          <t>Home based</t>
+          <t>HOME OFFICE</t>
         </is>
       </c>
       <c r="J3" s="22" t="n">
-        <v>46262</v>
+        <v>46267</v>
       </c>
       <c r="K3" s="22" t="n">
-        <v>46276</v>
+        <v>46278</v>
       </c>
       <c r="L3" s="23" t="inlineStr"/>
       <c r="M3" s="17" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="N3" s="20" t="inlineStr">
         <is>
-          <t>ugest@seduc.pi.gov.br</t>
+          <t>curriculos@consorcionordeste.gov.br</t>
         </is>
       </c>
       <c r="O3" s="24" t="inlineStr">
@@ -1006,16 +1006,16 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>146347</v>
+        <v>146353</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor (a) individual para apoiar tecnicamente a Superintendência de Ensino na realização das Olimpíadas do Conhecimento</t>
+          <t>TR - Mobilização Territorial/2026 - Suporte técnico especializado para Avaliação de Efetividade e Metodologias para Mobilização Territorial e Acesso a Instrumentos de Desenvolvimento</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E4" s="12" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr">
@@ -1038,14 +1038,14 @@
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Home based</t>
+          <t>Região Centro Oeste</t>
         </is>
       </c>
       <c r="J4" s="14" t="n">
-        <v>46262</v>
+        <v>46273</v>
       </c>
       <c r="K4" s="14" t="n">
-        <v>46276</v>
+        <v>46283</v>
       </c>
       <c r="L4" s="15" t="inlineStr"/>
       <c r="M4" s="9" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="N4" s="12" t="inlineStr">
         <is>
-          <t>ugest@seduc.pi.gov.br</t>
+          <t>prodocbra23018@sudeco.gov.br</t>
         </is>
       </c>
       <c r="O4" s="16" t="inlineStr">
@@ -1071,16 +1071,16 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>146349</v>
+        <v>146368</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>BRA/23/006 - CONSULTORIA TÉCNICA PARA O DESENVOLVIMENTO DE TECNOLOGIA APLICADA AO OBSERVATÓRIO DO NORDESTE</t>
+          <t>Edital 6/2026- UGP-PNUD/SENAD</t>
         </is>
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E5" s="20" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
@@ -1103,14 +1103,14 @@
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
-          <t>HOME OFFICE</t>
+          <t>null</t>
         </is>
       </c>
       <c r="J5" s="22" t="n">
-        <v>46267</v>
+        <v>46275</v>
       </c>
       <c r="K5" s="22" t="n">
-        <v>46278</v>
+        <v>46280</v>
       </c>
       <c r="L5" s="23" t="inlineStr"/>
       <c r="M5" s="17" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="N5" s="20" t="inlineStr">
         <is>
-          <t>curriculos@consorcionordeste.gov.br</t>
+          <t>cgep@mj.gov.br</t>
         </is>
       </c>
       <c r="O5" s="24" t="inlineStr">
@@ -1136,16 +1136,16 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>146353</v>
+        <v>146367</v>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>TR - Mobilização Territorial/2026 - Suporte técnico especializado para Avaliação de Efetividade e Metodologias para Mobilização Territorial e Acesso a Instrumentos de Desenvolvimento</t>
+          <t>EDITAL Nº 5/2026 - UGP-PNUD/SENAD</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -1168,14 +1168,14 @@
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Região Centro Oeste</t>
+          <t>Brasília/DF</t>
         </is>
       </c>
       <c r="J6" s="14" t="n">
-        <v>46273</v>
+        <v>46275</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>46283</v>
+        <v>46280</v>
       </c>
       <c r="L6" s="15" t="inlineStr"/>
       <c r="M6" s="9" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="N6" s="12" t="inlineStr">
         <is>
-          <t>prodocbra23018@sudeco.gov.br</t>
+          <t>cgep@mj.gov.br</t>
         </is>
       </c>
       <c r="O6" s="16" t="inlineStr">
@@ -1201,11 +1201,11 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>146368</v>
+        <v>146365</v>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>Edital 6/2026- UGP-PNUD/SENAD</t>
+          <t>EDITAL Nº 4/2026 - UGP-PNUD/SENAD</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="G7" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H7" s="19" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="N7" s="20" t="inlineStr">
         <is>
-          <t>cgep@mj.gov.br</t>
+          <t>dpagi@mj.gov.br</t>
         </is>
       </c>
       <c r="O7" s="24" t="inlineStr">
@@ -1266,11 +1266,11 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>146367</v>
+        <v>146364</v>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>EDITAL Nº 5/2026 - UGP-PNUD/SENAD</t>
+          <t>EDITAL Nº 3/2026 - UGP-PNUD/SENAD</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
@@ -1298,7 +1298,7 @@
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Brasília/DF</t>
+          <t>null</t>
         </is>
       </c>
       <c r="J8" s="14" t="n">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="N8" s="12" t="inlineStr">
         <is>
-          <t>cgep@mj.gov.br</t>
+          <t>dpagi@mj.gov.br</t>
         </is>
       </c>
       <c r="O8" s="16" t="inlineStr">
@@ -1331,11 +1331,11 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>146365</v>
+        <v>146363</v>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>EDITAL Nº 4/2026 - UGP-PNUD/SENAD</t>
+          <t>EDITAL Nº 2/2026 - UGP-PNUD/SENAD</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
@@ -1380,7 +1380,7 @@
       </c>
       <c r="N9" s="20" t="inlineStr">
         <is>
-          <t>dpagi@mj.gov.br</t>
+          <t>senad@mj.gov.br</t>
         </is>
       </c>
       <c r="O9" s="24" t="inlineStr">
@@ -1396,11 +1396,11 @@
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>146364</v>
+        <v>146369</v>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>EDITAL Nº 3/2026 - UGP-PNUD/SENAD</t>
+          <t>Edital nº 29/2026 – Contratação de Consultoria Individual para o desenho institucional da Secretaria de Serviços Compartilhados (SSC/MGI)</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1410,34 +1410,34 @@
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F10" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr"/>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J10" s="14" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>46280</v>
-      </c>
-      <c r="L10" s="15" t="inlineStr"/>
+        <v>46290</v>
+      </c>
+      <c r="L10" s="15" t="n">
+        <v>120000</v>
+      </c>
       <c r="M10" s="9" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1445,7 +1445,7 @@
       </c>
       <c r="N10" s="12" t="inlineStr">
         <is>
-          <t>dpagi@mj.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O10" s="16" t="inlineStr">
@@ -1461,11 +1461,11 @@
         </is>
       </c>
       <c r="B11" s="18" t="n">
-        <v>146363</v>
+        <v>146370</v>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>EDITAL Nº 2/2026 - UGP-PNUD/SENAD</t>
+          <t xml:space="preserve">Edital nº 25/2026 – Contratação de Consultoria Individual para avaliar os efeitos de intervenções comportamentais (políticas fiscais e de arquitetura de escolha) em mercado experimental para promover escolhas alimentares mais saudáveis. </t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
@@ -1475,34 +1475,34 @@
       </c>
       <c r="E11" s="20" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F11" s="21" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F11" s="21" t="inlineStr"/>
       <c r="G11" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H11" s="19" t="inlineStr">
         <is>
-          <t>Não identificado</t>
+          <t>MGI</t>
         </is>
       </c>
       <c r="I11" s="19" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>REMOTO</t>
         </is>
       </c>
       <c r="J11" s="22" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="K11" s="22" t="n">
-        <v>46280</v>
-      </c>
-      <c r="L11" s="23" t="inlineStr"/>
+        <v>46290</v>
+      </c>
+      <c r="L11" s="23" t="n">
+        <v>126000</v>
+      </c>
       <c r="M11" s="17" t="inlineStr">
         <is>
           <t>Aprovada</t>
@@ -1510,7 +1510,7 @@
       </c>
       <c r="N11" s="20" t="inlineStr">
         <is>
-          <t>senad@mj.gov.br</t>
+          <t>prodoc.mgi@gestao.gov.br</t>
         </is>
       </c>
       <c r="O11" s="24" t="inlineStr">
@@ -1522,15 +1522,17 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="n">
-        <v>146369</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>unesco:5c1d62c6-1efa-431c-b9e2-08df0436270c</t>
+        </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Edital nº 29/2026 – Contratação de Consultoria Individual para o desenho institucional da Secretaria de Serviços Compartilhados (SSC/MGI)</t>
+          <t>914BRZ1155 - EDITAL Nº 54/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
@@ -1540,62 +1542,56 @@
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F12" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>MGI</t>
-        </is>
-      </c>
-      <c r="I12" s="11" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr"/>
       <c r="J12" s="14" t="n">
-        <v>46276</v>
+        <v>46274</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>46290</v>
-      </c>
-      <c r="L12" s="15" t="n">
-        <v>120000</v>
-      </c>
+        <v>46278</v>
+      </c>
+      <c r="L12" s="15" t="inlineStr"/>
       <c r="M12" s="9" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N12" s="12" t="inlineStr">
-        <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N12" s="12" t="inlineStr"/>
       <c r="O12" s="16" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>PNUD</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="n">
-        <v>146370</v>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>unesco:1d72ac67-6c7d-4a8b-dd78-08df0757caed</t>
+        </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Edital nº 25/2026 – Contratação de Consultoria Individual para avaliar os efeitos de intervenções comportamentais (políticas fiscais e de arquitetura de escolha) em mercado experimental para promover escolhas alimentares mais saudáveis. </t>
+          <t>914BRZ1154 - Edital 05/2026 - 01 perfil - Consultoria Individual</t>
         </is>
       </c>
       <c r="D13" s="19" t="inlineStr">
@@ -1605,47 +1601,39 @@
       </c>
       <c r="E13" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F13" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F13" s="21" t="n">
+        <v>0.3</v>
+      </c>
       <c r="G13" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H13" s="19" t="inlineStr">
         <is>
-          <t>MGI</t>
-        </is>
-      </c>
-      <c r="I13" s="19" t="inlineStr">
-        <is>
-          <t>REMOTO</t>
-        </is>
-      </c>
+          <t>UNESCO</t>
+        </is>
+      </c>
+      <c r="I13" s="19" t="inlineStr"/>
       <c r="J13" s="22" t="n">
-        <v>46276</v>
+        <v>46268</v>
       </c>
       <c r="K13" s="22" t="n">
-        <v>46290</v>
-      </c>
-      <c r="L13" s="23" t="n">
-        <v>126000</v>
-      </c>
+        <v>46278</v>
+      </c>
+      <c r="L13" s="23" t="inlineStr"/>
       <c r="M13" s="17" t="inlineStr">
         <is>
-          <t>Aprovada</t>
-        </is>
-      </c>
-      <c r="N13" s="20" t="inlineStr">
-        <is>
-          <t>prodoc.mgi@gestao.gov.br</t>
-        </is>
-      </c>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="N13" s="20" t="inlineStr"/>
       <c r="O13" s="24" t="inlineStr">
         <is>
-          <t>https://parceiros.undp.org.br/opportunities</t>
+          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
         </is>
       </c>
     </row>
@@ -1657,12 +1645,12 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>unesco:5c1d62c6-1efa-431c-b9e2-08df0436270c</t>
+          <t>unesco:8c824e7b-7b9a-4a59-7ffc-08df082d82f3</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1155 - EDITAL Nº 54/2026 - 1 vaga - Consultor Individual</t>
+          <t>914BRZ1163 - Publicação -  Edital 68/2026 - 01 Vaga consultor Individual</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
@@ -1680,7 +1668,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1690,10 +1678,10 @@
       </c>
       <c r="I14" s="11" t="inlineStr"/>
       <c r="J14" s="14" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="L14" s="15" t="inlineStr"/>
       <c r="M14" s="9" t="inlineStr">
@@ -1716,12 +1704,12 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>unesco:83caba6b-babf-4307-dd76-08df0757caed</t>
+          <t>unesco:5907e744-d46d-4c01-2eaf-08df08e94b75</t>
         </is>
       </c>
       <c r="C15" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1164 - EDITAL 03/2026 - 2 VAGAS - Consultor Individual</t>
+          <t>914BRZ1159 - Publicação Edital 37/2026 - 2 vagas - Consultor Individual</t>
         </is>
       </c>
       <c r="D15" s="19" t="inlineStr">
@@ -1749,10 +1737,10 @@
       </c>
       <c r="I15" s="19" t="inlineStr"/>
       <c r="J15" s="22" t="n">
-        <v>46270</v>
+        <v>46277</v>
       </c>
       <c r="K15" s="22" t="n">
-        <v>46276</v>
+        <v>46283</v>
       </c>
       <c r="L15" s="23" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr">
@@ -1775,12 +1763,12 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>unesco:1d72ac67-6c7d-4a8b-dd78-08df0757caed</t>
+          <t>unesco:b0920c88-ab66-4545-2ead-08df08e94b75</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>914BRZ1154 - Edital 05/2026 - 01 perfil - Consultoria Individual</t>
+          <t>Projeto 914BRZ3050 - Edital N° 04/2026 - Consultor Individual PRORROGAÇÃO</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -1798,7 +1786,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1808,7 +1796,7 @@
       </c>
       <c r="I16" s="11" t="inlineStr"/>
       <c r="J16" s="14" t="n">
-        <v>46268</v>
+        <v>46274</v>
       </c>
       <c r="K16" s="14" t="n">
         <v>46278</v>
@@ -1834,12 +1822,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>unesco:8c824e7b-7b9a-4a59-7ffc-08df082d82f3</t>
+          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>914BRZ1163 - Publicação -  Edital 68/2026 - 01 Vaga consultor Individual</t>
+          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
@@ -1857,7 +1845,7 @@
       </c>
       <c r="G17" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H17" s="19" t="inlineStr">
@@ -1867,10 +1855,10 @@
       </c>
       <c r="I17" s="19" t="inlineStr"/>
       <c r="J17" s="22" t="n">
-        <v>46276</v>
+        <v>46253</v>
       </c>
       <c r="K17" s="22" t="n">
-        <v>46281</v>
+        <v>46283</v>
       </c>
       <c r="L17" s="23" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr">
@@ -1893,12 +1881,12 @@
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>unesco:b0920c88-ab66-4545-2ead-08df08e94b75</t>
+          <t>unesco:b260be61-61f9-4226-2eb0-08df08e94b75</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ3050 - Edital N° 04/2026 - Consultor Individual PRORROGAÇÃO</t>
+          <t>914BRZ3061 - EDITAL Nº 13/2026 - 01 VAGA - CONSULTOR INDIVIDUAL-REPUBLICACAO</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1908,15 +1896,13 @@
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F18" s="13" t="n">
-        <v>0.3</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr"/>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1926,7 +1912,7 @@
       </c>
       <c r="I18" s="11" t="inlineStr"/>
       <c r="J18" s="14" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="K18" s="14" t="n">
         <v>46278</v>
@@ -1947,22 +1933,22 @@
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>unesco:030ad7b8-d33f-491a-31d9-08defb16c1ac</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>Projeto 914BRZ5067 - Edital Nº 08/2026 - 1 vaga - Consultor Individual</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E19" s="20" t="inlineStr">
@@ -1971,52 +1957,62 @@
         </is>
       </c>
       <c r="F19" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I19" s="19" t="inlineStr"/>
+          <t>OEI</t>
+        </is>
+      </c>
+      <c r="I19" s="19" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J19" s="22" t="n">
-        <v>46253</v>
+        <v>46217</v>
       </c>
       <c r="K19" s="22" t="n">
-        <v>46283</v>
-      </c>
-      <c r="L19" s="23" t="inlineStr"/>
+        <v>46222</v>
+      </c>
+      <c r="L19" s="23" t="n">
+        <v>77100</v>
+      </c>
       <c r="M19" s="17" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N19" s="20" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N19" s="20" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O19" s="24" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>UNESCO</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>unesco:b260be61-61f9-4226-2eb0-08df08e94b75</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>914BRZ3061 - EDITAL Nº 13/2026 - 01 VAGA - CONSULTOR INDIVIDUAL-REPUBLICACAO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
@@ -2026,37 +2022,49 @@
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>UNESCO</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr"/>
+          <t>OEI/BRA</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>Brasília - DF</t>
+        </is>
+      </c>
       <c r="J20" s="14" t="n">
-        <v>46273</v>
+        <v>46223</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>46278</v>
-      </c>
-      <c r="L20" s="15" t="inlineStr"/>
+        <v>46238</v>
+      </c>
+      <c r="L20" s="15" t="n">
+        <v>100000</v>
+      </c>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="N20" s="12" t="inlineStr"/>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="N20" s="12" t="inlineStr">
+        <is>
+          <t>selecao.bra@oei.int</t>
+        </is>
+      </c>
       <c r="O20" s="16" t="inlineStr">
         <is>
-          <t>https://roster.brasilia.unesco.org/app/selection-process-list</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
         </is>
       </c>
     </row>
@@ -2135,17 +2143,17 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13062</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -2154,11 +2162,11 @@
         </is>
       </c>
       <c r="F22" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -2168,21 +2176,19 @@
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J22" s="14" t="n">
-        <v>46216</v>
+        <v>46221</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>46223</v>
-      </c>
-      <c r="L22" s="15" t="n">
-        <v>133000</v>
-      </c>
+        <v>46224</v>
+      </c>
+      <c r="L22" s="15" t="inlineStr"/>
       <c r="M22" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N22" s="12" t="inlineStr">
@@ -2192,7 +2198,7 @@
       </c>
       <c r="O22" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13062/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
         </is>
       </c>
     </row>
@@ -2204,12 +2210,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13078</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
@@ -2227,12 +2233,12 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I23" s="19" t="inlineStr">
@@ -2241,13 +2247,13 @@
         </is>
       </c>
       <c r="J23" s="22" t="n">
-        <v>46217</v>
+        <v>46220</v>
       </c>
       <c r="K23" s="22" t="n">
-        <v>46222</v>
+        <v>46225</v>
       </c>
       <c r="L23" s="23" t="n">
-        <v>77100</v>
+        <v>58800</v>
       </c>
       <c r="M23" s="17" t="inlineStr">
         <is>
@@ -2261,7 +2267,7 @@
       </c>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13078/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
         </is>
       </c>
     </row>
@@ -2273,12 +2279,12 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13015</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -2296,7 +2302,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2306,21 +2312,21 @@
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Brasília DF</t>
         </is>
       </c>
       <c r="J24" s="14" t="n">
-        <v>46220</v>
+        <v>46227</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>46225</v>
+        <v>46231</v>
       </c>
       <c r="L24" s="15" t="n">
-        <v>58800</v>
+        <v>150000</v>
       </c>
       <c r="M24" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N24" s="12" t="inlineStr">
@@ -2330,7 +2336,7 @@
       </c>
       <c r="O24" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003-tr13015/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
         </is>
       </c>
     </row>
@@ -2342,17 +2348,17 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/002 – TR 13098</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E25" s="20" t="inlineStr">
@@ -2361,11 +2367,11 @@
         </is>
       </c>
       <c r="F25" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
@@ -2375,19 +2381,21 @@
       </c>
       <c r="I25" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J25" s="22" t="n">
-        <v>46221</v>
+        <v>46225</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>46224</v>
-      </c>
-      <c r="L25" s="23" t="inlineStr"/>
+        <v>46229</v>
+      </c>
+      <c r="L25" s="23" t="n">
+        <v>114600</v>
+      </c>
       <c r="M25" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N25" s="20" t="inlineStr">
@@ -2397,7 +2405,7 @@
       </c>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-002-tr-13098/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
         </is>
       </c>
     </row>
@@ -2409,17 +2417,17 @@
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/16/002 – TR13077</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
@@ -2432,27 +2440,27 @@
       </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H26" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
         </is>
       </c>
       <c r="J26" s="14" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>46238</v>
+        <v>46233</v>
       </c>
       <c r="L26" s="15" t="n">
-        <v>100000</v>
+        <v>288000</v>
       </c>
       <c r="M26" s="9" t="inlineStr">
         <is>
@@ -2466,7 +2474,7 @@
       </c>
       <c r="O26" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-16-002-tr13077/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
         </is>
       </c>
     </row>
@@ -2478,12 +2486,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13107</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
@@ -2501,7 +2509,7 @@
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -2511,17 +2519,17 @@
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
         </is>
       </c>
       <c r="J27" s="22" t="n">
-        <v>46225</v>
+        <v>46232</v>
       </c>
       <c r="K27" s="22" t="n">
-        <v>46229</v>
+        <v>46237</v>
       </c>
       <c r="L27" s="23" t="n">
-        <v>114600</v>
+        <v>288000</v>
       </c>
       <c r="M27" s="17" t="inlineStr">
         <is>
@@ -2535,7 +2543,7 @@
       </c>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13107/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
         </is>
       </c>
     </row>
@@ -2547,12 +2555,12 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13105</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2562,15 +2570,13 @@
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F28" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="inlineStr"/>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2580,17 +2586,17 @@
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>Perfil 1: Amapá  AP Amapá - AP Perfil 2: Amazonas  AM Amazonas - AM Perfil 3: Bahia  BA Bahia - BA Perfil 4: Distrito Federal  DF Distrito Federal, DF Perfil 5: Mato Grosso do Sul (MS) Mato Grosso do Sul, MS Perfil 6 - Pará (PA) Para, PA Perfil 7: Paraíba (PB) Paraíba, PB Perfil 8: Pernambuco (PE) Pernambuco, PE Perfil 9: Rio Grande do Norte (RN) Rio Grande do Norte, RN Perfil 10: Rio Grande do Sul (RS) Rio Grande do Sul, RS Perfil 11: Roraima (RR) Roraima, RR Perfil 12: Santa Catarina (SC) Santa Catarina, SC</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J28" s="14" t="n">
-        <v>46224</v>
+        <v>46232</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>46233</v>
+        <v>46238</v>
       </c>
       <c r="L28" s="15" t="n">
-        <v>288000</v>
+        <v>30000</v>
       </c>
       <c r="M28" s="9" t="inlineStr">
         <is>
@@ -2604,7 +2610,7 @@
       </c>
       <c r="O28" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13105/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
         </is>
       </c>
     </row>
@@ -2616,17 +2622,17 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/002 – TR 13111</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
         </is>
       </c>
       <c r="D29" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E29" s="20" t="inlineStr">
@@ -2635,35 +2641,35 @@
         </is>
       </c>
       <c r="F29" s="21" t="n">
-        <v>0.4</v>
+        <v>0.343</v>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Brasília DF</t>
+          <t>Remoto, Brasília - DF</t>
         </is>
       </c>
       <c r="J29" s="22" t="n">
-        <v>46227</v>
+        <v>46232</v>
       </c>
       <c r="K29" s="22" t="n">
-        <v>46231</v>
+        <v>46238</v>
       </c>
       <c r="L29" s="23" t="n">
-        <v>150000</v>
+        <v>30000</v>
       </c>
       <c r="M29" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N29" s="20" t="inlineStr">
@@ -2673,7 +2679,7 @@
       </c>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-002-tr-13111/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
         </is>
       </c>
     </row>
@@ -2685,17 +2691,17 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13169</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Física (PF)</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -2704,11 +2710,11 @@
         </is>
       </c>
       <c r="F30" s="13" t="n">
-        <v>0.343</v>
+        <v>0.4</v>
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2718,17 +2724,17 @@
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J30" s="14" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K30" s="14" t="n">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="L30" s="15" t="n">
-        <v>30000</v>
+        <v>204000</v>
       </c>
       <c r="M30" s="9" t="inlineStr">
         <is>
@@ -2742,7 +2748,7 @@
       </c>
       <c r="O30" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13169/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
         </is>
       </c>
     </row>
@@ -2754,12 +2760,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO DEMOCRACIA PARTICIPATIVA/BRA/SGPR/24 – TR13173</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -2769,13 +2775,15 @@
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F31" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F31" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
@@ -2785,17 +2793,17 @@
       </c>
       <c r="I31" s="19" t="inlineStr">
         <is>
-          <t>Remoto, Brasília - DF</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J31" s="22" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K31" s="22" t="n">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="L31" s="23" t="n">
-        <v>30000</v>
+        <v>204000</v>
       </c>
       <c r="M31" s="17" t="inlineStr">
         <is>
@@ -2809,7 +2817,7 @@
       </c>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-democracia-participativa-bra-sgpr-24-tr13173/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
         </is>
       </c>
     </row>
@@ -2821,12 +2829,12 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13193</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
@@ -2844,7 +2852,7 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
@@ -2864,7 +2872,7 @@
         <v>46245</v>
       </c>
       <c r="L32" s="15" t="n">
-        <v>204000</v>
+        <v>80000</v>
       </c>
       <c r="M32" s="9" t="inlineStr">
         <is>
@@ -2878,7 +2886,7 @@
       </c>
       <c r="O32" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13193/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
         </is>
       </c>
     </row>
@@ -2890,12 +2898,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/003 – TR13165</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -2913,27 +2921,27 @@
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Articulação Estadual - Alagoas Alagoas Articulação Estadual - Espírito Santo Espírito Santo Articulação Estadual - Goiás Goiás Articulação Estadual - Maranhão Maranhão Articulação Estadual - Minas Gerais Minas Gerais Articulação Estadual - Rondônia Rondônia Articulação Estadual - São Paulo São Paulo Articulação Estadual - Tocantins Tocantins</t>
+          <t>Brasília - Df</t>
         </is>
       </c>
       <c r="J33" s="22" t="n">
-        <v>46232</v>
+        <v>46240</v>
       </c>
       <c r="K33" s="22" t="n">
-        <v>46237</v>
+        <v>46245</v>
       </c>
       <c r="L33" s="23" t="n">
-        <v>288000</v>
+        <v>80000</v>
       </c>
       <c r="M33" s="17" t="inlineStr">
         <is>
@@ -2947,7 +2955,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-003/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
         </is>
       </c>
     </row>
@@ -2959,12 +2967,12 @@
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13192</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
@@ -2982,7 +2990,7 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -3002,7 +3010,7 @@
         <v>46245</v>
       </c>
       <c r="L34" s="15" t="n">
-        <v>204000</v>
+        <v>100000</v>
       </c>
       <c r="M34" s="9" t="inlineStr">
         <is>
@@ -3016,7 +3024,7 @@
       </c>
       <c r="O34" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13192/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
         </is>
       </c>
     </row>
@@ -3028,17 +3036,17 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195</t>
+          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13195</t>
+          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E35" s="20" t="inlineStr">
@@ -3056,36 +3064,36 @@
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I35" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J35" s="22" t="n">
-        <v>46240</v>
+        <v>46244</v>
       </c>
       <c r="K35" s="22" t="n">
-        <v>46245</v>
+        <v>46296</v>
       </c>
       <c r="L35" s="23" t="n">
-        <v>80000</v>
+        <v>935000</v>
       </c>
       <c r="M35" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N35" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13195/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
         </is>
       </c>
     </row>
@@ -3097,12 +3105,12 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13194</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
@@ -3112,35 +3120,33 @@
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F36" s="13" t="n">
-        <v>0.4</v>
-      </c>
+          <t>Não Classificado</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="inlineStr"/>
       <c r="G36" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Não classificada</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Brasília - DF</t>
+          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
         </is>
       </c>
       <c r="J36" s="14" t="n">
-        <v>46240</v>
+        <v>46227</v>
       </c>
       <c r="K36" s="14" t="n">
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="L36" s="15" t="n">
-        <v>100000</v>
+        <v>286000</v>
       </c>
       <c r="M36" s="9" t="inlineStr">
         <is>
@@ -3154,7 +3160,7 @@
       </c>
       <c r="O36" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-13194/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
         </is>
       </c>
     </row>
@@ -3166,12 +3172,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196</t>
+          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
         </is>
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13196</t>
+          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -3185,11 +3191,11 @@
         </is>
       </c>
       <c r="F37" s="21" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G37" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H37" s="19" t="inlineStr">
@@ -3199,21 +3205,19 @@
       </c>
       <c r="I37" s="19" t="inlineStr">
         <is>
-          <t>Brasília - Df</t>
+          <t>Brasília - DF | Híbrido</t>
         </is>
       </c>
       <c r="J37" s="22" t="n">
-        <v>46240</v>
+        <v>46246</v>
       </c>
       <c r="K37" s="22" t="n">
-        <v>46245</v>
-      </c>
-      <c r="L37" s="23" t="n">
-        <v>80000</v>
-      </c>
+        <v>46250</v>
+      </c>
+      <c r="L37" s="23" t="inlineStr"/>
       <c r="M37" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N37" s="20" t="inlineStr">
@@ -3223,7 +3227,7 @@
       </c>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026-tr13196/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
         </is>
       </c>
     </row>
@@ -3235,17 +3239,17 @@
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13125-2026-oei-mdhc</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Concorrência nº 13125/2026 – OEI/MDHC – TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -3258,41 +3262,41 @@
       </c>
       <c r="G38" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J38" s="14" t="n">
-        <v>46244</v>
+        <v>46246</v>
       </c>
       <c r="K38" s="14" t="n">
-        <v>46296</v>
+        <v>46257</v>
       </c>
       <c r="L38" s="15" t="n">
-        <v>935000</v>
+        <v>54000</v>
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N38" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O38" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13125-2026-oei-mdhc/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
         </is>
       </c>
     </row>
@@ -3304,12 +3308,12 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor PROJETO FP-26-02 Ciência, Inovação e Desenvolvimento – TR 13199</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -3323,33 +3327,35 @@
         </is>
       </c>
       <c r="F39" s="21" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="G39" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H39" s="19" t="inlineStr">
         <is>
-          <t>OEI</t>
+          <t>OEI/BRA</t>
         </is>
       </c>
       <c r="I39" s="19" t="inlineStr">
         <is>
-          <t>Brasília - DF | Híbrido</t>
+          <t>Porto Alegre/RS</t>
         </is>
       </c>
       <c r="J39" s="22" t="n">
         <v>46246</v>
       </c>
       <c r="K39" s="22" t="n">
-        <v>46250</v>
-      </c>
-      <c r="L39" s="23" t="inlineStr"/>
+        <v>46257</v>
+      </c>
+      <c r="L39" s="23" t="n">
+        <v>54000</v>
+      </c>
       <c r="M39" s="17" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N39" s="20" t="inlineStr">
@@ -3359,7 +3365,7 @@
       </c>
       <c r="O39" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-projeto-fp-26-02-ciencia-inovacao-e-desenvolvimento-tr-13199/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
         </is>
       </c>
     </row>
@@ -3371,17 +3377,17 @@
       </c>
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13202</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Especializada (não especifica PF/PJ)</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
@@ -3394,7 +3400,7 @@
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H40" s="11" t="inlineStr">
@@ -3404,17 +3410,17 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Recife - PE</t>
         </is>
       </c>
       <c r="J40" s="14" t="n">
-        <v>46246</v>
+        <v>46251</v>
       </c>
       <c r="K40" s="14" t="n">
-        <v>46257</v>
+        <v>46256</v>
       </c>
       <c r="L40" s="15" t="n">
-        <v>54000</v>
+        <v>50000</v>
       </c>
       <c r="M40" s="9" t="inlineStr">
         <is>
@@ -3428,7 +3434,7 @@
       </c>
       <c r="O40" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13202/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
         </is>
       </c>
     </row>
@@ -3440,12 +3446,12 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13109</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -3455,13 +3461,15 @@
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>Não Classificado</t>
-        </is>
-      </c>
-      <c r="F41" s="21" t="inlineStr"/>
+          <t>Analista Powerbi</t>
+        </is>
+      </c>
+      <c r="F41" s="21" t="n">
+        <v>0.4</v>
+      </c>
       <c r="G41" s="19" t="inlineStr">
         <is>
-          <t>Não classificada</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H41" s="19" t="inlineStr">
@@ -3471,17 +3479,17 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>VAGA 1 - áreas DIPES, DIISE, DIORF, DIPLIC, DICON - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo VAGA 2 - áreas DRECID, EFAPE, SUPLAN E SUPED - Consultoria Técnica Especializada em Governança do Conhecimento e Inteligência Artificial São Paulo</t>
+          <t>São Paulo - SP</t>
         </is>
       </c>
       <c r="J41" s="22" t="n">
-        <v>46227</v>
+        <v>46252</v>
       </c>
       <c r="K41" s="22" t="n">
-        <v>46252</v>
+        <v>46259</v>
       </c>
       <c r="L41" s="23" t="n">
-        <v>286000</v>
+        <v>60000</v>
       </c>
       <c r="M41" s="17" t="inlineStr">
         <is>
@@ -3495,7 +3503,7 @@
       </c>
       <c r="O41" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13109/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
         </is>
       </c>
     </row>
@@ -3507,12 +3515,12 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13204</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
@@ -3530,7 +3538,7 @@
       </c>
       <c r="G42" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
+          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H42" s="11" t="inlineStr">
@@ -3547,14 +3555,14 @@
         <v>46246</v>
       </c>
       <c r="K42" s="14" t="n">
-        <v>46257</v>
+        <v>46272</v>
       </c>
       <c r="L42" s="15" t="n">
         <v>54000</v>
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N42" s="12" t="inlineStr">
@@ -3564,7 +3572,7 @@
       </c>
       <c r="O42" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13204/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
         </is>
       </c>
     </row>
@@ -3576,17 +3584,17 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200</t>
+          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/22/003 – TR13200</t>
+          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>Consultoria Especializada (não especifica PF/PJ)</t>
+          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
         </is>
       </c>
       <c r="E43" s="20" t="inlineStr">
@@ -3599,41 +3607,41 @@
       </c>
       <c r="G43" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Direito / Jurídico, Gestão / Administração Pública</t>
+          <t>Tecnologia da Informação / Dados</t>
         </is>
       </c>
       <c r="H43" s="19" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI/MDHC</t>
         </is>
       </c>
       <c r="I43" s="19" t="inlineStr">
         <is>
-          <t>Recife - PE</t>
+          <t>Nacional</t>
         </is>
       </c>
       <c r="J43" s="22" t="n">
-        <v>46251</v>
+        <v>46208</v>
       </c>
       <c r="K43" s="22" t="n">
-        <v>46256</v>
+        <v>46259</v>
       </c>
       <c r="L43" s="23" t="n">
-        <v>50000</v>
+        <v>500000</v>
       </c>
       <c r="M43" s="17" t="inlineStr">
         <is>
-          <t>En evaluación</t>
+          <t>En presentación</t>
         </is>
       </c>
       <c r="N43" s="20" t="inlineStr">
         <is>
-          <t>selecao.bra@oei.int</t>
+          <t>compras.bra@oei.int</t>
         </is>
       </c>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-22-003-tr13200/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3645,22 +3653,22 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/24/004 – TR13206</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>Consultoria (tipo não especificado)</t>
+          <t>Consultoria Pessoa Física (PF)</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Analista Powerbi</t>
+          <t>Economista</t>
         </is>
       </c>
       <c r="F44" s="13" t="n">
@@ -3668,27 +3676,27 @@
       </c>
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
         </is>
       </c>
       <c r="H44" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>São Paulo - SP</t>
+          <t>Remoto</t>
         </is>
       </c>
       <c r="J44" s="14" t="n">
-        <v>46252</v>
+        <v>46265</v>
       </c>
       <c r="K44" s="14" t="n">
-        <v>46259</v>
+        <v>46270</v>
       </c>
       <c r="L44" s="15" t="n">
-        <v>60000</v>
+        <v>30000</v>
       </c>
       <c r="M44" s="9" t="inlineStr">
         <is>
@@ -3702,7 +3710,7 @@
       </c>
       <c r="O44" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-24-004-tr13206/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
         </is>
       </c>
     </row>
@@ -3714,12 +3722,12 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13046/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -3737,7 +3745,7 @@
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
@@ -3751,17 +3759,17 @@
         </is>
       </c>
       <c r="J45" s="22" t="n">
-        <v>46208</v>
+        <v>46244</v>
       </c>
       <c r="K45" s="22" t="n">
-        <v>46259</v>
+        <v>46300</v>
       </c>
       <c r="L45" s="23" t="n">
-        <v>500000</v>
+        <v>350000</v>
       </c>
       <c r="M45" s="17" t="inlineStr">
         <is>
-          <t>En presentación</t>
+          <t>En fase de apresentação</t>
         </is>
       </c>
       <c r="N45" s="20" t="inlineStr">
@@ -3771,7 +3779,7 @@
       </c>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13046-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
         </is>
       </c>
     </row>
@@ -3783,17 +3791,17 @@
       </c>
       <c r="B46" s="10" t="inlineStr">
         <is>
-          <t>oei:concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco</t>
+          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
         </is>
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>CONCORRÊNCIA Nº 13126/2026- OEI/MDHC TÉCNICA E PREÇO</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>Consultoria Pessoa Jurídica (PJ) / Empresa</t>
+          <t>Consultoria (tipo não especificado)</t>
         </is>
       </c>
       <c r="E46" s="12" t="inlineStr">
@@ -3806,41 +3814,41 @@
       </c>
       <c r="G46" s="11" t="inlineStr">
         <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia</t>
+          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H46" s="11" t="inlineStr">
         <is>
-          <t>OEI/MDHC</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Brasília - DF</t>
         </is>
       </c>
       <c r="J46" s="14" t="n">
-        <v>46244</v>
+        <v>46275</v>
       </c>
       <c r="K46" s="14" t="n">
-        <v>46300</v>
+        <v>46280</v>
       </c>
       <c r="L46" s="15" t="n">
-        <v>350000</v>
+        <v>50000</v>
       </c>
       <c r="M46" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N46" s="12" t="inlineStr">
         <is>
-          <t>compras.bra@oei.int</t>
+          <t>selecao.bra@oei.int</t>
         </is>
       </c>
       <c r="O46" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/concorrencia-no-13126-2026-oei-mdhc-tecnica-e-preco/</t>
+          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
         </is>
       </c>
     </row>
@@ -3921,12 +3929,12 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203</t>
+          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
         </is>
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO OEI/BRA/25/001 – TR13203</t>
+          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13238</t>
         </is>
       </c>
       <c r="D48" s="11" t="inlineStr">
@@ -3940,35 +3948,33 @@
         </is>
       </c>
       <c r="F48" s="13" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="G48" s="11" t="inlineStr">
         <is>
-          <t>Estatística / Pesquisa / Metodologia, Meio Ambiente / Clima / Geografia</t>
+          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
         </is>
       </c>
       <c r="H48" s="11" t="inlineStr">
         <is>
-          <t>OEI/BRA</t>
+          <t>OEI</t>
         </is>
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Porto Alegre/RS</t>
+          <t>Porto Alegre - RS</t>
         </is>
       </c>
       <c r="J48" s="14" t="n">
-        <v>46246</v>
+        <v>46275</v>
       </c>
       <c r="K48" s="14" t="n">
-        <v>46272</v>
-      </c>
-      <c r="L48" s="15" t="n">
-        <v>54000</v>
-      </c>
+        <v>46281</v>
+      </c>
+      <c r="L48" s="15" t="inlineStr"/>
       <c r="M48" s="9" t="inlineStr">
         <is>
-          <t>En fase de apresentação</t>
+          <t>En evaluación</t>
         </is>
       </c>
       <c r="N48" s="12" t="inlineStr">
@@ -3978,219 +3984,12 @@
       </c>
       <c r="O48" s="16" t="inlineStr">
         <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-oei-bra-25-001-tr13203/</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B49" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211</t>
-        </is>
-      </c>
-      <c r="C49" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MEMP/SEBRAE/2024 – TR13211</t>
-        </is>
-      </c>
-      <c r="D49" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria Pessoa Física (PF)</t>
-        </is>
-      </c>
-      <c r="E49" s="20" t="inlineStr">
-        <is>
-          <t>Economista</t>
-        </is>
-      </c>
-      <c r="F49" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G49" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Economia / Finanças Públicas, Meio Ambiente / Clima / Geografia</t>
-        </is>
-      </c>
-      <c r="H49" s="19" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I49" s="19" t="inlineStr">
-        <is>
-          <t>Remoto</t>
-        </is>
-      </c>
-      <c r="J49" s="22" t="n">
-        <v>46265</v>
-      </c>
-      <c r="K49" s="22" t="n">
-        <v>46270</v>
-      </c>
-      <c r="L49" s="23" t="n">
-        <v>30000</v>
-      </c>
-      <c r="M49" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N49" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O49" s="24" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-memp-sebrae-2024-tr13211/</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="9" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B50" s="10" t="inlineStr">
-        <is>
-          <t>oei:ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026</t>
-        </is>
-      </c>
-      <c r="C50" s="11" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO MINC-CV-2026 – TR13230</t>
-        </is>
-      </c>
-      <c r="D50" s="11" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E50" s="12" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F50" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G50" s="11" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Estatística / Pesquisa / Metodologia, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H50" s="11" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I50" s="11" t="inlineStr">
-        <is>
-          <t>Brasília - DF</t>
-        </is>
-      </c>
-      <c r="J50" s="14" t="n">
-        <v>46275</v>
-      </c>
-      <c r="K50" s="14" t="n">
-        <v>46280</v>
-      </c>
-      <c r="L50" s="15" t="n">
-        <v>50000</v>
-      </c>
-      <c r="M50" s="9" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N50" s="12" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O50" s="16" t="inlineStr">
-        <is>
-          <t>https://oei.int/oficinas/brasil/contrataciones/ontratacao-de-consultor-na-modalidade-produto-projeto-minc-cv-2026/</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="17" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="B51" s="18" t="inlineStr">
-        <is>
-          <t>oei:contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238</t>
-        </is>
-      </c>
-      <c r="C51" s="19" t="inlineStr">
-        <is>
-          <t>Contratação de consultor na Modalidade PRODUTO PROJETO ACORDO EXEC MUSEDUCA RS – TR13238</t>
-        </is>
-      </c>
-      <c r="D51" s="19" t="inlineStr">
-        <is>
-          <t>Consultoria (tipo não especificado)</t>
-        </is>
-      </c>
-      <c r="E51" s="20" t="inlineStr">
-        <is>
-          <t>Analista Powerbi</t>
-        </is>
-      </c>
-      <c r="F51" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G51" s="19" t="inlineStr">
-        <is>
-          <t>Tecnologia da Informação / Dados, Gestão / Administração Pública</t>
-        </is>
-      </c>
-      <c r="H51" s="19" t="inlineStr">
-        <is>
-          <t>OEI</t>
-        </is>
-      </c>
-      <c r="I51" s="19" t="inlineStr">
-        <is>
-          <t>Porto Alegre - RS</t>
-        </is>
-      </c>
-      <c r="J51" s="22" t="n">
-        <v>46275</v>
-      </c>
-      <c r="K51" s="22" t="n">
-        <v>46281</v>
-      </c>
-      <c r="L51" s="23" t="n">
-        <v>180000</v>
-      </c>
-      <c r="M51" s="17" t="inlineStr">
-        <is>
-          <t>En evaluación</t>
-        </is>
-      </c>
-      <c r="N51" s="20" t="inlineStr">
-        <is>
-          <t>selecao.bra@oei.int</t>
-        </is>
-      </c>
-      <c r="O51" s="24" t="inlineStr">
-        <is>
           <t>https://oei.int/oficinas/brasil/contrataciones/contratacao-de-consultor-na-modalidade-produto-projeto-acordo-exec-museduca-rs-tr13238/</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O51"/>
+  <autoFilter ref="A1:O48"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId2"/>
@@ -4239,9 +4038,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4280,7 +4076,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3">
@@ -4290,7 +4086,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
@@ -4342,7 +4138,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3">
@@ -4404,7 +4200,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3">
@@ -4414,7 +4210,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4">
@@ -4476,7 +4272,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3">
@@ -4486,7 +4282,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -4496,7 +4292,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -4578,7 +4374,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -4598,7 +4394,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -4676,7 +4472,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -4691,7 +4487,7 @@
         </is>
       </c>
       <c r="B3" s="18" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C3" s="19" t="inlineStr">
         <is>
@@ -4706,7 +4502,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
@@ -4721,7 +4517,7 @@
         </is>
       </c>
       <c r="B5" s="18" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>

</xml_diff>